<commit_message>
Added reference to ADCS spec
</commit_message>
<xml_diff>
--- a/delegated_authorization_research.xlsx
+++ b/delegated_authorization_research.xlsx
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="6" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D11" s="7" t="n"/>
     </row>
@@ -3331,7 +3331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3530,27 +3530,27 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>AI Agents and the Multi-Hop Delegation Problem (WorkOS)</t>
+          <t>ADCS — Agent Delegation Chain Standard v1.0.0 (kahalewai)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>A WorkOS engineering blog post that catalogs the open IETF drafts and RFCs addressing multi-hop AI-agent delegation including identity chaining, attenuating tokens, and actor chains.</t>
+          <t>A vendor-neutral open specification for managing permissions across multi-agent AI workflows using cryptographic verification at each delegation hop. Core principle: scope can only narrow, never expand (monotonic restriction). Three cumulative conformance levels (core data model → JWT tokens → production infrastructure), a four-phase verification algorithm (structural, cryptographic, temporal, monotonic), seven standardized constraint types, and DID-based signing. Protocol bindings for MCP, A2A, ACP, and HTTP.</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>https://workos.com/blog/oauth-multi-hop-delegation-ai-agents</t>
+          <t>https://github.com/kahalewai/adcs/blob/main/spec/ADCS-Standard-v1.0.0.md</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Industry blog (WorkOS)</t>
+          <t>Open-source spec (Apache-2.0)</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Particularly useful index of currently-active drafts (April 2026) on the agent-delegation problem with NIST and EU AI Act compliance context.</t>
+          <t>Version 1.0.0 Public Draft for Community Review, dated 2026-04-11. Spec-only repository — no separate reference implementation. Advanced features include chain compaction, CAEP continuous revocation, multi-party quorum, and permission escalation. The monotonic-restriction guarantee is the same invariant as OVID-ME's Cedar-based subset proof and ZeroID's automatic scope attenuation — three independent approaches to the same core security property.</t>
         </is>
       </c>
     </row>
@@ -3560,27 +3560,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Mission-Bound OAuth MVP (McGuinness, 22 May 2026)</t>
+          <t>AI Agents and the Multi-Hop Delegation Problem (WorkOS)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>The protocol-level proposal. Five wire additions on top of existing OAuth: a 'mission_intent' RAR envelope (purpose, mission_expiry, context), a generic 'resource_access' RAR type, a durable Mission record at the Authorization Server, an opaque 'mission' claim (id + origin) on access tokens, and a Mission-state enforcement gate on refresh / exchange / introspection / assertion validation. Seven-state Mission lifecycle (pending_approval, active, suspended, revoked, expired, completed, rejected). proposal_hash (SHA-256 over JCS-canonical authorization_details) and consent_rendering_hash anchor what was approved versus what the user saw.</t>
+          <t>A WorkOS engineering blog post that catalogs the open IETF drafts and RFCs addressing multi-hop AI-agent delegation including identity chaining, attenuating tokens, and actor chains.</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>https://notes.karlmcguinness.com/notes/mission-bound-oauth-mvp/</t>
+          <t>https://workos.com/blog/oauth-multi-hop-delegation-ai-agents</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Architect blog (Karl McGuinness)</t>
+          <t>Industry blog (WorkOS)</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>76-min read; the substrate post for the whole series. Target I-D name: draft-mcguinness-oauth-mission-bound-minimum-profile. Conformance Ladder L0–L5 (L0 baseline OAuth → L5 verifiable governance with portable receipts). Cross-AS handoff uses ID-JAG for user-rooted flows or the Fletcher Transaction Token Chaining Profile for Txn-Token-rooted flows. Mission Expansion creates a successor Mission with 'mission.supersedes' rather than mutating in place. Three Resource Server tiers (RS-A OAuth-only → RS-D Mission-state aware via introspection or SSF/CAEP events). Architectural challenges acknowledged honestly: state-sync at scale, unknown-constraint brittleness, lethal-trifecta boundary.</t>
+          <t>Particularly useful index of currently-active drafts (April 2026) on the agent-delegation problem with NIST and EU AI Act compliance context.</t>
         </is>
       </c>
     </row>
@@ -3590,17 +3590,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>The Mission is the Missing OAuth Abstraction (McGuinness, 1 Jun 2026)</t>
+          <t>Mission-Bound OAuth MVP (McGuinness, 22 May 2026)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>The architectural frame: OAuth has no first-class object for 'the task the user approved' — only tokens, scopes, prompts, and logs that are downstream projections of it. The Mission is that durable, AS-stored, user-approved authority record. Argues this is what closes the gap that five prior bodies of his work (Power of Attorney, Mission Shaping, Open-World OAuth, Sessions Are Not Missions, the Mission-Bound architecture series) have circled from different angles. Two layers, one object: issuance-bound authority (MVP) plus runtime-enforced authority (the IBAC profile).</t>
+          <t>The protocol-level proposal. Five wire additions on top of existing OAuth: a 'mission_intent' RAR envelope (purpose, mission_expiry, context), a generic 'resource_access' RAR type, a durable Mission record at the Authorization Server, an opaque 'mission' claim (id + origin) on access tokens, and a Mission-state enforcement gate on refresh / exchange / introspection / assertion validation. Seven-state Mission lifecycle (pending_approval, active, suspended, revoked, expired, completed, rejected). proposal_hash (SHA-256 over JCS-canonical authorization_details) and consent_rendering_hash anchor what was approved versus what the user saw.</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>https://notes.karlmcguinness.com/notes/the-mission-is-the-missing-oauth-abstraction/</t>
+          <t>https://notes.karlmcguinness.com/notes/mission-bound-oauth-mvp/</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -3610,7 +3610,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Short (9-min) framing post that ties the whole programme together. The argument for why IBAC becomes practical when intent is compiled from an AS-validated Mission at consent time rather than inferred post-hoc from agent behaviour (where it's adversarial-input territory and the PDP has no user to ask). Best entry point for someone new to the series.</t>
+          <t>76-min read; the substrate post for the whole series. Target I-D name: draft-mcguinness-oauth-mission-bound-minimum-profile. Conformance Ladder L0–L5 (L0 baseline OAuth → L5 verifiable governance with portable receipts). Cross-AS handoff uses ID-JAG for user-rooted flows or the Fletcher Transaction Token Chaining Profile for Txn-Token-rooted flows. Mission Expansion creates a successor Mission with 'mission.supersedes' rather than mutating in place. Three Resource Server tiers (RS-A OAuth-only → RS-D Mission-state aware via introspection or SSF/CAEP events). Architectural challenges acknowledged honestly: state-sync at scale, unknown-constraint brittleness, lethal-trifecta boundary.</t>
         </is>
       </c>
     </row>
@@ -3620,17 +3620,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Mission-Bound OAuth Runtime Enforcement Profile (McGuinness, 1 Jun 2026)</t>
+          <t>The Mission is the Missing OAuth Abstraction (McGuinness, 1 Jun 2026)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>The IBAC layer layered on the MVP. Core (required for compliance): Intent-to-Policy Compilation (AS deterministically compiles approved authorization_details to an evaluable artifact at activation, stores policy_version on the Mission), Resource-Side Enforcement Contract (RS-B minimum, PDP evaluates every consequential request), Standard Subset Semantics per RAR Type with strict-refuse on unknown constraints (stricter than MVP's 'preserve or refuse'), Mission Introspection Profile (extended response with act chain, tenant, subject, policy_version), Runtime Denial and Escalation via ARAP (MUST), Local-Action Boundary requiring AuthZEN Access Evaluation for non-OAuth actions, Parameter Binding / TOCTOU Protection (parameter_digest bound to the permit), Decision Evidence Records (per-decision audit record bound to mission.id, proposal_hash, policy_version, decision, constraint clauses, act chain). Six Optional Modules: Tool Binding Profile, Decision Receipt Profile (W3C VC 2.0), Actor Provenance Profile, Purpose Registry Profile, Attestation Profile (RATS PTV + WIMSE), Policy Projection Profile (Cedar carriage).</t>
+          <t>The architectural frame: OAuth has no first-class object for 'the task the user approved' — only tokens, scopes, prompts, and logs that are downstream projections of it. The Mission is that durable, AS-stored, user-approved authority record. Argues this is what closes the gap that five prior bodies of his work (Power of Attorney, Mission Shaping, Open-World OAuth, Sessions Are Not Missions, the Mission-Bound architecture series) have circled from different angles. Two layers, one object: issuance-bound authority (MVP) plus runtime-enforced authority (the IBAC profile).</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>https://notes.karlmcguinness.com/notes/mission-bound-oauth-runtime-enforcement-profile/</t>
+          <t>https://notes.karlmcguinness.com/notes/the-mission-is-the-missing-oauth-abstraction/</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -3640,7 +3640,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>37-min read; target I-D name: draft-mcguinness-oauth-mission-bound-runtime-enforcement-profile. Six-class action classification (non-consequential → consequential read → consequential write → irreversible → external commitment → privileged administration) determines PDP-gate requirement and parameter binding. Four PDP deployment modes (AS-hosted, RS-hosted, tenant governance, federated). Goal pair: 'execution continuity' (every in-bounds action succeeds; every out-of-bounds becomes governed Mission Expansion) plus 'proof of authority' (per-decision cryptographic receipts). Acknowledges PDP latency overhead and tool-manifest fracturing as real challenges.</t>
+          <t>Short (9-min) framing post that ties the whole programme together. The argument for why IBAC becomes practical when intent is compiled from an AS-validated Mission at consent time rather than inferred post-hoc from agent behaviour (where it's adversarial-input territory and the PDP has no user to ask). Best entry point for someone new to the series.</t>
         </is>
       </c>
     </row>
@@ -3650,17 +3650,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Authorization Denied Is No Longer Enough (McGuinness, 2 Jun 2026)</t>
+          <t>Mission-Bound OAuth Runtime Enforcement Profile (McGuinness, 1 Jun 2026)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>The framing post for ARAP. In closed-world authorization, 'decision:false' was the end of the interaction. In open-world agentic systems with runtime discovery, sub-agent delegation, and evolving missions, denial is increasingly the beginning of a governance escalation — and the missing protocol primitive is a 'requestable denial': a deny that names where to ask and binds the request to the exact evaluation it remediates. Why CIBA isn't the answer (CIBA solves authentication freshness; this is about governance state). Why approvals aren't authority (reevaluation against current state, not standing entitlement).</t>
+          <t>The IBAC layer layered on the MVP. Core (required for compliance): Intent-to-Policy Compilation (AS deterministically compiles approved authorization_details to an evaluable artifact at activation, stores policy_version on the Mission), Resource-Side Enforcement Contract (RS-B minimum, PDP evaluates every consequential request), Standard Subset Semantics per RAR Type with strict-refuse on unknown constraints (stricter than MVP's 'preserve or refuse'), Mission Introspection Profile (extended response with act chain, tenant, subject, policy_version), Runtime Denial and Escalation via ARAP (MUST), Local-Action Boundary requiring AuthZEN Access Evaluation for non-OAuth actions, Parameter Binding / TOCTOU Protection (parameter_digest bound to the permit), Decision Evidence Records (per-decision audit record bound to mission.id, proposal_hash, policy_version, decision, constraint clauses, act chain). Six Optional Modules: Tool Binding Profile, Decision Receipt Profile (W3C VC 2.0), Actor Provenance Profile, Purpose Registry Profile, Attestation Profile (RATS PTV + WIMSE), Policy Projection Profile (Cedar carriage).</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>https://notes.karlmcguinness.com/notes/authorization-denied-is-no-longer-enough/</t>
+          <t>https://notes.karlmcguinness.com/notes/mission-bound-oauth-runtime-enforcement-profile/</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Confirms that the AuthZEN ARAP profile was adopted as a working group draft in May 2026 — material maturity signal. Useful as the 'why' read alongside the ARAP spec itself. Also positions the work against AARM (Autonomous Action Runtime Management, aarm.dev/spec) which intercepts every agent action and resolves to allow/deny/modify/step-up/defer — ARAP standardizes the deny+escalate boundary at the AuthZEN layer.</t>
+          <t>37-min read; target I-D name: draft-mcguinness-oauth-mission-bound-runtime-enforcement-profile. Six-class action classification (non-consequential → consequential read → consequential write → irreversible → external commitment → privileged administration) determines PDP-gate requirement and parameter binding. Four PDP deployment modes (AS-hosted, RS-hosted, tenant governance, federated). Goal pair: 'execution continuity' (every in-bounds action succeeds; every out-of-bounds becomes governed Mission Expansion) plus 'proof of authority' (per-decision cryptographic receipts). Acknowledges PDP latency overhead and tool-manifest fracturing as real challenges.</t>
         </is>
       </c>
     </row>
@@ -3680,17 +3680,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Re-Subjecting Is a Mint, Not an Attenuation (McGuinness, 8 Jun 2026)</t>
+          <t>Authorization Denied Is No Longer Enough (McGuinness, 2 Jun 2026)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Argues that crossing subject namespaces — mapping a user's identity from one application's identifier to another's — is a minting operation, not attenuation. Attenuation can narrow authority already represented by an existing artifact; it cannot authoritatively create a target-local identity binding the original issuer never supplied. Only a trusted IdP or broker can perform that translation. Distinguishes two topologies: caller-pushed (intermediate app returns to the IdP for a new assertion) and resource-pulled (destination resolves user identity through a broker). Separates workload identity (which service is calling) from user context (which person delegated the work) as requiring distinct claims.</t>
+          <t>The framing post for ARAP. In closed-world authorization, 'decision:false' was the end of the interaction. In open-world agentic systems with runtime discovery, sub-agent delegation, and evolving missions, denial is increasingly the beginning of a governance escalation — and the missing protocol primitive is a 'requestable denial': a deny that names where to ask and binds the request to the exact evaluation it remediates. Why CIBA isn't the answer (CIBA solves authentication freshness; this is about governance state). Why approvals aren't authority (reevaluation against current state, not standing entitlement).</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>https://notes.karlmcguinness.com/notes/re-subjecting-is-a-mint-not-an-attenuation/</t>
+          <t>https://notes.karlmcguinness.com/notes/authorization-denied-is-no-longer-enough/</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Published 8 Jun 2026; a standalone conceptual post outside the four-part Mission-Bound series but thematically continuous with it. Directly relevant to cross-AS delegation flows in the MVP post (ID-JAG for user-rooted re-subjecting) and to the token-exchange-target-service-discovery I-D. Privacy note: every intermediary-visible artifact should minimize identifiers that enable unauthorized cross-context linking.</t>
+          <t>Confirms that the AuthZEN ARAP profile was adopted as a working group draft in May 2026 — material maturity signal. Useful as the 'why' read alongside the ARAP spec itself. Also positions the work against AARM (Autonomous Action Runtime Management, aarm.dev/spec) which intercepts every agent action and resolves to allow/deny/modify/step-up/defer — ARAP standardizes the deny+escalate boundary at the AuthZEN layer.</t>
         </is>
       </c>
     </row>
@@ -3710,27 +3710,27 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Solving the Identity Crisis for AI Agents (Uber Engineering)</t>
+          <t>Re-Subjecting Is a Mint, Not an Attenuation (McGuinness, 8 Jun 2026)</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>A production engineering post from Uber describing their agent identity architecture: an Agent Registry (workload-to-agent mapping), a SPIRE-backed STS that issues short-lived JWTs with embedded actor chains at P99 below 40ms, an MCP Gateway as policy enforcement point, and an AI Agent Mesh for agent-to-agent communication. A standardized A2A client automates token exchange and chain propagation across agent hops.</t>
+          <t>Argues that crossing subject namespaces — mapping a user's identity from one application's identifier to another's — is a minting operation, not attenuation. Attenuation can narrow authority already represented by an existing artifact; it cannot authoritatively create a target-local identity binding the original issuer never supplied. Only a trusted IdP or broker can perform that translation. Distinguishes two topologies: caller-pushed (intermediate app returns to the IdP for a new assertion) and resource-pulled (destination resolves user identity through a broker). Separates workload identity (which service is calling) from user context (which person delegated the work) as requiring distinct claims.</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>https://www.uber.com/us/en/blog/solving-the-agent-identity-crisis/</t>
+          <t>https://notes.karlmcguinness.com/notes/re-subjecting-is-a-mint-not-an-attenuation/</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Industry blog (Uber Engineering)</t>
+          <t>Architect blog (Karl McGuinness)</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Published 21 May 2026; six-author post (Mathew, Borole, Huang, Burykin, Goel, Walsh) from Uber's platform engineering team. Architecture aligns with WIMSE workload identity (SPIRE as the credential foundation), RFC 8693 actor-chain propagation, and single-hop short-lived JWTs with audience-scoped claims. One of the few public disclosures of a production-grade agent identity system at hyperscaler scale — a real-world reference point for the corpus's delegation-chain design patterns.</t>
+          <t>Published 8 Jun 2026; a standalone conceptual post outside the four-part Mission-Bound series but thematically continuous with it. Directly relevant to cross-AS delegation flows in the MVP post (ID-JAG for user-rooted re-subjecting) and to the token-exchange-target-service-discovery I-D. Privacy note: every intermediary-visible artifact should minimize identifiers that enable unauthorized cross-context linking.</t>
         </is>
       </c>
     </row>
@@ -3740,27 +3740,27 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Agents Are Not Just Workloads (Patrick Parker, LinkedIn)</t>
+          <t>Solving the Identity Crisis for AI Agents (Uber Engineering)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Argues that classifying AI agents as 'workloads' is a category error that corrupts identity architecture: workloads are a what-runs-where concept, agents are a who-acts-on-whose-authority concept. Identifies five breakdown areas where workload-identity patterns fail for agents: intent captured as static token claims, delegation gaps (no purpose binding or revocation paths), overlooked tool-catalog authorization surface, bearer-credential custody ambiguity under prompt injection, and mutable logs insufficient as tamper-evident authorization evidence.</t>
+          <t>A production engineering post from Uber describing their agent identity architecture: an Agent Registry (workload-to-agent mapping), a SPIRE-backed STS that issues short-lived JWTs with embedded actor chains at P99 below 40ms, an MCP Gateway as policy enforcement point, and an AI Agent Mesh for agent-to-agent communication. A standardized A2A client automates token exchange and chain propagation across agent hops.</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/pulse/agents-just-workloads-patrick-parker-0qxte/</t>
+          <t>https://www.uber.com/us/en/blog/solving-the-agent-identity-crisis/</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Industry blog (LinkedIn)</t>
+          <t>Industry blog (Uber Engineering)</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Published 9 Jun 2026. Proposes signature-based receipts binding relationships, authority, tasks, and bounds; runtime validation of generated task intent; and AuthZEN gateway-based enforcement. A principled counterpoint to the WIMSE-as-sufficient-for-agents framing — pairs well with the Uber Engineering post (which uses SPIRE/WIMSE as the credential foundation but adds actor chains and MCP gateway enforcement on top).</t>
+          <t>Published 21 May 2026; six-author post (Mathew, Borole, Huang, Burykin, Goel, Walsh) from Uber's platform engineering team. Architecture aligns with WIMSE workload identity (SPIRE as the credential foundation), RFC 8693 actor-chain propagation, and single-hop short-lived JWTs with audience-scoped claims. One of the few public disclosures of a production-grade agent identity system at hyperscaler scale — a real-world reference point for the corpus's delegation-chain design patterns.</t>
         </is>
       </c>
     </row>
@@ -3770,27 +3770,27 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>AI Agent Authentication Gets the Hard Part Right. Authorization Is Still Your Problem. (Rock Cyber Musings)</t>
+          <t>Agents Are Not Just Workloads (Patrick Parker, LinkedIn)</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>An analyst article arguing the new IETF agent-auth draft solves authentication via SPIFFE+WIMSE+OAuth but leaves authorization and policy enforcement as an unsolved open problem.</t>
+          <t>Argues that classifying AI agents as 'workloads' is a category error that corrupts identity architecture: workloads are a what-runs-where concept, agents are a who-acts-on-whose-authority concept. Identifies five breakdown areas where workload-identity patterns fail for agents: intent captured as static token claims, delegation gaps (no purpose binding or revocation paths), overlooked tool-catalog authorization surface, bearer-credential custody ambiguity under prompt injection, and mutable logs insufficient as tamper-evident authorization evidence.</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>https://www.rockcybermusings.com/p/i-agent-authentication-authorization-gap</t>
+          <t>https://www.linkedin.com/pulse/agents-just-workloads-patrick-parker-0qxte/</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Industry analysis blog</t>
+          <t>Industry blog (LinkedIn)</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Maps the IETF draft against MCP and the Colorado AI Act 'reasonable care' standard; pragmatic implementer perspective.</t>
+          <t>Published 9 Jun 2026. Proposes signature-based receipts binding relationships, authority, tasks, and bounds; runtime validation of generated task intent; and AuthZEN gateway-based enforcement. A principled counterpoint to the WIMSE-as-sufficient-for-agents framing — pairs well with the Uber Engineering post (which uses SPIRE/WIMSE as the credential foundation but adds actor chains and MCP gateway enforcement on top).</t>
         </is>
       </c>
     </row>
@@ -3800,27 +3800,27 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Agent Authentication &amp; Delegated Access (Zylos Research, April 2026)</t>
+          <t>AI Agent Authentication Gets the Hard Part Right. Authorization Is Still Your Problem. (Rock Cyber Musings)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>A research-style industry article surveying OAuth flows, scoped tokens, and identity patterns specifically for AI agents, covering OAuth 2.1 baselines and chain-splicing risks.</t>
+          <t>An analyst article arguing the new IETF agent-auth draft solves authentication via SPIFFE+WIMSE+OAuth but leaves authorization and policy enforcement as an unsolved open problem.</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>https://zylos.ai/research/2026-04-11-agent-authentication-delegated-access-oauth-scoped-tokens</t>
+          <t>https://www.rockcybermusings.com/p/i-agent-authentication-authorization-gap</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Industry research blog</t>
+          <t>Industry analysis blog</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Documents the 'delegation chain splicing' attack against RFC 8693 actor-token chains formally raised on the OAuth WG list in early 2026.</t>
+          <t>Maps the IETF draft against MCP and the Colorado AI Act 'reasonable care' standard; pragmatic implementer perspective.</t>
         </is>
       </c>
     </row>
@@ -3830,27 +3830,27 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>AuthZEN + Shared Signals Framework Series (Andrew Doering)</t>
+          <t>Agent Authentication &amp; Delegated Access (Zylos Research, April 2026)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>A multi-part technical blog walking through how AuthZEN (synchronous PDP/PEP) and SSF/CAEP (asynchronous events) combine into a continuous-authorization loop in real Microsoft Entra/M365 deployments.</t>
+          <t>A research-style industry article surveying OAuth flows, scoped tokens, and identity patterns specifically for AI agents, covering OAuth 2.1 baselines and chain-splicing risks.</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>https://andrewdoering.org/blog/2026/authzen-shared-signals-framework-part-1-fundamentals/</t>
+          <t>https://zylos.ai/research/2026-04-11-agent-authentication-delegated-access-oauth-scoped-tokens</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Industry blog</t>
+          <t>Industry research blog</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Documents the 2026 asymmetry where Microsoft Entra is a CAEP transmitter for closed-loop CAE but not an external SSF receiver.</t>
+          <t>Documents the 'delegation chain splicing' attack against RFC 8693 actor-token chains formally raised on the OAuth WG list in early 2026.</t>
         </is>
       </c>
     </row>
@@ -3860,27 +3860,27 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Just-in-Time Authorization with OpenID SSE and CAEP (The New Stack, Tulshibagwale)</t>
+          <t>AuthZEN + Shared Signals Framework Series (Andrew Doering)</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>An article from CAEP's original inventor explaining how SSE+CAEP enable just-in-time authorization decisions instead of long-lived session-based access.</t>
+          <t>A multi-part technical blog walking through how AuthZEN (synchronous PDP/PEP) and SSF/CAEP (asynchronous events) combine into a continuous-authorization loop in real Microsoft Entra/M365 deployments.</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>https://thenewstack.io/just-in-time-authorization-with-openid-sse-and-caep/</t>
+          <t>https://andrewdoering.org/blog/2026/authzen-shared-signals-framework-part-1-fundamentals/</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Industry article (The New Stack)</t>
+          <t>Industry blog</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Background piece by Atul Tulshibagwale (SGNL CTO, CAEP inventor) explaining the architectural intent.</t>
+          <t>Documents the 2026 asymmetry where Microsoft Entra is a CAEP transmitter for closed-loop CAE but not an external SSF receiver.</t>
         </is>
       </c>
     </row>
@@ -3890,27 +3890,27 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>How AuthZEN, Shared Signals &amp; CAEP Complement Each Other (OpenID Foundation)</t>
+          <t>Just-in-Time Authorization with OpenID SSE and CAEP (The New Stack, Tulshibagwale)</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>An OpenID Foundation explainer arguing that AuthZEN and SSF/CAEP are complementary — sync access decisions vs async session updates — not competing standards.</t>
+          <t>An article from CAEP's original inventor explaining how SSE+CAEP enable just-in-time authorization decisions instead of long-lived session-based access.</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>https://openid.net/how-authzen-and-shared-signals-caep-complement-each-other/</t>
+          <t>https://thenewstack.io/just-in-time-authorization-with-openid-sse-and-caep/</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>OpenID Foundation</t>
+          <t>Industry article (The New Stack)</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Useful when explaining the layering to stakeholders confused by the OpenID alphabet soup.</t>
+          <t>Background piece by Atul Tulshibagwale (SGNL CTO, CAEP inventor) explaining the architectural intent.</t>
         </is>
       </c>
     </row>
@@ -3920,27 +3920,27 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>OAuth 2.1 Features You Can't Ignore in 2026 (Gutierrez, Medium)</t>
+          <t>How AuthZEN, Shared Signals &amp; CAEP Complement Each Other (OpenID Foundation)</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>A practitioner article summarizing why OAuth 2.1 — mandated PKCE, exact redirect matching, sender-constrained tokens — is the 2026 minimum bar for delegated authorization.</t>
+          <t>An OpenID Foundation explainer arguing that AuthZEN and SSF/CAEP are complementary — sync access decisions vs async session updates — not competing standards.</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>https://rgutierrez2004.medium.com/oauth-2-1-features-you-cant-ignore-in-2026-a15f852cb723</t>
+          <t>https://openid.net/how-authzen-and-shared-signals-caep-complement-each-other/</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Industry blog (Medium)</t>
+          <t>OpenID Foundation</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Author is Cyber Intelligence Lead — IAM/AI at Oracle; concise piece suitable for executive briefings.</t>
+          <t>Useful when explaining the layering to stakeholders confused by the OpenID alphabet soup.</t>
         </is>
       </c>
     </row>
@@ -3950,27 +3950,27 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>RFC 9396: OAuth 2.0 Rich Authorization Requests (CIAM Weekly)</t>
+          <t>OAuth 2.1 Features You Can't Ignore in 2026 (Gutierrez, Medium)</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>A practitioner deep-dive on RAR explaining why scopes alone don't carry transaction-level intent and how authorization_details is being adopted in payments and verifiable credentials.</t>
+          <t>A practitioner article summarizing why OAuth 2.1 — mandated PKCE, exact redirect matching, sender-constrained tokens — is the 2026 minimum bar for delegated authorization.</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>https://ciamweekly.substack.com/p/rfc-9396-oauth-20-rich-authorization</t>
+          <t>https://rgutierrez2004.medium.com/oauth-2-1-features-you-cant-ignore-in-2026-a15f852cb723</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Industry newsletter</t>
+          <t>Industry blog (Medium)</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Captures the current (March 2026) state of RAR adoption, including CAMARA telco APIs and DPV-purpose binding proposals.</t>
+          <t>Author is Cyber Intelligence Lead — IAM/AI at Oracle; concise piece suitable for executive briefings.</t>
         </is>
       </c>
     </row>
@@ -3980,27 +3980,27 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Technical Deconstruction of MCP Authorization (kane.mx, Nov 2025)</t>
+          <t>RFC 9396: OAuth 2.0 Rich Authorization Requests (CIAM Weekly)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>A long-form technical article showing that the Model Context Protocol's authorization spec is, in practice, an OAuth 2.1 profile combined with RFC 9728 protected-resource metadata and RFC 7591 dynamic registration.</t>
+          <t>A practitioner deep-dive on RAR explaining why scopes alone don't carry transaction-level intent and how authorization_details is being adopted in payments and verifiable credentials.</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>https://kane.mx/posts/2025/mcp-authorization-oauth-rfc-deep-dive/</t>
+          <t>https://ciamweekly.substack.com/p/rfc-9396-oauth-20-rich-authorization</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Independent technical blog</t>
+          <t>Industry newsletter</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Calls out RFC 8707 (Resource Indicators) as the critical compatibility bottleneck since most major IdPs use proprietary audience parameters.</t>
+          <t>Captures the current (March 2026) state of RAR adoption, including CAMARA telco APIs and DPV-purpose binding proposals.</t>
         </is>
       </c>
     </row>
@@ -4010,27 +4010,27 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>AI Agents Authentication: How Autonomous Systems Prove Identity (GitGuardian)</t>
+          <t>Technical Deconstruction of MCP Authorization (kane.mx, Nov 2025)</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>A GitGuardian engineering article arguing that delegated, short-lived OAuth grants are structurally safer than the static API keys that produced 28.65M secret leaks in 2025.</t>
+          <t>A long-form technical article showing that the Model Context Protocol's authorization spec is, in practice, an OAuth 2.1 profile combined with RFC 9728 protected-resource metadata and RFC 7591 dynamic registration.</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>https://blog.gitguardian.com/ai-agents-authentication-how-autonomous-systems-prove-identity/</t>
+          <t>https://kane.mx/posts/2025/mcp-authorization-oauth-rfc-deep-dive/</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Industry blog (GitGuardian)</t>
+          <t>Independent technical blog</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Useful for the 'why delegated authorization &gt; shared secrets' business case with concrete 2025 incident data.</t>
+          <t>Calls out RFC 8707 (Resource Indicators) as the critical compatibility bottleneck since most major IdPs use proprietary audience parameters.</t>
         </is>
       </c>
     </row>
@@ -4040,27 +4040,27 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Workload Identity – Key Takeaways from IETF 122 (Defakto)</t>
+          <t>AI Agents Authentication: How Autonomous Systems Prove Identity (GitGuardian)</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>A practitioner recap of IETF 122 covering the WIMSE Workload Identity Token, Credential Exchange, and side-meeting work on bot/agent web authentication.</t>
+          <t>A GitGuardian engineering article arguing that delegated, short-lived OAuth grants are structurally safer than the static API keys that produced 28.65M secret leaks in 2025.</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>https://www.defakto.security/blog/workload-identity-key-takeaways-from-ietf-122/</t>
+          <t>https://blog.gitguardian.com/ai-agents-authentication-how-autonomous-systems-prove-identity/</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Industry blog (Defakto)</t>
+          <t>Industry blog (GitGuardian)</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Author Pieter Kasselman is co-author of multiple key drafts (Transaction Tokens, First-Party Apps); strong primary-source view.</t>
+          <t>Useful for the 'why delegated authorization &gt; shared secrets' business case with concrete 2025 incident data.</t>
         </is>
       </c>
     </row>
@@ -4070,27 +4070,27 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>User-Managed Access (UMA) 2.0 Comprehensive Guide (SSOJet, Feb 2026)</t>
+          <t>Workload Identity – Key Takeaways from IETF 122 (Defakto)</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>A 2026 industry guide reframing UMA 2.0 for current CIAM contexts, covering resource-set registration, permission tickets, requesting-party tokens (RPTs), and policy externalization gains.</t>
+          <t>A practitioner recap of IETF 122 covering the WIMSE Workload Identity Token, Credential Exchange, and side-meeting work on bot/agent web authentication.</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>https://ssojet.com/blog/user-managed-access-uma-2-0-comprehensive-guide</t>
+          <t>https://www.defakto.security/blog/workload-identity-key-takeaways-from-ietf-122/</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Industry blog (SSOJet)</t>
+          <t>Industry blog (Defakto)</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Cites Kantara analysis showing centralized-policy moves can cut authorization code 80% — useful pitch material.</t>
+          <t>Author Pieter Kasselman is co-author of multiple key drafts (Transaction Tokens, First-Party Apps); strong primary-source view.</t>
         </is>
       </c>
     </row>
@@ -4100,27 +4100,27 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Decentralized Identity and Verifiable Credentials: The Enterprise Playbook 2026</t>
+          <t>User-Managed Access (UMA) 2.0 Comprehensive Guide (SSOJet, Feb 2026)</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>An enterprise-oriented guide explaining how W3C VCs, DIDs, and OpenID4VC enable the issuer-holder-verifier delegation model for digital credentials and EUDI Wallet acceptance.</t>
+          <t>A 2026 industry guide reframing UMA 2.0 for current CIAM contexts, covering resource-set registration, permission tickets, requesting-party tokens (RPTs), and policy externalization gains.</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>https://securityboulevard.com/2026/03/decentralized-identity-and-verifiable-credentials-the-enterprise-playbook-2026/</t>
+          <t>https://ssojet.com/blog/user-managed-access-uma-2-0-comprehensive-guide</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Industry article (Security Boulevard)</t>
+          <t>Industry blog (SSOJet)</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Critical 2027 EU compliance dates: banks, telecom, healthcare, and very-large platforms must accept EUDI Wallet.</t>
+          <t>Cites Kantara analysis showing centralized-policy moves can cut authorization code 80% — useful pitch material.</t>
         </is>
       </c>
     </row>
@@ -4130,27 +4130,27 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>OAuth 2.0 &amp; OpenID Connect: The Complete Guide to What the Standards Actually Say (Patil, Medium)</t>
+          <t>Decentralized Identity and Verifiable Credentials: The Enterprise Playbook 2026</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>A practitioner-friendly synthesis covering OAuth 2.0 core, the OAuth 2.1 draft, RFC 9068 JWT access tokens, RFC 8252 native apps, and RFC 8628 device authorization.</t>
+          <t>An enterprise-oriented guide explaining how W3C VCs, DIDs, and OpenID4VC enable the issuer-holder-verifier delegation model for digital credentials and EUDI Wallet acceptance.</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>https://mrutyunjaypatil.medium.com/oauth-2-0-openid-connect-the-complete-guide-to-what-the-standards-actually-say-e92f040a4251</t>
+          <t>https://securityboulevard.com/2026/03/decentralized-identity-and-verifiable-credentials-the-enterprise-playbook-2026/</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Industry blog (Medium)</t>
+          <t>Industry article (Security Boulevard)</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Good handoff document for engineers new to the area; cites the current standards rather than legacy patterns.</t>
+          <t>Critical 2027 EU compliance dates: banks, telecom, healthcare, and very-large platforms must accept EUDI Wallet.</t>
         </is>
       </c>
     </row>
@@ -4160,27 +4160,27 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>LinkedIn Engineering — OpenID Connect Authentication for Sign In with LinkedIn V2</t>
+          <t>OAuth 2.0 &amp; OpenID Connect: The Complete Guide to What the Standards Actually Say (Patil, Medium)</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>LinkedIn's own engineering write-up on adopting OpenID Connect on top of OAuth 2.0, explicitly distinguishing OAuth's delegated-access role from OIDC's identity-assertion role.</t>
+          <t>A practitioner-friendly synthesis covering OAuth 2.0 core, the OAuth 2.1 draft, RFC 9068 JWT access tokens, RFC 8252 native apps, and RFC 8628 device authorization.</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/developers/news/featured-updates/openid-connect-authentication</t>
+          <t>https://mrutyunjaypatil.medium.com/oauth-2-0-openid-connect-the-complete-guide-to-what-the-standards-actually-say-e92f040a4251</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Industry (LinkedIn Engineering)</t>
+          <t>Industry blog (Medium)</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Real-world example from LinkedIn explaining why they layered OIDC over an existing OAuth 2.0 delegated-access stack.</t>
+          <t>Good handoff document for engineers new to the area; cites the current standards rather than legacy patterns.</t>
         </is>
       </c>
     </row>
@@ -4190,27 +4190,27 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Rich Authorization Requests (RAR) — Authlete Knowledge Base</t>
+          <t>LinkedIn Engineering — OpenID Connect Authentication for Sign In with LinkedIn V2</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>A vendor knowledge-base article giving worked examples of RAR's authorization_details object, including locations, actions, datatypes, and identifier fields with their Authlete bindings.</t>
+          <t>LinkedIn's own engineering write-up on adopting OpenID Connect on top of OAuth 2.0, explicitly distinguishing OAuth's delegated-access role from OIDC's identity-assertion role.</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>https://www.authlete.com/kb/oauth-and-openid-connect/authorization-requests/rich-authorization-requests/</t>
+          <t>https://www.linkedin.com/developers/news/featured-updates/openid-connect-authentication</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Vendor documentation (Authlete)</t>
+          <t>Industry (LinkedIn Engineering)</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Authlete is one of the few certified FAPI 2.0 + RAR implementations; useful reference for concrete request bodies.</t>
+          <t>Real-world example from LinkedIn explaining why they layered OIDC over an existing OAuth 2.0 delegated-access stack.</t>
         </is>
       </c>
     </row>
@@ -4220,25 +4220,55 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
+          <t>Rich Authorization Requests (RAR) — Authlete Knowledge Base</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>A vendor knowledge-base article giving worked examples of RAR's authorization_details object, including locations, actions, datatypes, and identifier fields with their Authlete bindings.</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>https://www.authlete.com/kb/oauth-and-openid-connect/authorization-requests/rich-authorization-requests/</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Vendor documentation (Authlete)</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Authlete is one of the few certified FAPI 2.0 + RAR implementations; useful reference for concrete request bodies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
           <t>An Introduction to Authorization Exchange (AuthZEN) — Curity</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>A vendor explainer comparing externalized-authorization patterns (OPA, Cedar, XACML, Zanzibar) and showing how AuthZEN's API normalizes the PDP/PEP wire protocol across them.</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="D31" s="9" t="inlineStr">
         <is>
           <t>https://curity.io/resources/learn/authzen/</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>Vendor blog (Curity)</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>Curity is a member of the AuthZEN WG; positions AuthZEN as 'OpenID Connect for authorization' which has become the common framing.</t>
         </is>
@@ -4275,6 +4305,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added draft-hood-independent-agtp (AGTP) to transport cluster
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/delegated_authorization_research.xlsx
+++ b/delegated_authorization_research.xlsx
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="6" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D11" s="7" t="n"/>
     </row>
@@ -906,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2065,17 +2065,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>draft-ni-a2a-ai-agent-security-requirements — Security Requirements for AI Agents</t>
+          <t>draft-hood-independent-agtp — Agent Transfer Protocol (AGTP)</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft enumerating security requirements for AI agents, covering identity, authorization chaining across domains, and integration points with WIMSE, OAuth identity chaining, and the A2A OAuth profile.</t>
+          <t>An IETF individual draft proposing a dedicated application-layer protocol for AI agent traffic on port 4480 (TCP/TLS and QUIC) with an agtp:// URI scheme, arguing that HTTP is insufficient because agent-generated intent-driven traffic is indistinguishable from human-initiated requests. Defines a Runtime Contract Negotiation Substrate (RCNS) with eighteen methods split into cognitive verbs (QUERY, DISCOVER, DESCRIBE, SUMMARIZE, PLAN, PROPOSE) and mechanics verbs (EXECUTE, DELEGATE, ESCALATE, CONFIRM, SUSPEND, NOTIFY), mandatory agent identity headers, and protocol-level authority scope declaration.</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ni-a2a-ai-agent-security-requirements/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-independent-agtp/</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, February 2026; essential scaffolding for an eventual AI-agent WG. Well-connected to existing IETF work and authored by Ni and Liu, who also lead the WIMSE AI-agent identity draft.</t>
+          <t>Revision -08 (26 May 2026); supersedes draft-hood-independent-atp. Companion specs in the same family: AGTP-API, AGTP-CERT, AGTP-MERCHANT, AGTP-IDENTIFIERS, AGTP-TRUST. Mandatory TLS 1.3+. Ambitious scope — a new transport layer rather than an HTTP profile. The cognitive/mechanics verb split is a distinctive design choice; contrasts with draft-sharif-agent-transport-protocol which layers async store-and-forward on top of existing transports rather than replacing them.</t>
         </is>
       </c>
     </row>
@@ -2095,17 +2095,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>draft-rosenberg-aiproto-framework — Framework, Use Cases and Requirements for AI Agent Protocols</t>
+          <t>draft-ni-a2a-ai-agent-security-requirements — Security Requirements for AI Agents</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft providing a comprehensive AI-agent communications framework that covers user↔agent, agent↔API, and agent↔agent interactions; surveys MCP, A2A, and Agntcy; and sets the stage for IETF standards activity.</t>
+          <t>An IETF individual draft enumerating security requirements for AI agents, covering identity, authorization chaining across domains, and integration points with WIMSE, OAuth identity chaining, and the A2A OAuth profile.</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-framework/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ni-a2a-ai-agent-security-requirements/</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, October 2025; Rosenberg (Five9) and Jennings (Cisco) are credible long-time IETF contributors. Important landscape document but likely expired (April 2026); watch for a -01 refresh post-IETF 123.</t>
+          <t>Revision -01, February 2026; essential scaffolding for an eventual AI-agent WG. Well-connected to existing IETF work and authored by Ni and Liu, who also lead the WIMSE AI-agent identity draft.</t>
         </is>
       </c>
     </row>
@@ -2125,17 +2125,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>draft-rosenberg-aiproto-cheq — CHEQ: A Protocol for Confirmation of AI Agent Decisions (HITL)</t>
+          <t>draft-rosenberg-aiproto-framework — Framework, Use Cases and Requirements for AI Agent Protocols</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an out-of-band Human-in-the-Loop confirmation protocol for agent tool calls, eliminating LLM-hallucination risk for consequential actions and enabling sensitive operations (e.g., banking) without exposing data to the agent.</t>
+          <t>An IETF individual draft providing a comprehensive AI-agent communications framework that covers user↔agent, agent↔API, and agent↔agent interactions; surveys MCP, A2A, and Agntcy; and sets the stage for IETF standards activity.</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-cheq/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-framework/</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, October 2025; out-of-band HITL confirmation model is valuable and complements delegation frameworks. Likely expired (April 2026); worth tracking for a -01 refresh.</t>
+          <t>Revision -00, October 2025; Rosenberg (Five9) and Jennings (Cisco) are credible long-time IETF contributors. Important landscape document but likely expired (April 2026); watch for a -01 refresh post-IETF 123.</t>
         </is>
       </c>
     </row>
@@ -2155,27 +2155,27 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-payment-trust — Trust Scoring and Identity Verification for AI Agent Payment Transactions (SUPERSEDED)</t>
+          <t>draft-rosenberg-aiproto-cheq — CHEQ: A Protocol for Confirmation of AI Agent Decisions (HITL)</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft introducing an Agent Passport — a cryptographic delegation certificate intended to serve as the PSD2 'something you have' factor — and a trust-scoring model for payment transactions mapped to PCI DSS v4.0.1.</t>
+          <t>An IETF individual draft defining an out-of-band Human-in-the-Loop confirmation protocol for agent tool calls, eliminating LLM-hallucination risk for consequential actions and enabling sensitive operations (e.g., banking) without exposing data to the agent.</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-payment-trust/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-cheq/</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual, superseded)</t>
+          <t>IETF (individual)</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>SUPERSEDED by draft-sharif-attp-00 (April 2026). Retained for historical context — the Agent Passport concept is interesting but needs formal grounding; the ATTP successor generalizes it across transport bindings.</t>
+          <t>Revision -00, October 2025; out-of-band HITL confirmation model is valuable and complements delegation frameworks. Likely expired (April 2026); worth tracking for a -01 refresh.</t>
         </is>
       </c>
     </row>
@@ -2185,27 +2185,27 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>draft-stephan-ai-agent-6g — AI Agent Protocols for 6G Systems</t>
+          <t>draft-sharif-agent-payment-trust — Trust Scoring and Identity Verification for AI Agent Payment Transactions (SUPERSEDED)</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft translating use cases and service requirements from 3GPP TR 22.870 into IETF agent-protocol requirements, covering autonomous vehicles, privacy preservation, and anomaly detection.</t>
+          <t>An IETF individual draft introducing an Agent Passport — a cryptographic delegation certificate intended to serve as the PSD2 'something you have' factor — and a trust-scoring model for payment transactions mapped to PCI DSS v4.0.1.</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-stephan-ai-agent-6g/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-payment-trust/</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (individual, superseded)</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, October 2025; strong operator backing (Orange, Deutsche Telekom, Telefonica, China Mobile, Huawei). Requirements-oriented and important for 3GPP/IETF coordination. May be expired (April 2026); watch for an update.</t>
+          <t>SUPERSEDED by draft-sharif-attp-00 (April 2026). Retained for historical context — the Agent Passport concept is interesting but needs formal grounding; the ATTP successor generalizes it across transport bindings.</t>
         </is>
       </c>
     </row>
@@ -2215,17 +2215,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>draft-jimenez-t2trg-iot-agent — Agentic AI Operation of Constrained RESTful Environments</t>
+          <t>draft-stephan-ai-agent-6g — AI Agent Protocols for 6G Systems</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft (T2TRG affiliated) describing agentic AI (ReAct, smolagents) operating on CoAP/CoRE constrained-IoT environments, with a reference implementation provided.</t>
+          <t>An IETF individual draft translating use cases and service requirements from 3GPP TR 22.870 into IETF agent-protocol requirements, covering autonomous vehicles, privacy preservation, and anomaly detection.</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jimenez-t2trg-iot-agent/</t>
+          <t>https://datatracker.ietf.org/doc/draft-stephan-ai-agent-6g/</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 14 April 2026; unique in targeting constrained IoT environments. T2TRG affiliation and reference implementation are positive signals. Niche but fills an unaddressed gap.</t>
+          <t>Revision -02, October 2025; strong operator backing (Orange, Deutsche Telekom, Telefonica, China Mobile, Huawei). Requirements-oriented and important for 3GPP/IETF coordination. May be expired (April 2026); watch for an update.</t>
         </is>
       </c>
     </row>
@@ -2245,17 +2245,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>draft-li-oauth-delegated-authorization — OAuth 2.0 Delegated Authorization</t>
+          <t>draft-jimenez-t2trg-iot-agent — Agentic AI Operation of Constrained RESTful Environments</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Huawei authors that extends OAuth 2.0 with a hierarchical 'delegation token' model so a client can mint subordinate, narrowly-scoped access tokens for delegated parties.</t>
+          <t>An IETF individual draft (T2TRG affiliated) describing agentic AI (ReAct, smolagents) operating on CoAP/CoRE constrained-IoT environments, with a reference implementation provided.</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-li-oauth-delegated-authorization/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jimenez-t2trg-iot-agent/</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, March 2026 (Informational); directly addresses over-privileged tokens and is one of the few drafts using the literal term 'delegated authorization'.</t>
+          <t>Revision -00, 14 April 2026; unique in targeting constrained IoT environments. T2TRG affiliation and reference implementation are positive signals. Niche but fills an unaddressed gap.</t>
         </is>
       </c>
     </row>
@@ -2275,17 +2275,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>draft-araut-oauth-transaction-tokens-for-agents — Transaction Tokens For Agents</t>
+          <t>draft-li-oauth-delegated-authorization — OAuth 2.0 Delegated Authorization</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Ashay Raut (Amazon) profiling Transaction Tokens for agent-based workflows by adding 'act' for the agent identity, an 'agentic_ctx' claim carrying agent_type/intent/allowed_actions/environment_constraints, RFC 9396 RAR integration, and an 'actchain' claim for multi-agent delegation lineage.</t>
+          <t>An IETF individual draft from Huawei authors that extends OAuth 2.0 with a hierarchical 'delegation token' model so a client can mint subordinate, narrowly-scoped access tokens for delegated parties.</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-araut-oauth-transaction-tokens-for-agents/</t>
+          <t>https://datatracker.ietf.org/doc/draft-li-oauth-delegated-authorization/</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Revision -01 (May 2026) under the new slug — re-slugged from draft-oauth-transaction-tokens-for-agents-06; the -06 added the actchain delegation lineage, RAR-driven agentic_ctx, and a TTS check that blocks chain-splicing attacks. Conservative extension of the WG Transaction Tokens draft and an easier path to standardization.</t>
+          <t>Revision -01, March 2026 (Informational); directly addresses over-privileged tokens and is one of the few drafts using the literal term 'delegated authorization'.</t>
         </is>
       </c>
     </row>
@@ -2305,17 +2305,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>draft-oauth-ai-agents-on-behalf-of-user — On-Behalf-Of User Authorization for AI Agents</t>
+          <t>draft-araut-oauth-transaction-tokens-for-agents — Transaction Tokens For Agents</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft adding requested_actor and actor_token parameters to the OAuth authorization-code flow so the user gives explicit consent per agent, with the resulting delegation chain documented in the access-token claims.</t>
+          <t>An IETF individual draft from Ashay Raut (Amazon) profiling Transaction Tokens for agent-based workflows by adding 'act' for the agent identity, an 'agentic_ctx' claim carrying agent_type/intent/allowed_actions/environment_constraints, RFC 9396 RAR integration, and an 'actchain' claim for multi-agent delegation lineage.</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-oauth-ai-agents-on-behalf-of-user/</t>
+          <t>https://datatracker.ietf.org/doc/draft-araut-oauth-transaction-tokens-for-agents/</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Revision -02 was submitted August 2025; likely due for -03 refresh. Builds naturally on RFC 6749 + RFC 8693 + RFC 7636 PKCE — one of the most 'IETF-ready' delegation drafts and a strong WG-adoption candidate after the OAuth recharter.</t>
+          <t>Revision -01 (May 2026) under the new slug — re-slugged from draft-oauth-transaction-tokens-for-agents-06; the -06 added the actchain delegation lineage, RAR-driven agentic_ctx, and a TTS check that blocks chain-splicing attacks. Conservative extension of the WG Transaction Tokens draft and an easier path to standardization.</t>
         </is>
       </c>
     </row>
@@ -2335,17 +2335,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>draft-hardt-aauth-protocol — AAuth Protocol</t>
+          <t>draft-oauth-ai-agents-on-behalf-of-user — On-Behalf-Of User Authorization for AI Agents</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>A new clean-sheet authorization protocol from Dick Hardt (original OAuth author) defining proof-of-possession by default, resource-signed challenges, agent identity without pre-registration, deferred 202 responses, and AS-to-AS federation for the agent ecosystem.</t>
+          <t>An IETF individual draft adding requested_actor and actor_token parameters to the OAuth authorization-code flow so the user gives explicit consent per agent, with the resulting delegation chain documented in the access-token claims.</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hardt-aauth-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-oauth-ai-agents-on-behalf-of-user/</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, April 2026; the design rationale section explicitly explains why AAuth is not GNAP, not OAuth, not DPoP and not mTLS — important read for anyone planning a new agent-auth stack.</t>
+          <t>Revision -02 was submitted August 2025; likely due for -03 refresh. Builds naturally on RFC 6749 + RFC 8693 + RFC 7636 PKCE — one of the most 'IETF-ready' delegation drafts and a strong WG-adoption candidate after the OAuth recharter.</t>
         </is>
       </c>
     </row>
@@ -2365,17 +2365,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>draft-chen-oauth-roadmap — Comprehensive Roadmap for OAuth 2.0 Standards and Drafts</t>
+          <t>draft-hardt-aauth-protocol — AAuth Protocol</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>An IETF informational draft that maps the entire OAuth 2.0 ecosystem of RFCs, BCPs, and active drafts into functional layers from core to extensions to industry profiles.</t>
+          <t>A new clean-sheet authorization protocol from Dick Hardt (original OAuth author) defining proof-of-possession by default, resource-signed challenges, agent identity without pre-registration, deferred 202 responses, and AS-to-AS federation for the agent ecosystem.</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>https://www.ietf.org/archive/id/draft-chen-oauth-roadmap-00.html</t>
+          <t>https://datatracker.ietf.org/doc/draft-hardt-aauth-protocol/</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Brand-new -00 draft (May 2026); the single most useful index when starting work in this area.</t>
+          <t>Revision -00, April 2026; the design rationale section explicitly explains why AAuth is not GNAP, not OAuth, not DPoP and not mTLS — important read for anyone planning a new agent-auth stack.</t>
         </is>
       </c>
     </row>
@@ -2395,25 +2395,55 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
+          <t>draft-chen-oauth-roadmap — Comprehensive Roadmap for OAuth 2.0 Standards and Drafts</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>An IETF informational draft that maps the entire OAuth 2.0 ecosystem of RFCs, BCPs, and active drafts into functional layers from core to extensions to industry profiles.</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ietf.org/archive/id/draft-chen-oauth-roadmap-00.html</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Brand-new -00 draft (May 2026); the single most useful index when starting work in this area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
           <t>Charter: WIMSE — Workload Identity in Multi-System Environments (charter-ietf-wimse-01)</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>The formal IETF charter for the WIMSE WG covering architecture, JOSE-based WIMSE tokens for service-to-service traffic, local token issuance, and token exchange profiles (likely based on RFC 8693) for cross-trust-domain workload identity.</t>
         </is>
       </c>
-      <c r="D50" s="9" t="inlineStr">
+      <c r="D51" s="9" t="inlineStr">
         <is>
           <t>https://datatracker.ietf.org/doc/charter-ietf-wimse/01/</t>
         </is>
       </c>
-      <c r="E50" s="5" t="inlineStr">
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>IETF (WIMSE WG charter)</t>
         </is>
       </c>
-      <c r="F50" s="5" t="inlineStr">
+      <c r="F51" s="5" t="inlineStr">
         <is>
           <t>Approved 18 March 2026 (v01); explicitly liaises with OAuth, SCIM, SCITT, RATS, the OpenID Foundation, and CNCF/SPIFFE — the formal scope statement that anchors all WIMSE draft work.</t>
         </is>
@@ -2470,6 +2500,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Addecd link from Tom Jones
</commit_message>
<xml_diff>
--- a/delegated_authorization_research.xlsx
+++ b/delegated_authorization_research.xlsx
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="6" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D11" s="7" t="n"/>
     </row>
@@ -3362,7 +3362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3831,27 +3831,27 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>AI Agent Authentication Gets the Hard Part Right. Authorization Is Still Your Problem. (Rock Cyber Musings)</t>
+          <t>Creating a Relationship Binding (Tom Jones)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>An analyst article arguing the new IETF agent-auth draft solves authentication via SPIFFE+WIMSE+OAuth but leaves authorization and policy enforcement as an unsolved open problem.</t>
+          <t>A community whitepaper proposing a signed 'Consent to Create Binding' JWT/JWS message that establishes a subject-bound relationship identifier (UUID or DID) between a user and a set of agents or service providers. The message carries 16 mandatory/optional fields: issuer, subject, subject role, context (trust framework), permissions, device statement, identity proof, purpose of use, key material, and signature. Includes a lifecycle termination model (session, cookie, transaction, relationship, and legal-based retention scopes) and a companion 'Consent Receipt with Binding' response. A second section argues that relationship-based governance — binding actors through mutual obligations, escalation paths, and accountability chains — is more resilient for AI agent systems than representational approaches (policies, classifications, static maps).</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>https://www.rockcybermusings.com/p/i-agent-authentication-authorization-gap</t>
+          <t>https://docs.google.com/document/d/1CwBDRbw147YlNld-UOlJ4lGvmpDIOCSI/edit#heading=h.kp911j18z01y</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Industry analysis blog</t>
+          <t>Community whitepaper</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Maps the IETF draft against MCP and the Colorado AI Act 'reasonable care' standard; pragmatic implementer perspective.</t>
+          <t>No publication date in the document; primary use case is healthcare (NIST IAL2/AAL2). Draws on Kantara's Distribute Assurance Specification for identity assurance levels and references OpenID Connect id_token as the closest existing message shape. The Consent to Create Binding message adds purpose of use, device statement, and lifecycle termination semantics that id_token lacks. Companion doc 'Digital Contracts Made Legally Valid' (separate Google Doc) covers giving the binding legal status. Relationship-governance argument is thematically aligned with Parker's 'Agents Are Not Just Workloads' — both argue that accountability chains and mutual obligations are the right governance primitive for agentic systems.</t>
         </is>
       </c>
     </row>
@@ -3861,27 +3861,27 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Agent Authentication &amp; Delegated Access (Zylos Research, April 2026)</t>
+          <t>AI Agent Authentication Gets the Hard Part Right. Authorization Is Still Your Problem. (Rock Cyber Musings)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>A research-style industry article surveying OAuth flows, scoped tokens, and identity patterns specifically for AI agents, covering OAuth 2.1 baselines and chain-splicing risks.</t>
+          <t>An analyst article arguing the new IETF agent-auth draft solves authentication via SPIFFE+WIMSE+OAuth but leaves authorization and policy enforcement as an unsolved open problem.</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>https://zylos.ai/research/2026-04-11-agent-authentication-delegated-access-oauth-scoped-tokens</t>
+          <t>https://www.rockcybermusings.com/p/i-agent-authentication-authorization-gap</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Industry research blog</t>
+          <t>Industry analysis blog</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Documents the 'delegation chain splicing' attack against RFC 8693 actor-token chains formally raised on the OAuth WG list in early 2026.</t>
+          <t>Maps the IETF draft against MCP and the Colorado AI Act 'reasonable care' standard; pragmatic implementer perspective.</t>
         </is>
       </c>
     </row>
@@ -3891,27 +3891,27 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>AuthZEN + Shared Signals Framework Series (Andrew Doering)</t>
+          <t>Agent Authentication &amp; Delegated Access (Zylos Research, April 2026)</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>A multi-part technical blog walking through how AuthZEN (synchronous PDP/PEP) and SSF/CAEP (asynchronous events) combine into a continuous-authorization loop in real Microsoft Entra/M365 deployments.</t>
+          <t>A research-style industry article surveying OAuth flows, scoped tokens, and identity patterns specifically for AI agents, covering OAuth 2.1 baselines and chain-splicing risks.</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>https://andrewdoering.org/blog/2026/authzen-shared-signals-framework-part-1-fundamentals/</t>
+          <t>https://zylos.ai/research/2026-04-11-agent-authentication-delegated-access-oauth-scoped-tokens</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Industry blog</t>
+          <t>Industry research blog</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Documents the 2026 asymmetry where Microsoft Entra is a CAEP transmitter for closed-loop CAE but not an external SSF receiver.</t>
+          <t>Documents the 'delegation chain splicing' attack against RFC 8693 actor-token chains formally raised on the OAuth WG list in early 2026.</t>
         </is>
       </c>
     </row>
@@ -3921,27 +3921,27 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Just-in-Time Authorization with OpenID SSE and CAEP (The New Stack, Tulshibagwale)</t>
+          <t>AuthZEN + Shared Signals Framework Series (Andrew Doering)</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>An article from CAEP's original inventor explaining how SSE+CAEP enable just-in-time authorization decisions instead of long-lived session-based access.</t>
+          <t>A multi-part technical blog walking through how AuthZEN (synchronous PDP/PEP) and SSF/CAEP (asynchronous events) combine into a continuous-authorization loop in real Microsoft Entra/M365 deployments.</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>https://thenewstack.io/just-in-time-authorization-with-openid-sse-and-caep/</t>
+          <t>https://andrewdoering.org/blog/2026/authzen-shared-signals-framework-part-1-fundamentals/</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Industry article (The New Stack)</t>
+          <t>Industry blog</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Background piece by Atul Tulshibagwale (SGNL CTO, CAEP inventor) explaining the architectural intent.</t>
+          <t>Documents the 2026 asymmetry where Microsoft Entra is a CAEP transmitter for closed-loop CAE but not an external SSF receiver.</t>
         </is>
       </c>
     </row>
@@ -3951,27 +3951,27 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>How AuthZEN, Shared Signals &amp; CAEP Complement Each Other (OpenID Foundation)</t>
+          <t>Just-in-Time Authorization with OpenID SSE and CAEP (The New Stack, Tulshibagwale)</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>An OpenID Foundation explainer arguing that AuthZEN and SSF/CAEP are complementary — sync access decisions vs async session updates — not competing standards.</t>
+          <t>An article from CAEP's original inventor explaining how SSE+CAEP enable just-in-time authorization decisions instead of long-lived session-based access.</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>https://openid.net/how-authzen-and-shared-signals-caep-complement-each-other/</t>
+          <t>https://thenewstack.io/just-in-time-authorization-with-openid-sse-and-caep/</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>OpenID Foundation</t>
+          <t>Industry article (The New Stack)</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Useful when explaining the layering to stakeholders confused by the OpenID alphabet soup.</t>
+          <t>Background piece by Atul Tulshibagwale (SGNL CTO, CAEP inventor) explaining the architectural intent.</t>
         </is>
       </c>
     </row>
@@ -3981,27 +3981,27 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>OAuth 2.1 Features You Can't Ignore in 2026 (Gutierrez, Medium)</t>
+          <t>How AuthZEN, Shared Signals &amp; CAEP Complement Each Other (OpenID Foundation)</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>A practitioner article summarizing why OAuth 2.1 — mandated PKCE, exact redirect matching, sender-constrained tokens — is the 2026 minimum bar for delegated authorization.</t>
+          <t>An OpenID Foundation explainer arguing that AuthZEN and SSF/CAEP are complementary — sync access decisions vs async session updates — not competing standards.</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>https://rgutierrez2004.medium.com/oauth-2-1-features-you-cant-ignore-in-2026-a15f852cb723</t>
+          <t>https://openid.net/how-authzen-and-shared-signals-caep-complement-each-other/</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Industry blog (Medium)</t>
+          <t>OpenID Foundation</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Author is Cyber Intelligence Lead — IAM/AI at Oracle; concise piece suitable for executive briefings.</t>
+          <t>Useful when explaining the layering to stakeholders confused by the OpenID alphabet soup.</t>
         </is>
       </c>
     </row>
@@ -4011,27 +4011,27 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>RFC 9396: OAuth 2.0 Rich Authorization Requests (CIAM Weekly)</t>
+          <t>OAuth 2.1 Features You Can't Ignore in 2026 (Gutierrez, Medium)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>A practitioner deep-dive on RAR explaining why scopes alone don't carry transaction-level intent and how authorization_details is being adopted in payments and verifiable credentials.</t>
+          <t>A practitioner article summarizing why OAuth 2.1 — mandated PKCE, exact redirect matching, sender-constrained tokens — is the 2026 minimum bar for delegated authorization.</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>https://ciamweekly.substack.com/p/rfc-9396-oauth-20-rich-authorization</t>
+          <t>https://rgutierrez2004.medium.com/oauth-2-1-features-you-cant-ignore-in-2026-a15f852cb723</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Industry newsletter</t>
+          <t>Industry blog (Medium)</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Captures the current (March 2026) state of RAR adoption, including CAMARA telco APIs and DPV-purpose binding proposals.</t>
+          <t>Author is Cyber Intelligence Lead — IAM/AI at Oracle; concise piece suitable for executive briefings.</t>
         </is>
       </c>
     </row>
@@ -4041,27 +4041,27 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Technical Deconstruction of MCP Authorization (kane.mx, Nov 2025)</t>
+          <t>RFC 9396: OAuth 2.0 Rich Authorization Requests (CIAM Weekly)</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>A long-form technical article showing that the Model Context Protocol's authorization spec is, in practice, an OAuth 2.1 profile combined with RFC 9728 protected-resource metadata and RFC 7591 dynamic registration.</t>
+          <t>A practitioner deep-dive on RAR explaining why scopes alone don't carry transaction-level intent and how authorization_details is being adopted in payments and verifiable credentials.</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>https://kane.mx/posts/2025/mcp-authorization-oauth-rfc-deep-dive/</t>
+          <t>https://ciamweekly.substack.com/p/rfc-9396-oauth-20-rich-authorization</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Independent technical blog</t>
+          <t>Industry newsletter</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Calls out RFC 8707 (Resource Indicators) as the critical compatibility bottleneck since most major IdPs use proprietary audience parameters.</t>
+          <t>Captures the current (March 2026) state of RAR adoption, including CAMARA telco APIs and DPV-purpose binding proposals.</t>
         </is>
       </c>
     </row>
@@ -4071,27 +4071,27 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>AI Agents Authentication: How Autonomous Systems Prove Identity (GitGuardian)</t>
+          <t>Technical Deconstruction of MCP Authorization (kane.mx, Nov 2025)</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>A GitGuardian engineering article arguing that delegated, short-lived OAuth grants are structurally safer than the static API keys that produced 28.65M secret leaks in 2025.</t>
+          <t>A long-form technical article showing that the Model Context Protocol's authorization spec is, in practice, an OAuth 2.1 profile combined with RFC 9728 protected-resource metadata and RFC 7591 dynamic registration.</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>https://blog.gitguardian.com/ai-agents-authentication-how-autonomous-systems-prove-identity/</t>
+          <t>https://kane.mx/posts/2025/mcp-authorization-oauth-rfc-deep-dive/</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Industry blog (GitGuardian)</t>
+          <t>Independent technical blog</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Useful for the 'why delegated authorization &gt; shared secrets' business case with concrete 2025 incident data.</t>
+          <t>Calls out RFC 8707 (Resource Indicators) as the critical compatibility bottleneck since most major IdPs use proprietary audience parameters.</t>
         </is>
       </c>
     </row>
@@ -4101,27 +4101,27 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Workload Identity – Key Takeaways from IETF 122 (Defakto)</t>
+          <t>AI Agents Authentication: How Autonomous Systems Prove Identity (GitGuardian)</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>A practitioner recap of IETF 122 covering the WIMSE Workload Identity Token, Credential Exchange, and side-meeting work on bot/agent web authentication.</t>
+          <t>A GitGuardian engineering article arguing that delegated, short-lived OAuth grants are structurally safer than the static API keys that produced 28.65M secret leaks in 2025.</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>https://www.defakto.security/blog/workload-identity-key-takeaways-from-ietf-122/</t>
+          <t>https://blog.gitguardian.com/ai-agents-authentication-how-autonomous-systems-prove-identity/</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Industry blog (Defakto)</t>
+          <t>Industry blog (GitGuardian)</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Author Pieter Kasselman is co-author of multiple key drafts (Transaction Tokens, First-Party Apps); strong primary-source view.</t>
+          <t>Useful for the 'why delegated authorization &gt; shared secrets' business case with concrete 2025 incident data.</t>
         </is>
       </c>
     </row>
@@ -4131,27 +4131,27 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>User-Managed Access (UMA) 2.0 Comprehensive Guide (SSOJet, Feb 2026)</t>
+          <t>Workload Identity – Key Takeaways from IETF 122 (Defakto)</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>A 2026 industry guide reframing UMA 2.0 for current CIAM contexts, covering resource-set registration, permission tickets, requesting-party tokens (RPTs), and policy externalization gains.</t>
+          <t>A practitioner recap of IETF 122 covering the WIMSE Workload Identity Token, Credential Exchange, and side-meeting work on bot/agent web authentication.</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>https://ssojet.com/blog/user-managed-access-uma-2-0-comprehensive-guide</t>
+          <t>https://www.defakto.security/blog/workload-identity-key-takeaways-from-ietf-122/</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Industry blog (SSOJet)</t>
+          <t>Industry blog (Defakto)</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Cites Kantara analysis showing centralized-policy moves can cut authorization code 80% — useful pitch material.</t>
+          <t>Author Pieter Kasselman is co-author of multiple key drafts (Transaction Tokens, First-Party Apps); strong primary-source view.</t>
         </is>
       </c>
     </row>
@@ -4161,27 +4161,27 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Decentralized Identity and Verifiable Credentials: The Enterprise Playbook 2026</t>
+          <t>User-Managed Access (UMA) 2.0 Comprehensive Guide (SSOJet, Feb 2026)</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>An enterprise-oriented guide explaining how W3C VCs, DIDs, and OpenID4VC enable the issuer-holder-verifier delegation model for digital credentials and EUDI Wallet acceptance.</t>
+          <t>A 2026 industry guide reframing UMA 2.0 for current CIAM contexts, covering resource-set registration, permission tickets, requesting-party tokens (RPTs), and policy externalization gains.</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>https://securityboulevard.com/2026/03/decentralized-identity-and-verifiable-credentials-the-enterprise-playbook-2026/</t>
+          <t>https://ssojet.com/blog/user-managed-access-uma-2-0-comprehensive-guide</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Industry article (Security Boulevard)</t>
+          <t>Industry blog (SSOJet)</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Critical 2027 EU compliance dates: banks, telecom, healthcare, and very-large platforms must accept EUDI Wallet.</t>
+          <t>Cites Kantara analysis showing centralized-policy moves can cut authorization code 80% — useful pitch material.</t>
         </is>
       </c>
     </row>
@@ -4191,27 +4191,27 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>OAuth 2.0 &amp; OpenID Connect: The Complete Guide to What the Standards Actually Say (Patil, Medium)</t>
+          <t>Decentralized Identity and Verifiable Credentials: The Enterprise Playbook 2026</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>A practitioner-friendly synthesis covering OAuth 2.0 core, the OAuth 2.1 draft, RFC 9068 JWT access tokens, RFC 8252 native apps, and RFC 8628 device authorization.</t>
+          <t>An enterprise-oriented guide explaining how W3C VCs, DIDs, and OpenID4VC enable the issuer-holder-verifier delegation model for digital credentials and EUDI Wallet acceptance.</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>https://mrutyunjaypatil.medium.com/oauth-2-0-openid-connect-the-complete-guide-to-what-the-standards-actually-say-e92f040a4251</t>
+          <t>https://securityboulevard.com/2026/03/decentralized-identity-and-verifiable-credentials-the-enterprise-playbook-2026/</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Industry blog (Medium)</t>
+          <t>Industry article (Security Boulevard)</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Good handoff document for engineers new to the area; cites the current standards rather than legacy patterns.</t>
+          <t>Critical 2027 EU compliance dates: banks, telecom, healthcare, and very-large platforms must accept EUDI Wallet.</t>
         </is>
       </c>
     </row>
@@ -4221,27 +4221,27 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>LinkedIn Engineering — OpenID Connect Authentication for Sign In with LinkedIn V2</t>
+          <t>OAuth 2.0 &amp; OpenID Connect: The Complete Guide to What the Standards Actually Say (Patil, Medium)</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>LinkedIn's own engineering write-up on adopting OpenID Connect on top of OAuth 2.0, explicitly distinguishing OAuth's delegated-access role from OIDC's identity-assertion role.</t>
+          <t>A practitioner-friendly synthesis covering OAuth 2.0 core, the OAuth 2.1 draft, RFC 9068 JWT access tokens, RFC 8252 native apps, and RFC 8628 device authorization.</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/developers/news/featured-updates/openid-connect-authentication</t>
+          <t>https://mrutyunjaypatil.medium.com/oauth-2-0-openid-connect-the-complete-guide-to-what-the-standards-actually-say-e92f040a4251</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Industry (LinkedIn Engineering)</t>
+          <t>Industry blog (Medium)</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Real-world example from LinkedIn explaining why they layered OIDC over an existing OAuth 2.0 delegated-access stack.</t>
+          <t>Good handoff document for engineers new to the area; cites the current standards rather than legacy patterns.</t>
         </is>
       </c>
     </row>
@@ -4251,27 +4251,27 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Rich Authorization Requests (RAR) — Authlete Knowledge Base</t>
+          <t>LinkedIn Engineering — OpenID Connect Authentication for Sign In with LinkedIn V2</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>A vendor knowledge-base article giving worked examples of RAR's authorization_details object, including locations, actions, datatypes, and identifier fields with their Authlete bindings.</t>
+          <t>LinkedIn's own engineering write-up on adopting OpenID Connect on top of OAuth 2.0, explicitly distinguishing OAuth's delegated-access role from OIDC's identity-assertion role.</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>https://www.authlete.com/kb/oauth-and-openid-connect/authorization-requests/rich-authorization-requests/</t>
+          <t>https://www.linkedin.com/developers/news/featured-updates/openid-connect-authentication</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Vendor documentation (Authlete)</t>
+          <t>Industry (LinkedIn Engineering)</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Authlete is one of the few certified FAPI 2.0 + RAR implementations; useful reference for concrete request bodies.</t>
+          <t>Real-world example from LinkedIn explaining why they layered OIDC over an existing OAuth 2.0 delegated-access stack.</t>
         </is>
       </c>
     </row>
@@ -4281,25 +4281,55 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
+          <t>Rich Authorization Requests (RAR) — Authlete Knowledge Base</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>A vendor knowledge-base article giving worked examples of RAR's authorization_details object, including locations, actions, datatypes, and identifier fields with their Authlete bindings.</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>https://www.authlete.com/kb/oauth-and-openid-connect/authorization-requests/rich-authorization-requests/</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Vendor documentation (Authlete)</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Authlete is one of the few certified FAPI 2.0 + RAR implementations; useful reference for concrete request bodies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
           <t>An Introduction to Authorization Exchange (AuthZEN) — Curity</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>A vendor explainer comparing externalized-authorization patterns (OPA, Cedar, XACML, Zanzibar) and showing how AuthZEN's API normalizes the PDP/PEP wire protocol across them.</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D32" s="9" t="inlineStr">
         <is>
           <t>https://curity.io/resources/learn/authzen/</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>Vendor blog (Curity)</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
         <is>
           <t>Curity is a member of the AuthZEN WG; positions AuthZEN as 'OpenID Connect for authorization' which has become the common framing.</t>
         </is>
@@ -4337,6 +4367,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added oauth txn challenge
</commit_message>
<xml_diff>
--- a/delegated_authorization_research.xlsx
+++ b/delegated_authorization_research.xlsx
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="6" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D11" s="7" t="n"/>
     </row>
@@ -906,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2365,17 +2365,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>draft-hardt-aauth-protocol — AAuth Protocol</t>
+          <t>draft-rosomakho-oauth-txn-challenge — OAuth Transaction Authorization Challenge</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>A new clean-sheet authorization protocol from Dick Hardt (original OAuth author) defining proof-of-possession by default, resource-signed challenges, agent identity without pre-registration, deferred 202 responses, and AS-to-AS federation for the agent ecosystem.</t>
+          <t>An OAuth mechanism enabling protected resources to demand transaction-specific authorization through challenges. When a request involves an agent or automated workflow, the RS returns a challenge to the client; the client presents it to the AS, which validates it, obtains human approval, and issues an access token with RFC 9396 authorization_details describing the approved operation. Positions as complementary to RFC 9470 (Step-Up Authentication) — that spec handles authentication freshness; this one handles authorization specificity.</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hardt-aauth-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rosomakho-oauth-txn-challenge/</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, April 2026; the design rationale section explicitly explains why AAuth is not GNAP, not OAuth, not DPoP and not mTLS — important read for anyone planning a new agent-auth stack.</t>
+          <t>Revision -00, submitted 25 June 2026. Authors: Yaroslav Rosomakho (Zscaler), Brian Campbell (Ping Identity), Karl McGuinness (Independent), Pieter Kasselman (Defakto). Strong author lineup — Campbell is a prolific OAuth WG contributor, Kasselman co-authored Transaction Tokens and First-Party Apps, McGuinness brings the Mission-Bound OAuth context. The RS-initiated challenge model is distinct from ARAP (which operates at the PDP/PEP layer via AuthZEN) but addresses the same 'denial is not the end' problem — here at the OAuth RS/AS layer rather than the AuthZEN layer.</t>
         </is>
       </c>
     </row>
@@ -2395,17 +2395,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>draft-chen-oauth-roadmap — Comprehensive Roadmap for OAuth 2.0 Standards and Drafts</t>
+          <t>draft-hardt-aauth-protocol — AAuth Protocol</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>An IETF informational draft that maps the entire OAuth 2.0 ecosystem of RFCs, BCPs, and active drafts into functional layers from core to extensions to industry profiles.</t>
+          <t>A new clean-sheet authorization protocol from Dick Hardt (original OAuth author) defining proof-of-possession by default, resource-signed challenges, agent identity without pre-registration, deferred 202 responses, and AS-to-AS federation for the agent ecosystem.</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>https://www.ietf.org/archive/id/draft-chen-oauth-roadmap-00.html</t>
+          <t>https://datatracker.ietf.org/doc/draft-hardt-aauth-protocol/</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Brand-new -00 draft (May 2026); the single most useful index when starting work in this area.</t>
+          <t>Revision -00, April 2026; the design rationale section explicitly explains why AAuth is not GNAP, not OAuth, not DPoP and not mTLS — important read for anyone planning a new agent-auth stack.</t>
         </is>
       </c>
     </row>
@@ -2425,25 +2425,55 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
+          <t>draft-chen-oauth-roadmap — Comprehensive Roadmap for OAuth 2.0 Standards and Drafts</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>An IETF informational draft that maps the entire OAuth 2.0 ecosystem of RFCs, BCPs, and active drafts into functional layers from core to extensions to industry profiles.</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ietf.org/archive/id/draft-chen-oauth-roadmap-00.html</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>Brand-new -00 draft (May 2026); the single most useful index when starting work in this area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
           <t>Charter: WIMSE — Workload Identity in Multi-System Environments (charter-ietf-wimse-01)</t>
         </is>
       </c>
-      <c r="C51" s="5" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>The formal IETF charter for the WIMSE WG covering architecture, JOSE-based WIMSE tokens for service-to-service traffic, local token issuance, and token exchange profiles (likely based on RFC 8693) for cross-trust-domain workload identity.</t>
         </is>
       </c>
-      <c r="D51" s="9" t="inlineStr">
+      <c r="D52" s="9" t="inlineStr">
         <is>
           <t>https://datatracker.ietf.org/doc/charter-ietf-wimse/01/</t>
         </is>
       </c>
-      <c r="E51" s="5" t="inlineStr">
+      <c r="E52" s="5" t="inlineStr">
         <is>
           <t>IETF (WIMSE WG charter)</t>
         </is>
       </c>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="F52" s="5" t="inlineStr">
         <is>
           <t>Approved 18 March 2026 (v01); explicitly liaises with OAuth, SCIM, SCITT, RATS, the OpenID Foundation, and CNCF/SPIFFE — the formal scope statement that anchors all WIMSE draft work.</t>
         </is>
@@ -2501,6 +2531,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId51"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated based on recently submitted individual drafts
</commit_message>
<xml_diff>
--- a/delegated_authorization_research.xlsx
+++ b/delegated_authorization_research.xlsx
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="6" t="n">
-        <v>109</v>
+        <v>141</v>
       </c>
       <c r="D11" s="7" t="n"/>
     </row>
@@ -906,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1585,17 +1585,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>draft-mishra-oauth-agent-grants — Delegated Agent Authorization Protocol (DAAP)</t>
+          <t>draft-mcguinness-oauth-insufficient-claims — OAuth 2.0 Insufficient Claims Challenge</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft addressing runtime agent identity for dynamically-spawned agents, multi-agent sub-delegation with depth-limiting, and cascade revocation of an entire delegation subtree when any ancestor is revoked.</t>
+          <t>A McGuinness individual draft defining an insufficient_claims error code and required_claims parameter enabling authorization servers and protected resources to signal precisely which claims are missing from a presented credential. Allows resource servers to request enriched credentials carrying specific missing attributes rather than returning a generic 401.</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mishra-oauth-agent-grants/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-insufficient-claims/</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Revision -01 (March 2026); registers new JWT claims (agt, dev, grnt, scp, bdg) — a more aggressive alternative to RFC 8693 with budget-bounded grants. Overlaps with draft-niyikiza-oauth-attenuating-agent-tokens; OAuth WG will likely expect consolidation.</t>
+          <t>Revision -00, 27 May 2026. Enables just-in-time claim negotiation in multi-agent delegation chains where the acting party must assemble claims from multiple sources. Natural companion to the Actor Profile and Client Instance Assertion — those drafts define the identity structure; this one provides the feedback loop when that structure is incomplete at the RS.</t>
         </is>
       </c>
     </row>
@@ -1615,17 +1615,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>draft-kuehlewind-audit-architecture — Architecture for Auditing AI Agent Delegation and Interactions</t>
+          <t>draft-mishra-oauth-agent-grants — Delegated Agent Authorization Protocol (DAAP)</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Mirja Kühlewind (Ericsson, former IETF TSV-AD) and Henk Birkholz (Fraunhofer SIT, lead author of RFC 9334 RATS and SCITT architecture) defining four record types — Interaction, Action, Delegation, and Authorization Transition — and an Audit Context that propagates across OAuth + WIMSE + RATS + SCITT to make agent behaviour verifiably auditable end-to-end.</t>
+          <t>An IETF individual draft addressing runtime agent identity for dynamically-spawned agents, multi-agent sub-delegation with depth-limiting, and cascade revocation of an entire delegation subtree when any ancestor is revoked.</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-kuehlewind-audit-architecture/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mishra-oauth-agent-grants/</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Revision -00 published 18 May 2026; the cross-layer integration piece — explicitly composes the McGuinness Actor Profile, Transaction Tokens, identity-chaining, ID-JAG, WIMSE, RATS, and SCITT into a single auditable architecture with 11 proposed work items. The treats-Agent-as-untrusted threat model is what regulators (SOX, PSD2, EU AI Act) actually want.</t>
+          <t>Revision -01 (March 2026); registers new JWT claims (agt, dev, grnt, scp, bdg) — a more aggressive alternative to RFC 8693 with budget-bounded grants. Overlaps with draft-niyikiza-oauth-attenuating-agent-tokens; OAuth WG will likely expect consolidation.</t>
         </is>
       </c>
     </row>
@@ -1645,17 +1645,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>draft-birkholz-verifiable-agent-conversations — Verifiable Agent Conversation Records</t>
+          <t>draft-kuehlewind-audit-architecture — Architecture for Auditing AI Agent Delegation and Interactions</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft (Birkholz/Heldt/Steele) defining a CDDL data format — with both JSON and CBOR encodings — for tamper-evident, verifiably-signed records of agent conversations, agent reasoning traces, tool calls, and system events that support long-term evidentiary value across chains of custody.</t>
+          <t>An IETF individual draft from Mirja Kühlewind (Ericsson, former IETF TSV-AD) and Henk Birkholz (Fraunhofer SIT, lead author of RFC 9334 RATS and SCITT architecture) defining four record types — Interaction, Action, Delegation, and Authorization Transition — and an Audit Context that propagates across OAuth + WIMSE + RATS + SCITT to make agent behaviour verifiably auditable end-to-end.</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-birkholz-verifiable-agent-conversations/</t>
+          <t>https://datatracker.ietf.org/doc/draft-kuehlewind-audit-architecture/</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Revision -00 published 25 Feb 2026; presented at IETF 125 dispatch and hotrfc. The canonical Interaction-Record format for the Kuehlewind audit architecture. Motivating examples are concrete: agents acting beyond scope, CoT divergence, and 'sandbagging' during evaluations.</t>
+          <t>Revision -00 published 18 May 2026; the cross-layer integration piece — explicitly composes the McGuinness Actor Profile, Transaction Tokens, identity-chaining, ID-JAG, WIMSE, RATS, and SCITT into a single auditable architecture with 11 proposed work items. The treats-Agent-as-untrusted threat model is what regulators (SOX, PSD2, EU AI Act) actually want.</t>
         </is>
       </c>
     </row>
@@ -1675,17 +1675,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>draft-klrc-aiagent-auth — AI Agent Authentication and Authorization</t>
+          <t>draft-birkholz-verifiable-agent-conversations — Verifiable Agent Conversation Records</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft that does not invent new protocols but composes WIMSE/SPIFFE workload identity, OAuth 2.x, and OpenID SSF to authenticate and delegate authority to AI agents.</t>
+          <t>An IETF individual draft (Birkholz/Heldt/Steele) defining a CDDL data format — with both JSON and CBOR encodings — for tamper-evident, verifiably-signed records of agent conversations, agent reasoning traces, tool calls, and system events that support long-term evidentiary value across chains of custody.</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/html/draft-klrc-aiagent-auth-00</t>
+          <t>https://datatracker.ietf.org/doc/draft-birkholz-verifiable-agent-conversations/</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, March 2026; introduces 'Agent Identity Management System (AIMS)' and is the cleanest standards-based framing of agent-as-workload.</t>
+          <t>Revision -00 published 25 Feb 2026; presented at IETF 125 dispatch and hotrfc. The canonical Interaction-Record format for the Kuehlewind audit architecture. Motivating examples are concrete: agents acting beyond scope, CoT divergence, and 'sandbagging' during evaluations.</t>
         </is>
       </c>
     </row>
@@ -1705,17 +1705,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>draft-niyikiza-oauth-attenuating-agent-tokens — Attenuating Authorization Tokens for Agentic Delegation Chains</t>
+          <t>draft-klrc-aiagent-auth — AI Agent Authentication and Authorization</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft extending RFC 9396 Rich Authorization Requests with monotonic attenuation at each delegation hop, offline chain verification, and a typed constraint vocabulary for tool-level argument restrictions.</t>
+          <t>An IETF individual draft that does not invent new protocols but composes WIMSE/SPIFFE workload identity, OAuth 2.x, and OpenID SSF to authenticate and delegate authority to AI agents.</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-niyikiza-oauth-attenuating-agent-tokens/</t>
+          <t>https://datatracker.ietf.org/doc/html/draft-klrc-aiagent-auth-00</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, March 2026; arguably the strongest purely-OAuth-grounded delegation draft — offline verification is a key scalability property. Good path to OAuth WG adoption; overlaps with draft-mishra-oauth-agent-grants and will likely need to be consolidated with it.</t>
+          <t>Revision -00, March 2026; introduces 'Agent Identity Management System (AIMS)' and is the cleanest standards-based framing of agent-as-workload.</t>
         </is>
       </c>
     </row>
@@ -1735,17 +1735,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>draft-singla-agent-identity-protocol — AIP: Decentralized Identity and Delegation for AI Agents</t>
+          <t>draft-niyikiza-oauth-attenuating-agent-tokens — Attenuating Authorization Tokens for Agentic Delegation Chains</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft proposing a six-layer model (identity through reputation) for AI agents with W3C DID anchoring, a Delegation Depth counter, three Grant ceremony tiers (G1/G2/G3), DPoP proof-of-possession, and an MCP integration layer.</t>
+          <t>An IETF individual draft extending RFC 9396 Rich Authorization Requests with monotonic attenuation at each delegation hop, offline chain verification, and a typed constraint vocabulary for tool-level argument restrictions.</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-singla-agent-identity-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-niyikiza-oauth-attenuating-agent-tokens/</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 17 April 2026; the most comprehensive identity framework in the set. The W3C DID dependency will face IETF pushback, the 75+ page scope needs reduction, and the 'AIP' name collision with two other drafts (draft-prakash-aip, draft-aip-agent-identity-protocol) must be resolved.</t>
+          <t>Revision -00, March 2026; arguably the strongest purely-OAuth-grounded delegation draft — offline verification is a key scalability property. Good path to OAuth WG adoption; overlaps with draft-mishra-oauth-agent-grants and will likely need to be consolidated with it.</t>
         </is>
       </c>
     </row>
@@ -1765,17 +1765,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>draft-prakash-aip — AIP: Verifiable Delegation for AI Agent Systems</t>
+          <t>draft-singla-agent-identity-protocol — AIP: Decentralized Identity and Delegation for AI Agents</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft introducing Invocation-Bound Capability Tokens (IBCTs) in two modes — compact (JWT/Ed25519) for single-hop and chained (Biscuit + Datalog) for multi-hop — with bindings for MCP, A2A, and HTTP APIs.</t>
+          <t>An IETF individual draft proposing a six-layer model (identity through reputation) for AI agents with W3C DID anchoring, a Delegation Depth counter, three Grant ceremony tiers (G1/G2/G3), DPoP proof-of-possession, and an MCP integration layer.</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-prakash-aip/</t>
+          <t>https://datatracker.ietf.org/doc/draft-singla-agent-identity-protocol/</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 27 March 2026; technically strong — Biscuit + Datalog is well-suited to scope attenuation. The 'AIP' name collision with draft-singla-agent-identity-protocol and draft-aip-agent-identity-protocol is a blocking issue for WG adoption.</t>
+          <t>Revision -00, 17 April 2026; the most comprehensive identity framework in the set. The W3C DID dependency will face IETF pushback, the 75+ page scope needs reduction, and the 'AIP' name collision with two other drafts (draft-prakash-aip, draft-aip-agent-identity-protocol) must be resolved.</t>
         </is>
       </c>
     </row>
@@ -1795,17 +1795,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>draft-goswami-agentic-jwt — Secure Intent Protocol: JWT-Compatible Agentic Identity and Workflow Management</t>
+          <t>draft-prakash-aip — AIP: Verifiable Delegation for AI Agent Systems</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an Agentic JWT extension to OAuth 2.0 with a Supervisor Agent role for sub-agent coordination, explicitly addressing the 'intent-execution separation' gap and adding workflow-step authorization.</t>
+          <t>An IETF individual draft introducing Invocation-Bound Capability Tokens (IBCTs) in two modes — compact (JWT/Ed25519) for single-hop and chained (Biscuit + Datalog) for multi-hop — with bindings for MCP, A2A, and HTTP APIs.</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-goswami-agentic-jwt/</t>
+          <t>https://datatracker.ietf.org/doc/draft-prakash-aip/</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, December 2025; the intent-execution-separation framing is insightful and distinguishing. The workflow-step authorization approach is novel but may face skepticism in the OAuth WG.</t>
+          <t>Revision -00, 27 March 2026; technically strong — Biscuit + Datalog is well-suited to scope attenuation. The 'AIP' name collision with draft-singla-agent-identity-protocol and draft-aip-agent-identity-protocol is a blocking issue for WG adoption.</t>
         </is>
       </c>
     </row>
@@ -1825,17 +1825,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>draft-ni-wimse-ai-agent-identity — WIMSE Applicability for AI Agents</t>
+          <t>draft-goswami-agentic-jwt — Secure Intent Protocol: JWT-Compatible Agentic Identity and Workflow Management</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft mapping the WIMSE workload-identity architecture to AI-agent use cases and establishing credential-management mechanisms for agentic AI within the WIMSE framework.</t>
+          <t>An IETF individual draft defining an Agentic JWT extension to OAuth 2.0 with a Supervisor Agent role for sub-agent coordination, explicitly addressing the 'intent-execution separation' gap and adding workflow-step authorization.</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ni-wimse-ai-agent-identity/</t>
+          <t>https://datatracker.ietf.org/doc/draft-goswami-agentic-jwt/</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, February 2026; an important bridge between the WIMSE WG and the AI agent space. If an AI-agent WG is ever chartered, this applicability statement is essential groundwork. Co-authored with Liu, who also leads the related security-requirements draft.</t>
+          <t>Revision -00, December 2025; the intent-execution-separation framing is insightful and distinguishing. The workflow-step authorization approach is novel but may face skepticism in the OAuth WG.</t>
         </is>
       </c>
     </row>
@@ -1855,17 +1855,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-identity-framework — Agent Identity Framework: Trust and Identity for Autonomous AI Agents</t>
+          <t>draft-ni-wimse-ai-agent-identity — WIMSE Applicability for AI Agents</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft proposing a five-layer model (identity, authorization, attestation, evidence, trust) for autonomous AI agents, with a gap analysis between current Internet standards and agent requirements.</t>
+          <t>An IETF individual draft mapping the WIMSE workload-identity architecture to AI-agent use cases and establishing credential-management mechanisms for agentic AI within the WIMSE framework.</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-identity-framework/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ni-wimse-ai-agent-identity/</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 6 April 2026; more gap-analysis than protocol spec. Useful as problem statement. Five-layer model is a reasonable decomposition but insufficient as a standalone contribution. Part of the Sharif cluster (with -agent-audit-trail, -attp, etc.).</t>
+          <t>Revision -02, February 2026; an important bridge between the WIMSE WG and the AI agent space. If an AI-agent WG is ever chartered, this applicability statement is essential groundwork. Co-authored with Liu, who also leads the related security-requirements draft.</t>
         </is>
       </c>
     </row>
@@ -1885,17 +1885,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>draft-aip-agent-identity-protocol — AIP: Agentic Authentication and Authorized Policy Enforcement</t>
+          <t>draft-sharif-agent-identity-framework — Agent Identity Framework: Trust and Identity for Autonomous AI Agents</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an AIP Token signed per tool call (agent ID, tool, nonce, timestamp, signature), an AgentPolicy YAML format for per-tool argument constraints and DLP rules, and a Human-in-the-Loop proxy enforcement model.</t>
+          <t>An IETF individual draft proposing a five-layer model (identity, authorization, attestation, evidence, trust) for autonomous AI agents, with a gap analysis between current Internet standards and agent requirements.</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-aip-agent-identity-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-identity-framework/</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 16 March 2026; implementation-focused. YAML policy approach is pragmatic but not interoperable-by-design. HITL integration is a valuable safety feature. Third member of the 'AIP' name-collision triple — must be resolved before any can progress.</t>
+          <t>Revision -00, 6 April 2026; more gap-analysis than protocol spec. Useful as problem statement. Five-layer model is a reasonable decomposition but insufficient as a standalone contribution. Part of the Sharif cluster (with -agent-audit-trail, -attp, etc.).</t>
         </is>
       </c>
     </row>
@@ -1915,17 +1915,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>draft-serra-mcp-discovery-uri — The mcp URI Scheme and MCP Server Discovery Mechanism</t>
+          <t>draft-aip-agent-identity-protocol — AIP: Agentic Authentication and Authorized Policy Enforcement</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an 'mcp://' URI scheme combined with /.well-known/mcp-server (RFC 8615) and a DNS TXT fallback for discovery of Model Context Protocol servers.</t>
+          <t>An IETF individual draft defining an AIP Token signed per tool call (agent ID, tool, nonce, timestamp, signature), an AgentPolicy YAML format for per-tool argument constraints and DLP rules, and a Human-in-the-Loop proxy enforcement model.</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-serra-mcp-discovery-uri/</t>
+          <t>https://datatracker.ietf.org/doc/draft-aip-agent-identity-protocol/</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Already at revision -04 (March 2026), suggesting active iteration; narrow scope, clean design, and the strongest IANA-registration candidate in the set. OAuth 2.1 for auth is deliberately out of scope.</t>
+          <t>Revision -00, 16 March 2026; implementation-focused. YAML policy approach is pragmatic but not interoperable-by-design. HITL integration is a valuable safety feature. Third member of the 'AIP' name-collision triple — must be resolved before any can progress.</t>
         </is>
       </c>
     </row>
@@ -1945,17 +1945,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-attp — ATTP: Agent Trust Transport Protocol</t>
+          <t>draft-liu-oauth-chain-delegation — Delegation Chain for OAuth 2.0</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining trust levels L0–L4 mapped to PSD2 Strong Customer Authentication requirements, with bindings for MCP (MCPS), REST, A2A, gRPC, and GraphQL; supersedes draft-sharif-agent-payment-trust.</t>
+          <t>Introduces a delegation_chain JWT claim as a structured companion to RFC 8693's act claim; delegation_chain records the complete delegation history as an ordered array with per-hop authorization constraints and optional cryptographic confirmation from each delegating agent. Supports cross-domain delegation with integrated user consent interaction.</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-attp/</t>
+          <t>https://datatracker.ietf.org/doc/draft-liu-oauth-chain-delegation/</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, April 2026; regulatory mapping appendices (PSD2, PCI DSS) are notable — one of the few drafts engaging financial regulation directly. Ambitious scope. Part of the Sharif cluster.</t>
+          <t>Revision -00, 6 Jun 2026; authors: Dapeng Liu, Judy Zhu, Suresh Krishnan (Ericsson), Aaron Parecki (Okta). Provides the structured delegation lineage that act alone cannot express; strong overlap with draft-mw-oauth-actor-chain and draft-niyikiza-oauth-attenuating-agent-tokens — OAuth WG will likely expect consolidation across these three.</t>
         </is>
       </c>
     </row>
@@ -1975,17 +1975,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-transport-protocol — Agent Transport Protocol (ATP): Async Store-and-Forward for AI Agents</t>
+          <t>draft-fletcher-transaction-token-chaining-profile — Transaction Token Authorization Grant Profile for OAuth Identity and Authorization Chaining</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining async store-and-forward messaging semantics with cryptographic identity per relay hop, trust scoring at ingress, capability negotiation, and interop with Google A2A, MCP, and FIPA ACL; transport-agnostic over TCP/TLS/QUIC.</t>
+          <t>Establishes a framework for using Transaction Tokens as subject credentials in OAuth 2.0 Token Exchange requests (RFC 8693), enabling services within one trust domain to obtain JWT authorization grants for accessing resources across domain boundaries without exposing internal token formats.</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-transport-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-fletcher-transaction-token-chaining-profile/</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 28 March 2026; addresses a real gap — most agent protocols assume synchronous availability, and store-and-forward is appropriate for long-running agentic tasks. Scope is broad and needs narrowing.</t>
+          <t>Revision -01, 20 Jun 2026; authors: George Fletcher (Practical Identity LLC), Pieter Kasselman (Defakto Security), Sean O'Dell (CVS Health). Directly bridges draft-ietf-oauth-transaction-tokens and draft-ietf-oauth-identity-chaining (both in corpus), closing the 'how do TX Tokens actually cross domains' gap. Note: lead author is the corpus maintainer.</t>
         </is>
       </c>
     </row>
@@ -2005,17 +2005,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-audit-trail — Agent Audit Trail (AAT): Standard Logging Format for Autonomous AI Systems</t>
+          <t>draft-zhu-oauth-async-delegation — Sender-Constrained Delegation Handle for Asynchronous OAuth 2.0 Identity Chaining</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining a JSON-based audit record with mandatory fields (agent identity, action classification, outcome tracking, trust level) using RFC 8785 JSON Canonicalization and RFC 9562 UUIDs.</t>
+          <t>Introduces a Delegation Handle — a sender-constrained, audience-locked JWT issued by authorization servers — enabling acting clients to refresh chained access tokens without re-prompting an offline end user while maintaining strict policy bounds and identity chains.</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-audit-trail/</t>
+          <t>https://datatracker.ietf.org/doc/draft-zhu-oauth-async-delegation/</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 29 March 2026; orthogonal to delegation but important for compliance — standardized audit-log format is a genuine gap. Complements identity frameworks well. A sibling/alternative to the Kuehlewind audit architecture which takes a far more ambitious cross-layer approach.</t>
+          <t>Revision -00, 22 May 2026; authors: Larry Zhu, Sam Currie (Atlassian). Addresses a concrete gap in agent delegation: what happens when the delegating human is not present to re-authorize. Directly relevant to long-running agentic workflows using draft-ietf-oauth-identity-chaining.</t>
         </is>
       </c>
     </row>
@@ -2035,17 +2035,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>draft-aiendpoint-ai-discovery — The AI Discovery Endpoint</t>
+          <t>draft-chen-oauth-agent-revocation — OAuth 2.0 Agent Authorization Explicit Revocation</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining a /.well-known/ai URI suffix for programmatic service capability discovery by AI agents — letting agents discover what an endpoint supports without having to parse human-oriented documentation; requests IANA well-known URI registration.</t>
+          <t>Extends RFC 7009 token revocation for agent-based scenarios: introduces batch revocation by agent ID, cascading revocation across delegation chains, conditional revocation options, and verifiable audit trails.</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-aiendpoint-ai-discovery/</t>
+          <t>https://datatracker.ietf.org/doc/draft-chen-oauth-agent-revocation/</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, March 2026; complementary to MCP discovery but broader (not MCP-specific). Needs differentiation from OpenAPI/service-description work to gain traction.</t>
+          <t>Revision -00, 27 Apr 2026; authors: Meiling Chen, Li Su (China Mobile). Fills the lifecycle management gap — existing RFC 7009 revocation is single-token and client-centric, but agent delegation chains require cascade semantics. Natural companion to draft-ietf-oauth-transaction-tokens and draft-niyikiza-oauth-attenuating-agent-tokens.</t>
         </is>
       </c>
     </row>
@@ -2065,17 +2065,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>draft-hood-independent-agtp — Agent Transfer Protocol (AGTP)</t>
+          <t>draft-jiang-oauth-intent-admission — Intent Admission Assertions for Agentic Systems</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft proposing a dedicated application-layer protocol for AI agent traffic on port 4480 (TCP/TLS and QUIC) with an agtp:// URI scheme, arguing that HTTP is insufficient because agent-generated intent-driven traffic is indistinguishable from human-initiated requests. Defines a Runtime Contract Negotiation Substrate (RCNS) with eighteen methods split into cognitive verbs (QUERY, DISCOVER, DESCRIBE, SUMMARIZE, PLAN, PROPOSE) and mechanics verbs (EXECUTE, DELEGATE, ESCALATE, CONFIRM, SUSPEND, NOTIFY), mandatory agent identity headers, and protocol-level authority scope declaration.</t>
+          <t>Defines a signed, verifiable Intent Admission Assertion (IAA) that an admission point creates after verifying agent identity, evaluating permissions against policy, and — when required — obtaining explicit user consent; the IAA is transmitted to the execution endpoint which re-validates before proceeding. Leverages OAuth and RFC 9396 Rich Authorization Requests.</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hood-independent-agtp/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jiang-oauth-intent-admission/</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Revision -08 (26 May 2026); supersedes draft-hood-independent-atp. Companion specs in the same family: AGTP-API, AGTP-CERT, AGTP-MERCHANT, AGTP-IDENTIFIERS, AGTP-TRUST. Mandatory TLS 1.3+. Ambitious scope — a new transport layer rather than an HTTP profile. The cognitive/mechanics verb split is a distinctive design choice; contrasts with draft-sharif-agent-transport-protocol which layers async store-and-forward on top of existing transports rather than replacing them.</t>
+          <t>Revision -00, 23 Jun 2026; authors: Yuning Jiang, Lun Li, Yurong Song, Faye Liu (Huawei). The required_consent path maps directly to the HITL pattern central to the corpus. Companion to draft-jiang-intent-security (threat model) from the same Huawei group.</t>
         </is>
       </c>
     </row>
@@ -2095,17 +2095,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>draft-ni-a2a-ai-agent-security-requirements — Security Requirements for AI Agents</t>
+          <t>draft-kroehl-agentic-trust-aae — Agent Authorization Envelope (AAE)</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft enumerating security requirements for AI agents, covering identity, authorization chaining across domains, and integration points with WIMSE, OAuth identity chaining, and the A2A OAuth profile.</t>
+          <t>Specifies the AAE, a structured authorization container with three mandatory components — MANDATE, CONSTRAINTS, and VALIDITY — providing a machine-evaluable, cryptographically verifiable authorization assertion using W3C DIDs and Verifiable Credentials.</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ni-a2a-ai-agent-security-requirements/</t>
+          <t>https://datatracker.ietf.org/doc/draft-kroehl-agentic-trust-aae/</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, February 2026; essential scaffolding for an eventual AI-agent WG. Well-connected to existing IETF work and authored by Ni and Liu, who also lead the WIMSE AI-agent identity draft.</t>
+          <t>Revision -00, 21 May 2026; author: Lars Kersten Kroehl (CryptoKRI GmbH). Occupies similar design space to draft-mcguinness-oauth-actor-profile but uses a DID/VC substrate rather than OAuth — provides a useful alternative approach for non-OAuth deployments.</t>
         </is>
       </c>
     </row>
@@ -2125,17 +2125,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>draft-rosenberg-aiproto-framework — Framework, Use Cases and Requirements for AI Agent Protocols</t>
+          <t>draft-pidlisnyi-aps — Agent Passport System (APS)</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft providing a comprehensive AI-agent communications framework that covers user↔agent, agent↔API, and agent↔agent interactions; surveys MCP, A2A, and Agntcy; and sets the stage for IETF standards activity.</t>
+          <t>Specifies Ed25519-based agent passports, scoped delegation chains with constraints across seven dimensions (a lattice model where delegation monotonically narrows capabilities), cascade revocation, a three-signature policy chain, signed receipts, and MCP bindings; includes reference implementations in TypeScript and Python.</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-framework/</t>
+          <t>https://datatracker.ietf.org/doc/draft-pidlisnyi-aps/</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, October 2025; Rosenberg (Five9) and Jennings (Cisco) are credible long-time IETF contributors. Important landscape document but likely expired (April 2026); watch for a -01 refresh post-IETF 123.</t>
+          <t>Revision -01, 14 May 2026; author: Tymofii Pidlisnyi (AEOESS). Among the most comprehensive standalone agent authz specs in the wave — the seven-dimension constraint lattice and MCP binding make it directly implementable against Model Context Protocol deployments alongside draft-serra-mcp-discovery-uri.</t>
         </is>
       </c>
     </row>
@@ -2155,17 +2155,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>draft-rosenberg-aiproto-cheq — CHEQ: A Protocol for Confirmation of AI Agent Decisions (HITL)</t>
+          <t>draft-serra-mcp-discovery-uri — The mcp URI Scheme and MCP Server Discovery Mechanism</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an out-of-band Human-in-the-Loop confirmation protocol for agent tool calls, eliminating LLM-hallucination risk for consequential actions and enabling sensitive operations (e.g., banking) without exposing data to the agent.</t>
+          <t>An IETF individual draft defining an 'mcp://' URI scheme combined with /.well-known/mcp-server (RFC 8615) and a DNS TXT fallback for discovery of Model Context Protocol servers.</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-cheq/</t>
+          <t>https://datatracker.ietf.org/doc/draft-serra-mcp-discovery-uri/</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, October 2025; out-of-band HITL confirmation model is valuable and complements delegation frameworks. Likely expired (April 2026); worth tracking for a -01 refresh.</t>
+          <t>Already at revision -04 (March 2026), suggesting active iteration; narrow scope, clean design, and the strongest IANA-registration candidate in the set. OAuth 2.1 for auth is deliberately out of scope.</t>
         </is>
       </c>
     </row>
@@ -2185,27 +2185,27 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-payment-trust — Trust Scoring and Identity Verification for AI Agent Payment Transactions (SUPERSEDED)</t>
+          <t>draft-sharif-attp — ATTP: Agent Trust Transport Protocol</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft introducing an Agent Passport — a cryptographic delegation certificate intended to serve as the PSD2 'something you have' factor — and a trust-scoring model for payment transactions mapped to PCI DSS v4.0.1.</t>
+          <t>An IETF individual draft defining trust levels L0–L4 mapped to PSD2 Strong Customer Authentication requirements, with bindings for MCP (MCPS), REST, A2A, gRPC, and GraphQL; supersedes draft-sharif-agent-payment-trust.</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-payment-trust/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-attp/</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual, superseded)</t>
+          <t>IETF (individual)</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>SUPERSEDED by draft-sharif-attp-00 (April 2026). Retained for historical context — the Agent Passport concept is interesting but needs formal grounding; the ATTP successor generalizes it across transport bindings.</t>
+          <t>Revision -00, April 2026; regulatory mapping appendices (PSD2, PCI DSS) are notable — one of the few drafts engaging financial regulation directly. Ambitious scope. Part of the Sharif cluster.</t>
         </is>
       </c>
     </row>
@@ -2215,17 +2215,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>draft-stephan-ai-agent-6g — AI Agent Protocols for 6G Systems</t>
+          <t>draft-sharif-agent-transport-protocol — Agent Transport Protocol (ATP): Async Store-and-Forward for AI Agents</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft translating use cases and service requirements from 3GPP TR 22.870 into IETF agent-protocol requirements, covering autonomous vehicles, privacy preservation, and anomaly detection.</t>
+          <t>An IETF individual draft defining async store-and-forward messaging semantics with cryptographic identity per relay hop, trust scoring at ingress, capability negotiation, and interop with Google A2A, MCP, and FIPA ACL; transport-agnostic over TCP/TLS/QUIC.</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-stephan-ai-agent-6g/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-transport-protocol/</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, October 2025; strong operator backing (Orange, Deutsche Telekom, Telefonica, China Mobile, Huawei). Requirements-oriented and important for 3GPP/IETF coordination. May be expired (April 2026); watch for an update.</t>
+          <t>Revision -00, 28 March 2026; addresses a real gap — most agent protocols assume synchronous availability, and store-and-forward is appropriate for long-running agentic tasks. Scope is broad and needs narrowing.</t>
         </is>
       </c>
     </row>
@@ -2245,17 +2245,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>draft-jimenez-t2trg-iot-agent — Agentic AI Operation of Constrained RESTful Environments</t>
+          <t>draft-sharif-agent-audit-trail — Agent Audit Trail (AAT): Standard Logging Format for Autonomous AI Systems</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft (T2TRG affiliated) describing agentic AI (ReAct, smolagents) operating on CoAP/CoRE constrained-IoT environments, with a reference implementation provided.</t>
+          <t>An IETF individual draft defining a JSON-based audit record with mandatory fields (agent identity, action classification, outcome tracking, trust level) using RFC 8785 JSON Canonicalization and RFC 9562 UUIDs.</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jimenez-t2trg-iot-agent/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-audit-trail/</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 14 April 2026; unique in targeting constrained IoT environments. T2TRG affiliation and reference implementation are positive signals. Niche but fills an unaddressed gap.</t>
+          <t>Revision -00, 29 March 2026; orthogonal to delegation but important for compliance — standardized audit-log format is a genuine gap. Complements identity frameworks well. A sibling/alternative to the Kuehlewind audit architecture which takes a far more ambitious cross-layer approach.</t>
         </is>
       </c>
     </row>
@@ -2275,17 +2275,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>draft-li-oauth-delegated-authorization — OAuth 2.0 Delegated Authorization</t>
+          <t>draft-aiendpoint-ai-discovery — The AI Discovery Endpoint</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Huawei authors that extends OAuth 2.0 with a hierarchical 'delegation token' model so a client can mint subordinate, narrowly-scoped access tokens for delegated parties.</t>
+          <t>An IETF individual draft defining a /.well-known/ai URI suffix for programmatic service capability discovery by AI agents — letting agents discover what an endpoint supports without having to parse human-oriented documentation; requests IANA well-known URI registration.</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-li-oauth-delegated-authorization/</t>
+          <t>https://datatracker.ietf.org/doc/draft-aiendpoint-ai-discovery/</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, March 2026 (Informational); directly addresses over-privileged tokens and is one of the few drafts using the literal term 'delegated authorization'.</t>
+          <t>Revision -00, March 2026; complementary to MCP discovery but broader (not MCP-specific). Needs differentiation from OpenAPI/service-description work to gain traction.</t>
         </is>
       </c>
     </row>
@@ -2305,17 +2305,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>draft-araut-oauth-transaction-tokens-for-agents — Transaction Tokens For Agents</t>
+          <t>draft-hood-independent-agtp — Agent Transfer Protocol (AGTP)</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Ashay Raut (Amazon) profiling Transaction Tokens for agent-based workflows by adding 'act' for the agent identity, an 'agentic_ctx' claim carrying agent_type/intent/allowed_actions/environment_constraints, RFC 9396 RAR integration, and an 'actchain' claim for multi-agent delegation lineage.</t>
+          <t>An IETF individual draft proposing a dedicated application-layer protocol for AI agent traffic on port 4480 (TCP/TLS and QUIC) with an agtp:// URI scheme, arguing that HTTP is insufficient because agent-generated intent-driven traffic is indistinguishable from human-initiated requests. Defines a Runtime Contract Negotiation Substrate (RCNS) with eighteen methods split into cognitive verbs (QUERY, DISCOVER, DESCRIBE, SUMMARIZE, PLAN, PROPOSE) and mechanics verbs (EXECUTE, DELEGATE, ESCALATE, CONFIRM, SUSPEND, NOTIFY), mandatory agent identity headers, and protocol-level authority scope declaration.</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-araut-oauth-transaction-tokens-for-agents/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-independent-agtp/</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Revision -01 (May 2026) under the new slug — re-slugged from draft-oauth-transaction-tokens-for-agents-06; the -06 added the actchain delegation lineage, RAR-driven agentic_ctx, and a TTS check that blocks chain-splicing attacks. Conservative extension of the WG Transaction Tokens draft and an easier path to standardization.</t>
+          <t>Revision -08 (26 May 2026); supersedes draft-hood-independent-atp. Companion specs in the same family: AGTP-API, AGTP-CERT, AGTP-MERCHANT, AGTP-IDENTIFIERS, AGTP-TRUST. Mandatory TLS 1.3+. Ambitious scope — a new transport layer rather than an HTTP profile. The cognitive/mechanics verb split is a distinctive design choice; contrasts with draft-sharif-agent-transport-protocol which layers async store-and-forward on top of existing transports rather than replacing them.</t>
         </is>
       </c>
     </row>
@@ -2335,17 +2335,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>draft-oauth-ai-agents-on-behalf-of-user — On-Behalf-Of User Authorization for AI Agents</t>
+          <t>draft-hood-agtp-ard — ARD Binding for AGTP: Agentic Resource Discovery over the Agent Transfer Protocol</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft adding requested_actor and actor_token parameters to the OAuth authorization-code flow so the user gives explicit consent per agent, with the resulting delegation chain documented in the access-token claims.</t>
+          <t>Specifies how Agentic Resource Discovery (ARD) composes with AGTP, defining a catalog entry type for ARD manifests, aligning AGTP's identity model with ARD's trustManifest, and providing an AGTP-native binding for publishing ARD catalogs over AGTP substrate rather than HTTPS.</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-oauth-ai-agents-on-behalf-of-user/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-ard/</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Revision -02 was submitted August 2025; likely due for -03 refresh. Builds naturally on RFC 6749 + RFC 8693 + RFC 7636 PKCE — one of the most 'IETF-ready' delegation drafts and a strong WG-adoption candidate after the OAuth recharter.</t>
+          <t>Revision -00, 18 Jun 2026; author: Chris Hood (Nomotic). Extends the AGTP family (draft-hood-independent-agtp in corpus). The trustManifest identity alignment is the piece relevant to the agent identity thread; the rest is transport-layer plumbing for AGTP deployments.</t>
         </is>
       </c>
     </row>
@@ -2365,17 +2365,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>draft-rosomakho-oauth-txn-challenge — OAuth Transaction Authorization Challenge</t>
+          <t>draft-ni-a2a-ai-agent-security-requirements — Security Requirements for AI Agents</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>An OAuth mechanism enabling protected resources to demand transaction-specific authorization through challenges. When a request involves an agent or automated workflow, the RS returns a challenge to the client; the client presents it to the AS, which validates it, obtains human approval, and issues an access token with RFC 9396 authorization_details describing the approved operation. Positions as complementary to RFC 9470 (Step-Up Authentication) — that spec handles authentication freshness; this one handles authorization specificity.</t>
+          <t>An IETF individual draft enumerating security requirements for AI agents, covering identity, authorization chaining across domains, and integration points with WIMSE, OAuth identity chaining, and the A2A OAuth profile.</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rosomakho-oauth-txn-challenge/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ni-a2a-ai-agent-security-requirements/</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, submitted 25 June 2026. Authors: Yaroslav Rosomakho (Zscaler), Brian Campbell (Ping Identity), Karl McGuinness (Independent), Pieter Kasselman (Defakto). Strong author lineup — Campbell is a prolific OAuth WG contributor, Kasselman co-authored Transaction Tokens and First-Party Apps, McGuinness brings the Mission-Bound OAuth context. The RS-initiated challenge model is distinct from ARAP (which operates at the PDP/PEP layer via AuthZEN) but addresses the same 'denial is not the end' problem — here at the OAuth RS/AS layer rather than the AuthZEN layer.</t>
+          <t>Revision -01, February 2026; essential scaffolding for an eventual AI-agent WG. Well-connected to existing IETF work and authored by Ni and Liu, who also lead the WIMSE AI-agent identity draft.</t>
         </is>
       </c>
     </row>
@@ -2395,17 +2395,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>draft-hardt-aauth-protocol — AAuth Protocol</t>
+          <t>draft-rosenberg-aiproto-framework — Framework, Use Cases and Requirements for AI Agent Protocols</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>A new clean-sheet authorization protocol from Dick Hardt (original OAuth author) defining proof-of-possession by default, resource-signed challenges, agent identity without pre-registration, deferred 202 responses, and AS-to-AS federation for the agent ecosystem.</t>
+          <t>An IETF individual draft providing a comprehensive AI-agent communications framework that covers user↔agent, agent↔API, and agent↔agent interactions; surveys MCP, A2A, and Agntcy; and sets the stage for IETF standards activity.</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hardt-aauth-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-framework/</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, April 2026; the design rationale section explicitly explains why AAuth is not GNAP, not OAuth, not DPoP and not mTLS — important read for anyone planning a new agent-auth stack.</t>
+          <t>Revision -00, October 2025; Rosenberg (Five9) and Jennings (Cisco) are credible long-time IETF contributors. Important landscape document but likely expired (April 2026); watch for a -01 refresh post-IETF 123.</t>
         </is>
       </c>
     </row>
@@ -2425,17 +2425,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>draft-chen-oauth-roadmap — Comprehensive Roadmap for OAuth 2.0 Standards and Drafts</t>
+          <t>draft-rosenberg-aiproto-cheq — CHEQ: A Protocol for Confirmation of AI Agent Decisions (HITL)</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>An IETF informational draft that maps the entire OAuth 2.0 ecosystem of RFCs, BCPs, and active drafts into functional layers from core to extensions to industry profiles.</t>
+          <t>An IETF individual draft defining an out-of-band Human-in-the-Loop confirmation protocol for agent tool calls, eliminating LLM-hallucination risk for consequential actions and enabling sensitive operations (e.g., banking) without exposing data to the agent.</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>https://www.ietf.org/archive/id/draft-chen-oauth-roadmap-00.html</t>
+          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-cheq/</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Brand-new -00 draft (May 2026); the single most useful index when starting work in this area.</t>
+          <t>Revision -00, October 2025; out-of-band HITL confirmation model is valuable and complements delegation frameworks. Likely expired (April 2026); worth tracking for a -01 refresh.</t>
         </is>
       </c>
     </row>
@@ -2455,25 +2455,985 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
+          <t>draft-sharif-agent-payment-trust — Trust Scoring and Identity Verification for AI Agent Payment Transactions (SUPERSEDED)</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>An IETF individual draft introducing an Agent Passport — a cryptographic delegation certificate intended to serve as the PSD2 'something you have' factor — and a trust-scoring model for payment transactions mapped to PCI DSS v4.0.1.</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-payment-trust/</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual, superseded)</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>SUPERSEDED by draft-sharif-attp-00 (April 2026). Retained for historical context — the Agent Passport concept is interesting but needs formal grounding; the ATTP successor generalizes it across transport bindings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>draft-stephan-ai-agent-6g — AI Agent Protocols for 6G Systems</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>An IETF individual draft translating use cases and service requirements from 3GPP TR 22.870 into IETF agent-protocol requirements, covering autonomous vehicles, privacy preservation, and anomaly detection.</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-stephan-ai-agent-6g/</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, October 2025; strong operator backing (Orange, Deutsche Telekom, Telefonica, China Mobile, Huawei). Requirements-oriented and important for 3GPP/IETF coordination. May be expired (April 2026); watch for an update.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>draft-jimenez-t2trg-iot-agent — Agentic AI Operation of Constrained RESTful Environments</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>An IETF individual draft (T2TRG affiliated) describing agentic AI (ReAct, smolagents) operating on CoAP/CoRE constrained-IoT environments, with a reference implementation provided.</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-jimenez-t2trg-iot-agent/</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 14 April 2026; unique in targeting constrained IoT environments. T2TRG affiliation and reference implementation are positive signals. Niche but fills an unaddressed gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>draft-li-oauth-delegated-authorization — OAuth 2.0 Delegated Authorization</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>An IETF individual draft from Huawei authors that extends OAuth 2.0 with a hierarchical 'delegation token' model so a client can mint subordinate, narrowly-scoped access tokens for delegated parties.</t>
+        </is>
+      </c>
+      <c r="D55" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-li-oauth-delegated-authorization/</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, March 2026 (Informational); directly addresses over-privileged tokens and is one of the few drafts using the literal term 'delegated authorization'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>draft-araut-oauth-transaction-tokens-for-agents — Transaction Tokens For Agents</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>An IETF individual draft from Ashay Raut (Amazon) profiling Transaction Tokens for agent-based workflows by adding 'act' for the agent identity, an 'agentic_ctx' claim carrying agent_type/intent/allowed_actions/environment_constraints, RFC 9396 RAR integration, and an 'actchain' claim for multi-agent delegation lineage.</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-araut-oauth-transaction-tokens-for-agents/</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01 (May 2026) under the new slug — re-slugged from draft-oauth-transaction-tokens-for-agents-06; the -06 added the actchain delegation lineage, RAR-driven agentic_ctx, and a TTS check that blocks chain-splicing attacks. Conservative extension of the WG Transaction Tokens draft and an easier path to standardization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>draft-oauth-ai-agents-on-behalf-of-user — On-Behalf-Of User Authorization for AI Agents</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>An IETF individual draft adding requested_actor and actor_token parameters to the OAuth authorization-code flow so the user gives explicit consent per agent, with the resulting delegation chain documented in the access-token claims.</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-oauth-ai-agents-on-behalf-of-user/</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02 was submitted August 2025; likely due for -03 refresh. Builds naturally on RFC 6749 + RFC 8693 + RFC 7636 PKCE — one of the most 'IETF-ready' delegation drafts and a strong WG-adoption candidate after the OAuth recharter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>draft-rosomakho-oauth-txn-challenge — OAuth Transaction Authorization Challenge</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>An OAuth mechanism enabling protected resources to demand transaction-specific authorization through challenges. When a request involves an agent or automated workflow, the RS returns a challenge to the client; the client presents it to the AS, which validates it, obtains human approval, and issues an access token with RFC 9396 authorization_details describing the approved operation. Positions as complementary to RFC 9470 (Step-Up Authentication) — that spec handles authentication freshness; this one handles authorization specificity.</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-rosomakho-oauth-txn-challenge/</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, submitted 25 June 2026. Authors: Yaroslav Rosomakho (Zscaler), Brian Campbell (Ping Identity), Karl McGuinness (Independent), Pieter Kasselman (Defakto). Strong author lineup — Campbell is a prolific OAuth WG contributor, Kasselman co-authored Transaction Tokens and First-Party Apps, McGuinness brings the Mission-Bound OAuth context. The RS-initiated challenge model is distinct from ARAP (which operates at the PDP/PEP layer via AuthZEN) but addresses the same 'denial is not the end' problem — here at the OAuth RS/AS layer rather than the AuthZEN layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>draft-lee-orprg-permit-receipts — Permit Receipts for Permit-Before-Commit Authorization</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Defines requirements and an abstract data model for PermitReceipts: a verifier evaluates canonicalized effect requests, action digests, policy epochs, validity intervals, and revocation status before any protected effect is committed at an effect boundary. Covers verifier behavior, failure semantics, and candidate registries.</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-lee-orprg-permit-receipts/</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 4 Jun 2026; author: Yong Bok Lee (Meridian Verity Group). The most complete standalone framework for pre-commit authorization in the current wave; intended to ground IETF discussion on scope and profiles. Seeks guidance on appropriate organizational placement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>draft-nelson-agent-delegation-receipts — Delegation Receipt Protocol for AI Agent Authorization</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Specifies the Delegation Receipt Protocol (DRP) where users sign Authorization Objects (containing scope boundaries, time constraints, instruction hashes, and model state commitments) that are published to an append-only log before the agent runtime gains control. Removes operators as trusted intermediaries by making the user's private key the sole signing authority.</t>
+        </is>
+      </c>
+      <c r="D60" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-nelson-agent-delegation-receipts/</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>Revision -10, 13 Jun 2026; author: Ryan Nelson (Authproof). At version 10, the most iterated individual draft in the pre-action authorization space. The commitment-before-execution architecture — sign before the agent runs, not after — is distinctive and directly addresses the prompt-injection attack surface.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>draft-williams-intent-token — The Intent Token: A Cryptographic Authorization Primitive for Autonomous Agents</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Specifies a cryptographic authorization primitive that binds an autonomous agent action to a cryptographically signed, human-declared authorization envelope before execution. Addresses the gap in OAuth 2.0 frameworks that govern access to resources but not what agents are permitted to do at the moment of action. Positioned as complementary to OAuth, not a replacement.</t>
+        </is>
+      </c>
+      <c r="D61" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-williams-intent-token/</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 22 Jun 2026; author: Jeffrey Williams (Independent). Overlaps conceptually with draft-kroehl-agentic-trust-aae and draft-nelson-agent-delegation-receipts; worth tracking as a lighter-weight alternative to both.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>draft-reece-wimse-cross-org-delegation — Cross-Organizational Delegation for Workload and Agent Identity</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>A problem statement and requirements draft identifying that existing workload and token-based authorization mechanisms were designed for a single trust domain, describing the cross-organizational agent delegation gap, and enumerating requirements for solutions — without proposing specific technical approaches.</t>
+        </is>
+      </c>
+      <c r="D62" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-reece-wimse-cross-org-delegation/</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 25 Jun 2026; author: Morgan Reece (TowerGuardian Consulting). The problem-statement companion to the corpus's operational drafts; likely to feed into WIMSE WG scope expansion and is directly in scope for draft-kuehlewind-audit-architecture's composition graph.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>draft-jiang-wimse-heterogeneous-credential — Heterogeneous Credential Verification for Workload and Agentic Systems</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Specifies mechanisms for representing credential sets, identifying credential types, determining appropriate verifiers, normalizing verification results across different formats (workload tokens, OAuth, X.509, attestation), and combining results into a single handling decision.</t>
+        </is>
+      </c>
+      <c r="D63" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-jiang-wimse-heterogeneous-credential/</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 23 Jun 2026; authors: Yuning Jiang, Donghui Wang, Yurong Song, Faye Liu (Huawei). Solves the practical problem of agentic systems receiving credentials in multiple formats from different issuers. Fills a gap left by draft-ni-wimse-ai-agent-identity (corpus) which describes the identity problem but not multi-format credential handling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>draft-munoz-wimse-authorization-evidence — Signed Authorization-Evidence Records for WIMSE-Authorized AI Agent Actions</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Specifies a signed authorization-evidence record (Permit) for WIMSE-authorized AI actions, cryptographically binding to the dispatched request bytes via HTTP Message Signatures, OAuth access tokens, and Shared Signals Framework eventing — without modifying existing standards.</t>
+        </is>
+      </c>
+      <c r="D64" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-munoz-wimse-authorization-evidence/</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 15 May 2026; author: Christian Munoz (Keel API). Profiles WIMSE for AI agent actions and satisfies audit requirements; companion to the SCITT permit profile below. Extends the corpus WIMSE thread (draft-ni-wimse-ai-agent-identity) with a concrete evidence artifact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>draft-munoz-scitt-permit-profile — A SCITT Profile for Pre-Execution AI Action Authorization Records</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>SCITT profile for the Pre-Execution Authorization Record (Permit), documenting policy-evaluated decisions before AI agent action dispatch with cryptographic binding proving 'authorized request equals dispatched request.' Composes with adjacent profiles for human-authority binding, post-execution evidence, and content-refusal events via referencing mechanisms.</t>
+        </is>
+      </c>
+      <c r="D65" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-munoz-scitt-permit-profile/</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 15 May 2026; author: Christian Munoz (Keel API). SCITT-anchored analog of the WIMSE evidence record; companion to draft-munoz-wimse-authorization-evidence from the same author. Connects to draft-sharif-agent-audit-trail and draft-kuehlewind-audit-architecture (both in corpus).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>draft-marques-asqav-compliance-receipts — Compliance Profile of Signed Action Receipts for AI Agents</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Establishes a compliance framework for signed action receipts from AI agents, mandating specific fields, cryptographic anchoring, hash-chain linkage, risk/incident classification, cross-agent envelope binding, and enforcement attestation with retention floors tied to EU AI Act, DORA, NIST AI RMF, HIPAA, SEC Rule 17a-4, and CIRCIA.</t>
+        </is>
+      </c>
+      <c r="D66" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-marques-asqav-compliance-receipts/</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>Revision -05, 31 May 2026; author: João André Gomes Marques. The most legally grounded receipt profile in the wave — at revision 05, relatively mature. Complements draft-sharif-agent-audit-trail (corpus) with a multi-regulation compliance overlay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>draft-mih-scitt-agent-action-capsule — An Agent Action Capsule Profile for SCITT</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Defines a SCITT statement profile (Agent Action Capsule) documenting agent actions with outcome status (executed, blocked, denied, errored, timed out), evaluated constraints, committed-effect binding, and a human-in-the-loop flag; records a Capsule for every verdict including refusals. COSE Signed Statement format; registrable in SCITT Transparency Services.</t>
+        </is>
+      </c>
+      <c r="D67" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-mih-scitt-agent-action-capsule/</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 19 Jun 2026; author: Steven Mih (Action State Group). Provides auditor-grade evidence that decision gates functioned. The HITL flag directly tracks the corpus theme; the most complete single-draft SCITT audit story in this batch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>draft-car-rer-artifact — RER Run Artifact Format: Hash-Chained, Signed Records of AI Inference Execution</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Specifies a cryptographically signed JSON record for AI inference runs including a signed envelope declaring permissions and limits, a hash-chained event log covering all model and tool calls, and a runtime signature binding envelope and log to the producing implementation. Enables offline verification by parties uninvolved in the original run.</t>
+        </is>
+      </c>
+      <c r="D68" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-car-rer-artifact/</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 12 Jun 2026; author: Kayla Cardillo (Tech Enrichment). Relevant for post-hoc audit of what permissions an agent claimed during execution; companion to the SCITT profiles but more focused on inference traceability than authorization decisions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>draft-noa-scitt-ai-agent-receipt — A SCITT Profile for AI-Agent Action Receipts</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Defines a minimal SCITT profile: COSE_Sign1 Signed Statements with canonicalized payloads, hash-chained for ordering, registrable in SCITT Transparency Services. Explicitly does NOT assert agent correctness, safety, or real-world outcomes — only tamper-evident, signature-verifiable records of action, principal, policy identity, and verdict.</t>
+        </is>
+      </c>
+      <c r="D69" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-noa-scitt-ai-agent-receipt/</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 23 Jun 2026; author: Tora Toraman (NordenSoft). The minimalist end of the SCITT profile spectrum; useful for corpus completeness alongside the more comprehensive draft-mih-scitt-agent-action-capsule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>draft-sato-soos-mjwt — The Mandate JWT (MJWT) for Agentic AI Systems</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Introduces the Mandate JWT — a WIMSE workload credential profile binding agent authority to specific Sovereign Object instances under named human principals, with cryptographically enforced delegation ceilings and a six-dimensional Narrowing Property preventing sub-agents from exceeding root authority.</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-mjwt/</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). The authorization token primitive for the SOOS governance protocol family. Directly comparable to draft-mcguinness-oauth-client-instance-assertion but uses a WIMSE/Sovereign Object substrate rather than OAuth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>draft-sato-soos-mad — Multi-Agent Delegation in Sovereign Object Systems</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Specifies three core mechanisms for multi-agent delegation accountability: the Narrowing Property (capability non-amplification), five formally defined object topology patterns for runtime relationships, and cluster coordination primitives for parallel execution with aggregation rules. Version 02 adds revocation-during-execution handling and partial-completion routing to human oversight.</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-mad/</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). Claims to address gaps the OpenID Foundation identifies as unsolved in multi-agent authorization. The five topology patterns are a useful vocabulary for describing agent-to-agent relationship structures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>draft-sato-soos-hem — The Human Escalation Mechanism (HEM) for Agentic AI Systems</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Defines a kernel-enforced mechanism placing agent sessions in a pending state when human judgment is required, routing structured escalation requests to designated human decision-makers, and prohibiting all state transitions until a human decision is received. Defines five decision types and a dual-layer architecture (LLM-HEM and SOOS-HEM).</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-hem/</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>Revision -04, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). The most normative HITL protocol in the current wave; explicitly aligns with EU AI Act Article 14 requirements for high-risk AI system oversight. Counterpart to ARAP (AuthZEN WG) at the protocol level vs. the OAuth/AuthZEN layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>draft-sato-soos-idp — The Intent Declaration Primitive (IDP) for Agentic AI Systems</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Specifies a structured declaration mechanism committing AI agent intent to tamper-evident logs before actions are taken, enabling post-hoc review and EU AI Act Article 12 compliance for high-risk systems.</t>
+        </is>
+      </c>
+      <c r="D73" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-idp/</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>Revision -04, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). The log-before-execute pattern mirrors draft-nelson-agent-delegation-receipts but operates at the intent declaration level rather than the user-authorization level. Pairs with GAR (below) to form a complete pre/post audit trail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>draft-sato-soos-gar — The Governance Audit Record (GAR) for Agentic AI Systems</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Defines GAR, an audit framework with five audit types, a Session Audit Record, and an Audit Alert mechanism; collects, signs, and makes governance events from IDP, HEM, and associated SOOS primitives available for regulatory inspection via an append-only, non-suppressible SCITT-anchored audit stream with Authority Lifecycle Events covering the complete revocation-recovery cycle.</t>
+        </is>
+      </c>
+      <c r="D74" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-gar/</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). The integrator for the SOOS family, analogous to how draft-kuehlewind-audit-architecture (in corpus) integrates the broader IETF agent draft landscape. SCITT-anchored audit stream is a concrete architectural choice distinguishing it from the Kuehlewind approach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>draft-jiang-intent-security — Security Considerations and Requirements for Intent-Based Requests in Agentic Systems</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Solution-agnostic threat analysis covering tampering, privilege escalation, constraint violations, and intent drift in intent-based agentic systems, with a reference model, attack scenarios, and security requirements covering authentication, admission control, constraint validation, and multi-hop integrity.</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-jiang-intent-security/</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>Revision -03, 22 Jun 2026; authors: Yuning Jiang, Lun Li, Yurong Song, Faye Liu (Huawei). The threat-model companion to draft-jiang-oauth-intent-admission from the same group; likely intended to inform the broader IETF agentic AI security discussion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>draft-somoza-dmsc-atn-agent-trust-negotiation — Agent Trust Negotiation: Capability, Delegation, and Provenance Binding</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Specifies the Agent Trust Negotiation (ATN) protocol, which binds four artifacts — capability manifests, delegation chains, provenance attestations, and session receipts — to agent identities via a handshake state machine producing mutually verified, scope-bounded sessions with SCITT-suitable audit records.</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-somoza-dmsc-atn-agent-trust-negotiation/</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 29 May 2026; author: Enrique Somoza (Independent). Operates above discovery mechanisms and positions itself between the discovery layer (DAWN, MCP) and the authorization layer (WIMSE, OAuth). Relevant as an agent-to-agent trust establishment handshake protocol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>draft-mcgraw-httpapi-agent-budget — The Delegation HTTP Authentication Scheme for Request-Bound Authority</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>Defines the 'Delegation' HTTP authentication scheme and response semantics for delegated-authority challenges using HTTP status codes and Problem Details, plus a CBOR/COSE proof format. The initial authority profile is 'Budget,' using post-quantum ML-DSA to prove spending or resource-consumption limits.</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-mcgraw-httpapi-agent-budget/</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, 15 Jun 2026; author: John Paul McGraw Jr. (TaskHawk Systems). HTTP-layer bounded delegation with post-quantum crypto; distinct from OAuth-layer delegation in that the authority proof travels in the Authorization header. Complements x401 (Industry tab) at the HTTP challenge-response layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>draft-vauban-x402-delegation-binding — x402 Delegation Binding for Agentic HTTP Pipelines</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Addresses the security gap where x402 V2 payment grants issued to one agent could be misused by another in the same pipeline, introducing three binding mechanisms: a JCS-derived agent identity pseudonym, a nonce for anti-replay, and a depth-limiting field for transitive delegation.</t>
+        </is>
+      </c>
+      <c r="D78" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-vauban-x402-delegation-binding/</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 25 May 2026; author: Vauban Research. Narrowly scoped to payment pipelines but the delegation-binding pattern (pseudonymous identity + anti-replay + depth-limit) is applicable broadly. Validated across five language runtimes with A2A and MCP integration guidance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>draft-samal-vap — Verifiable Agent Protocol (VAP): Intent-Bound Admission Control and Audit for Agent Tool Invocation</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Specifies VAP as a defense-in-depth layer adding declarations of purpose and session budget commitments to tool invocation requests (targeting MCP-style protocols), enabling servers to perform admission control before execution via four messages carried in existing protocol metadata.</t>
+        </is>
+      </c>
+      <c r="D79" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-samal-vap/</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 3 Jun 2026; author: Kruttidipta Samal (Independent). Lightweight and protocol-agnostic; addresses erroneous agent behavior, cost control, and audit trails without replacing existing auth mechanisms. Practical tool-invocation-level authorization layer for MCP deployments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>draft-khera-aurora — Agent Unification, Runtime, and Operational Responsibility Attestation (AURORA)</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>A two-layer framework unifying hardware-enclave-backed Runtime Integrity Attestation with scoped, cryptographically bound Authority Delegation; enables agents to prove both operational authority and runtime integrity simultaneously.</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-khera-aurora/</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 5 Jun 2026; author: Ankur Khera. Addresses the gap where delegation tokens don't prove the runtime environment is trustworthy — relevant where delegation must be paired with platform attestation (enterprise/regulated deployments). Bridges the RATS attestation thread and the OAuth delegation thread.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>draft-borthwick-msebenzi-environment-state — Verifiable Intent — environment.* Constraint Family</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>Defines the environment.* constraint family for agent-authorization mandate vocabularies, covering external conditions at transaction execution time (venue availability, wallet funding) that existing transactional constraints cannot address. Extends agent authorization mandate frameworks with environmental precondition checking.</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-borthwick-msebenzi-environment-state/</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 13 Jun 2026; authors: Douglas Cameron Borthwick (InsumerAPI), Michael Msebenzi (Headless Oracle). Narrow but practically important for financial and commerce agent workflows; connects to draft-mcgraw-httpapi-agent-budget and draft-vauban-x402-delegation-binding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>draft-hardt-aauth-protocol — AAuth Protocol</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>A new clean-sheet authorization protocol from Dick Hardt (original OAuth author) defining proof-of-possession by default, resource-signed challenges, agent identity without pre-registration, deferred 202 responses, and AS-to-AS federation for the agent ecosystem.</t>
+        </is>
+      </c>
+      <c r="D82" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-hardt-aauth-protocol/</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, April 2026; the design rationale section explicitly explains why AAuth is not GNAP, not OAuth, not DPoP and not mTLS — important read for anyone planning a new agent-auth stack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>draft-chen-oauth-roadmap — Comprehensive Roadmap for OAuth 2.0 Standards and Drafts</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>An IETF informational draft that maps the entire OAuth 2.0 ecosystem of RFCs, BCPs, and active drafts into functional layers from core to extensions to industry profiles.</t>
+        </is>
+      </c>
+      <c r="D83" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ietf.org/archive/id/draft-chen-oauth-roadmap-00.html</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>Brand-new -00 draft (May 2026); the single most useful index when starting work in this area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
           <t>Charter: WIMSE — Workload Identity in Multi-System Environments (charter-ietf-wimse-01)</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C84" s="5" t="inlineStr">
         <is>
           <t>The formal IETF charter for the WIMSE WG covering architecture, JOSE-based WIMSE tokens for service-to-service traffic, local token issuance, and token exchange profiles (likely based on RFC 8693) for cross-trust-domain workload identity.</t>
         </is>
       </c>
-      <c r="D52" s="9" t="inlineStr">
+      <c r="D84" s="9" t="inlineStr">
         <is>
           <t>https://datatracker.ietf.org/doc/charter-ietf-wimse/01/</t>
         </is>
       </c>
-      <c r="E52" s="5" t="inlineStr">
+      <c r="E84" s="5" t="inlineStr">
         <is>
           <t>IETF (WIMSE WG charter)</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
+      <c r="F84" s="5" t="inlineStr">
         <is>
           <t>Approved 18 March 2026 (v01); explicitly liaises with OAuth, SCIM, SCITT, RATS, the OpenID Foundation, and CNCF/SPIFFE — the formal scope statement that anchors all WIMSE draft work.</t>
         </is>
@@ -2532,6 +3492,38 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId83"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added ACLX governance framework
</commit_message>
<xml_diff>
--- a/delegated_authorization_research.xlsx
+++ b/delegated_authorization_research.xlsx
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="6" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D11" s="7" t="n"/>
     </row>
@@ -4385,7 +4385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5385,6 +5385,36 @@
       <c r="F33" s="5" t="inlineStr">
         <is>
           <t>Curity is a member of the AuthZEN WG; positions AuthZEN as 'OpenID Connect for authorization' which has become the common framing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>ACLX — AI Output Governance (Proprietary)</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>A proprietary enforcement layer that intercepts AI-generated content between inference and delivery, evaluating it against OPA/Cedar policies, identity context, and a three-phase sensitivity detection stack: deterministic regex rules → ontology-based compilation-risk scoring → semantic LLM evaluation for novel synthesis. Four enforcement outcomes: ALLOW, REDACT, BLOCK, or ESCALATE to human review. Treats agents as first-class principals evaluated at the output boundary regardless of whether a session or IDP exists.</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>https://aclx.ai/</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Proprietary product</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>No published specification. Identifies a gap the corpus standards map does not yet cover: identity (OIDC/SCIM/SPIFFE), signals (CAEP/SSF), policy (OAuth/AuthZEN/OPA), and enforcement (ZTA/RATS/SCITT) all have standards, but output evaluation — governing what the AI synthesizes rather than what the user was authorized to ask — has none. The synthesis-detection layer (AI compiling across individually-authorized sources to produce content crossing a higher sensitivity boundary) is a novel problem the corpus's existing standards do not address.</t>
         </is>
       </c>
     </row>
@@ -5422,6 +5452,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated with recent IETF datatracker updates
</commit_message>
<xml_diff>
--- a/delegated_authorization_research.xlsx
+++ b/delegated_authorization_research.xlsx
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="6" t="n">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="D11" s="7" t="n"/>
     </row>
@@ -906,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:F94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Active WG draft (-08, expires Aug 2026); the canonical multi-domain delegation pattern referenced by most agent and zero-trust drafts.</t>
+          <t>IESG-approved; currently in RFC Editor queue (status: Waiting on Authors — outstanding SECDIR 'Has issues' and OPSDIR 'Not ready' flags unresolved; no RFC number assigned yet as of Jul 2026). The canonical multi-domain delegation pattern referenced by most agent and zero-trust drafts.</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Revision -08 published March 2026; co-authored by Tulshibagwale (CAEP inventor), Fletcher, and Kasselman — pairs with AuthZEN/CAEP for zero-trust microservices.</t>
+          <t>Revision -09 published 6 Jul 2026 (was -08 Mar 2026); co-authored by Tulshibagwale (CAEP inventor), Fletcher, and Kasselman. -09 reorganized the Request Context section, changed JWT body claims from OPTIONAL to RECOMMENDED, and enhanced security considerations for invalidated access tokens. Still in WGLC; IESG submission milestone Dec 2026.</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>97-page -00 submitted 1 May 2026 (re-slugged from draft-mw-spice-actor-chain-05); a complementary alternative to the McGuinness Actor Profile that directly addresses RFC 8693's chain-splicing weakness by making the chain itself cryptographically verifiable rather than just informational.</t>
+          <t>Revision -01, 30 Jun 2026 (was -00 May 2026; re-slugged from draft-mw-spice-actor-chain-05); a complementary alternative to the McGuinness Actor Profile that directly addresses RFC 8693's chain-splicing weakness by making the chain itself cryptographically verifiable rather than just informational.</t>
         </is>
       </c>
     </row>
@@ -1565,17 +1565,17 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>https://mcguinness.github.io/draft-mcguinness-oauth-actor-profile/draft-mcguinness-oauth-actor-receipts.html</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-actor-receipts/</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Pre-publication (author's GitHub)</t>
+          <t>IETF (individual)</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>NOT YET ON DATATRACKER. McGuinness described it on the OAUTH-WG list on 1 May 2026 as 'a very early work in progress'. Recommended companion to the Actor Profile when a deployment needs Verified Full Disclosure mode (per the Mission-Bound OAuth Runtime Enforcement Profile's Actor Provenance Module). Watch for an IETF submission later in 2026.</t>
+          <t>Revision -00, 4 Jul 2026; now formally on IETF Datatracker (was GitHub-only pre-publication through Jun 2026). Recommended companion to the Actor Profile when a deployment needs Verified Full Disclosure mode (per the Mission-Bound OAuth Runtime Enforcement Profile's Actor Provenance Module). Completes a triad with actor-profile and actor-proofs — receipts provide provenance, proofs provide cryptographic per-hop accountability.</t>
         </is>
       </c>
     </row>
@@ -1585,17 +1585,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-insufficient-claims — OAuth 2.0 Insufficient Claims Challenge</t>
+          <t>draft-mcguinness-oauth-actor-proofs — OAuth Actor-Signed Hop Proofs</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>A McGuinness individual draft defining an insufficient_claims error code and required_claims parameter enabling authorization servers and protected resources to signal precisely which claims are missing from a presented credential. Allows resource servers to request enriched credentials carrying specific missing attributes rather than returning a generic 401.</t>
+          <t>Introduces the 'actor_proofs' claim — a signed per-hop proof chain where each actor signs its own participation and the target binding it authorized for that hop; proofs are hash-chained and validated using actor verification keys from trusted sources, with optional references to sibling actor receipts.</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-insufficient-claims/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-actor-proofs/</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 27 May 2026. Enables just-in-time claim negotiation in multi-agent delegation chains where the acting party must assemble claims from multiple sources. Natural companion to the Actor Profile and Client Instance Assertion — those drafts define the identity structure; this one provides the feedback loop when that structure is incomplete at the RS.</t>
+          <t>Revision -00, 4 Jul 2026; McGuinness's 7th individual I-D on IETF Datatracker. Completes the actor triad with actor-profile (chain structure) and actor-receipts (provenance) — actor-proofs closes the cryptographic accountability gap. Was not previously on the Pending Watch List; a new design direction beyond the original Mission-Bound OAuth blog series.</t>
         </is>
       </c>
     </row>
@@ -1615,17 +1615,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>draft-mishra-oauth-agent-grants — Delegated Agent Authorization Protocol (DAAP)</t>
+          <t>draft-mcguinness-oauth-insufficient-claims — OAuth 2.0 Insufficient Claims Challenge</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft addressing runtime agent identity for dynamically-spawned agents, multi-agent sub-delegation with depth-limiting, and cascade revocation of an entire delegation subtree when any ancestor is revoked.</t>
+          <t>A McGuinness individual draft defining an insufficient_claims error code and required_claims parameter enabling authorization servers and protected resources to signal precisely which claims are missing from a presented credential. Allows resource servers to request enriched credentials carrying specific missing attributes rather than returning a generic 401.</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mishra-oauth-agent-grants/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-insufficient-claims/</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Revision -01 (March 2026); registers new JWT claims (agt, dev, grnt, scp, bdg) — a more aggressive alternative to RFC 8693 with budget-bounded grants. Overlaps with draft-niyikiza-oauth-attenuating-agent-tokens; OAuth WG will likely expect consolidation.</t>
+          <t>Revision -00, 27 May 2026. Enables just-in-time claim negotiation in multi-agent delegation chains where the acting party must assemble claims from multiple sources. Natural companion to the Actor Profile and Client Instance Assertion — those drafts define the identity structure; this one provides the feedback loop when that structure is incomplete at the RS.</t>
         </is>
       </c>
     </row>
@@ -1645,17 +1645,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>draft-kuehlewind-audit-architecture — Architecture for Auditing AI Agent Delegation and Interactions</t>
+          <t>draft-mishra-oauth-agent-grants — Delegated Agent Authorization Protocol (DAAP)</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Mirja Kühlewind (Ericsson, former IETF TSV-AD) and Henk Birkholz (Fraunhofer SIT, lead author of RFC 9334 RATS and SCITT architecture) defining four record types — Interaction, Action, Delegation, and Authorization Transition — and an Audit Context that propagates across OAuth + WIMSE + RATS + SCITT to make agent behaviour verifiably auditable end-to-end.</t>
+          <t>An IETF individual draft addressing runtime agent identity for dynamically-spawned agents, multi-agent sub-delegation with depth-limiting, and cascade revocation of an entire delegation subtree when any ancestor is revoked.</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-kuehlewind-audit-architecture/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mishra-oauth-agent-grants/</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Revision -00 published 18 May 2026; the cross-layer integration piece — explicitly composes the McGuinness Actor Profile, Transaction Tokens, identity-chaining, ID-JAG, WIMSE, RATS, and SCITT into a single auditable architecture with 11 proposed work items. The treats-Agent-as-untrusted threat model is what regulators (SOX, PSD2, EU AI Act) actually want.</t>
+          <t>Revision -01 (March 2026); registers new JWT claims (agt, dev, grnt, scp, bdg) — a more aggressive alternative to RFC 8693 with budget-bounded grants. Overlaps with draft-niyikiza-oauth-attenuating-agent-tokens; OAuth WG will likely expect consolidation.</t>
         </is>
       </c>
     </row>
@@ -1675,17 +1675,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>draft-birkholz-verifiable-agent-conversations — Verifiable Agent Conversation Records</t>
+          <t>draft-kuehlewind-audit-architecture — Architecture for Auditing AI Agent Delegation and Interactions</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft (Birkholz/Heldt/Steele) defining a CDDL data format — with both JSON and CBOR encodings — for tamper-evident, verifiably-signed records of agent conversations, agent reasoning traces, tool calls, and system events that support long-term evidentiary value across chains of custody.</t>
+          <t>An IETF individual draft from Mirja Kühlewind (Ericsson, former IETF TSV-AD) and Henk Birkholz (Fraunhofer SIT, lead author of RFC 9334 RATS and SCITT architecture) defining four record types — Interaction, Action, Delegation, and Authorization Transition — and an Audit Context that propagates across OAuth + WIMSE + RATS + SCITT to make agent behaviour verifiably auditable end-to-end.</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-birkholz-verifiable-agent-conversations/</t>
+          <t>https://datatracker.ietf.org/doc/draft-kuehlewind-audit-architecture/</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Revision -00 published 25 Feb 2026; presented at IETF 125 dispatch and hotrfc. The canonical Interaction-Record format for the Kuehlewind audit architecture. Motivating examples are concrete: agents acting beyond scope, CoT divergence, and 'sandbagging' during evaluations.</t>
+          <t>Revision -00 published 18 May 2026; the cross-layer integration piece — explicitly composes the McGuinness Actor Profile, Transaction Tokens, identity-chaining, ID-JAG, WIMSE, RATS, and SCITT into a single auditable architecture with 11 proposed work items. The treats-Agent-as-untrusted threat model is what regulators (SOX, PSD2, EU AI Act) actually want.</t>
         </is>
       </c>
     </row>
@@ -1705,17 +1705,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>draft-klrc-aiagent-auth — AI Agent Authentication and Authorization</t>
+          <t>draft-birkholz-verifiable-agent-conversations — Verifiable Agent Conversation Records</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft that does not invent new protocols but composes WIMSE/SPIFFE workload identity, OAuth 2.x, and OpenID SSF to authenticate and delegate authority to AI agents.</t>
+          <t>An IETF individual draft (Birkholz/Heldt/Steele) defining a CDDL data format — with both JSON and CBOR encodings — for tamper-evident, verifiably-signed records of agent conversations, agent reasoning traces, tool calls, and system events that support long-term evidentiary value across chains of custody.</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/html/draft-klrc-aiagent-auth-00</t>
+          <t>https://datatracker.ietf.org/doc/draft-birkholz-verifiable-agent-conversations/</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, March 2026; introduces 'Agent Identity Management System (AIMS)' and is the cleanest standards-based framing of agent-as-workload.</t>
+          <t>Revision -00 published 25 Feb 2026; presented at IETF 125 dispatch and hotrfc. The canonical Interaction-Record format for the Kuehlewind audit architecture. Motivating examples are concrete: agents acting beyond scope, CoT divergence, and 'sandbagging' during evaluations.</t>
         </is>
       </c>
     </row>
@@ -1735,17 +1735,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>draft-niyikiza-oauth-attenuating-agent-tokens — Attenuating Authorization Tokens for Agentic Delegation Chains</t>
+          <t>draft-klrc-aiagent-auth — AI Agent Authentication and Authorization</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft extending RFC 9396 Rich Authorization Requests with monotonic attenuation at each delegation hop, offline chain verification, and a typed constraint vocabulary for tool-level argument restrictions.</t>
+          <t>An IETF individual draft that does not invent new protocols but composes WIMSE/SPIFFE workload identity, OAuth 2.x, and OpenID SSF to authenticate and delegate authority to AI agents.</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-niyikiza-oauth-attenuating-agent-tokens/</t>
+          <t>https://datatracker.ietf.org/doc/html/draft-klrc-aiagent-auth-00</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, March 2026; arguably the strongest purely-OAuth-grounded delegation draft — offline verification is a key scalability property. Good path to OAuth WG adoption; overlaps with draft-mishra-oauth-agent-grants and will likely need to be consolidated with it.</t>
+          <t>Revision -00, March 2026; introduces 'Agent Identity Management System (AIMS)' and is the cleanest standards-based framing of agent-as-workload.</t>
         </is>
       </c>
     </row>
@@ -1765,17 +1765,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>draft-singla-agent-identity-protocol — AIP: Decentralized Identity and Delegation for AI Agents</t>
+          <t>draft-niyikiza-oauth-attenuating-agent-tokens — Attenuating Authorization Tokens for Agentic Delegation Chains</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft proposing a six-layer model (identity through reputation) for AI agents with W3C DID anchoring, a Delegation Depth counter, three Grant ceremony tiers (G1/G2/G3), DPoP proof-of-possession, and an MCP integration layer.</t>
+          <t>An IETF individual draft extending RFC 9396 Rich Authorization Requests with monotonic attenuation at each delegation hop, offline chain verification, and a typed constraint vocabulary for tool-level argument restrictions.</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-singla-agent-identity-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-niyikiza-oauth-attenuating-agent-tokens/</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 17 April 2026; the most comprehensive identity framework in the set. The W3C DID dependency will face IETF pushback, the 75+ page scope needs reduction, and the 'AIP' name collision with two other drafts (draft-prakash-aip, draft-aip-agent-identity-protocol) must be resolved.</t>
+          <t>Revision -00, March 2026; arguably the strongest purely-OAuth-grounded delegation draft — offline verification is a key scalability property. Good path to OAuth WG adoption; overlaps with draft-mishra-oauth-agent-grants and will likely need to be consolidated with it.</t>
         </is>
       </c>
     </row>
@@ -1795,17 +1795,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>draft-prakash-aip — AIP: Verifiable Delegation for AI Agent Systems</t>
+          <t>draft-singla-agent-identity-protocol — AIP: Decentralized Identity and Delegation for AI Agents</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft introducing Invocation-Bound Capability Tokens (IBCTs) in two modes — compact (JWT/Ed25519) for single-hop and chained (Biscuit + Datalog) for multi-hop — with bindings for MCP, A2A, and HTTP APIs.</t>
+          <t>An IETF individual draft proposing a six-layer model (identity through reputation) for AI agents with W3C DID anchoring, a Delegation Depth counter, three Grant ceremony tiers (G1/G2/G3), DPoP proof-of-possession, and an MCP integration layer.</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-prakash-aip/</t>
+          <t>https://datatracker.ietf.org/doc/draft-singla-agent-identity-protocol/</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 27 March 2026; technically strong — Biscuit + Datalog is well-suited to scope attenuation. The 'AIP' name collision with draft-singla-agent-identity-protocol and draft-aip-agent-identity-protocol is a blocking issue for WG adoption.</t>
+          <t>Revision -00, 17 April 2026; the most comprehensive identity framework in the set. The W3C DID dependency will face IETF pushback, the 75+ page scope needs reduction, and the 'AIP' name collision with two other drafts (draft-prakash-aip, draft-aip-agent-identity-protocol) must be resolved.</t>
         </is>
       </c>
     </row>
@@ -1825,17 +1825,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>draft-goswami-agentic-jwt — Secure Intent Protocol: JWT-Compatible Agentic Identity and Workflow Management</t>
+          <t>draft-prakash-aip — AIP: Verifiable Delegation for AI Agent Systems</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an Agentic JWT extension to OAuth 2.0 with a Supervisor Agent role for sub-agent coordination, explicitly addressing the 'intent-execution separation' gap and adding workflow-step authorization.</t>
+          <t>An IETF individual draft introducing Invocation-Bound Capability Tokens (IBCTs) in two modes — compact (JWT/Ed25519) for single-hop and chained (Biscuit + Datalog) for multi-hop — with bindings for MCP, A2A, and HTTP APIs.</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-goswami-agentic-jwt/</t>
+          <t>https://datatracker.ietf.org/doc/draft-prakash-aip/</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, December 2025; the intent-execution-separation framing is insightful and distinguishing. The workflow-step authorization approach is novel but may face skepticism in the OAuth WG.</t>
+          <t>Revision -00, 27 March 2026; technically strong — Biscuit + Datalog is well-suited to scope attenuation. The 'AIP' name collision with draft-singla-agent-identity-protocol and draft-aip-agent-identity-protocol is a blocking issue for WG adoption.</t>
         </is>
       </c>
     </row>
@@ -1855,17 +1855,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>draft-ni-wimse-ai-agent-identity — WIMSE Applicability for AI Agents</t>
+          <t>draft-goswami-agentic-jwt — Secure Intent Protocol: JWT-Compatible Agentic Identity and Workflow Management</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft mapping the WIMSE workload-identity architecture to AI-agent use cases and establishing credential-management mechanisms for agentic AI within the WIMSE framework.</t>
+          <t>An IETF individual draft defining an Agentic JWT extension to OAuth 2.0 with a Supervisor Agent role for sub-agent coordination, explicitly addressing the 'intent-execution separation' gap and adding workflow-step authorization.</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ni-wimse-ai-agent-identity/</t>
+          <t>https://datatracker.ietf.org/doc/draft-goswami-agentic-jwt/</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, February 2026; an important bridge between the WIMSE WG and the AI agent space. If an AI-agent WG is ever chartered, this applicability statement is essential groundwork. Co-authored with Liu, who also leads the related security-requirements draft.</t>
+          <t>Revision -00, December 2025; the intent-execution-separation framing is insightful and distinguishing. The workflow-step authorization approach is novel but may face skepticism in the OAuth WG.</t>
         </is>
       </c>
     </row>
@@ -1885,17 +1885,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-identity-framework — Agent Identity Framework: Trust and Identity for Autonomous AI Agents</t>
+          <t>draft-ni-wimse-ai-agent-identity — WIMSE Applicability for AI Agents</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft proposing a five-layer model (identity, authorization, attestation, evidence, trust) for autonomous AI agents, with a gap analysis between current Internet standards and agent requirements.</t>
+          <t>An IETF individual draft mapping the WIMSE workload-identity architecture to AI-agent use cases and establishing credential-management mechanisms for agentic AI within the WIMSE framework.</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-identity-framework/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ni-wimse-ai-agent-identity/</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 6 April 2026; more gap-analysis than protocol spec. Useful as problem statement. Five-layer model is a reasonable decomposition but insufficient as a standalone contribution. Part of the Sharif cluster (with -agent-audit-trail, -attp, etc.).</t>
+          <t>Revision -02, February 2026; an important bridge between the WIMSE WG and the AI agent space. If an AI-agent WG is ever chartered, this applicability statement is essential groundwork. Co-authored with Liu, who also leads the related security-requirements draft.</t>
         </is>
       </c>
     </row>
@@ -1915,17 +1915,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>draft-aip-agent-identity-protocol — AIP: Agentic Authentication and Authorized Policy Enforcement</t>
+          <t>draft-sharif-agent-identity-framework — Agent Identity Framework: Trust and Identity for Autonomous AI Agents</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an AIP Token signed per tool call (agent ID, tool, nonce, timestamp, signature), an AgentPolicy YAML format for per-tool argument constraints and DLP rules, and a Human-in-the-Loop proxy enforcement model.</t>
+          <t>An IETF individual draft proposing a five-layer model (identity, authorization, attestation, evidence, trust) for autonomous AI agents, with a gap analysis between current Internet standards and agent requirements.</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-aip-agent-identity-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-identity-framework/</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 16 March 2026; implementation-focused. YAML policy approach is pragmatic but not interoperable-by-design. HITL integration is a valuable safety feature. Third member of the 'AIP' name-collision triple — must be resolved before any can progress.</t>
+          <t>Revision -00, 6 April 2026; more gap-analysis than protocol spec. Useful as problem statement. Five-layer model is a reasonable decomposition but insufficient as a standalone contribution. Part of the Sharif cluster (with -agent-audit-trail, -attp, etc.).</t>
         </is>
       </c>
     </row>
@@ -1945,17 +1945,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>draft-liu-oauth-chain-delegation — Delegation Chain for OAuth 2.0</t>
+          <t>draft-aip-agent-identity-protocol — AIP: Agentic Authentication and Authorized Policy Enforcement</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Introduces a delegation_chain JWT claim as a structured companion to RFC 8693's act claim; delegation_chain records the complete delegation history as an ordered array with per-hop authorization constraints and optional cryptographic confirmation from each delegating agent. Supports cross-domain delegation with integrated user consent interaction.</t>
+          <t>An IETF individual draft defining an AIP Token signed per tool call (agent ID, tool, nonce, timestamp, signature), an AgentPolicy YAML format for per-tool argument constraints and DLP rules, and a Human-in-the-Loop proxy enforcement model.</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-liu-oauth-chain-delegation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-aip-agent-identity-protocol/</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 6 Jun 2026; authors: Dapeng Liu, Judy Zhu, Suresh Krishnan (Ericsson), Aaron Parecki (Okta). Provides the structured delegation lineage that act alone cannot express; strong overlap with draft-mw-oauth-actor-chain and draft-niyikiza-oauth-attenuating-agent-tokens — OAuth WG will likely expect consolidation across these three.</t>
+          <t>Revision -00, 16 March 2026; implementation-focused. YAML policy approach is pragmatic but not interoperable-by-design. HITL integration is a valuable safety feature. Third member of the 'AIP' name-collision triple — must be resolved before any can progress.</t>
         </is>
       </c>
     </row>
@@ -1975,17 +1975,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>draft-fletcher-transaction-token-chaining-profile — Transaction Token Authorization Grant Profile for OAuth Identity and Authorization Chaining</t>
+          <t>draft-liu-oauth-chain-delegation — Delegation Chain for OAuth 2.0</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Establishes a framework for using Transaction Tokens as subject credentials in OAuth 2.0 Token Exchange requests (RFC 8693), enabling services within one trust domain to obtain JWT authorization grants for accessing resources across domain boundaries without exposing internal token formats.</t>
+          <t>Introduces a delegation_chain JWT claim as a structured companion to RFC 8693's act claim; delegation_chain records the complete delegation history as an ordered array with per-hop authorization constraints and optional cryptographic confirmation from each delegating agent. Supports cross-domain delegation with integrated user consent interaction.</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-fletcher-transaction-token-chaining-profile/</t>
+          <t>https://datatracker.ietf.org/doc/draft-liu-oauth-chain-delegation/</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 20 Jun 2026; authors: George Fletcher (Practical Identity LLC), Pieter Kasselman (Defakto Security), Sean O'Dell (CVS Health). Directly bridges draft-ietf-oauth-transaction-tokens and draft-ietf-oauth-identity-chaining (both in corpus), closing the 'how do TX Tokens actually cross domains' gap. Note: lead author is the corpus maintainer.</t>
+          <t>Revision -00, 6 Jun 2026; authors: Dapeng Liu, Judy Zhu, Suresh Krishnan (Ericsson), Aaron Parecki (Okta). Provides the structured delegation lineage that act alone cannot express; strong overlap with draft-mw-oauth-actor-chain and draft-niyikiza-oauth-attenuating-agent-tokens — OAuth WG will likely expect consolidation across these three.</t>
         </is>
       </c>
     </row>
@@ -2005,17 +2005,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>draft-zhu-oauth-async-delegation — Sender-Constrained Delegation Handle for Asynchronous OAuth 2.0 Identity Chaining</t>
+          <t>draft-fletcher-transaction-token-chaining-profile — Transaction Token Authorization Grant Profile for OAuth Identity and Authorization Chaining</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Introduces a Delegation Handle — a sender-constrained, audience-locked JWT issued by authorization servers — enabling acting clients to refresh chained access tokens without re-prompting an offline end user while maintaining strict policy bounds and identity chains.</t>
+          <t>Establishes a framework for using Transaction Tokens as subject credentials in OAuth 2.0 Token Exchange requests (RFC 8693), enabling services within one trust domain to obtain JWT authorization grants for accessing resources across domain boundaries without exposing internal token formats.</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-zhu-oauth-async-delegation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-fletcher-transaction-token-chaining-profile/</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 22 May 2026; authors: Larry Zhu, Sam Currie (Atlassian). Addresses a concrete gap in agent delegation: what happens when the delegating human is not present to re-authorize. Directly relevant to long-running agentic workflows using draft-ietf-oauth-identity-chaining.</t>
+          <t>Revision -02, 6 Jul 2026 (was -01 Jun 2026); authors: George Fletcher (Practical Identity LLC), Pieter Kasselman (Defakto Security), Sean O'Dell (CVS Health). Directly bridges draft-ietf-oauth-transaction-tokens and draft-ietf-oauth-identity-chaining (both in corpus), closing the 'how do TX Tokens actually cross domains' gap. Note: lead author is the corpus maintainer.</t>
         </is>
       </c>
     </row>
@@ -2035,17 +2035,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>draft-chen-oauth-agent-revocation — OAuth 2.0 Agent Authorization Explicit Revocation</t>
+          <t>draft-zhu-oauth-async-delegation — Sender-Constrained Delegation Handle for Asynchronous OAuth 2.0 Identity Chaining</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Extends RFC 7009 token revocation for agent-based scenarios: introduces batch revocation by agent ID, cascading revocation across delegation chains, conditional revocation options, and verifiable audit trails.</t>
+          <t>Introduces a Delegation Handle — a sender-constrained, audience-locked JWT issued by authorization servers — enabling acting clients to refresh chained access tokens without re-prompting an offline end user while maintaining strict policy bounds and identity chains.</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-chen-oauth-agent-revocation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-zhu-oauth-async-delegation/</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 27 Apr 2026; authors: Meiling Chen, Li Su (China Mobile). Fills the lifecycle management gap — existing RFC 7009 revocation is single-token and client-centric, but agent delegation chains require cascade semantics. Natural companion to draft-ietf-oauth-transaction-tokens and draft-niyikiza-oauth-attenuating-agent-tokens.</t>
+          <t>Revision -00, 22 May 2026; authors: Larry Zhu, Sam Currie (Atlassian). Addresses a concrete gap in agent delegation: what happens when the delegating human is not present to re-authorize. Directly relevant to long-running agentic workflows using draft-ietf-oauth-identity-chaining.</t>
         </is>
       </c>
     </row>
@@ -2065,17 +2065,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>draft-jiang-oauth-intent-admission — Intent Admission Assertions for Agentic Systems</t>
+          <t>draft-chen-oauth-agent-revocation — OAuth 2.0 Agent Authorization Explicit Revocation</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Defines a signed, verifiable Intent Admission Assertion (IAA) that an admission point creates after verifying agent identity, evaluating permissions against policy, and — when required — obtaining explicit user consent; the IAA is transmitted to the execution endpoint which re-validates before proceeding. Leverages OAuth and RFC 9396 Rich Authorization Requests.</t>
+          <t>Extends RFC 7009 token revocation for agent-based scenarios: introduces batch revocation by agent ID, cascading revocation across delegation chains, conditional revocation options, and verifiable audit trails.</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jiang-oauth-intent-admission/</t>
+          <t>https://datatracker.ietf.org/doc/draft-chen-oauth-agent-revocation/</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 23 Jun 2026; authors: Yuning Jiang, Lun Li, Yurong Song, Faye Liu (Huawei). The required_consent path maps directly to the HITL pattern central to the corpus. Companion to draft-jiang-intent-security (threat model) from the same Huawei group.</t>
+          <t>Revision -00, 27 Apr 2026; authors: Meiling Chen, Li Su (China Mobile). Fills the lifecycle management gap — existing RFC 7009 revocation is single-token and client-centric, but agent delegation chains require cascade semantics. Natural companion to draft-ietf-oauth-transaction-tokens and draft-niyikiza-oauth-attenuating-agent-tokens.</t>
         </is>
       </c>
     </row>
@@ -2095,17 +2095,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>draft-kroehl-agentic-trust-aae — Agent Authorization Envelope (AAE)</t>
+          <t>draft-jiang-oauth-intent-admission — Intent Admission Assertions for Agentic Systems</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Specifies the AAE, a structured authorization container with three mandatory components — MANDATE, CONSTRAINTS, and VALIDITY — providing a machine-evaluable, cryptographically verifiable authorization assertion using W3C DIDs and Verifiable Credentials.</t>
+          <t>Defines a signed, verifiable Intent Admission Assertion (IAA) that an admission point creates after verifying agent identity, evaluating permissions against policy, and — when required — obtaining explicit user consent; the IAA is transmitted to the execution endpoint which re-validates before proceeding. Leverages OAuth and RFC 9396 Rich Authorization Requests.</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-kroehl-agentic-trust-aae/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jiang-oauth-intent-admission/</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 21 May 2026; author: Lars Kersten Kroehl (CryptoKRI GmbH). Occupies similar design space to draft-mcguinness-oauth-actor-profile but uses a DID/VC substrate rather than OAuth — provides a useful alternative approach for non-OAuth deployments.</t>
+          <t>Revision -00, 23 Jun 2026; authors: Yuning Jiang, Lun Li, Yurong Song, Faye Liu (Huawei). The required_consent path maps directly to the HITL pattern central to the corpus. Companion to draft-jiang-intent-security (threat model) from the same Huawei group.</t>
         </is>
       </c>
     </row>
@@ -2125,17 +2125,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>draft-pidlisnyi-aps — Agent Passport System (APS)</t>
+          <t>draft-song-oauth-ai-agent-collaborate-authz — OAuth 2.0 Extension for Multi-AI Agent Collaboration</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Specifies Ed25519-based agent passports, scoped delegation chains with constraints across seven dimensions (a lattice model where delegation monotonically narrows capabilities), cascade revocation, a three-signature policy chain, signed receipts, and MCP bindings; includes reference implementations in TypeScript and Python.</t>
+          <t>Extends OAuth 2.0 for coordinated multi-agent task groups: defines a collaborative authorization flow allowing a lead agent to obtain delegation tokens for sub-agents, with shared task context, coordinated scope attenuation, and cross-agent session binding.</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-pidlisnyi-aps/</t>
+          <t>https://datatracker.ietf.org/doc/draft-song-oauth-ai-agent-collaborate-authz/</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 14 May 2026; author: Tymofii Pidlisnyi (AEOESS). Among the most comprehensive standalone agent authz specs in the wave — the seven-dimension constraint lattice and MCP binding make it directly implementable against Model Context Protocol deployments alongside draft-serra-mcp-discovery-uri.</t>
+          <t>Revision -02, Jun/Jul 2026; authors: Yurong Song (Huawei) and colleagues. Addresses the multi-agent coordination gap at the OAuth layer — complements draft-jiang-oauth-intent-admission from the same Huawei group. Distinct from single-hop delegation drafts in explicitly modeling lead-agent-to-sub-agent scope sharing.</t>
         </is>
       </c>
     </row>
@@ -2155,17 +2155,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>draft-serra-mcp-discovery-uri — The mcp URI Scheme and MCP Server Discovery Mechanism</t>
+          <t>draft-kroehl-agentic-trust-aae — Agent Authorization Envelope (AAE)</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an 'mcp://' URI scheme combined with /.well-known/mcp-server (RFC 8615) and a DNS TXT fallback for discovery of Model Context Protocol servers.</t>
+          <t>Specifies the AAE, a structured authorization container with three mandatory components — MANDATE, CONSTRAINTS, and VALIDITY — providing a machine-evaluable, cryptographically verifiable authorization assertion using W3C DIDs and Verifiable Credentials.</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-serra-mcp-discovery-uri/</t>
+          <t>https://datatracker.ietf.org/doc/draft-kroehl-agentic-trust-aae/</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Already at revision -04 (March 2026), suggesting active iteration; narrow scope, clean design, and the strongest IANA-registration candidate in the set. OAuth 2.1 for auth is deliberately out of scope.</t>
+          <t>Revision -00, 21 May 2026; author: Lars Kersten Kroehl (CryptoKRI GmbH). Occupies similar design space to draft-mcguinness-oauth-actor-profile but uses a DID/VC substrate rather than OAuth — provides a useful alternative approach for non-OAuth deployments.</t>
         </is>
       </c>
     </row>
@@ -2185,17 +2185,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-attp — ATTP: Agent Trust Transport Protocol</t>
+          <t>draft-pidlisnyi-aps — Agent Passport System (APS)</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining trust levels L0–L4 mapped to PSD2 Strong Customer Authentication requirements, with bindings for MCP (MCPS), REST, A2A, gRPC, and GraphQL; supersedes draft-sharif-agent-payment-trust.</t>
+          <t>Specifies Ed25519-based agent passports, scoped delegation chains with constraints across seven dimensions (a lattice model where delegation monotonically narrows capabilities), cascade revocation, a three-signature policy chain, signed receipts, and MCP bindings; includes reference implementations in TypeScript and Python.</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-attp/</t>
+          <t>https://datatracker.ietf.org/doc/draft-pidlisnyi-aps/</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, April 2026; regulatory mapping appendices (PSD2, PCI DSS) are notable — one of the few drafts engaging financial regulation directly. Ambitious scope. Part of the Sharif cluster.</t>
+          <t>Revision -01, 14 May 2026; author: Tymofii Pidlisnyi (AEOESS). Among the most comprehensive standalone agent authz specs in the wave — the seven-dimension constraint lattice and MCP binding make it directly implementable against Model Context Protocol deployments alongside draft-serra-mcp-discovery-uri.</t>
         </is>
       </c>
     </row>
@@ -2215,17 +2215,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-transport-protocol — Agent Transport Protocol (ATP): Async Store-and-Forward for AI Agents</t>
+          <t>draft-serra-mcp-discovery-uri — The mcp URI Scheme and MCP Server Discovery Mechanism</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining async store-and-forward messaging semantics with cryptographic identity per relay hop, trust scoring at ingress, capability negotiation, and interop with Google A2A, MCP, and FIPA ACL; transport-agnostic over TCP/TLS/QUIC.</t>
+          <t>An IETF individual draft defining an 'mcp://' URI scheme combined with /.well-known/mcp-server (RFC 8615) and a DNS TXT fallback for discovery of Model Context Protocol servers.</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-transport-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-serra-mcp-discovery-uri/</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 28 March 2026; addresses a real gap — most agent protocols assume synchronous availability, and store-and-forward is appropriate for long-running agentic tasks. Scope is broad and needs narrowing.</t>
+          <t>Already at revision -04 (March 2026), suggesting active iteration; narrow scope, clean design, and the strongest IANA-registration candidate in the set. OAuth 2.1 for auth is deliberately out of scope.</t>
         </is>
       </c>
     </row>
@@ -2245,17 +2245,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-audit-trail — Agent Audit Trail (AAT): Standard Logging Format for Autonomous AI Systems</t>
+          <t>draft-sharif-attp — ATTP: Agent Trust Transport Protocol</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining a JSON-based audit record with mandatory fields (agent identity, action classification, outcome tracking, trust level) using RFC 8785 JSON Canonicalization and RFC 9562 UUIDs.</t>
+          <t>An IETF individual draft defining trust levels L0–L4 mapped to PSD2 Strong Customer Authentication requirements, with bindings for MCP (MCPS), REST, A2A, gRPC, and GraphQL; supersedes draft-sharif-agent-payment-trust.</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-audit-trail/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-attp/</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 29 March 2026; orthogonal to delegation but important for compliance — standardized audit-log format is a genuine gap. Complements identity frameworks well. A sibling/alternative to the Kuehlewind audit architecture which takes a far more ambitious cross-layer approach.</t>
+          <t>Revision -00, April 2026; regulatory mapping appendices (PSD2, PCI DSS) are notable — one of the few drafts engaging financial regulation directly. Ambitious scope. Part of the Sharif cluster.</t>
         </is>
       </c>
     </row>
@@ -2275,17 +2275,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>draft-aiendpoint-ai-discovery — The AI Discovery Endpoint</t>
+          <t>draft-sharif-agent-transport-protocol — Agent Transport Protocol (ATP): Async Store-and-Forward for AI Agents</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining a /.well-known/ai URI suffix for programmatic service capability discovery by AI agents — letting agents discover what an endpoint supports without having to parse human-oriented documentation; requests IANA well-known URI registration.</t>
+          <t>An IETF individual draft defining async store-and-forward messaging semantics with cryptographic identity per relay hop, trust scoring at ingress, capability negotiation, and interop with Google A2A, MCP, and FIPA ACL; transport-agnostic over TCP/TLS/QUIC.</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-aiendpoint-ai-discovery/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-transport-protocol/</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, March 2026; complementary to MCP discovery but broader (not MCP-specific). Needs differentiation from OpenAPI/service-description work to gain traction.</t>
+          <t>Revision -00, 28 March 2026; addresses a real gap — most agent protocols assume synchronous availability, and store-and-forward is appropriate for long-running agentic tasks. Scope is broad and needs narrowing.</t>
         </is>
       </c>
     </row>
@@ -2305,17 +2305,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>draft-hood-independent-agtp — Agent Transfer Protocol (AGTP)</t>
+          <t>draft-sharif-agent-audit-trail — Agent Audit Trail (AAT): Standard Logging Format for Autonomous AI Systems</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft proposing a dedicated application-layer protocol for AI agent traffic on port 4480 (TCP/TLS and QUIC) with an agtp:// URI scheme, arguing that HTTP is insufficient because agent-generated intent-driven traffic is indistinguishable from human-initiated requests. Defines a Runtime Contract Negotiation Substrate (RCNS) with eighteen methods split into cognitive verbs (QUERY, DISCOVER, DESCRIBE, SUMMARIZE, PLAN, PROPOSE) and mechanics verbs (EXECUTE, DELEGATE, ESCALATE, CONFIRM, SUSPEND, NOTIFY), mandatory agent identity headers, and protocol-level authority scope declaration.</t>
+          <t>An IETF individual draft defining a JSON-based audit record with mandatory fields (agent identity, action classification, outcome tracking, trust level) using RFC 8785 JSON Canonicalization and RFC 9562 UUIDs.</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hood-independent-agtp/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-audit-trail/</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Revision -08 (26 May 2026); supersedes draft-hood-independent-atp. Companion specs in the same family: AGTP-API, AGTP-CERT, AGTP-MERCHANT, AGTP-IDENTIFIERS, AGTP-TRUST. Mandatory TLS 1.3+. Ambitious scope — a new transport layer rather than an HTTP profile. The cognitive/mechanics verb split is a distinctive design choice; contrasts with draft-sharif-agent-transport-protocol which layers async store-and-forward on top of existing transports rather than replacing them.</t>
+          <t>Revision -00, 29 March 2026; orthogonal to delegation but important for compliance — standardized audit-log format is a genuine gap. Complements identity frameworks well. A sibling/alternative to the Kuehlewind audit architecture which takes a far more ambitious cross-layer approach.</t>
         </is>
       </c>
     </row>
@@ -2335,17 +2335,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>draft-hood-agtp-ard — ARD Binding for AGTP: Agentic Resource Discovery over the Agent Transfer Protocol</t>
+          <t>draft-aiendpoint-ai-discovery — The AI Discovery Endpoint</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Specifies how Agentic Resource Discovery (ARD) composes with AGTP, defining a catalog entry type for ARD manifests, aligning AGTP's identity model with ARD's trustManifest, and providing an AGTP-native binding for publishing ARD catalogs over AGTP substrate rather than HTTPS.</t>
+          <t>An IETF individual draft defining a /.well-known/ai URI suffix for programmatic service capability discovery by AI agents — letting agents discover what an endpoint supports without having to parse human-oriented documentation; requests IANA well-known URI registration.</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-ard/</t>
+          <t>https://datatracker.ietf.org/doc/draft-aiendpoint-ai-discovery/</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 18 Jun 2026; author: Chris Hood (Nomotic). Extends the AGTP family (draft-hood-independent-agtp in corpus). The trustManifest identity alignment is the piece relevant to the agent identity thread; the rest is transport-layer plumbing for AGTP deployments.</t>
+          <t>Revision -00, March 2026; complementary to MCP discovery but broader (not MCP-specific). Needs differentiation from OpenAPI/service-description work to gain traction.</t>
         </is>
       </c>
     </row>
@@ -2365,17 +2365,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>draft-ni-a2a-ai-agent-security-requirements — Security Requirements for AI Agents</t>
+          <t>draft-hood-independent-agtp — Agent Transfer Protocol (AGTP)</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft enumerating security requirements for AI agents, covering identity, authorization chaining across domains, and integration points with WIMSE, OAuth identity chaining, and the A2A OAuth profile.</t>
+          <t>An IETF individual draft proposing a dedicated application-layer protocol for AI agent traffic on port 4480 (TCP/TLS and QUIC) with an agtp:// URI scheme, arguing that HTTP is insufficient because agent-generated intent-driven traffic is indistinguishable from human-initiated requests. Defines a Runtime Contract Negotiation Substrate (RCNS) with eighteen methods split into cognitive verbs (QUERY, DISCOVER, DESCRIBE, SUMMARIZE, PLAN, PROPOSE) and mechanics verbs (EXECUTE, DELEGATE, ESCALATE, CONFIRM, SUSPEND, NOTIFY), mandatory agent identity headers, and protocol-level authority scope declaration.</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ni-a2a-ai-agent-security-requirements/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-independent-agtp/</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, February 2026; essential scaffolding for an eventual AI-agent WG. Well-connected to existing IETF work and authored by Ni and Liu, who also lead the WIMSE AI-agent identity draft.</t>
+          <t>Revision -09, 28 Jun 2026 (was -08 May 2026); supersedes draft-hood-independent-atp. Companion specs in the same family: AGTP-API, AGTP-CERT, AGTP-MERCHANT, AGTP-IDENTIFIERS, AGTP-TRUST. Mandatory TLS 1.3+. Ambitious scope — a new transport layer rather than an HTTP profile. The cognitive/mechanics verb split is a distinctive design choice; contrasts with draft-sharif-agent-transport-protocol which layers async store-and-forward on top of existing transports rather than replacing them.</t>
         </is>
       </c>
     </row>
@@ -2395,17 +2395,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>draft-rosenberg-aiproto-framework — Framework, Use Cases and Requirements for AI Agent Protocols</t>
+          <t>draft-hood-agtp-ard — ARD Binding for AGTP: Agentic Resource Discovery over the Agent Transfer Protocol</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft providing a comprehensive AI-agent communications framework that covers user↔agent, agent↔API, and agent↔agent interactions; surveys MCP, A2A, and Agntcy; and sets the stage for IETF standards activity.</t>
+          <t>Specifies how Agentic Resource Discovery (ARD) composes with AGTP, defining a catalog entry type for ARD manifests, aligning AGTP's identity model with ARD's trustManifest, and providing an AGTP-native binding for publishing ARD catalogs over AGTP substrate rather than HTTPS.</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-framework/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-ard/</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, October 2025; Rosenberg (Five9) and Jennings (Cisco) are credible long-time IETF contributors. Important landscape document but likely expired (April 2026); watch for a -01 refresh post-IETF 123.</t>
+          <t>Revision -00, 18 Jun 2026; author: Chris Hood (Nomotic). Extends the AGTP family (draft-hood-independent-agtp in corpus). The trustManifest identity alignment is the piece relevant to the agent identity thread; the rest is transport-layer plumbing for AGTP deployments.</t>
         </is>
       </c>
     </row>
@@ -2425,17 +2425,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>draft-rosenberg-aiproto-cheq — CHEQ: A Protocol for Confirmation of AI Agent Decisions (HITL)</t>
+          <t>draft-jernalczyk-intentweb-agent-manifest — IntentWeb AgentManifest</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an out-of-band Human-in-the-Loop confirmation protocol for agent tool calls, eliminating LLM-hallucination risk for consequential actions and enabling sensitive operations (e.g., banking) without exposing data to the agent.</t>
+          <t>Defines a JSON document that websites publish to describe identity, trusted knowledge, agent-facing capabilities, structured bindings, risk levels, consent requirements, authentication expectations, audit rules, and policies — enabling AI agents to comprehend website functionality and safely perform actions without scraping or fragile UI automation.</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-cheq/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jernalczyk-intentweb-agent-manifest/</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, October 2025; out-of-band HITL confirmation model is valuable and complements delegation frameworks. Likely expired (April 2026); worth tracking for a -01 refresh.</t>
+          <t>Revision -00, 6 Jul 2026; author: Mariusz Jernalczyk (IntentWeb). Website-side complement to agent identity drafts; sits in the Discovery &amp; Transport cluster alongside draft-hood-agtp-ard and the DAWN/.well-known discovery thread. Single author, no-affiliation submission — early stage but addresses a real discovery gap.</t>
         </is>
       </c>
     </row>
@@ -2455,27 +2455,27 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-payment-trust — Trust Scoring and Identity Verification for AI Agent Payment Transactions (SUPERSEDED)</t>
+          <t>draft-ni-a2a-ai-agent-security-requirements — Security Requirements for AI Agents</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft introducing an Agent Passport — a cryptographic delegation certificate intended to serve as the PSD2 'something you have' factor — and a trust-scoring model for payment transactions mapped to PCI DSS v4.0.1.</t>
+          <t>An IETF individual draft enumerating security requirements for AI agents, covering identity, authorization chaining across domains, and integration points with WIMSE, OAuth identity chaining, and the A2A OAuth profile.</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-payment-trust/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ni-a2a-ai-agent-security-requirements/</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual, superseded)</t>
+          <t>IETF (individual)</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>SUPERSEDED by draft-sharif-attp-00 (April 2026). Retained for historical context — the Agent Passport concept is interesting but needs formal grounding; the ATTP successor generalizes it across transport bindings.</t>
+          <t>Revision -01, February 2026; essential scaffolding for an eventual AI-agent WG. Well-connected to existing IETF work and authored by Ni and Liu, who also lead the WIMSE AI-agent identity draft.</t>
         </is>
       </c>
     </row>
@@ -2485,17 +2485,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>draft-stephan-ai-agent-6g — AI Agent Protocols for 6G Systems</t>
+          <t>draft-rosenberg-aiproto-framework — Framework, Use Cases and Requirements for AI Agent Protocols</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft translating use cases and service requirements from 3GPP TR 22.870 into IETF agent-protocol requirements, covering autonomous vehicles, privacy preservation, and anomaly detection.</t>
+          <t>An IETF individual draft providing a comprehensive AI-agent communications framework that covers user↔agent, agent↔API, and agent↔agent interactions; surveys MCP, A2A, and Agntcy; and sets the stage for IETF standards activity.</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-stephan-ai-agent-6g/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-framework/</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, October 2025; strong operator backing (Orange, Deutsche Telekom, Telefonica, China Mobile, Huawei). Requirements-oriented and important for 3GPP/IETF coordination. May be expired (April 2026); watch for an update.</t>
+          <t>Revision -00, October 2025; Rosenberg (Five9) and Jennings (Cisco) are credible long-time IETF contributors. Important landscape document but likely expired (April 2026); watch for a -01 refresh post-IETF 123.</t>
         </is>
       </c>
     </row>
@@ -2515,17 +2515,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>draft-jimenez-t2trg-iot-agent — Agentic AI Operation of Constrained RESTful Environments</t>
+          <t>draft-rosenberg-aiproto-cheq — CHEQ: A Protocol for Confirmation of AI Agent Decisions (HITL)</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft (T2TRG affiliated) describing agentic AI (ReAct, smolagents) operating on CoAP/CoRE constrained-IoT environments, with a reference implementation provided.</t>
+          <t>An IETF individual draft defining an out-of-band Human-in-the-Loop confirmation protocol for agent tool calls, eliminating LLM-hallucination risk for consequential actions and enabling sensitive operations (e.g., banking) without exposing data to the agent.</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jimenez-t2trg-iot-agent/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-cheq/</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 14 April 2026; unique in targeting constrained IoT environments. T2TRG affiliation and reference implementation are positive signals. Niche but fills an unaddressed gap.</t>
+          <t>Revision -00, October 2025; out-of-band HITL confirmation model is valuable and complements delegation frameworks. Likely expired (April 2026); worth tracking for a -01 refresh.</t>
         </is>
       </c>
     </row>
@@ -2545,27 +2545,27 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>draft-li-oauth-delegated-authorization — OAuth 2.0 Delegated Authorization</t>
+          <t>draft-sharif-agent-payment-trust — Trust Scoring and Identity Verification for AI Agent Payment Transactions (SUPERSEDED)</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Huawei authors that extends OAuth 2.0 with a hierarchical 'delegation token' model so a client can mint subordinate, narrowly-scoped access tokens for delegated parties.</t>
+          <t>An IETF individual draft introducing an Agent Passport — a cryptographic delegation certificate intended to serve as the PSD2 'something you have' factor — and a trust-scoring model for payment transactions mapped to PCI DSS v4.0.1.</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-li-oauth-delegated-authorization/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-payment-trust/</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (individual, superseded)</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, March 2026 (Informational); directly addresses over-privileged tokens and is one of the few drafts using the literal term 'delegated authorization'.</t>
+          <t>SUPERSEDED by draft-sharif-attp-00 (April 2026). Retained for historical context — the Agent Passport concept is interesting but needs formal grounding; the ATTP successor generalizes it across transport bindings.</t>
         </is>
       </c>
     </row>
@@ -2575,17 +2575,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>draft-araut-oauth-transaction-tokens-for-agents — Transaction Tokens For Agents</t>
+          <t>draft-stephan-ai-agent-6g — AI Agent Protocols for 6G Systems</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Ashay Raut (Amazon) profiling Transaction Tokens for agent-based workflows by adding 'act' for the agent identity, an 'agentic_ctx' claim carrying agent_type/intent/allowed_actions/environment_constraints, RFC 9396 RAR integration, and an 'actchain' claim for multi-agent delegation lineage.</t>
+          <t>An IETF individual draft translating use cases and service requirements from 3GPP TR 22.870 into IETF agent-protocol requirements, covering autonomous vehicles, privacy preservation, and anomaly detection.</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-araut-oauth-transaction-tokens-for-agents/</t>
+          <t>https://datatracker.ietf.org/doc/draft-stephan-ai-agent-6g/</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>Revision -01 (May 2026) under the new slug — re-slugged from draft-oauth-transaction-tokens-for-agents-06; the -06 added the actchain delegation lineage, RAR-driven agentic_ctx, and a TTS check that blocks chain-splicing attacks. Conservative extension of the WG Transaction Tokens draft and an easier path to standardization.</t>
+          <t>Revision -02, October 2025; strong operator backing (Orange, Deutsche Telekom, Telefonica, China Mobile, Huawei). Requirements-oriented and important for 3GPP/IETF coordination. May be expired (April 2026); watch for an update.</t>
         </is>
       </c>
     </row>
@@ -2605,17 +2605,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>draft-oauth-ai-agents-on-behalf-of-user — On-Behalf-Of User Authorization for AI Agents</t>
+          <t>draft-jimenez-t2trg-iot-agent — Agentic AI Operation of Constrained RESTful Environments</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft adding requested_actor and actor_token parameters to the OAuth authorization-code flow so the user gives explicit consent per agent, with the resulting delegation chain documented in the access-token claims.</t>
+          <t>An IETF individual draft (T2TRG affiliated) describing agentic AI (ReAct, smolagents) operating on CoAP/CoRE constrained-IoT environments, with a reference implementation provided.</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-oauth-ai-agents-on-behalf-of-user/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jimenez-t2trg-iot-agent/</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Revision -02 was submitted August 2025; likely due for -03 refresh. Builds naturally on RFC 6749 + RFC 8693 + RFC 7636 PKCE — one of the most 'IETF-ready' delegation drafts and a strong WG-adoption candidate after the OAuth recharter.</t>
+          <t>Revision -00, 14 April 2026; unique in targeting constrained IoT environments. T2TRG affiliation and reference implementation are positive signals. Niche but fills an unaddressed gap.</t>
         </is>
       </c>
     </row>
@@ -2635,17 +2635,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>draft-rosomakho-oauth-txn-challenge — OAuth Transaction Authorization Challenge</t>
+          <t>draft-li-oauth-delegated-authorization — OAuth 2.0 Delegated Authorization</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>An OAuth mechanism enabling protected resources to demand transaction-specific authorization through challenges. When a request involves an agent or automated workflow, the RS returns a challenge to the client; the client presents it to the AS, which validates it, obtains human approval, and issues an access token with RFC 9396 authorization_details describing the approved operation. Positions as complementary to RFC 9470 (Step-Up Authentication) — that spec handles authentication freshness; this one handles authorization specificity.</t>
+          <t>An IETF individual draft from Huawei authors that extends OAuth 2.0 with a hierarchical 'delegation token' model so a client can mint subordinate, narrowly-scoped access tokens for delegated parties.</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rosomakho-oauth-txn-challenge/</t>
+          <t>https://datatracker.ietf.org/doc/draft-li-oauth-delegated-authorization/</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, submitted 25 June 2026. Authors: Yaroslav Rosomakho (Zscaler), Brian Campbell (Ping Identity), Karl McGuinness (Independent), Pieter Kasselman (Defakto). Strong author lineup — Campbell is a prolific OAuth WG contributor, Kasselman co-authored Transaction Tokens and First-Party Apps, McGuinness brings the Mission-Bound OAuth context. The RS-initiated challenge model is distinct from ARAP (which operates at the PDP/PEP layer via AuthZEN) but addresses the same 'denial is not the end' problem — here at the OAuth RS/AS layer rather than the AuthZEN layer.</t>
+          <t>Revision -01, March 2026 (Informational); directly addresses over-privileged tokens and is one of the few drafts using the literal term 'delegated authorization'.</t>
         </is>
       </c>
     </row>
@@ -2665,17 +2665,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>draft-lee-orprg-permit-receipts — Permit Receipts for Permit-Before-Commit Authorization</t>
+          <t>draft-araut-oauth-transaction-tokens-for-agents — Transaction Tokens For Agents</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Defines requirements and an abstract data model for PermitReceipts: a verifier evaluates canonicalized effect requests, action digests, policy epochs, validity intervals, and revocation status before any protected effect is committed at an effect boundary. Covers verifier behavior, failure semantics, and candidate registries.</t>
+          <t>An IETF individual draft from Ashay Raut (Amazon) profiling Transaction Tokens for agent-based workflows by adding 'act' for the agent identity, an 'agentic_ctx' claim carrying agent_type/intent/allowed_actions/environment_constraints, RFC 9396 RAR integration, and an 'actchain' claim for multi-agent delegation lineage.</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-lee-orprg-permit-receipts/</t>
+          <t>https://datatracker.ietf.org/doc/draft-araut-oauth-transaction-tokens-for-agents/</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 4 Jun 2026; author: Yong Bok Lee (Meridian Verity Group). The most complete standalone framework for pre-commit authorization in the current wave; intended to ground IETF discussion on scope and profiles. Seeks guidance on appropriate organizational placement.</t>
+          <t>Revision -01 (May 2026) under the new slug — re-slugged from draft-oauth-transaction-tokens-for-agents-06; the -06 added the actchain delegation lineage, RAR-driven agentic_ctx, and a TTS check that blocks chain-splicing attacks. Conservative extension of the WG Transaction Tokens draft and an easier path to standardization.</t>
         </is>
       </c>
     </row>
@@ -2695,17 +2695,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>draft-nelson-agent-delegation-receipts — Delegation Receipt Protocol for AI Agent Authorization</t>
+          <t>draft-oauth-ai-agents-on-behalf-of-user — On-Behalf-Of User Authorization for AI Agents</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Specifies the Delegation Receipt Protocol (DRP) where users sign Authorization Objects (containing scope boundaries, time constraints, instruction hashes, and model state commitments) that are published to an append-only log before the agent runtime gains control. Removes operators as trusted intermediaries by making the user's private key the sole signing authority.</t>
+          <t>An IETF individual draft adding requested_actor and actor_token parameters to the OAuth authorization-code flow so the user gives explicit consent per agent, with the resulting delegation chain documented in the access-token claims.</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-nelson-agent-delegation-receipts/</t>
+          <t>https://datatracker.ietf.org/doc/draft-oauth-ai-agents-on-behalf-of-user/</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Revision -10, 13 Jun 2026; author: Ryan Nelson (Authproof). At version 10, the most iterated individual draft in the pre-action authorization space. The commitment-before-execution architecture — sign before the agent runs, not after — is distinctive and directly addresses the prompt-injection attack surface.</t>
+          <t>Revision -02 was submitted August 2025; likely due for -03 refresh. Builds naturally on RFC 6749 + RFC 8693 + RFC 7636 PKCE — one of the most 'IETF-ready' delegation drafts and a strong WG-adoption candidate after the OAuth recharter.</t>
         </is>
       </c>
     </row>
@@ -2725,17 +2725,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>draft-williams-intent-token — The Intent Token: A Cryptographic Authorization Primitive for Autonomous Agents</t>
+          <t>draft-rosomakho-oauth-txn-challenge — OAuth Transaction Authorization Challenge</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Specifies a cryptographic authorization primitive that binds an autonomous agent action to a cryptographically signed, human-declared authorization envelope before execution. Addresses the gap in OAuth 2.0 frameworks that govern access to resources but not what agents are permitted to do at the moment of action. Positioned as complementary to OAuth, not a replacement.</t>
+          <t>An OAuth mechanism enabling protected resources to demand transaction-specific authorization through challenges. When a request involves an agent or automated workflow, the RS returns a challenge to the client; the client presents it to the AS, which validates it, obtains human approval, and issues an access token with RFC 9396 authorization_details describing the approved operation. Positions as complementary to RFC 9470 (Step-Up Authentication) — that spec handles authentication freshness; this one handles authorization specificity.</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-williams-intent-token/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rosomakho-oauth-txn-challenge/</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 22 Jun 2026; author: Jeffrey Williams (Independent). Overlaps conceptually with draft-kroehl-agentic-trust-aae and draft-nelson-agent-delegation-receipts; worth tracking as a lighter-weight alternative to both.</t>
+          <t>Revision -00, submitted 25 June 2026. Authors: Yaroslav Rosomakho (Zscaler), Brian Campbell (Ping Identity), Karl McGuinness (Independent), Pieter Kasselman (Defakto). Strong author lineup — Campbell is a prolific OAuth WG contributor, Kasselman co-authored Transaction Tokens and First-Party Apps, McGuinness brings the Mission-Bound OAuth context. The RS-initiated challenge model is distinct from ARAP (which operates at the PDP/PEP layer via AuthZEN) but addresses the same 'denial is not the end' problem — here at the OAuth RS/AS layer rather than the AuthZEN layer.</t>
         </is>
       </c>
     </row>
@@ -2755,17 +2755,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>draft-reece-wimse-cross-org-delegation — Cross-Organizational Delegation for Workload and Agent Identity</t>
+          <t>draft-lee-orprg-permit-receipts — Permit Receipts for Permit-Before-Commit Authorization</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>A problem statement and requirements draft identifying that existing workload and token-based authorization mechanisms were designed for a single trust domain, describing the cross-organizational agent delegation gap, and enumerating requirements for solutions — without proposing specific technical approaches.</t>
+          <t>Defines requirements and an abstract data model for PermitReceipts: a verifier evaluates canonicalized effect requests, action digests, policy epochs, validity intervals, and revocation status before any protected effect is committed at an effect boundary. Covers verifier behavior, failure semantics, and candidate registries.</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-reece-wimse-cross-org-delegation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-lee-orprg-permit-receipts/</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -2775,7 +2775,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 25 Jun 2026; author: Morgan Reece (TowerGuardian Consulting). The problem-statement companion to the corpus's operational drafts; likely to feed into WIMSE WG scope expansion and is directly in scope for draft-kuehlewind-audit-architecture's composition graph.</t>
+          <t>Revision -00, 4 Jun 2026; author: Yong Bok Lee (Meridian Verity Group). The most complete standalone framework for pre-commit authorization in the current wave; intended to ground IETF discussion on scope and profiles. Seeks guidance on appropriate organizational placement.</t>
         </is>
       </c>
     </row>
@@ -2785,17 +2785,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>draft-jiang-wimse-heterogeneous-credential — Heterogeneous Credential Verification for Workload and Agentic Systems</t>
+          <t>draft-nelson-agent-delegation-receipts — Delegation Receipt Protocol for AI Agent Authorization</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Specifies mechanisms for representing credential sets, identifying credential types, determining appropriate verifiers, normalizing verification results across different formats (workload tokens, OAuth, X.509, attestation), and combining results into a single handling decision.</t>
+          <t>Specifies the Delegation Receipt Protocol (DRP) where users sign Authorization Objects (containing scope boundaries, time constraints, instruction hashes, and model state commitments) that are published to an append-only log before the agent runtime gains control. Removes operators as trusted intermediaries by making the user's private key the sole signing authority.</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jiang-wimse-heterogeneous-credential/</t>
+          <t>https://datatracker.ietf.org/doc/draft-nelson-agent-delegation-receipts/</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 23 Jun 2026; authors: Yuning Jiang, Donghui Wang, Yurong Song, Faye Liu (Huawei). Solves the practical problem of agentic systems receiving credentials in multiple formats from different issuers. Fills a gap left by draft-ni-wimse-ai-agent-identity (corpus) which describes the identity problem but not multi-format credential handling.</t>
+          <t>Revision -10, 13 Jun 2026; author: Ryan Nelson (Authproof). At version 10, the most iterated individual draft in the pre-action authorization space. The commitment-before-execution architecture — sign before the agent runs, not after — is distinctive and directly addresses the prompt-injection attack surface.</t>
         </is>
       </c>
     </row>
@@ -2815,17 +2815,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>draft-munoz-wimse-authorization-evidence — Signed Authorization-Evidence Records for WIMSE-Authorized AI Agent Actions</t>
+          <t>draft-williams-intent-token — The Intent Token: A Cryptographic Authorization Primitive for Autonomous Agents</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Specifies a signed authorization-evidence record (Permit) for WIMSE-authorized AI actions, cryptographically binding to the dispatched request bytes via HTTP Message Signatures, OAuth access tokens, and Shared Signals Framework eventing — without modifying existing standards.</t>
+          <t>Specifies a cryptographic authorization primitive that binds an autonomous agent action to a cryptographically signed, human-declared authorization envelope before execution. Addresses the gap in OAuth 2.0 frameworks that govern access to resources but not what agents are permitted to do at the moment of action. Positioned as complementary to OAuth, not a replacement.</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-munoz-wimse-authorization-evidence/</t>
+          <t>https://datatracker.ietf.org/doc/draft-williams-intent-token/</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 15 May 2026; author: Christian Munoz (Keel API). Profiles WIMSE for AI agent actions and satisfies audit requirements; companion to the SCITT permit profile below. Extends the corpus WIMSE thread (draft-ni-wimse-ai-agent-identity) with a concrete evidence artifact.</t>
+          <t>Revision -01, 22 Jun 2026; author: Jeffrey Williams (Independent). Overlaps conceptually with draft-kroehl-agentic-trust-aae and draft-nelson-agent-delegation-receipts; worth tracking as a lighter-weight alternative to both.</t>
         </is>
       </c>
     </row>
@@ -2845,17 +2845,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>draft-munoz-scitt-permit-profile — A SCITT Profile for Pre-Execution AI Action Authorization Records</t>
+          <t>draft-pereira-licet-human-intent — LICET: Multi-Modal Physiological Human-Intent Verification for Autonomous AI Agent Authorization</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>SCITT profile for the Pre-Execution Authorization Record (Permit), documenting policy-evaluated decisions before AI agent action dispatch with cryptographic binding proving 'authorized request equals dispatched request.' Composes with adjacent profiles for human-authority binding, post-execution evidence, and content-refusal events via referencing mechanisms.</t>
+          <t>Proposes a biometric HITL protocol fusing ECG, electrodermal activity, and Mahalanobis statistical distance to cryptographically verify genuine human intent — not just credential possession — before authorizing autonomous AI agent actions, with ZK proofs enabling third-party audit without exposing raw biometric data.</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-munoz-scitt-permit-profile/</t>
+          <t>https://datatracker.ietf.org/doc/draft-pereira-licet-human-intent/</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -2865,7 +2865,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 15 May 2026; author: Christian Munoz (Keel API). SCITT-anchored analog of the WIMSE evidence record; companion to draft-munoz-wimse-authorization-evidence from the same author. Connects to draft-sharif-agent-audit-trail and draft-kuehlewind-audit-architecture (both in corpus).</t>
+          <t>Revision -01, 2 Jul 2026. The most novel and technically niche HITL proposal in the current wave — complements draft-rosenberg-aiproto-cheq (out-of-band HITL confirmation) and draft-sato-soos-hem (kernel-enforced escalation) by grounding human intent in physiological signal rather than credential or UI interaction.</t>
         </is>
       </c>
     </row>
@@ -2875,17 +2875,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>draft-marques-asqav-compliance-receipts — Compliance Profile of Signed Action Receipts for AI Agents</t>
+          <t>draft-reece-wimse-cross-org-delegation — Cross-Organizational Delegation for Workload and Agent Identity</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Establishes a compliance framework for signed action receipts from AI agents, mandating specific fields, cryptographic anchoring, hash-chain linkage, risk/incident classification, cross-agent envelope binding, and enforcement attestation with retention floors tied to EU AI Act, DORA, NIST AI RMF, HIPAA, SEC Rule 17a-4, and CIRCIA.</t>
+          <t>A problem statement and requirements draft identifying that existing workload and token-based authorization mechanisms were designed for a single trust domain, describing the cross-organizational agent delegation gap, and enumerating requirements for solutions — without proposing specific technical approaches.</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-marques-asqav-compliance-receipts/</t>
+          <t>https://datatracker.ietf.org/doc/draft-reece-wimse-cross-org-delegation/</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>Revision -05, 31 May 2026; author: João André Gomes Marques. The most legally grounded receipt profile in the wave — at revision 05, relatively mature. Complements draft-sharif-agent-audit-trail (corpus) with a multi-regulation compliance overlay.</t>
+          <t>Revision -00, 25 Jun 2026; author: Morgan Reece (TowerGuardian Consulting). The problem-statement companion to the corpus's operational drafts; likely to feed into WIMSE WG scope expansion and is directly in scope for draft-kuehlewind-audit-architecture's composition graph.</t>
         </is>
       </c>
     </row>
@@ -2905,17 +2905,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>draft-mih-scitt-agent-action-capsule — An Agent Action Capsule Profile for SCITT</t>
+          <t>draft-jiang-wimse-heterogeneous-credential — Heterogeneous Credential Verification for Workload and Agentic Systems</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Defines a SCITT statement profile (Agent Action Capsule) documenting agent actions with outcome status (executed, blocked, denied, errored, timed out), evaluated constraints, committed-effect binding, and a human-in-the-loop flag; records a Capsule for every verdict including refusals. COSE Signed Statement format; registrable in SCITT Transparency Services.</t>
+          <t>Specifies mechanisms for representing credential sets, identifying credential types, determining appropriate verifiers, normalizing verification results across different formats (workload tokens, OAuth, X.509, attestation), and combining results into a single handling decision.</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mih-scitt-agent-action-capsule/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jiang-wimse-heterogeneous-credential/</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 19 Jun 2026; author: Steven Mih (Action State Group). Provides auditor-grade evidence that decision gates functioned. The HITL flag directly tracks the corpus theme; the most complete single-draft SCITT audit story in this batch.</t>
+          <t>Revision -01, 30 Jun 2026 (was -00 Jun 2026); authors: Yuning Jiang, Donghui Wang, Yurong Song, Faye Liu (Huawei). Solves the practical problem of agentic systems receiving credentials in multiple formats from different issuers. Fills a gap left by draft-ni-wimse-ai-agent-identity (corpus) which describes the identity problem but not multi-format credential handling.</t>
         </is>
       </c>
     </row>
@@ -2935,17 +2935,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>draft-car-rer-artifact — RER Run Artifact Format: Hash-Chained, Signed Records of AI Inference Execution</t>
+          <t>draft-munoz-wimse-authorization-evidence — Signed Authorization-Evidence Records for WIMSE-Authorized AI Agent Actions</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Specifies a cryptographically signed JSON record for AI inference runs including a signed envelope declaring permissions and limits, a hash-chained event log covering all model and tool calls, and a runtime signature binding envelope and log to the producing implementation. Enables offline verification by parties uninvolved in the original run.</t>
+          <t>Specifies a signed authorization-evidence record (Permit) for WIMSE-authorized AI actions, cryptographically binding to the dispatched request bytes via HTTP Message Signatures, OAuth access tokens, and Shared Signals Framework eventing — without modifying existing standards.</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-car-rer-artifact/</t>
+          <t>https://datatracker.ietf.org/doc/draft-munoz-wimse-authorization-evidence/</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 12 Jun 2026; author: Kayla Cardillo (Tech Enrichment). Relevant for post-hoc audit of what permissions an agent claimed during execution; companion to the SCITT profiles but more focused on inference traceability than authorization decisions.</t>
+          <t>Revision -00, 15 May 2026; author: Christian Munoz (Keel API). Profiles WIMSE for AI agent actions and satisfies audit requirements; companion to the SCITT permit profile below. Extends the corpus WIMSE thread (draft-ni-wimse-ai-agent-identity) with a concrete evidence artifact.</t>
         </is>
       </c>
     </row>
@@ -2965,17 +2965,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>draft-noa-scitt-ai-agent-receipt — A SCITT Profile for AI-Agent Action Receipts</t>
+          <t>draft-schwenkschuster-wimse-trust-domain-discovery — WIMSE Trust Domain Discovery</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Defines a minimal SCITT profile: COSE_Sign1 Signed Statements with canonicalized payloads, hash-chained for ordering, registrable in SCITT Transparency Services. Explicitly does NOT assert agent correctness, safety, or real-world outcomes — only tamper-evident, signature-verifiable records of action, principal, policy identity, and verdict.</t>
+          <t>Fills a gap in the WIMSE architecture by defining how relying parties obtain cryptographic trust anchors for workload identity credentials; specifies the WIMSE Trust Bundle (a JSON document with freshness metadata) and a well-known HTTPS discovery endpoint resolving trust domain names to their trust bundles, following OpenID Connect Discovery / OAuth 2.0 patterns.</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-noa-scitt-ai-agent-receipt/</t>
+          <t>https://datatracker.ietf.org/doc/draft-schwenkschuster-wimse-trust-domain-discovery/</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 23 Jun 2026; author: Tora Toraman (NordenSoft). The minimalist end of the SCITT profile spectrum; useful for corpus completeness alongside the more comprehensive draft-mih-scitt-agent-action-capsule.</t>
+          <t>Revision -00, 3 Jul 2026; authors: Arndt Schwenkschuster (Defakto Security), Yaroslav Rosomakho (Zscaler). Directly complements draft-schwenkschuster-wimse-credential-exchange (corpus). The kuehlewind-audit-architecture HUB assumes resolvable trust anchors — this provides the discovery mechanism. Rosomakho co-authorship ties it to draft-rosomakho-oauth-txn-challenge.</t>
         </is>
       </c>
     </row>
@@ -2995,17 +2995,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-mjwt — The Mandate JWT (MJWT) for Agentic AI Systems</t>
+          <t>draft-winmagic-wimse-condition-bounded-credentials — Condition-Bounded Credentials for Workload and Agent Identity</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Introduces the Mandate JWT — a WIMSE workload credential profile binding agent authority to specific Sovereign Object instances under named human principals, with cryptographically enforced delegation ceilings and a six-dimensional Narrowing Property preventing sub-agents from exceeding root authority.</t>
+          <t>Proposes hardware-rooted, non-exfiltratable workload credentials whose validity is conditioned on attested runtime posture rather than expiration time — so a credential becomes invalid if the workload's attestation evidence degrades, regardless of the stated expiry.</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-mjwt/</t>
+          <t>https://datatracker.ietf.org/doc/draft-winmagic-wimse-condition-bounded-credentials/</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). The authorization token primitive for the SOOS governance protocol family. Directly comparable to draft-mcguinness-oauth-client-instance-assertion but uses a WIMSE/Sovereign Object substrate rather than OAuth.</t>
+          <t>Revision -01, 6 Jul 2026; author: WinMagic. Extends the WIMSE credential model with posture-conditioned validity — distinct from time-bounded credentials in that security policy changes at the hardware/attestation layer instantly invalidate the credential. Bridges the RATS attestation thread and the WIMSE identity thread in the corpus.</t>
         </is>
       </c>
     </row>
@@ -3025,17 +3025,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-mad — Multi-Agent Delegation in Sovereign Object Systems</t>
+          <t>draft-munoz-scitt-permit-profile — A SCITT Profile for Pre-Execution AI Action Authorization Records</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Specifies three core mechanisms for multi-agent delegation accountability: the Narrowing Property (capability non-amplification), five formally defined object topology patterns for runtime relationships, and cluster coordination primitives for parallel execution with aggregation rules. Version 02 adds revocation-during-execution handling and partial-completion routing to human oversight.</t>
+          <t>SCITT profile for the Pre-Execution Authorization Record (Permit), documenting policy-evaluated decisions before AI agent action dispatch with cryptographic binding proving 'authorized request equals dispatched request.' Composes with adjacent profiles for human-authority binding, post-execution evidence, and content-refusal events via referencing mechanisms.</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-mad/</t>
+          <t>https://datatracker.ietf.org/doc/draft-munoz-scitt-permit-profile/</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). Claims to address gaps the OpenID Foundation identifies as unsolved in multi-agent authorization. The five topology patterns are a useful vocabulary for describing agent-to-agent relationship structures.</t>
+          <t>Revision -00, 15 May 2026; author: Christian Munoz (Keel API). SCITT-anchored analog of the WIMSE evidence record; companion to draft-munoz-wimse-authorization-evidence from the same author. Connects to draft-sharif-agent-audit-trail and draft-kuehlewind-audit-architecture (both in corpus).</t>
         </is>
       </c>
     </row>
@@ -3055,17 +3055,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-hem — The Human Escalation Mechanism (HEM) for Agentic AI Systems</t>
+          <t>draft-marques-asqav-compliance-receipts — Compliance Profile of Signed Action Receipts for AI Agents</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Defines a kernel-enforced mechanism placing agent sessions in a pending state when human judgment is required, routing structured escalation requests to designated human decision-makers, and prohibiting all state transitions until a human decision is received. Defines five decision types and a dual-layer architecture (LLM-HEM and SOOS-HEM).</t>
+          <t>Establishes a compliance framework for signed action receipts from AI agents, mandating specific fields, cryptographic anchoring, hash-chain linkage, risk/incident classification, cross-agent envelope binding, and enforcement attestation with retention floors tied to EU AI Act, DORA, NIST AI RMF, HIPAA, SEC Rule 17a-4, and CIRCIA.</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-hem/</t>
+          <t>https://datatracker.ietf.org/doc/draft-marques-asqav-compliance-receipts/</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -3075,7 +3075,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>Revision -04, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). The most normative HITL protocol in the current wave; explicitly aligns with EU AI Act Article 14 requirements for high-risk AI system oversight. Counterpart to ARAP (AuthZEN WG) at the protocol level vs. the OAuth/AuthZEN layer.</t>
+          <t>Revision -06, 1 Jul 2026 (was -05 May 2026); author: João André Gomes Marques. The most legally grounded receipt profile in the wave — at revision 06, relatively mature. Complements draft-sharif-agent-audit-trail (corpus) with a multi-regulation compliance overlay.</t>
         </is>
       </c>
     </row>
@@ -3085,17 +3085,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-idp — The Intent Declaration Primitive (IDP) for Agentic AI Systems</t>
+          <t>draft-mih-scitt-agent-action-capsule — An Agent Action Capsule Profile for SCITT</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Specifies a structured declaration mechanism committing AI agent intent to tamper-evident logs before actions are taken, enabling post-hoc review and EU AI Act Article 12 compliance for high-risk systems.</t>
+          <t>Defines a SCITT statement profile (Agent Action Capsule) documenting agent actions with outcome status (executed, blocked, denied, errored, timed out), evaluated constraints, committed-effect binding, and a human-in-the-loop flag; records a Capsule for every verdict including refusals. COSE Signed Statement format; registrable in SCITT Transparency Services.</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-idp/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mih-scitt-agent-action-capsule/</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>Revision -04, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). The log-before-execute pattern mirrors draft-nelson-agent-delegation-receipts but operates at the intent declaration level rather than the user-authorization level. Pairs with GAR (below) to form a complete pre/post audit trail.</t>
+          <t>Revision -02, 6 Jul 2026 (was -01 Jun 2026); author: Steven Mih (Action State Group). -02 added an 'honest human-in-the-loop' flag distinguishing actual HITL from automated policy. Provides auditor-grade evidence that decision gates functioned; the HITL flag directly tracks the corpus theme.</t>
         </is>
       </c>
     </row>
@@ -3115,17 +3115,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-gar — The Governance Audit Record (GAR) for Agentic AI Systems</t>
+          <t>draft-car-rer-artifact — RER Run Artifact Format: Hash-Chained, Signed Records of AI Inference Execution</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Defines GAR, an audit framework with five audit types, a Session Audit Record, and an Audit Alert mechanism; collects, signs, and makes governance events from IDP, HEM, and associated SOOS primitives available for regulatory inspection via an append-only, non-suppressible SCITT-anchored audit stream with Authority Lifecycle Events covering the complete revocation-recovery cycle.</t>
+          <t>Specifies a cryptographically signed JSON record for AI inference runs including a signed envelope declaring permissions and limits, a hash-chained event log covering all model and tool calls, and a runtime signature binding envelope and log to the producing implementation. Enables offline verification by parties uninvolved in the original run.</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-gar/</t>
+          <t>https://datatracker.ietf.org/doc/draft-car-rer-artifact/</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). The integrator for the SOOS family, analogous to how draft-kuehlewind-audit-architecture (in corpus) integrates the broader IETF agent draft landscape. SCITT-anchored audit stream is a concrete architectural choice distinguishing it from the Kuehlewind approach.</t>
+          <t>Revision -01, 12 Jun 2026; author: Kayla Cardillo (Tech Enrichment). Relevant for post-hoc audit of what permissions an agent claimed during execution; companion to the SCITT profiles but more focused on inference traceability than authorization decisions.</t>
         </is>
       </c>
     </row>
@@ -3145,17 +3145,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>draft-jiang-intent-security — Security Considerations and Requirements for Intent-Based Requests in Agentic Systems</t>
+          <t>draft-noa-scitt-ai-agent-receipt — A SCITT Profile for AI-Agent Action Receipts</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Solution-agnostic threat analysis covering tampering, privilege escalation, constraint violations, and intent drift in intent-based agentic systems, with a reference model, attack scenarios, and security requirements covering authentication, admission control, constraint validation, and multi-hop integrity.</t>
+          <t>Defines a minimal SCITT profile: COSE_Sign1 Signed Statements with canonicalized payloads, hash-chained for ordering, registrable in SCITT Transparency Services. Explicitly does NOT assert agent correctness, safety, or real-world outcomes — only tamper-evident, signature-verifiable records of action, principal, policy identity, and verdict.</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jiang-intent-security/</t>
+          <t>https://datatracker.ietf.org/doc/draft-noa-scitt-ai-agent-receipt/</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>Revision -03, 22 Jun 2026; authors: Yuning Jiang, Lun Li, Yurong Song, Faye Liu (Huawei). The threat-model companion to draft-jiang-oauth-intent-admission from the same group; likely intended to inform the broader IETF agentic AI security discussion.</t>
+          <t>Revision -00, 23 Jun 2026; author: Tora Toraman (NordenSoft). The minimalist end of the SCITT profile spectrum; useful for corpus completeness alongside the more comprehensive draft-mih-scitt-agent-action-capsule.</t>
         </is>
       </c>
     </row>
@@ -3175,17 +3175,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>draft-somoza-dmsc-atn-agent-trust-negotiation — Agent Trust Negotiation: Capability, Delegation, and Provenance Binding</t>
+          <t>draft-rampalli-scitt-capsule-provenance-binding — Binding Per-Action Authorization and Memory Provenance into Agent Action Capsules</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Specifies the Agent Trust Negotiation (ATN) protocol, which binds four artifacts — capability manifests, delegation chains, provenance attestations, and session receipts — to agent identities via a handshake state machine producing mutually verified, scope-bounded sessions with SCITT-suitable audit records.</t>
+          <t>Specifies how to bind three components into AAC records: what was executed ('did'), whether it was authorized ('may'), and the source of the belief that motivated the action ('why-believed'); uses optional payload extensions carrying authorization token references, memory chain roots, and quarantine attestations without modifying AAC core protected-header claims.</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-somoza-dmsc-atn-agent-trust-negotiation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rampalli-scitt-capsule-provenance-binding/</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 29 May 2026; author: Enrique Somoza (Independent). Operates above discovery mechanisms and positions itself between the discovery layer (DAWN, MCP) and the authorization layer (WIMSE, OAuth). Relevant as an agent-to-agent trust establishment handshake protocol.</t>
+          <t>Revision -00, 5 Jul 2026; author: Karthik Rampalli (Glyphzero, Inc.). Extends draft-mih-scitt-agent-action-capsule with memory provenance — the 'why-believed' component is novel among SCITT profiles. Includes a defensive publication notice waiving patent claims on the core binding technique.</t>
         </is>
       </c>
     </row>
@@ -3205,17 +3205,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>draft-mcgraw-httpapi-agent-budget — The Delegation HTTP Authentication Scheme for Request-Bound Authority</t>
+          <t>draft-nobuo-scitt-composite-evidence-verification — Composite Evidence Verification for SCITT Statement Graphs</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Defines the 'Delegation' HTTP authentication scheme and response semantics for delegated-authority challenges using HTTP status codes and Problem Details, plus a CBOR/COSE proof format. The initial authority profile is 'Budget,' using post-quantum ML-DSA to prove spending or resource-consumption limits.</t>
+          <t>Defines a composite verifier function for checking collections of SCITT Signed Statements, receipts, object bindings, and relationship edges under a named verification profile; provides structured reporting on validation status, missing evidence, outdated information, and conflicting claims — targeting auditors needing to evaluate multiple interconnected statements.</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcgraw-httpapi-agent-budget/</t>
+          <t>https://datatracker.ietf.org/doc/draft-nobuo-scitt-composite-evidence-verification/</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, 15 Jun 2026; author: John Paul McGraw Jr. (TaskHawk Systems). HTTP-layer bounded delegation with post-quantum crypto; distinct from OAuth-layer delegation in that the authority proof travels in the Authorization header. Complements x401 (Industry tab) at the HTTP challenge-response layer.</t>
+          <t>Revision -00, 7 Jul 2026; author: Nobuo Aoki (SOKENDAI). Operates above individual SCITT profiles (AAC, permits, compliance receipts all in corpus) — the 'how do you verify all of them together' layer that draft-kuehlewind-audit-architecture implies but does not yet specify. Watch for Kühlewind/Birkholz pickup.</t>
         </is>
       </c>
     </row>
@@ -3235,17 +3235,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>draft-vauban-x402-delegation-binding — x402 Delegation Binding for Agentic HTTP Pipelines</t>
+          <t>draft-sato-soos-mjwt — The Mandate JWT (MJWT) for Agentic AI Systems</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Addresses the security gap where x402 V2 payment grants issued to one agent could be misused by another in the same pipeline, introducing three binding mechanisms: a JCS-derived agent identity pseudonym, a nonce for anti-replay, and a depth-limiting field for transitive delegation.</t>
+          <t>Introduces the Mandate JWT — a WIMSE workload credential profile binding agent authority to specific Sovereign Object instances under named human principals, with cryptographically enforced delegation ceilings and a six-dimensional Narrowing Property preventing sub-agents from exceeding root authority.</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-vauban-x402-delegation-binding/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-mjwt/</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -3255,7 +3255,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 25 May 2026; author: Vauban Research. Narrowly scoped to payment pipelines but the delegation-binding pattern (pseudonymous identity + anti-replay + depth-limit) is applicable broadly. Validated across five language runtimes with A2A and MCP integration guidance.</t>
+          <t>Revision -01, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). The authorization token primitive for the SOOS governance protocol family. Directly comparable to draft-mcguinness-oauth-client-instance-assertion but uses a WIMSE/Sovereign Object substrate rather than OAuth.</t>
         </is>
       </c>
     </row>
@@ -3265,17 +3265,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>draft-samal-vap — Verifiable Agent Protocol (VAP): Intent-Bound Admission Control and Audit for Agent Tool Invocation</t>
+          <t>draft-sato-soos-mad — Multi-Agent Delegation in Sovereign Object Systems</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Specifies VAP as a defense-in-depth layer adding declarations of purpose and session budget commitments to tool invocation requests (targeting MCP-style protocols), enabling servers to perform admission control before execution via four messages carried in existing protocol metadata.</t>
+          <t>Specifies three core mechanisms for multi-agent delegation accountability: the Narrowing Property (capability non-amplification), five formally defined object topology patterns for runtime relationships, and cluster coordination primitives for parallel execution with aggregation rules. Version 02 adds revocation-during-execution handling and partial-completion routing to human oversight.</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-samal-vap/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-mad/</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 3 Jun 2026; author: Kruttidipta Samal (Independent). Lightweight and protocol-agnostic; addresses erroneous agent behavior, cost control, and audit trails without replacing existing auth mechanisms. Practical tool-invocation-level authorization layer for MCP deployments.</t>
+          <t>Revision -02, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). Claims to address gaps the OpenID Foundation identifies as unsolved in multi-agent authorization. The five topology patterns are a useful vocabulary for describing agent-to-agent relationship structures.</t>
         </is>
       </c>
     </row>
@@ -3295,17 +3295,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>draft-khera-aurora — Agent Unification, Runtime, and Operational Responsibility Attestation (AURORA)</t>
+          <t>draft-sato-soos-hem — The Human Escalation Mechanism (HEM) for Agentic AI Systems</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>A two-layer framework unifying hardware-enclave-backed Runtime Integrity Attestation with scoped, cryptographically bound Authority Delegation; enables agents to prove both operational authority and runtime integrity simultaneously.</t>
+          <t>Defines a kernel-enforced mechanism placing agent sessions in a pending state when human judgment is required, routing structured escalation requests to designated human decision-makers, and prohibiting all state transitions until a human decision is received. Defines five decision types and a dual-layer architecture (LLM-HEM and SOOS-HEM).</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-khera-aurora/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-hem/</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 5 Jun 2026; author: Ankur Khera. Addresses the gap where delegation tokens don't prove the runtime environment is trustworthy — relevant where delegation must be paired with platform attestation (enterprise/regulated deployments). Bridges the RATS attestation thread and the OAuth delegation thread.</t>
+          <t>Revision -05, 30 Jun 2026 (was -04 Jun 2026); author: Tom Sato (MyAuberge K.K.). The most normative HITL protocol in the current wave; explicitly aligns with EU AI Act Article 14 requirements for high-risk AI system oversight. Counterpart to ARAP (AuthZEN WG) at the protocol level vs. the OAuth/AuthZEN layer.</t>
         </is>
       </c>
     </row>
@@ -3325,17 +3325,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>draft-borthwick-msebenzi-environment-state — Verifiable Intent — environment.* Constraint Family</t>
+          <t>draft-sato-soos-idp — The Intent Declaration Primitive (IDP) for Agentic AI Systems</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Defines the environment.* constraint family for agent-authorization mandate vocabularies, covering external conditions at transaction execution time (venue availability, wallet funding) that existing transactional constraints cannot address. Extends agent authorization mandate frameworks with environmental precondition checking.</t>
+          <t>Specifies a structured declaration mechanism committing AI agent intent to tamper-evident logs before actions are taken, enabling post-hoc review and EU AI Act Article 12 compliance for high-risk systems.</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-borthwick-msebenzi-environment-state/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-idp/</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 13 Jun 2026; authors: Douglas Cameron Borthwick (InsumerAPI), Michael Msebenzi (Headless Oracle). Narrow but practically important for financial and commerce agent workflows; connects to draft-mcgraw-httpapi-agent-budget and draft-vauban-x402-delegation-binding.</t>
+          <t>Revision -05, 30 Jun 2026 (was -04 Jun 2026); author: Tom Sato (MyAuberge K.K.). The log-before-execute pattern mirrors draft-nelson-agent-delegation-receipts but operates at the intent declaration level rather than the user-authorization level. Pairs with GAR (below) to form a complete pre/post audit trail.</t>
         </is>
       </c>
     </row>
@@ -3355,17 +3355,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>draft-hardt-aauth-protocol — AAuth Protocol</t>
+          <t>draft-sato-soos-gar — The Governance Audit Record (GAR) for Agentic AI Systems</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>A new clean-sheet authorization protocol from Dick Hardt (original OAuth author) defining proof-of-possession by default, resource-signed challenges, agent identity without pre-registration, deferred 202 responses, and AS-to-AS federation for the agent ecosystem.</t>
+          <t>Defines GAR, an audit framework with five audit types, a Session Audit Record, and an Audit Alert mechanism; collects, signs, and makes governance events from IDP, HEM, and associated SOOS primitives available for regulatory inspection via an append-only, non-suppressible SCITT-anchored audit stream with Authority Lifecycle Events covering the complete revocation-recovery cycle.</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hardt-aauth-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-gar/</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -3375,7 +3375,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, April 2026; the design rationale section explicitly explains why AAuth is not GNAP, not OAuth, not DPoP and not mTLS — important read for anyone planning a new agent-auth stack.</t>
+          <t>Revision -02, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). The integrator for the SOOS family, analogous to how draft-kuehlewind-audit-architecture (in corpus) integrates the broader IETF agent draft landscape. SCITT-anchored audit stream is a concrete architectural choice distinguishing it from the Kuehlewind approach.</t>
         </is>
       </c>
     </row>
@@ -3385,17 +3385,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>draft-chen-oauth-roadmap — Comprehensive Roadmap for OAuth 2.0 Standards and Drafts</t>
+          <t>draft-jiang-intent-security — Security Considerations and Requirements for Intent-Based Requests in Agentic Systems</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>An IETF informational draft that maps the entire OAuth 2.0 ecosystem of RFCs, BCPs, and active drafts into functional layers from core to extensions to industry profiles.</t>
+          <t>Solution-agnostic threat analysis covering tampering, privilege escalation, constraint violations, and intent drift in intent-based agentic systems, with a reference model, attack scenarios, and security requirements covering authentication, admission control, constraint validation, and multi-hop integrity.</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>https://www.ietf.org/archive/id/draft-chen-oauth-roadmap-00.html</t>
+          <t>https://datatracker.ietf.org/doc/draft-jiang-intent-security/</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -3405,7 +3405,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>Brand-new -00 draft (May 2026); the single most useful index when starting work in this area.</t>
+          <t>Revision -03, 22 Jun 2026; authors: Yuning Jiang, Lun Li, Yurong Song, Faye Liu (Huawei). The threat-model companion to draft-jiang-oauth-intent-admission from the same group; likely intended to inform the broader IETF agentic AI security discussion.</t>
         </is>
       </c>
     </row>
@@ -3415,25 +3415,325 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
+          <t>draft-somoza-dmsc-atn-agent-trust-negotiation — Agent Trust Negotiation: Capability, Delegation, and Provenance Binding</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Specifies the Agent Trust Negotiation (ATN) protocol, which binds four artifacts — capability manifests, delegation chains, provenance attestations, and session receipts — to agent identities via a handshake state machine producing mutually verified, scope-bounded sessions with SCITT-suitable audit records.</t>
+        </is>
+      </c>
+      <c r="D84" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-somoza-dmsc-atn-agent-trust-negotiation/</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 29 May 2026; author: Enrique Somoza (Independent). Operates above discovery mechanisms and positions itself between the discovery layer (DAWN, MCP) and the authorization layer (WIMSE, OAuth). Relevant as an agent-to-agent trust establishment handshake protocol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>draft-mcgraw-httpapi-agent-budget — The Delegation HTTP Authentication Scheme for Request-Bound Authority</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>Defines the 'Delegation' HTTP authentication scheme and response semantics for delegated-authority challenges using HTTP status codes and Problem Details, plus a CBOR/COSE proof format. The initial authority profile is 'Budget,' using post-quantum ML-DSA to prove spending or resource-consumption limits.</t>
+        </is>
+      </c>
+      <c r="D85" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-mcgraw-httpapi-agent-budget/</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, 15 Jun 2026; author: John Paul McGraw Jr. (TaskHawk Systems). HTTP-layer bounded delegation with post-quantum crypto; distinct from OAuth-layer delegation in that the authority proof travels in the Authorization header. Complements x401 (Industry tab) at the HTTP challenge-response layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>draft-vauban-x402-delegation-binding — x402 Delegation Binding for Agentic HTTP Pipelines</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Addresses the security gap where x402 V2 payment grants issued to one agent could be misused by another in the same pipeline, introducing three binding mechanisms: a JCS-derived agent identity pseudonym, a nonce for anti-replay, and a depth-limiting field for transitive delegation.</t>
+        </is>
+      </c>
+      <c r="D86" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-vauban-x402-delegation-binding/</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 25 May 2026; author: Vauban Research. Narrowly scoped to payment pipelines but the delegation-binding pattern (pseudonymous identity + anti-replay + depth-limit) is applicable broadly. Validated across five language runtimes with A2A and MCP integration guidance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>draft-samal-vap — Verifiable Agent Protocol (VAP): Intent-Bound Admission Control and Audit for Agent Tool Invocation</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Specifies VAP as a defense-in-depth layer adding declarations of purpose and session budget commitments to tool invocation requests (targeting MCP-style protocols), enabling servers to perform admission control before execution via four messages carried in existing protocol metadata.</t>
+        </is>
+      </c>
+      <c r="D87" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-samal-vap/</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 3 Jun 2026; author: Kruttidipta Samal (Independent). Lightweight and protocol-agnostic; addresses erroneous agent behavior, cost control, and audit trails without replacing existing auth mechanisms. Practical tool-invocation-level authorization layer for MCP deployments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>draft-khera-aurora — Agent Unification, Runtime, and Operational Responsibility Attestation (AURORA)</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>A two-layer framework unifying hardware-enclave-backed Runtime Integrity Attestation with scoped, cryptographically bound Authority Delegation; enables agents to prove both operational authority and runtime integrity simultaneously.</t>
+        </is>
+      </c>
+      <c r="D88" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-khera-aurora/</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 5 Jun 2026; author: Ankur Khera. Addresses the gap where delegation tokens don't prove the runtime environment is trustworthy — relevant where delegation must be paired with platform attestation (enterprise/regulated deployments). Bridges the RATS attestation thread and the OAuth delegation thread.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>draft-borthwick-msebenzi-environment-state — Verifiable Intent — environment.* Constraint Family</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Defines the environment.* constraint family for agent-authorization mandate vocabularies, covering external conditions at transaction execution time (venue availability, wallet funding) that existing transactional constraints cannot address. Extends agent authorization mandate frameworks with environmental precondition checking.</t>
+        </is>
+      </c>
+      <c r="D89" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-borthwick-msebenzi-environment-state/</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 13 Jun 2026; authors: Douglas Cameron Borthwick (InsumerAPI), Michael Msebenzi (Headless Oracle). Narrow but practically important for financial and commerce agent workflows; connects to draft-mcgraw-httpapi-agent-budget and draft-vauban-x402-delegation-binding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>draft-chen-oauth-agent-authz-use-cases — Agent Authorization Use Cases and Gap Analysis for OAuth 2.0</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>A framework-level analysis enumerating agentic authorization use cases — delegated task execution, multi-agent coordination, long-running workflows, capability attenuation — and mapping each against current OAuth 2.0 mechanisms to identify gaps that require new extensions or profiles.</t>
+        </is>
+      </c>
+      <c r="D90" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-chen-oauth-agent-authz-use-cases/</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 5 Jul 2026; useful problem-statement companion to the OAuth recharter's 'Complex Delegation' milestone. Gap analysis directly motivates several other drafts in this corpus — a natural reference document for the OAuth WG scoping discussion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>draft-agnihotri-oauth-agent-impl-status — Implementation Status of OAuth Identity Chaining and Transaction Tokens</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>An RFC 7942–compliant implementation status report tracking open-source implementations of draft-ietf-oauth-identity-chaining and draft-ietf-oauth-transaction-tokens against the relevant spec requirements.</t>
+        </is>
+      </c>
+      <c r="D91" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-agnihotri-oauth-agent-impl-status/</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, Jun 2026; provides the implementation evidence required to advance both WG drafts toward IESG submission. Informational companion to the two WG drafts — not a protocol spec but tracking their standardization progress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>draft-hardt-aauth-protocol — AAuth Protocol</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>A new clean-sheet authorization protocol from Dick Hardt (original OAuth author) defining proof-of-possession by default, resource-signed challenges, agent identity without pre-registration, deferred 202 responses, and AS-to-AS federation for the agent ecosystem.</t>
+        </is>
+      </c>
+      <c r="D92" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-hardt-aauth-protocol/</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, April 2026; the design rationale section explicitly explains why AAuth is not GNAP, not OAuth, not DPoP and not mTLS — important read for anyone planning a new agent-auth stack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>draft-chen-oauth-roadmap — Comprehensive Roadmap for OAuth 2.0 Standards and Drafts</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>An IETF informational draft that maps the entire OAuth 2.0 ecosystem of RFCs, BCPs, and active drafts into functional layers from core to extensions to industry profiles.</t>
+        </is>
+      </c>
+      <c r="D93" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ietf.org/archive/id/draft-chen-oauth-roadmap-00.html</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>Brand-new -00 draft (May 2026); the single most useful index when starting work in this area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
           <t>Charter: WIMSE — Workload Identity in Multi-System Environments (charter-ietf-wimse-01)</t>
         </is>
       </c>
-      <c r="C84" s="5" t="inlineStr">
+      <c r="C94" s="5" t="inlineStr">
         <is>
           <t>The formal IETF charter for the WIMSE WG covering architecture, JOSE-based WIMSE tokens for service-to-service traffic, local token issuance, and token exchange profiles (likely based on RFC 8693) for cross-trust-domain workload identity.</t>
         </is>
       </c>
-      <c r="D84" s="9" t="inlineStr">
+      <c r="D94" s="9" t="inlineStr">
         <is>
           <t>https://datatracker.ietf.org/doc/charter-ietf-wimse/01/</t>
         </is>
       </c>
-      <c r="E84" s="5" t="inlineStr">
+      <c r="E94" s="5" t="inlineStr">
         <is>
           <t>IETF (WIMSE WG charter)</t>
         </is>
       </c>
-      <c r="F84" s="5" t="inlineStr">
+      <c r="F94" s="5" t="inlineStr">
         <is>
           <t>Approved 18 March 2026 (v01); explicitly liaises with OAuth, SCIM, SCITT, RATS, the OpenID Foundation, and CNCF/SPIFFE — the formal scope statement that anchors all WIMSE draft work.</t>
         </is>
@@ -3524,6 +3824,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId93"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Proposed boundaries between IETF groups
</commit_message>
<xml_diff>
--- a/delegated_authorization_research.xlsx
+++ b/delegated_authorization_research.xlsx
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>99</v>
+        <v>117</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="6" t="n">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="D11" s="7" t="n"/>
     </row>
@@ -906,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1015,27 +1015,27 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Charter: AI Preferences WG (charter-ietf-aipref-01)</t>
+          <t>draft-nottingham-webbotauth-use-cases — Use Cases for Authentication of Web Bots</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>The formal IETF charter for the AIPREF WG, standardizing vocabulary and protocol mechanisms (e.g., extending the Robots Exclusion Protocol and HTTP headers) for content owners to express preferences about AI training, deployment, and use of their content.</t>
+          <t>Frames the key questions for WebBotAuth WG scope: what sites need (mitigating bot abuse, access control for human-gated content), what bot operators need (IP mobility, non-IP-based identity), and the tension between them when a bot operator wants to be recognized but not tracked.</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/charter-ietf-aipref/01/</t>
+          <t>https://datatracker.ietf.org/doc/draft-nottingham-webbotauth-use-cases/</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>IETF (AIPREF WG charter)</t>
+          <t>IETF (WebBotAuth WG)</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Approved April 2025; the charter explicitly puts 'authenticating or authorizing clients and/or crawlers' out of scope — included here for ecosystem context, not because it's delegated-authz work per se. Sibling WG to WebBotAuth.</t>
+          <t>Revision -02, Apr 2026; author: Mark Nottingham (Melbourne). The foundational use-case framing for the WG; scopes out the design space that the registry, httpsig-protocol, and anonymous-auth drafts are responding to.</t>
         </is>
       </c>
     </row>
@@ -1045,27 +1045,27 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>draft-king-dawn-requirements — Requirements for Discovery of Agents, Workloads, and Named Entities (DAWN)</t>
+          <t>draft-meunier-webbotauth-registry — Registry and Signature Agent Card for Web Bot Auth</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>An individual IETF draft from Adrian Farrel and Daniel King setting out solution-neutral requirements for discovering AI agents, services, and workloads across administrative boundaries — what must be discoverable, what trust properties apply, and what architectural constraints exist.</t>
+          <t>Defines the 'Signature Agent Card,' a JSON metadata document enabling bots to publish their identity, capabilities, and public keys; establishes a IANA registry drawing from OAuth client metadata extended with bot-specific fields including crawl-rate declarations and data-use purpose.</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-king-dawn-requirements/01/</t>
+          <t>https://datatracker.ietf.org/doc/draft-meunier-webbotauth-registry/</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (WebBotAuth WG)</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, April 2026; intentionally NOT a protocol — sits one layer below auth. Authentication and authorization of discovered entities are out of scope, but DAWN discovery happens *before* auth/authz can begin.</t>
+          <t>Revision -03, Jun 26 2026 (most mature WG document); authors: Maxime Guerreiro, Thibault Meunier (Cloudflare), Ulas Kirazci (Amazon). The Agent Card is the identity artifact that the httpsig-protocol references; together they form the core WebBotAuth authentication architecture.</t>
         </is>
       </c>
     </row>
@@ -1075,27 +1075,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>draft-ietf-oauth-v2-1 — The OAuth 2.1 Authorization Framework</t>
+          <t>draft-meunier-webbotauth-httpsig-protocol — HTTP Message Signatures for Automated Traffic</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>An IETF WG draft that obsoletes RFC 6749/6750 by mandating PKCE for the authorization code grant, removing implicit and ROPC, and requiring exact redirect-URI matching.</t>
+          <t>Defines the core WebBotAuth authentication architecture: automated agents sign HTTP requests with private keys bound to their Agent Card; origin servers verify agent identity through public key discovery via the registry. Intended to replace IP allowlisting and User-Agent string matching as the primary bot identification mechanism.</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-v2-1/</t>
+          <t>https://datatracker.ietf.org/doc/draft-meunier-webbotauth-httpsig-protocol/</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>IETF (OAuth WG)</t>
+          <t>IETF (WebBotAuth WG)</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Revision -15 (March 2026) is the current baseline that MCP, FAPI 2.0, and most agent specs profile against.</t>
+          <t>Revision -00, Jun 26 2026; authors: Thibault Meunier (Cloudflare), Sandor Major (Google). Replaces draft-meunier-web-bot-auth-architecture. Pairs with draft-meunier-webbotauth-httpsig-directory for key discovery.</t>
         </is>
       </c>
     </row>
@@ -1105,27 +1105,27 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>draft-ietf-oauth-identity-chaining — OAuth Identity and Authorization Chaining Across Domains</t>
+          <t>draft-meunier-webbotauth-httpsig-directory — HTTP Message Signatures Directory</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>An IETF WG draft that defines how to preserve identity and authorization context across trust domains by combining RFC 8693 token exchange with RFC 7521/7523 JWT assertions.</t>
+          <t>Defines a JWKS-based key directory, a well-known URI for key discovery (/.well-known/bot-auth-directory), and a new HTTP header field for in-band signing-key location communication, enabling origin servers to resolve a bot's signing key without prior configuration.</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-identity-chaining/</t>
+          <t>https://datatracker.ietf.org/doc/draft-meunier-webbotauth-httpsig-directory/</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>IETF (OAuth WG)</t>
+          <t>IETF (WebBotAuth WG)</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>IESG-approved; currently in RFC Editor queue (status: Waiting on Authors — outstanding SECDIR 'Has issues' and OPSDIR 'Not ready' flags unresolved; no RFC number assigned yet as of Jul 2026). The canonical multi-domain delegation pattern referenced by most agent and zero-trust drafts.</t>
+          <t>Revision -00, Jun 26 2026; authors: Thibault Meunier (Cloudflare), Sandor Major (Google). Replaces draft-meunier-http-message-signatures-directory. The key-discovery complement to httpsig-protocol.</t>
         </is>
       </c>
     </row>
@@ -1135,27 +1135,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>draft-ietf-oauth-identity-assertion-authz-grant — Identity Assertion JWT Authorization Grant (ID-JAG)</t>
+          <t>draft-rescorla-anonymous-webbotauth — Anonymous Bot Authentication: Authorization and Rate Limiting for Web Agents</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>An IETF WG draft (Parecki/McGuinness/Campbell) defining how an app uses an identity assertion to obtain an access token for a third-party API by coordinating through a shared enterprise IdP.</t>
+          <t>Proposes Anonymous Bot Authentication (ABA) using Privacy Pass tokens and Anonymous Rate-Limited Credentials, enabling sites to enforce rate limits and access controls on bots without identifying individual operators. Decouples 'is this a legitimate bot' from 'which bot is this,' preserving privacy while preventing abuse.</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-identity-assertion-authz-grant/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rescorla-anonymous-webbotauth/</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>IETF (OAuth WG)</t>
+          <t>IETF (WebBotAuth WG)</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Revision -03, April 2026; the cross-IdP SSO-to-API bridge that the McGuinness Actor Profile draft layers on top of, and that WorkOS's auth.md uses as one of its three discovery flows.</t>
+          <t>Revision -00, Apr 7 2026; authors: Eric Rescorla (Independent), Richard L. Barnes (Cisco). Proposes the privacy-preserving counterpart to the httpsig identity approach — the WG will need to decide where the identity/anonymity balance lies.</t>
         </is>
       </c>
     </row>
@@ -1165,27 +1165,27 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>draft-ietf-oauth-transaction-tokens — Transaction Tokens (Txn-Tokens)</t>
+          <t>Charter: AI Preferences WG (charter-ietf-aipref-01)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>An IETF WG draft defining short-lived signed JWTs that propagate immutable user identity and authorization context through internal call chains within a trust domain.</t>
+          <t>The formal IETF charter for the AIPREF WG, standardizing vocabulary and protocol mechanisms (e.g., extending the Robots Exclusion Protocol and HTTP headers) for content owners to express preferences about AI training, deployment, and use of their content.</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-transaction-tokens/</t>
+          <t>https://datatracker.ietf.org/doc/charter-ietf-aipref/01/</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>IETF (OAuth WG)</t>
+          <t>IETF (AIPREF WG charter)</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Revision -09 published 6 Jul 2026 (was -08 Mar 2026); co-authored by Tulshibagwale (CAEP inventor), Fletcher, and Kasselman. -09 reorganized the Request Context section, changed JWT body claims from OPTIONAL to RECOMMENDED, and enhanced security considerations for invalidated access tokens. Still in WGLC; IESG submission milestone Dec 2026.</t>
+          <t>Approved April 2025; the charter explicitly puts 'authenticating or authorizing clients and/or crawlers' out of scope — included here for ecosystem context, not because it's delegated-authz work per se. Sibling WG to WebBotAuth.</t>
         </is>
       </c>
     </row>
@@ -1195,27 +1195,27 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>draft-ietf-oauth-first-party-apps — OAuth 2.0 for First-Party Applications</t>
+          <t>draft-king-dawn-requirements — Requirements for Discovery of Agents, Workloads, and Named Entities (DAWN)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>An IETF WG draft defining an Authorization Challenge Endpoint that lets first-party native apps drive a browserless OAuth flow while still supporting step-up authentication via RFC 9470.</t>
+          <t>An individual IETF draft from Adrian Farrel and Daniel King setting out solution-neutral requirements for discovering AI agents, services, and workloads across administrative boundaries — what must be discoverable, what trust properties apply, and what architectural constraints exist.</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-first-party-apps/</t>
+          <t>https://datatracker.ietf.org/doc/draft-king-dawn-requirements/01/</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>IETF (OAuth WG)</t>
+          <t>IETF (individual)</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Revision -04, published 1 Jul 2026; explicitly excluded for third-party use because it requires high AS↔client trust.</t>
+          <t>Revision -01, April 2026; intentionally NOT a protocol — sits one layer below auth. Authentication and authorization of discovered entities are out of scope, but DAWN discovery happens *before* auth/authz can begin.</t>
         </is>
       </c>
     </row>
@@ -1225,27 +1225,27 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>draft-ietf-oauth-attestation-based-client-auth — OAuth 2.0 Attestation-Based Client Authentication</t>
+          <t>draft-farrel-dawn-terminology — Terminology for the Discovery of Agents, Workloads, and Named Entities (DAWN)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>An IETF WG draft (Looker/Bastian/Bormann) introducing two JWTs — a Client Attestation issued by a Client Attester and a Client Attestation PoP signed by the client instance — that travel in HTTP headers to let traditionally-public clients authenticate to the AS without a shared secret.</t>
+          <t>Establishes standardized vocabulary across DAWN specifications: agents, workloads, named entities, capabilities, discovery processes, and registration functions. Defines the entities-to-be-discovered and the properties discovery must convey, without specifying protocol mechanics.</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-attestation-based-client-auth/</t>
+          <t>https://datatracker.ietf.org/doc/draft-farrel-dawn-terminology/</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>IETF (OAuth WG)</t>
+          <t>IETF (individual)</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Revision -10, Jul 2026 (was -08 Mar 2026). -10 added a 'client_attestation_pop_methods_supported' metadata parameter, created a new 'OAuth Client Attestation Proof-of-Possession Methods' registry, clarified that PoP mechanisms from other specs are permitted, and refined DPoP combined-mode handling. Relates to the RATS Passport Model per RFC 9334; RATS attestation procedures themselves are deliberately out of scope. The 'client instance' framing pairs naturally with the McGuinness Client Instance Assertion and AI Agent Instance drafts.</t>
+          <t>Revision -03, Jul 5 2026; authors: Adrian Farrel (Old Dog Consulting), Kehan Yao (China Mobile), Roland Schott (Deutsche Telekom), Nic Williams (Infoblox). At rev 03 the most mature DAWN document after the requirements draft; Farrel/Williams authorship signals serious WG momentum. IETF 126 (Bangkok, Jul 2026) has DAWN BoF time.</t>
         </is>
       </c>
     </row>
@@ -1255,27 +1255,27 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>draft-ietf-oauth-spiffe-client-auth — OAuth SPIFFE Client Authentication</t>
+          <t>draft-akhavain-moussa-dawn-problem-statement — Problem Statement for the Discovery of Agents, Workloads, and Named Entities (DAWN)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>An IETF WG draft (Schwenkschuster/Kasselman/Rose-NIST/Thorgersen-IBM) profiling RFC 7521, RFC 7523, and OAuth attestation-based client auth so that SPIFFE-enabled workloads can authenticate to OAuth ASes using JWT-SVID, WIT-SVID, or X.509-SVID credentials instead of shared client secrets.</t>
+          <t>Articulates cross-domain discovery challenges for the DAWN problem space: scalability across administrative boundaries, trust in discovered information, and the absence of a unified discovery model for heterogeneous AI agents and workloads. Establishes functional requirements that protocol proposals must satisfy.</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-spiffe-client-auth/</t>
+          <t>https://datatracker.ietf.org/doc/draft-akhavain-moussa-dawn-problem-statement/</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>IETF (OAuth WG)</t>
+          <t>IETF (individual)</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, March 2026 (re-slugged from draft-schwenkschuster-oauth-spiffe-client-auth after WG adoption); the protocol bridge between SPIFFE/WIMSE workload identity and the OAuth client-auth surface.</t>
+          <t>Revision -04, Jun 12 2026; authors: Arashmid Akhavain, Hesham Moussa (Huawei Canada), Daniel King (Old Dog Consulting). King co-authorship ties this to draft-king-dawn-requirements already in corpus; together they are the two foundational DAWN framing documents.</t>
         </is>
       </c>
     </row>
@@ -1285,17 +1285,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>draft-kahrer-oauth-client-challenge-protocol — OAuth Client Challenge Protocol</t>
+          <t>draft-moussa-dawn-gap-analysis — Gap Analysis and Applicability Statement for Discovery Protocols of DAWN</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Judith Kahrer (Curity) defining a new 'insufficient_client_authorization' error code so the authorization server can dynamically challenge the client mid-flow for an additional assertion, verifiable presentation, or proof-of-possession material — enabling just-in-time and step-up client authorization.</t>
+          <t>Evaluates DNS, mDNS/DNS-SD, SSDP/UPnP, and other existing discovery protocols against DAWN requirements, identifying security gaps (no agent-specific trust model), privacy gaps (broadcast exposure), and applicability limits (local-scope vs. global cross-domain scenarios); proposes hybrid patterns and mitigations.</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-kahrer-oauth-client-challenge-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-moussa-dawn-gap-analysis/</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Revision -00 published 19 May 2026; deliberately distinct from first-party-apps (challenges the CLIENT, not the user) and works for both first- and third-party clients. Cites Mastercard Verifiable Intent as a use case, linking it directly to the mandate/RAR pattern OVID implements.</t>
+          <t>Revision -01, Jun 12 2026; authors: Hesham Moussa, Arashmid Akhavain (Huawei Canada). Directly informs which existing protocol building blocks DAWN can reuse vs. what must be specified fresh. Key input for understanding why a new WG is needed rather than profiling DNS or mDNS.</t>
         </is>
       </c>
     </row>
@@ -1315,27 +1315,27 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>draft-ietf-oauth-browser-based-apps — OAuth 2.0 for Browser-Based Applications</t>
+          <t>draft-jimenez-dawn-discovery-landscape — A Survey of AI Agent Discovery Mechanisms</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>An IETF WG draft establishing the Backend-for-Frontend (BFF) and other architectural patterns as current best practice for SPAs given browser-resident token-storage limitations.</t>
+          <t>Surveys discovery mechanisms across standardization bodies and open-source projects (MCP, A2A, robots.txt, Well-Known URIs, registry services), comparing approaches by model, scope, and semantic capability, and identifying remaining standardization gaps that DAWN must address.</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-browser-based-apps/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jimenez-dawn-discovery-landscape/</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>IETF (OAuth WG)</t>
+          <t>IETF (individual)</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Revision -26 (Dec 2025); critical for any delegated-authorization design touching SPAs because it codifies why pure-browser refresh tokens are deprecated.</t>
+          <t>Revision -00, Jul 3 2026; authors: Jaime Jimenez, Jim Feng, Jari Arkko, Mirja Kühlewind, Rajat Kandoi (all Ericsson). Kühlewind co-authorship (same as kuehlewind-audit-architecture in corpus) is notable — the audit architecture team is tracking the discovery space. Useful as the landscape reference for the boundaries analysis.</t>
         </is>
       </c>
     </row>
@@ -1345,17 +1345,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>draft-ietf-oauth-security-topics-update — Updates to OAuth 2.0 Security BCP</t>
+          <t>draft-ietf-oauth-v2-1 — The OAuth 2.1 Authorization Framework</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>An IETF WG draft that extends RFC 9700 with new countermeasures, notably rules against audience-injection attacks where a client authenticates to multiple authorization servers.</t>
+          <t>An IETF WG draft that obsoletes RFC 6749/6750 by mandating PKCE for the authorization code grant, removing implicit and ROPC, and requiring exact redirect-URI matching.</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-security-topics-update/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-v2-1/</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, March 2026; co-authored by University of Stuttgart (FAPI formal-analysis team) so the recommendations are formally grounded.</t>
+          <t>Revision -15 (March 2026) is the current baseline that MCP, FAPI 2.0, and most agent specs profile against.</t>
         </is>
       </c>
     </row>
@@ -1375,27 +1375,27 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-actor-profile — OAuth Actor Profile for Delegation</t>
+          <t>draft-ietf-oauth-identity-chaining — OAuth Identity and Authorization Chaining Across Domains</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Karl McGuinness's individual draft profiling the RFC 8693 'act' claim with required iss, optional sub_profile entity classification, and uniform processing across JWT assertion grants, JWT access tokens, and Transaction Tokens.</t>
+          <t>An IETF WG draft that defines how to preserve identity and authorization context across trust domains by combining RFC 8693 token exchange with RFC 7521/7523 JWT assertions.</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/html/draft-mcguinness-oauth-actor-profile-00</t>
+          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-identity-chaining/</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (OAuth WG)</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Revision -00 published 30 April 2026; defines depth-1+ chain validation, cycle-aware construction, and bearer-to-PoP upgrade — the most complete actor-representation profile to date.</t>
+          <t>IESG-approved; currently in RFC Editor queue (status: Waiting on Authors — outstanding SECDIR 'Has issues' and OPSDIR 'Not ready' flags unresolved; no RFC number assigned yet as of Jul 2026). The canonical multi-domain delegation pattern referenced by most agent and zero-trust drafts.</t>
         </is>
       </c>
     </row>
@@ -1405,27 +1405,27 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>draft-mw-oauth-actor-chain — Cryptographically Verifiable Actor Chains for OAuth 2.0 Token Exchange</t>
+          <t>draft-ietf-oauth-identity-assertion-authz-grant — Identity Assertion JWT Authorization Grant (ID-JAG)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft (Prasad/Krishnan/Lopez/Addepalli) defining six actor-chain profiles for RFC 8693 — Declared/Verified × Full/Subset/Actor-Only Disclosure — that preserve and cryptographically validate delegation-path continuity across successive token exchanges instead of relying on RFC 8693's informational-only nested act claims.</t>
+          <t>An IETF WG draft (Parecki/McGuinness/Campbell) defining how an app uses an identity assertion to obtain an access token for a third-party API by coordinating through a shared enterprise IdP.</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mw-oauth-actor-chain/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-identity-assertion-authz-grant/</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (OAuth WG)</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 30 Jun 2026 (was -00 May 2026; re-slugged from draft-mw-spice-actor-chain-05); a complementary alternative to the McGuinness Actor Profile that directly addresses RFC 8693's chain-splicing weakness by making the chain itself cryptographically verifiable rather than just informational.</t>
+          <t>Revision -03, April 2026; the cross-IdP SSO-to-API bridge that the McGuinness Actor Profile draft layers on top of, and that WorkOS's auth.md uses as one of its three discovery flows.</t>
         </is>
       </c>
     </row>
@@ -1435,27 +1435,27 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-client-instance-assertion — OAuth Client Instance Assertion</t>
+          <t>draft-ietf-oauth-transaction-tokens — Transaction Tokens (Txn-Tokens)</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Karl McGuinness's individual draft for representing a specific running instance of an OAuth client (rather than just the client registration) so authorization servers can bind grants to a concrete instance.</t>
+          <t>An IETF WG draft defining short-lived signed JWTs that propagate immutable user identity and authorization context through internal call chains within a trust domain.</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-client-instance-assertion/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-transaction-tokens/</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (OAuth WG)</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Note: full draft text was not retrievable through automated fetch at time of writing — recommend reading directly. Companion to the Actor Profile draft and to attestation-based client auth.</t>
+          <t>Revision -09 published 6 Jul 2026 (was -08 Mar 2026); co-authored by Tulshibagwale (CAEP inventor), Fletcher, and Kasselman. -09 reorganized the Request Context section, changed JWT body claims from OPTIONAL to RECOMMENDED, and enhanced security considerations for invalidated access tokens. Still in WGLC; IESG submission milestone Dec 2026.</t>
         </is>
       </c>
     </row>
@@ -1465,27 +1465,27 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-resource-token-resp — OAuth 2.0 Resource Parameter in Access Token Response</t>
+          <t>draft-ietf-oauth-first-party-apps — OAuth 2.0 for First-Party Applications</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>A McGuinness/Skokan individual draft adding a 'resource' parameter to the OAuth access token response so clients can confirm which resource the issued token is valid for, mitigating resource mix-up attacks especially in deployments that use RFC 8707 Resource Indicators.</t>
+          <t>An IETF WG draft defining an Authorization Challenge Endpoint that lets first-party native apps drive a browserless OAuth flow while still supporting step-up authentication via RFC 9470.</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-resource-token-resp/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-first-party-apps/</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (OAuth WG)</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Revision -03 (March 2026). Filip Skokan added as co-author in -03. Complements RFC 8707 / RFC 9700 / RFC 9207 by adding issuance-time confirmation to the discovery-time mechanisms. Notable for the agent-authz corpus because dynamic resource discovery is a core agent pattern and resource-mix-up attacks are amplified when agents juggle many short-lived tokens.</t>
+          <t>Revision -04, published 1 Jul 2026; explicitly excluded for third-party use because it requires high AS↔client trust.</t>
         </is>
       </c>
     </row>
@@ -1495,27 +1495,27 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-rfc9728bis — Update to OAuth 2.0 Protected Resource Metadata Resource Identifier Validation</t>
+          <t>draft-ietf-oauth-attestation-based-client-auth — OAuth 2.0 Attestation-Based Client Authentication</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>A McGuinness individual draft updating Section 3.3 of RFC 9728 (Protected Resource Metadata) so the resource value can be any URI sharing the same TLS origin as the requested URL whose path is a prefix of it — broadening the set of WWW-Authenticate response use cases without changing the rest of RFC 9728.</t>
+          <t>An IETF WG draft (Looker/Bastian/Bormann) introducing two JWTs — a Client Attestation issued by a Client Attester and a Client Attestation PoP signed by the client instance — that travel in HTTP headers to let traditionally-public clients authenticate to the AS without a shared secret.</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-rfc9728bis/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-attestation-based-client-auth/</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (OAuth WG)</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Revision -01 (Feb 2026). A small targeted correction to the PRM validation rule. Notable as supporting infrastructure for the McGuinness Mission-Bound OAuth work — PRM is the substrate for Resource AS / Resource Server discovery of required RAR types under that profile.</t>
+          <t>Revision -10, Jul 2026 (was -08 Mar 2026). -10 added a 'client_attestation_pop_methods_supported' metadata parameter, created a new 'OAuth Client Attestation Proof-of-Possession Methods' registry, clarified that PoP mechanisms from other specs are permitted, and refined DPoP combined-mode handling. Relates to the RATS Passport Model per RFC 9334; RATS attestation procedures themselves are deliberately out of scope. The 'client instance' framing pairs naturally with the McGuinness Client Instance Assertion and AI Agent Instance drafts.</t>
         </is>
       </c>
     </row>
@@ -1525,27 +1525,27 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-token-xchg-target-svc-disco — OAuth 2.0 Token Exchange Target Service Discovery</t>
+          <t>draft-ietf-oauth-spiffe-client-auth — OAuth SPIFFE Client Authentication</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>A McGuinness/Parecki individual draft defining a discovery endpoint that, given a subject token, returns the set of available target services (audiences, resources, scopes) the holder can request via RFC 8693 Token Exchange — accepting any registered subject_token_type so it supports advanced flows including identity chaining and cross-domain delegation.</t>
+          <t>An IETF WG draft (Schwenkschuster/Kasselman/Rose-NIST/Thorgersen-IBM) profiling RFC 7521, RFC 7523, and OAuth attestation-based client auth so that SPIFFE-enabled workloads can authenticate to OAuth ASes using JWT-SVID, WIT-SVID, or X.509-SVID credentials instead of shared client secrets.</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-token-xchg-target-svc-disco/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-spiffe-client-auth/</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (OAuth WG)</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Revision -01 (Feb 2026), co-authored with Aaron Parecki (Okta). Fills a discovery gap that ID-JAG and the Transaction Token Chaining Profile both implicitly assume — clients today must know which audience to request, which doesn't compose with open-world agentic flows where the right downstream service is determined at runtime.</t>
+          <t>Revision -01, March 2026 (re-slugged from draft-schwenkschuster-oauth-spiffe-client-auth after WG adoption); the protocol bridge between SPIFFE/WIMSE workload identity and the OAuth client-auth surface.</t>
         </is>
       </c>
     </row>
@@ -1555,17 +1555,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-actor-receipts — OAuth Actor Receipts for Delegation Provenance</t>
+          <t>draft-kahrer-oauth-client-challenge-protocol — OAuth Client Challenge Protocol</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>A McGuinness companion draft to the Actor Profile, aiming to provide per-hop signed receipts as the verifiable provenance layer that the Actor Profile (which keeps the 'act' chain informational) deliberately leaves out. Pulls over the provenance gap from the core profile so each principal in a delegation chain can produce independent cryptographic evidence.</t>
+          <t>An IETF individual draft from Judith Kahrer (Curity) defining a new 'insufficient_client_authorization' error code so the authorization server can dynamically challenge the client mid-flow for an additional assertion, verifiable presentation, or proof-of-possession material — enabling just-in-time and step-up client authorization.</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-actor-receipts/</t>
+          <t>https://datatracker.ietf.org/doc/draft-kahrer-oauth-client-challenge-protocol/</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 4 Jul 2026; now formally on IETF Datatracker (was GitHub-only pre-publication through Jun 2026). Recommended companion to the Actor Profile when a deployment needs Verified Full Disclosure mode (per the Mission-Bound OAuth Runtime Enforcement Profile's Actor Provenance Module). Completes a triad with actor-profile and actor-proofs — receipts provide provenance, proofs provide cryptographic per-hop accountability.</t>
+          <t>Revision -00 published 19 May 2026; deliberately distinct from first-party-apps (challenges the CLIENT, not the user) and works for both first- and third-party clients. Cites Mastercard Verifiable Intent as a use case, linking it directly to the mandate/RAR pattern OVID implements.</t>
         </is>
       </c>
     </row>
@@ -1585,27 +1585,27 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-actor-proofs — OAuth Actor-Signed Hop Proofs</t>
+          <t>draft-ietf-oauth-browser-based-apps — OAuth 2.0 for Browser-Based Applications</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Introduces the 'actor_proofs' claim — a signed per-hop proof chain where each actor signs its own participation and the target binding it authorized for that hop; proofs are hash-chained and validated using actor verification keys from trusted sources, with optional references to sibling actor receipts.</t>
+          <t>An IETF WG draft establishing the Backend-for-Frontend (BFF) and other architectural patterns as current best practice for SPAs given browser-resident token-storage limitations.</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-actor-proofs/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-browser-based-apps/</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (OAuth WG)</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 4 Jul 2026. Completes the actor triad with actor-profile (chain structure) and actor-receipts (provenance) — actor-proofs closes the cryptographic accountability gap. Filed the same day as ai-agent-instance, id-assertion-framework, and domain-authorized-issuer — McGuinness submitted four new I-Ds on Jul 4-6, bringing his total to 11 individual I-Ds on Datatracker.</t>
+          <t>Revision -26 (Dec 2025); critical for any delegated-authorization design touching SPAs because it codifies why pure-browser refresh tokens are deprecated.</t>
         </is>
       </c>
     </row>
@@ -1615,27 +1615,27 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-insufficient-claims — OAuth 2.0 Insufficient Claims Challenge</t>
+          <t>draft-ietf-oauth-security-topics-update — Updates to OAuth 2.0 Security BCP</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>A McGuinness individual draft defining an insufficient_claims error code and required_claims parameter enabling authorization servers and protected resources to signal precisely which claims are missing from a presented credential. Allows resource servers to request enriched credentials carrying specific missing attributes rather than returning a generic 401.</t>
+          <t>An IETF WG draft that extends RFC 9700 with new countermeasures, notably rules against audience-injection attacks where a client authenticates to multiple authorization servers.</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-insufficient-claims/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-security-topics-update/</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (OAuth WG)</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 27 May 2026. Enables just-in-time claim negotiation in multi-agent delegation chains where the acting party must assemble claims from multiple sources. Natural companion to the Actor Profile and Client Instance Assertion — those drafts define the identity structure; this one provides the feedback loop when that structure is incomplete at the RS.</t>
+          <t>Revision -01, March 2026; co-authored by University of Stuttgart (FAPI formal-analysis team) so the recommendations are formally grounded.</t>
         </is>
       </c>
     </row>
@@ -1645,17 +1645,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-ai-agent-instance — OAuth 2.0 AI Agent Instance Profile</t>
+          <t>draft-mcguinness-oauth-actor-profile — OAuth Actor Profile for Delegation</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Profiles OAuth 2.0 for deployments where a single client ID represents an agent platform running many concurrent agent instances; defines claims conveying attested agent instance identity and provenance from an agent attester to the AS, with delegation-chain semantics for sub-agents. Claims are carrier-independent, compatible with both Client Instance Assertions and Client Attestation JWT.</t>
+          <t>Karl McGuinness's individual draft profiling the RFC 8693 'act' claim with required iss, optional sub_profile entity classification, and uniform processing across JWT assertion grants, JWT access tokens, and Transaction Tokens.</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-ai-agent-instance/</t>
+          <t>https://datatracker.ietf.org/doc/html/draft-mcguinness-oauth-actor-profile-00</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 4 Jul 2026. Fills the gap between a registered OAuth client ID (platform-level) and a running agent instance (runtime-level) — the level at which delegation chains, attestation, and revocation actually operate. Companion to draft-mcguinness-oauth-client-instance-assertion (general instance framing) and draft-mcguinness-oauth-actor-profile (chain representation).</t>
+          <t>Revision -00 published 30 April 2026; defines depth-1+ chain validation, cycle-aware construction, and bearer-to-PoP upgrade — the most complete actor-representation profile to date.</t>
         </is>
       </c>
     </row>
@@ -1675,17 +1675,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-id-assertion-framework — OAuth Identity Assertion Trust Framework</t>
+          <t>draft-mw-oauth-actor-chain — Cryptographically Verifiable Actor Chains for OAuth 2.0 Token Exchange</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Addresses the gap where issuer authentication alone does not prove AS authority over subject namespaces; defines an Authority Delegation Model with independent trust-evaluation categories and an Identity Assertion Issuer Trust Policy (JSON document declaring required trust methods) that Resource ASes evaluate before accepting identity assertions.</t>
+          <t>An IETF individual draft (Prasad/Krishnan/Lopez/Addepalli) defining six actor-chain profiles for RFC 8693 — Declared/Verified × Full/Subset/Actor-Only Disclosure — that preserve and cryptographically validate delegation-path continuity across successive token exchanges instead of relying on RFC 8693's informational-only nested act claims.</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-id-assertion-framework/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mw-oauth-actor-chain/</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 4 Jul 2026. Directly motivates and companions draft-mcguinness-oauth-domain-authorized-issuer (below) which provides a DNS-based trust method. Addresses the 'who is allowed to assert identities in this namespace?' question that ID-JAG and the identity-chaining WG draft assume resolved but do not specify.</t>
+          <t>Revision -01, 30 Jun 2026 (was -00 May 2026; re-slugged from draft-mw-spice-actor-chain-05); a complementary alternative to the McGuinness Actor Profile that directly addresses RFC 8693's chain-splicing weakness by making the chain itself cryptographically verifiable rather than just informational.</t>
         </is>
       </c>
     </row>
@@ -1705,17 +1705,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-domain-authorized-issuer — OAuth Domain-Authorized Issuer Trust Method</t>
+          <t>draft-mcguinness-oauth-client-instance-assertion — OAuth Client Instance Assertion</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>DNS domain owners publish a policy (DNS TXT record at _oauth-issuer-policy.{domain} or HTTPS well-known fallback) listing the OAuth ASes authorized to assert identities in that namespace; Resource ASes use this to validate assertion issuers before accepting identity assertions or chaining tokens. Pattern echoes CAA/SPF/DKIM. Non-transitive — flat authorization, no delegation chains.</t>
+          <t>Karl McGuinness's individual draft for representing a specific running instance of an OAuth client (rather than just the client registration) so authorization servers can bind grants to a concrete instance.</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-domain-authorized-issuer/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-client-instance-assertion/</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 4 Jul 2026. Implements one trust method for draft-mcguinness-oauth-id-assertion-framework. DNS-based approach is lightweight and operationally familiar; the non-transitive design avoids the amplification risks of transitive trust chains. Closes the 'how do you know the AS is allowed to speak for this domain?' gap that cross-domain identity chaining has always assumed away.</t>
+          <t>Note: full draft text was not retrievable through automated fetch at time of writing — recommend reading directly. Companion to the Actor Profile draft and to attestation-based client auth.</t>
         </is>
       </c>
     </row>
@@ -1735,17 +1735,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-mission — Mission-Bound Authorization for OAuth 2.0</t>
+          <t>draft-mcguinness-oauth-resource-token-resp — OAuth 2.0 Resource Parameter in Access Token Response</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Introduces 'Mission' — a durable, integrity-bound artifact stored at the AS representing an approved task; clients submit Mission Intent via PAR, ASes derive concrete permissions, and approvers grant consent via integrity anchors. Access tokens carry a 'mission' claim; issuance is gated by the Mission's lifecycle state, enabling revocation governance and audit trails for multi-step agent operations.</t>
+          <t>A McGuinness/Skokan individual draft adding a 'resource' parameter to the OAuth access token response so clients can confirm which resource the issued token is valid for, mitigating resource mix-up attacks especially in deployments that use RFC 8707 Resource Indicators.</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-mission/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-resource-token-resp/</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 6 Jul 2026. This is the formal I-D target for the 'Mission-Bound OAuth MVP' blog post (May 2026, Industry tab) — the five-wire-addition protocol that makes the user-approved task a first-class OAuth object. Paired with the runtime enforcement profile (still not on Datatracker as of Jul 10). The Mission lifecycle (pending_approval → active → suspended → revoked → expired → completed → rejected) and the proposal_hash/consent_rendering_hash binding anchor what was approved versus what the user saw.</t>
+          <t>Revision -03 (March 2026). Filip Skokan added as co-author in -03. Complements RFC 8707 / RFC 9700 / RFC 9207 by adding issuance-time confirmation to the discovery-time mechanisms. Notable for the agent-authz corpus because dynamic resource discovery is a core agent pattern and resource-mix-up attacks are amplified when agents juggle many short-lived tokens.</t>
         </is>
       </c>
     </row>
@@ -1765,17 +1765,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>draft-mishra-oauth-agent-grants — Delegated Agent Authorization Protocol (DAAP)</t>
+          <t>draft-mcguinness-oauth-rfc9728bis — Update to OAuth 2.0 Protected Resource Metadata Resource Identifier Validation</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft addressing runtime agent identity for dynamically-spawned agents, multi-agent sub-delegation with depth-limiting, and cascade revocation of an entire delegation subtree when any ancestor is revoked.</t>
+          <t>A McGuinness individual draft updating Section 3.3 of RFC 9728 (Protected Resource Metadata) so the resource value can be any URI sharing the same TLS origin as the requested URL whose path is a prefix of it — broadening the set of WWW-Authenticate response use cases without changing the rest of RFC 9728.</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mishra-oauth-agent-grants/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-rfc9728bis/</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Revision -01 (March 2026); registers new JWT claims (agt, dev, grnt, scp, bdg) — a more aggressive alternative to RFC 8693 with budget-bounded grants. Overlaps with draft-niyikiza-oauth-attenuating-agent-tokens; OAuth WG will likely expect consolidation.</t>
+          <t>Revision -01 (Feb 2026). A small targeted correction to the PRM validation rule. Notable as supporting infrastructure for the McGuinness Mission-Bound OAuth work — PRM is the substrate for Resource AS / Resource Server discovery of required RAR types under that profile.</t>
         </is>
       </c>
     </row>
@@ -1795,17 +1795,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>draft-kuehlewind-audit-architecture — Architecture for Auditing AI Agent Delegation and Interactions</t>
+          <t>draft-mcguinness-token-xchg-target-svc-disco — OAuth 2.0 Token Exchange Target Service Discovery</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Mirja Kühlewind (Ericsson, former IETF TSV-AD) and Henk Birkholz (Fraunhofer SIT, lead author of RFC 9334 RATS and SCITT architecture) defining four record types — Interaction, Action, Delegation, and Authorization Transition — and an Audit Context that propagates across OAuth + WIMSE + RATS + SCITT to make agent behaviour verifiably auditable end-to-end.</t>
+          <t>A McGuinness/Parecki individual draft defining a discovery endpoint that, given a subject token, returns the set of available target services (audiences, resources, scopes) the holder can request via RFC 8693 Token Exchange — accepting any registered subject_token_type so it supports advanced flows including identity chaining and cross-domain delegation.</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-kuehlewind-audit-architecture/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-token-xchg-target-svc-disco/</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Revision -00 published 18 May 2026; the cross-layer integration piece — explicitly composes the McGuinness Actor Profile, Transaction Tokens, identity-chaining, ID-JAG, WIMSE, RATS, and SCITT into a single auditable architecture with 11 proposed work items. The treats-Agent-as-untrusted threat model is what regulators (SOX, PSD2, EU AI Act) actually want.</t>
+          <t>Revision -01 (Feb 2026), co-authored with Aaron Parecki (Okta). Fills a discovery gap that ID-JAG and the Transaction Token Chaining Profile both implicitly assume — clients today must know which audience to request, which doesn't compose with open-world agentic flows where the right downstream service is determined at runtime.</t>
         </is>
       </c>
     </row>
@@ -1825,17 +1825,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>draft-birkholz-verifiable-agent-conversations — Verifiable Agent Conversation Records</t>
+          <t>draft-mcguinness-oauth-actor-receipts — OAuth Actor Receipts for Delegation Provenance</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft (Birkholz/Heldt/Steele) defining a CDDL data format — with both JSON and CBOR encodings — for tamper-evident, verifiably-signed records of agent conversations, agent reasoning traces, tool calls, and system events that support long-term evidentiary value across chains of custody.</t>
+          <t>A McGuinness companion draft to the Actor Profile, aiming to provide per-hop signed receipts as the verifiable provenance layer that the Actor Profile (which keeps the 'act' chain informational) deliberately leaves out. Pulls over the provenance gap from the core profile so each principal in a delegation chain can produce independent cryptographic evidence.</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-birkholz-verifiable-agent-conversations/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-actor-receipts/</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Revision -00 published 25 Feb 2026; presented at IETF 125 dispatch and hotrfc. The canonical Interaction-Record format for the Kuehlewind audit architecture. Motivating examples are concrete: agents acting beyond scope, CoT divergence, and 'sandbagging' during evaluations.</t>
+          <t>Revision -00, 4 Jul 2026; now formally on IETF Datatracker (was GitHub-only pre-publication through Jun 2026). Recommended companion to the Actor Profile when a deployment needs Verified Full Disclosure mode (per the Mission-Bound OAuth Runtime Enforcement Profile's Actor Provenance Module). Completes a triad with actor-profile and actor-proofs — receipts provide provenance, proofs provide cryptographic per-hop accountability.</t>
         </is>
       </c>
     </row>
@@ -1855,17 +1855,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>draft-klrc-aiagent-auth — AI Agent Authentication and Authorization</t>
+          <t>draft-mcguinness-oauth-actor-proofs — OAuth Actor-Signed Hop Proofs</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft that does not invent new protocols but composes WIMSE/SPIFFE workload identity, OAuth 2.x, and OpenID SSF to authenticate and delegate authority to AI agents.</t>
+          <t>Introduces the 'actor_proofs' claim — a signed per-hop proof chain where each actor signs its own participation and the target binding it authorized for that hop; proofs are hash-chained and validated using actor verification keys from trusted sources, with optional references to sibling actor receipts.</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/html/draft-klrc-aiagent-auth-00</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-actor-proofs/</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, March 2026; introduces 'Agent Identity Management System (AIMS)' and is the cleanest standards-based framing of agent-as-workload.</t>
+          <t>Revision -00, 4 Jul 2026. Completes the actor triad with actor-profile (chain structure) and actor-receipts (provenance) — actor-proofs closes the cryptographic accountability gap. Filed the same day as ai-agent-instance, id-assertion-framework, and domain-authorized-issuer — McGuinness submitted four new I-Ds on Jul 4-6, bringing his total to 11 individual I-Ds on Datatracker.</t>
         </is>
       </c>
     </row>
@@ -1885,17 +1885,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>draft-niyikiza-oauth-attenuating-agent-tokens — Attenuating Authorization Tokens for Agentic Delegation Chains</t>
+          <t>draft-mcguinness-oauth-insufficient-claims — OAuth 2.0 Insufficient Claims Challenge</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft extending RFC 9396 Rich Authorization Requests with monotonic attenuation at each delegation hop, offline chain verification, and a typed constraint vocabulary for tool-level argument restrictions.</t>
+          <t>A McGuinness individual draft defining an insufficient_claims error code and required_claims parameter enabling authorization servers and protected resources to signal precisely which claims are missing from a presented credential. Allows resource servers to request enriched credentials carrying specific missing attributes rather than returning a generic 401.</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-niyikiza-oauth-attenuating-agent-tokens/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-insufficient-claims/</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, March 2026; arguably the strongest purely-OAuth-grounded delegation draft — offline verification is a key scalability property. Good path to OAuth WG adoption; overlaps with draft-mishra-oauth-agent-grants and will likely need to be consolidated with it.</t>
+          <t>Revision -00, 27 May 2026. Enables just-in-time claim negotiation in multi-agent delegation chains where the acting party must assemble claims from multiple sources. Natural companion to the Actor Profile and Client Instance Assertion — those drafts define the identity structure; this one provides the feedback loop when that structure is incomplete at the RS.</t>
         </is>
       </c>
     </row>
@@ -1915,17 +1915,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>draft-singla-agent-identity-protocol — AIP: Decentralized Identity and Delegation for AI Agents</t>
+          <t>draft-mcguinness-oauth-ai-agent-instance — OAuth 2.0 AI Agent Instance Profile</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft proposing a six-layer model (identity through reputation) for AI agents with W3C DID anchoring, a Delegation Depth counter, three Grant ceremony tiers (G1/G2/G3), DPoP proof-of-possession, and an MCP integration layer.</t>
+          <t>Profiles OAuth 2.0 for deployments where a single client ID represents an agent platform running many concurrent agent instances; defines claims conveying attested agent instance identity and provenance from an agent attester to the AS, with delegation-chain semantics for sub-agents. Claims are carrier-independent, compatible with both Client Instance Assertions and Client Attestation JWT.</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-singla-agent-identity-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-ai-agent-instance/</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 17 April 2026; the most comprehensive identity framework in the set. The W3C DID dependency will face IETF pushback, the 75+ page scope needs reduction, and the 'AIP' name collision with two other drafts (draft-prakash-aip, draft-aip-agent-identity-protocol) must be resolved.</t>
+          <t>Revision -00, 4 Jul 2026. Fills the gap between a registered OAuth client ID (platform-level) and a running agent instance (runtime-level) — the level at which delegation chains, attestation, and revocation actually operate. Companion to draft-mcguinness-oauth-client-instance-assertion (general instance framing) and draft-mcguinness-oauth-actor-profile (chain representation).</t>
         </is>
       </c>
     </row>
@@ -1945,17 +1945,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>draft-prakash-aip — AIP: Verifiable Delegation for AI Agent Systems</t>
+          <t>draft-mcguinness-oauth-id-assertion-framework — OAuth Identity Assertion Trust Framework</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft introducing Invocation-Bound Capability Tokens (IBCTs) in two modes — compact (JWT/Ed25519) for single-hop and chained (Biscuit + Datalog) for multi-hop — with bindings for MCP, A2A, and HTTP APIs.</t>
+          <t>Addresses the gap where issuer authentication alone does not prove AS authority over subject namespaces; defines an Authority Delegation Model with independent trust-evaluation categories and an Identity Assertion Issuer Trust Policy (JSON document declaring required trust methods) that Resource ASes evaluate before accepting identity assertions.</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-prakash-aip/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-id-assertion-framework/</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 27 March 2026; technically strong — Biscuit + Datalog is well-suited to scope attenuation. The 'AIP' name collision with draft-singla-agent-identity-protocol and draft-aip-agent-identity-protocol is a blocking issue for WG adoption.</t>
+          <t>Revision -00, 4 Jul 2026. Directly motivates and companions draft-mcguinness-oauth-domain-authorized-issuer (below) which provides a DNS-based trust method. Addresses the 'who is allowed to assert identities in this namespace?' question that ID-JAG and the identity-chaining WG draft assume resolved but do not specify.</t>
         </is>
       </c>
     </row>
@@ -1975,17 +1975,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>draft-goswami-agentic-jwt — Secure Intent Protocol: JWT-Compatible Agentic Identity and Workflow Management</t>
+          <t>draft-mcguinness-oauth-domain-authorized-issuer — OAuth Domain-Authorized Issuer Trust Method</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an Agentic JWT extension to OAuth 2.0 with a Supervisor Agent role for sub-agent coordination, explicitly addressing the 'intent-execution separation' gap and adding workflow-step authorization.</t>
+          <t>DNS domain owners publish a policy (DNS TXT record at _oauth-issuer-policy.{domain} or HTTPS well-known fallback) listing the OAuth ASes authorized to assert identities in that namespace; Resource ASes use this to validate assertion issuers before accepting identity assertions or chaining tokens. Pattern echoes CAA/SPF/DKIM. Non-transitive — flat authorization, no delegation chains.</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-goswami-agentic-jwt/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-domain-authorized-issuer/</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, December 2025; the intent-execution-separation framing is insightful and distinguishing. The workflow-step authorization approach is novel but may face skepticism in the OAuth WG.</t>
+          <t>Revision -00, 4 Jul 2026. Implements one trust method for draft-mcguinness-oauth-id-assertion-framework. DNS-based approach is lightweight and operationally familiar; the non-transitive design avoids the amplification risks of transitive trust chains. Closes the 'how do you know the AS is allowed to speak for this domain?' gap that cross-domain identity chaining has always assumed away.</t>
         </is>
       </c>
     </row>
@@ -2005,17 +2005,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>draft-ni-wimse-ai-agent-identity — WIMSE Applicability for AI Agents</t>
+          <t>draft-mcguinness-oauth-mission — Mission-Bound Authorization for OAuth 2.0</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft mapping the WIMSE workload-identity architecture to AI-agent use cases and establishing credential-management mechanisms for agentic AI within the WIMSE framework.</t>
+          <t>Introduces 'Mission' — a durable, integrity-bound artifact stored at the AS representing an approved task; clients submit Mission Intent via PAR, ASes derive concrete permissions, and approvers grant consent via integrity anchors. Access tokens carry a 'mission' claim; issuance is gated by the Mission's lifecycle state, enabling revocation governance and audit trails for multi-step agent operations.</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ni-wimse-ai-agent-identity/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-mission/</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, February 2026; an important bridge between the WIMSE WG and the AI agent space. If an AI-agent WG is ever chartered, this applicability statement is essential groundwork. Co-authored with Liu, who also leads the related security-requirements draft.</t>
+          <t>Revision -00, 6 Jul 2026. This is the formal I-D target for the 'Mission-Bound OAuth MVP' blog post (May 2026, Industry tab) — the five-wire-addition protocol that makes the user-approved task a first-class OAuth object. Paired with the runtime enforcement profile (still not on Datatracker as of Jul 10). The Mission lifecycle (pending_approval → active → suspended → revoked → expired → completed → rejected) and the proposal_hash/consent_rendering_hash binding anchor what was approved versus what the user saw.</t>
         </is>
       </c>
     </row>
@@ -2035,17 +2035,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-identity-framework — Agent Identity Framework: Trust and Identity for Autonomous AI Agents</t>
+          <t>draft-mishra-oauth-agent-grants — Delegated Agent Authorization Protocol (DAAP)</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft proposing a five-layer model (identity, authorization, attestation, evidence, trust) for autonomous AI agents, with a gap analysis between current Internet standards and agent requirements.</t>
+          <t>An IETF individual draft addressing runtime agent identity for dynamically-spawned agents, multi-agent sub-delegation with depth-limiting, and cascade revocation of an entire delegation subtree when any ancestor is revoked.</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-identity-framework/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mishra-oauth-agent-grants/</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 6 April 2026; more gap-analysis than protocol spec. Useful as problem statement. Five-layer model is a reasonable decomposition but insufficient as a standalone contribution. Part of the Sharif cluster (with -agent-audit-trail, -attp, etc.).</t>
+          <t>Revision -01 (March 2026); registers new JWT claims (agt, dev, grnt, scp, bdg) — a more aggressive alternative to RFC 8693 with budget-bounded grants. Overlaps with draft-niyikiza-oauth-attenuating-agent-tokens; OAuth WG will likely expect consolidation.</t>
         </is>
       </c>
     </row>
@@ -2065,17 +2065,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>draft-aip-agent-identity-protocol — AIP: Agentic Authentication and Authorized Policy Enforcement</t>
+          <t>draft-kuehlewind-audit-architecture — Architecture for Auditing AI Agent Delegation and Interactions</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an AIP Token signed per tool call (agent ID, tool, nonce, timestamp, signature), an AgentPolicy YAML format for per-tool argument constraints and DLP rules, and a Human-in-the-Loop proxy enforcement model.</t>
+          <t>An IETF individual draft from Mirja Kühlewind (Ericsson, former IETF TSV-AD) and Henk Birkholz (Fraunhofer SIT, lead author of RFC 9334 RATS and SCITT architecture) defining four record types — Interaction, Action, Delegation, and Authorization Transition — and an Audit Context that propagates across OAuth + WIMSE + RATS + SCITT to make agent behaviour verifiably auditable end-to-end.</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-aip-agent-identity-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-kuehlewind-audit-architecture/</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 16 March 2026; implementation-focused. YAML policy approach is pragmatic but not interoperable-by-design. HITL integration is a valuable safety feature. Third member of the 'AIP' name-collision triple — must be resolved before any can progress.</t>
+          <t>Revision -00 published 18 May 2026; the cross-layer integration piece — explicitly composes the McGuinness Actor Profile, Transaction Tokens, identity-chaining, ID-JAG, WIMSE, RATS, and SCITT into a single auditable architecture with 11 proposed work items. The treats-Agent-as-untrusted threat model is what regulators (SOX, PSD2, EU AI Act) actually want.</t>
         </is>
       </c>
     </row>
@@ -2095,17 +2095,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>draft-liu-oauth-chain-delegation — Delegation Chain for OAuth 2.0</t>
+          <t>draft-birkholz-verifiable-agent-conversations — Verifiable Agent Conversation Records</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Introduces a delegation_chain JWT claim as a structured companion to RFC 8693's act claim; delegation_chain records the complete delegation history as an ordered array with per-hop authorization constraints and optional cryptographic confirmation from each delegating agent. Supports cross-domain delegation with integrated user consent interaction.</t>
+          <t>An IETF individual draft (Birkholz/Heldt/Steele) defining a CDDL data format — with both JSON and CBOR encodings — for tamper-evident, verifiably-signed records of agent conversations, agent reasoning traces, tool calls, and system events that support long-term evidentiary value across chains of custody.</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-liu-oauth-chain-delegation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-birkholz-verifiable-agent-conversations/</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 6 Jun 2026; authors: Dapeng Liu, Judy Zhu, Suresh Krishnan (Ericsson), Aaron Parecki (Okta). Provides the structured delegation lineage that act alone cannot express; strong overlap with draft-mw-oauth-actor-chain and draft-niyikiza-oauth-attenuating-agent-tokens — OAuth WG will likely expect consolidation across these three.</t>
+          <t>Revision -00 published 25 Feb 2026; presented at IETF 125 dispatch and hotrfc. The canonical Interaction-Record format for the Kuehlewind audit architecture. Motivating examples are concrete: agents acting beyond scope, CoT divergence, and 'sandbagging' during evaluations.</t>
         </is>
       </c>
     </row>
@@ -2125,17 +2125,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>draft-fletcher-transaction-token-chaining-profile — Transaction Token Authorization Grant Profile for OAuth Identity and Authorization Chaining</t>
+          <t>draft-klrc-aiagent-auth — AI Agent Authentication and Authorization</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Establishes a framework for using Transaction Tokens as subject credentials in OAuth 2.0 Token Exchange requests (RFC 8693), enabling services within one trust domain to obtain JWT authorization grants for accessing resources across domain boundaries without exposing internal token formats.</t>
+          <t>An IETF individual draft that does not invent new protocols but composes WIMSE/SPIFFE workload identity, OAuth 2.x, and OpenID SSF to authenticate and delegate authority to AI agents.</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-fletcher-transaction-token-chaining-profile/</t>
+          <t>https://datatracker.ietf.org/doc/html/draft-klrc-aiagent-auth-00</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, 6 Jul 2026 (was -01 Jun 2026); authors: George Fletcher (Practical Identity LLC), Pieter Kasselman (Defakto Security), Sean O'Dell (CVS Health). Directly bridges draft-ietf-oauth-transaction-tokens and draft-ietf-oauth-identity-chaining (both in corpus), closing the 'how do TX Tokens actually cross domains' gap. Note: lead author is the corpus maintainer.</t>
+          <t>Revision -00, March 2026; introduces 'Agent Identity Management System (AIMS)' and is the cleanest standards-based framing of agent-as-workload.</t>
         </is>
       </c>
     </row>
@@ -2155,17 +2155,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>draft-zhu-oauth-async-delegation — Sender-Constrained Delegation Handle for Asynchronous OAuth 2.0 Identity Chaining</t>
+          <t>draft-niyikiza-oauth-attenuating-agent-tokens — Attenuating Authorization Tokens for Agentic Delegation Chains</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Introduces a Delegation Handle — a sender-constrained, audience-locked JWT issued by authorization servers — enabling acting clients to refresh chained access tokens without re-prompting an offline end user while maintaining strict policy bounds and identity chains.</t>
+          <t>An IETF individual draft extending RFC 9396 Rich Authorization Requests with monotonic attenuation at each delegation hop, offline chain verification, and a typed constraint vocabulary for tool-level argument restrictions.</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-zhu-oauth-async-delegation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-niyikiza-oauth-attenuating-agent-tokens/</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 22 May 2026; authors: Larry Zhu, Sam Currie (Atlassian). Addresses a concrete gap in agent delegation: what happens when the delegating human is not present to re-authorize. Directly relevant to long-running agentic workflows using draft-ietf-oauth-identity-chaining.</t>
+          <t>Revision -00, March 2026; arguably the strongest purely-OAuth-grounded delegation draft — offline verification is a key scalability property. Good path to OAuth WG adoption; overlaps with draft-mishra-oauth-agent-grants and will likely need to be consolidated with it.</t>
         </is>
       </c>
     </row>
@@ -2185,17 +2185,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>draft-chen-oauth-agent-revocation — OAuth 2.0 Agent Authorization Explicit Revocation</t>
+          <t>draft-singla-agent-identity-protocol — AIP: Decentralized Identity and Delegation for AI Agents</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Extends RFC 7009 token revocation for agent-based scenarios: introduces batch revocation by agent ID, cascading revocation across delegation chains, conditional revocation options, and verifiable audit trails.</t>
+          <t>An IETF individual draft proposing a six-layer model (identity through reputation) for AI agents with W3C DID anchoring, a Delegation Depth counter, three Grant ceremony tiers (G1/G2/G3), DPoP proof-of-possession, and an MCP integration layer.</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-chen-oauth-agent-revocation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-singla-agent-identity-protocol/</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 27 Apr 2026; authors: Meiling Chen, Li Su (China Mobile). Fills the lifecycle management gap — existing RFC 7009 revocation is single-token and client-centric, but agent delegation chains require cascade semantics. Natural companion to draft-ietf-oauth-transaction-tokens and draft-niyikiza-oauth-attenuating-agent-tokens.</t>
+          <t>Revision -00, 17 April 2026; the most comprehensive identity framework in the set. The W3C DID dependency will face IETF pushback, the 75+ page scope needs reduction, and the 'AIP' name collision with two other drafts (draft-prakash-aip, draft-aip-agent-identity-protocol) must be resolved.</t>
         </is>
       </c>
     </row>
@@ -2215,17 +2215,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>draft-jiang-oauth-intent-admission — Intent Admission Assertions for Agentic Systems</t>
+          <t>draft-prakash-aip — AIP: Verifiable Delegation for AI Agent Systems</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Defines a signed, verifiable Intent Admission Assertion (IAA) that an admission point creates after verifying agent identity, evaluating permissions against policy, and — when required — obtaining explicit user consent; the IAA is transmitted to the execution endpoint which re-validates before proceeding. Leverages OAuth and RFC 9396 Rich Authorization Requests.</t>
+          <t>An IETF individual draft introducing Invocation-Bound Capability Tokens (IBCTs) in two modes — compact (JWT/Ed25519) for single-hop and chained (Biscuit + Datalog) for multi-hop — with bindings for MCP, A2A, and HTTP APIs.</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jiang-oauth-intent-admission/</t>
+          <t>https://datatracker.ietf.org/doc/draft-prakash-aip/</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 23 Jun 2026; authors: Yuning Jiang, Lun Li, Yurong Song, Faye Liu (Huawei). The required_consent path maps directly to the HITL pattern central to the corpus. Companion to draft-jiang-intent-security (threat model) from the same Huawei group.</t>
+          <t>Revision -00, 27 March 2026; technically strong — Biscuit + Datalog is well-suited to scope attenuation. The 'AIP' name collision with draft-singla-agent-identity-protocol and draft-aip-agent-identity-protocol is a blocking issue for WG adoption.</t>
         </is>
       </c>
     </row>
@@ -2245,17 +2245,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>draft-ni-oauth-batch-authorization-delegation — Batch Authorization Delegation</t>
+          <t>draft-goswami-agentic-jwt — Secure Intent Protocol: JWT-Compatible Agentic Identity and Workflow Management</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Defines a mechanism for delegating a batch of fine-grained, actor-bound permissions in a single request across multiple collaborating actors; uses RFC 9396 RAR to carry per-actor authorization_details and RFC 8693 Token Exchange for sub-agent delegation, targeting multi-agent orchestration where a leader-agent receives batch permissions and delegates subsets to sub-agents.</t>
+          <t>An IETF individual draft defining an Agentic JWT extension to OAuth 2.0 with a Supervisor Agent role for sub-agent coordination, explicitly addressing the 'intent-execution separation' gap and adding workflow-step authorization.</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ni-oauth-batch-authorization-delegation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-goswami-agentic-jwt/</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 3 Jul 2026; authors: Ni Yuan, Peter Chunchi Liu (Huawei). Addresses the round-trip overhead problem in large-scale multi-agent orchestration — individual delegation exchanges per sub-agent don't scale. Complements draft-song-oauth-ai-agent-collaborate-authz (same Huawei group, coordination focus) and draft-niyikiza-oauth-attenuating-agent-tokens (attenuation semantics). The RAR-based batch approach aligns well with the OAuth WG's RAR investment.</t>
+          <t>Revision -00, December 2025; the intent-execution-separation framing is insightful and distinguishing. The workflow-step authorization approach is novel but may face skepticism in the OAuth WG.</t>
         </is>
       </c>
     </row>
@@ -2275,17 +2275,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>draft-liu-oauth-a2a-profile — Agent-to-Agent (A2A) Profile for OAuth Transaction Tokens</t>
+          <t>draft-ni-wimse-ai-agent-identity — WIMSE Applicability for AI Agents</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Defines a profile for using OAuth Transaction Tokens in distributed agent-to-agent communication scenarios; specifies mechanisms for embedding call-chain context within tokens to preserve agent identity, authorization information, and operational flow across agent workloads in trusted environments.</t>
+          <t>An IETF individual draft mapping the WIMSE workload-identity architecture to AI-agent use cases and establishing credential-management mechanisms for agentic AI within the WIMSE framework.</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-liu-oauth-a2a-profile/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ni-wimse-ai-agent-identity/</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>EXPIRED. Revision -00, Oct 2025; authors: Peter Chunchi Liu, Ni Yuan (Huawei) — same author pair as draft-ni-oauth-batch-authorization-delegation. Directly profiles draft-ietf-oauth-transaction-tokens for A2A use; overlaps significantly with draft-araut-oauth-transaction-tokens-for-agents. Never revised; likely deferred rather than abandoned given both authors remain active in the corpus through Jul 2026.</t>
+          <t>Revision -02, February 2026; an important bridge between the WIMSE WG and the AI agent space. If an AI-agent WG is ever chartered, this applicability statement is essential groundwork. Co-authored with Liu, who also leads the related security-requirements draft.</t>
         </is>
       </c>
     </row>
@@ -2305,17 +2305,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>draft-song-oauth-ai-agent-collaborate-authz — OAuth 2.0 Extension for Multi-AI Agent Collaboration</t>
+          <t>draft-sharif-agent-identity-framework — Agent Identity Framework: Trust and Identity for Autonomous AI Agents</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Extends OAuth 2.0 for coordinated multi-agent task groups: defines a collaborative authorization flow allowing a lead agent to obtain delegation tokens for sub-agents, with shared task context, coordinated scope attenuation, and cross-agent session binding.</t>
+          <t>An IETF individual draft proposing a five-layer model (identity, authorization, attestation, evidence, trust) for autonomous AI agents, with a gap analysis between current Internet standards and agent requirements.</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-song-oauth-ai-agent-collaborate-authz/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-identity-framework/</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, Jun/Jul 2026; authors: Yurong Song (Huawei) and colleagues. Addresses the multi-agent coordination gap at the OAuth layer — complements draft-jiang-oauth-intent-admission from the same Huawei group. Distinct from single-hop delegation drafts in explicitly modeling lead-agent-to-sub-agent scope sharing.</t>
+          <t>Revision -00, 6 April 2026; more gap-analysis than protocol spec. Useful as problem statement. Five-layer model is a reasonable decomposition but insufficient as a standalone contribution. Part of the Sharif cluster (with -agent-audit-trail, -attp, etc.).</t>
         </is>
       </c>
     </row>
@@ -2335,17 +2335,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>draft-kroehl-agentic-trust-aae — Agent Authorization Envelope (AAE)</t>
+          <t>draft-aip-agent-identity-protocol — AIP: Agentic Authentication and Authorized Policy Enforcement</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Specifies the AAE, a structured authorization container with three mandatory components — MANDATE, CONSTRAINTS, and VALIDITY — providing a machine-evaluable, cryptographically verifiable authorization assertion using W3C DIDs and Verifiable Credentials.</t>
+          <t>An IETF individual draft defining an AIP Token signed per tool call (agent ID, tool, nonce, timestamp, signature), an AgentPolicy YAML format for per-tool argument constraints and DLP rules, and a Human-in-the-Loop proxy enforcement model.</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-kroehl-agentic-trust-aae/</t>
+          <t>https://datatracker.ietf.org/doc/draft-aip-agent-identity-protocol/</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 21 May 2026; author: Lars Kersten Kroehl (CryptoKRI GmbH). Occupies similar design space to draft-mcguinness-oauth-actor-profile but uses a DID/VC substrate rather than OAuth — provides a useful alternative approach for non-OAuth deployments.</t>
+          <t>Revision -00, 16 March 2026; implementation-focused. YAML policy approach is pragmatic but not interoperable-by-design. HITL integration is a valuable safety feature. Third member of the 'AIP' name-collision triple — must be resolved before any can progress.</t>
         </is>
       </c>
     </row>
@@ -2365,17 +2365,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>draft-pidlisnyi-aps — Agent Passport System (APS)</t>
+          <t>draft-liu-oauth-chain-delegation — Delegation Chain for OAuth 2.0</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Specifies Ed25519-based agent passports, scoped delegation chains with constraints across seven dimensions (a lattice model where delegation monotonically narrows capabilities), cascade revocation, a three-signature policy chain, signed receipts, and MCP bindings; includes reference implementations in TypeScript and Python.</t>
+          <t>Introduces a delegation_chain JWT claim as a structured companion to RFC 8693's act claim; delegation_chain records the complete delegation history as an ordered array with per-hop authorization constraints and optional cryptographic confirmation from each delegating agent. Supports cross-domain delegation with integrated user consent interaction.</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-pidlisnyi-aps/</t>
+          <t>https://datatracker.ietf.org/doc/draft-liu-oauth-chain-delegation/</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 14 May 2026; author: Tymofii Pidlisnyi (AEOESS). Among the most comprehensive standalone agent authz specs in the wave — the seven-dimension constraint lattice and MCP binding make it directly implementable against Model Context Protocol deployments alongside draft-serra-mcp-discovery-uri.</t>
+          <t>Revision -00, 6 Jun 2026; authors: Dapeng Liu, Judy Zhu, Suresh Krishnan (Ericsson), Aaron Parecki (Okta). Provides the structured delegation lineage that act alone cannot express; strong overlap with draft-mw-oauth-actor-chain and draft-niyikiza-oauth-attenuating-agent-tokens — OAuth WG will likely expect consolidation across these three.</t>
         </is>
       </c>
     </row>
@@ -2395,17 +2395,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>draft-serra-mcp-discovery-uri — The mcp URI Scheme and MCP Server Discovery Mechanism</t>
+          <t>draft-fletcher-transaction-token-chaining-profile — Transaction Token Authorization Grant Profile for OAuth Identity and Authorization Chaining</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an 'mcp://' URI scheme combined with /.well-known/mcp-server (RFC 8615) and a DNS TXT fallback for discovery of Model Context Protocol servers.</t>
+          <t>Establishes a framework for using Transaction Tokens as subject credentials in OAuth 2.0 Token Exchange requests (RFC 8693), enabling services within one trust domain to obtain JWT authorization grants for accessing resources across domain boundaries without exposing internal token formats.</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-serra-mcp-discovery-uri/</t>
+          <t>https://datatracker.ietf.org/doc/draft-fletcher-transaction-token-chaining-profile/</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Already at revision -04 (March 2026), suggesting active iteration; narrow scope, clean design, and the strongest IANA-registration candidate in the set. OAuth 2.1 for auth is deliberately out of scope.</t>
+          <t>Revision -02, 6 Jul 2026 (was -01 Jun 2026); authors: George Fletcher (Practical Identity LLC), Pieter Kasselman (Defakto Security), Sean O'Dell (CVS Health). Directly bridges draft-ietf-oauth-transaction-tokens and draft-ietf-oauth-identity-chaining (both in corpus), closing the 'how do TX Tokens actually cross domains' gap. Note: lead author is the corpus maintainer.</t>
         </is>
       </c>
     </row>
@@ -2425,17 +2425,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-attp — ATTP: Agent Trust Transport Protocol</t>
+          <t>draft-zhu-oauth-async-delegation — Sender-Constrained Delegation Handle for Asynchronous OAuth 2.0 Identity Chaining</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining trust levels L0–L4 mapped to PSD2 Strong Customer Authentication requirements, with bindings for MCP (MCPS), REST, A2A, gRPC, and GraphQL; supersedes draft-sharif-agent-payment-trust.</t>
+          <t>Introduces a Delegation Handle — a sender-constrained, audience-locked JWT issued by authorization servers — enabling acting clients to refresh chained access tokens without re-prompting an offline end user while maintaining strict policy bounds and identity chains.</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-attp/</t>
+          <t>https://datatracker.ietf.org/doc/draft-zhu-oauth-async-delegation/</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, April 2026; regulatory mapping appendices (PSD2, PCI DSS) are notable — one of the few drafts engaging financial regulation directly. Ambitious scope. Part of the Sharif cluster.</t>
+          <t>Revision -00, 22 May 2026; authors: Larry Zhu, Sam Currie (Atlassian). Addresses a concrete gap in agent delegation: what happens when the delegating human is not present to re-authorize. Directly relevant to long-running agentic workflows using draft-ietf-oauth-identity-chaining.</t>
         </is>
       </c>
     </row>
@@ -2455,17 +2455,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-transport-protocol — Agent Transport Protocol (ATP): Async Store-and-Forward for AI Agents</t>
+          <t>draft-chen-oauth-agent-revocation — OAuth 2.0 Agent Authorization Explicit Revocation</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining async store-and-forward messaging semantics with cryptographic identity per relay hop, trust scoring at ingress, capability negotiation, and interop with Google A2A, MCP, and FIPA ACL; transport-agnostic over TCP/TLS/QUIC.</t>
+          <t>Extends RFC 7009 token revocation for agent-based scenarios: introduces batch revocation by agent ID, cascading revocation across delegation chains, conditional revocation options, and verifiable audit trails.</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-transport-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-chen-oauth-agent-revocation/</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 28 March 2026; addresses a real gap — most agent protocols assume synchronous availability, and store-and-forward is appropriate for long-running agentic tasks. Scope is broad and needs narrowing.</t>
+          <t>Revision -00, 27 Apr 2026; authors: Meiling Chen, Li Su (China Mobile). Fills the lifecycle management gap — existing RFC 7009 revocation is single-token and client-centric, but agent delegation chains require cascade semantics. Natural companion to draft-ietf-oauth-transaction-tokens and draft-niyikiza-oauth-attenuating-agent-tokens.</t>
         </is>
       </c>
     </row>
@@ -2485,17 +2485,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-audit-trail — Agent Audit Trail (AAT): Standard Logging Format for Autonomous AI Systems</t>
+          <t>draft-jiang-oauth-intent-admission — Intent Admission Assertions for Agentic Systems</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining a JSON-based audit record with mandatory fields (agent identity, action classification, outcome tracking, trust level) using RFC 8785 JSON Canonicalization and RFC 9562 UUIDs.</t>
+          <t>Defines a signed, verifiable Intent Admission Assertion (IAA) that an admission point creates after verifying agent identity, evaluating permissions against policy, and — when required — obtaining explicit user consent; the IAA is transmitted to the execution endpoint which re-validates before proceeding. Leverages OAuth and RFC 9396 Rich Authorization Requests.</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-audit-trail/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jiang-oauth-intent-admission/</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 29 March 2026; orthogonal to delegation but important for compliance — standardized audit-log format is a genuine gap. Complements identity frameworks well. A sibling/alternative to the Kuehlewind audit architecture which takes a far more ambitious cross-layer approach.</t>
+          <t>Revision -00, 23 Jun 2026; authors: Yuning Jiang, Lun Li, Yurong Song, Faye Liu (Huawei). The required_consent path maps directly to the HITL pattern central to the corpus. Companion to draft-jiang-intent-security (threat model) from the same Huawei group.</t>
         </is>
       </c>
     </row>
@@ -2515,17 +2515,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>draft-aiendpoint-ai-discovery — The AI Discovery Endpoint</t>
+          <t>draft-ni-oauth-batch-authorization-delegation — Batch Authorization Delegation</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining a /.well-known/ai URI suffix for programmatic service capability discovery by AI agents — letting agents discover what an endpoint supports without having to parse human-oriented documentation; requests IANA well-known URI registration.</t>
+          <t>Defines a mechanism for delegating a batch of fine-grained, actor-bound permissions in a single request across multiple collaborating actors; uses RFC 9396 RAR to carry per-actor authorization_details and RFC 8693 Token Exchange for sub-agent delegation, targeting multi-agent orchestration where a leader-agent receives batch permissions and delegates subsets to sub-agents.</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-aiendpoint-ai-discovery/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ni-oauth-batch-authorization-delegation/</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, March 2026; complementary to MCP discovery but broader (not MCP-specific). Needs differentiation from OpenAPI/service-description work to gain traction.</t>
+          <t>Revision -00, 3 Jul 2026; authors: Ni Yuan, Peter Chunchi Liu (Huawei). Addresses the round-trip overhead problem in large-scale multi-agent orchestration — individual delegation exchanges per sub-agent don't scale. Complements draft-song-oauth-ai-agent-collaborate-authz (same Huawei group, coordination focus) and draft-niyikiza-oauth-attenuating-agent-tokens (attenuation semantics). The RAR-based batch approach aligns well with the OAuth WG's RAR investment.</t>
         </is>
       </c>
     </row>
@@ -2545,17 +2545,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>draft-hood-independent-agtp — Agent Transfer Protocol (AGTP)</t>
+          <t>draft-liu-oauth-a2a-profile — Agent-to-Agent (A2A) Profile for OAuth Transaction Tokens</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft proposing a dedicated application-layer protocol for AI agent traffic on port 4480 (TCP/TLS and QUIC) with an agtp:// URI scheme, arguing that HTTP is insufficient because agent-generated intent-driven traffic is indistinguishable from human-initiated requests. Defines a Runtime Contract Negotiation Substrate (RCNS) with eighteen methods split into cognitive verbs (QUERY, DISCOVER, DESCRIBE, SUMMARIZE, PLAN, PROPOSE) and mechanics verbs (EXECUTE, DELEGATE, ESCALATE, CONFIRM, SUSPEND, NOTIFY), mandatory agent identity headers, and protocol-level authority scope declaration.</t>
+          <t>Defines a profile for using OAuth Transaction Tokens in distributed agent-to-agent communication scenarios; specifies mechanisms for embedding call-chain context within tokens to preserve agent identity, authorization information, and operational flow across agent workloads in trusted environments.</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hood-independent-agtp/</t>
+          <t>https://datatracker.ietf.org/doc/draft-liu-oauth-a2a-profile/</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Revision -09, 28 Jun 2026 (was -08 May 2026); supersedes draft-hood-independent-atp. Companion specs in the same family: AGTP-API, AGTP-CERT, AGTP-MERCHANT, AGTP-IDENTIFIERS, AGTP-TRUST. Mandatory TLS 1.3+. Ambitious scope — a new transport layer rather than an HTTP profile. The cognitive/mechanics verb split is a distinctive design choice; contrasts with draft-sharif-agent-transport-protocol which layers async store-and-forward on top of existing transports rather than replacing them.</t>
+          <t>EXPIRED. Revision -00, Oct 2025; authors: Peter Chunchi Liu, Ni Yuan (Huawei) — same author pair as draft-ni-oauth-batch-authorization-delegation. Directly profiles draft-ietf-oauth-transaction-tokens for A2A use; overlaps significantly with draft-araut-oauth-transaction-tokens-for-agents. Never revised; likely deferred rather than abandoned given both authors remain active in the corpus through Jul 2026.</t>
         </is>
       </c>
     </row>
@@ -2575,17 +2575,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>draft-hood-agtp-ard — ARD Binding for AGTP: Agentic Resource Discovery over the Agent Transfer Protocol</t>
+          <t>draft-song-oauth-ai-agent-collaborate-authz — OAuth 2.0 Extension for Multi-AI Agent Collaboration</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Specifies how Agentic Resource Discovery (ARD) composes with AGTP, defining a catalog entry type for ARD manifests, aligning AGTP's identity model with ARD's trustManifest, and providing an AGTP-native binding for publishing ARD catalogs over AGTP substrate rather than HTTPS.</t>
+          <t>Extends OAuth 2.0 for coordinated multi-agent task groups: defines a collaborative authorization flow allowing a lead agent to obtain delegation tokens for sub-agents, with shared task context, coordinated scope attenuation, and cross-agent session binding.</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-ard/</t>
+          <t>https://datatracker.ietf.org/doc/draft-song-oauth-ai-agent-collaborate-authz/</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 18 Jun 2026; author: Chris Hood (Nomotic). Extends the AGTP family (draft-hood-independent-agtp in corpus). The trustManifest identity alignment is the piece relevant to the agent identity thread; the rest is transport-layer plumbing for AGTP deployments.</t>
+          <t>Revision -02, Jun/Jul 2026; authors: Yurong Song (Huawei) and colleagues. Addresses the multi-agent coordination gap at the OAuth layer — complements draft-jiang-oauth-intent-admission from the same Huawei group. Distinct from single-hop delegation drafts in explicitly modeling lead-agent-to-sub-agent scope sharing.</t>
         </is>
       </c>
     </row>
@@ -2605,17 +2605,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>draft-jernalczyk-intentweb-agent-manifest — IntentWeb AgentManifest</t>
+          <t>draft-kroehl-agentic-trust-aae — Agent Authorization Envelope (AAE)</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Defines a JSON document that websites publish to describe identity, trusted knowledge, agent-facing capabilities, structured bindings, risk levels, consent requirements, authentication expectations, audit rules, and policies — enabling AI agents to comprehend website functionality and safely perform actions without scraping or fragile UI automation.</t>
+          <t>Specifies the AAE, a structured authorization container with three mandatory components — MANDATE, CONSTRAINTS, and VALIDITY — providing a machine-evaluable, cryptographically verifiable authorization assertion using W3C DIDs and Verifiable Credentials.</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jernalczyk-intentweb-agent-manifest/</t>
+          <t>https://datatracker.ietf.org/doc/draft-kroehl-agentic-trust-aae/</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 6 Jul 2026; author: Mariusz Jernalczyk (IntentWeb). Website-side complement to agent identity drafts; sits in the Discovery &amp; Transport cluster alongside draft-hood-agtp-ard and the DAWN/.well-known discovery thread. Single author, no-affiliation submission — early stage but addresses a real discovery gap.</t>
+          <t>Revision -00, 21 May 2026; author: Lars Kersten Kroehl (CryptoKRI GmbH). Occupies similar design space to draft-mcguinness-oauth-actor-profile but uses a DID/VC substrate rather than OAuth — provides a useful alternative approach for non-OAuth deployments.</t>
         </is>
       </c>
     </row>
@@ -2635,17 +2635,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>draft-ni-a2a-ai-agent-security-requirements — Security Requirements for AI Agents</t>
+          <t>draft-pidlisnyi-aps — Agent Passport System (APS)</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft enumerating security requirements for AI agents, covering identity, authorization chaining across domains, and integration points with WIMSE, OAuth identity chaining, and the A2A OAuth profile.</t>
+          <t>Specifies Ed25519-based agent passports, scoped delegation chains with constraints across seven dimensions (a lattice model where delegation monotonically narrows capabilities), cascade revocation, a three-signature policy chain, signed receipts, and MCP bindings; includes reference implementations in TypeScript and Python.</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ni-a2a-ai-agent-security-requirements/</t>
+          <t>https://datatracker.ietf.org/doc/draft-pidlisnyi-aps/</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, February 2026; essential scaffolding for an eventual AI-agent WG. Well-connected to existing IETF work and authored by Ni and Liu, who also lead the WIMSE AI-agent identity draft.</t>
+          <t>Revision -01, 14 May 2026; author: Tymofii Pidlisnyi (AEOESS). Among the most comprehensive standalone agent authz specs in the wave — the seven-dimension constraint lattice and MCP binding make it directly implementable against Model Context Protocol deployments alongside draft-serra-mcp-discovery-uri.</t>
         </is>
       </c>
     </row>
@@ -2665,17 +2665,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>draft-rosenberg-aiproto-framework — Framework, Use Cases and Requirements for AI Agent Protocols</t>
+          <t>draft-serra-mcp-discovery-uri — The mcp URI Scheme and MCP Server Discovery Mechanism</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft providing a comprehensive AI-agent communications framework that covers user↔agent, agent↔API, and agent↔agent interactions; surveys MCP, A2A, and Agntcy; and sets the stage for IETF standards activity.</t>
+          <t>An IETF individual draft defining an 'mcp://' URI scheme combined with /.well-known/mcp-server (RFC 8615) and a DNS TXT fallback for discovery of Model Context Protocol servers.</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-framework/</t>
+          <t>https://datatracker.ietf.org/doc/draft-serra-mcp-discovery-uri/</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, October 2025; Rosenberg (Five9) and Jennings (Cisco) are credible long-time IETF contributors. Important landscape document but likely expired (April 2026); watch for a -01 refresh post-IETF 123.</t>
+          <t>Already at revision -04 (March 2026), suggesting active iteration; narrow scope, clean design, and the strongest IANA-registration candidate in the set. OAuth 2.1 for auth is deliberately out of scope.</t>
         </is>
       </c>
     </row>
@@ -2695,17 +2695,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>draft-rosenberg-aiproto-cheq — CHEQ: A Protocol for Confirmation of AI Agent Decisions (HITL)</t>
+          <t>draft-sharif-attp — ATTP: Agent Trust Transport Protocol</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an out-of-band Human-in-the-Loop confirmation protocol for agent tool calls, eliminating LLM-hallucination risk for consequential actions and enabling sensitive operations (e.g., banking) without exposing data to the agent.</t>
+          <t>An IETF individual draft defining trust levels L0–L4 mapped to PSD2 Strong Customer Authentication requirements, with bindings for MCP (MCPS), REST, A2A, gRPC, and GraphQL; supersedes draft-sharif-agent-payment-trust.</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-cheq/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-attp/</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, October 2025; out-of-band HITL confirmation model is valuable and complements delegation frameworks. Likely expired (April 2026); worth tracking for a -01 refresh.</t>
+          <t>Revision -00, April 2026; regulatory mapping appendices (PSD2, PCI DSS) are notable — one of the few drafts engaging financial regulation directly. Ambitious scope. Part of the Sharif cluster.</t>
         </is>
       </c>
     </row>
@@ -2725,27 +2725,27 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-payment-trust — Trust Scoring and Identity Verification for AI Agent Payment Transactions (SUPERSEDED)</t>
+          <t>draft-sharif-agent-transport-protocol — Agent Transport Protocol (ATP): Async Store-and-Forward for AI Agents</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft introducing an Agent Passport — a cryptographic delegation certificate intended to serve as the PSD2 'something you have' factor — and a trust-scoring model for payment transactions mapped to PCI DSS v4.0.1.</t>
+          <t>An IETF individual draft defining async store-and-forward messaging semantics with cryptographic identity per relay hop, trust scoring at ingress, capability negotiation, and interop with Google A2A, MCP, and FIPA ACL; transport-agnostic over TCP/TLS/QUIC.</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-payment-trust/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-transport-protocol/</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual, superseded)</t>
+          <t>IETF (individual)</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>SUPERSEDED by draft-sharif-attp-00 (April 2026). Retained for historical context — the Agent Passport concept is interesting but needs formal grounding; the ATTP successor generalizes it across transport bindings.</t>
+          <t>Revision -00, 28 March 2026; addresses a real gap — most agent protocols assume synchronous availability, and store-and-forward is appropriate for long-running agentic tasks. Scope is broad and needs narrowing.</t>
         </is>
       </c>
     </row>
@@ -2755,17 +2755,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>draft-stephan-ai-agent-6g — AI Agent Protocols for 6G Systems</t>
+          <t>draft-sharif-agent-audit-trail — Agent Audit Trail (AAT): Standard Logging Format for Autonomous AI Systems</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft translating use cases and service requirements from 3GPP TR 22.870 into IETF agent-protocol requirements, covering autonomous vehicles, privacy preservation, and anomaly detection.</t>
+          <t>An IETF individual draft defining a JSON-based audit record with mandatory fields (agent identity, action classification, outcome tracking, trust level) using RFC 8785 JSON Canonicalization and RFC 9562 UUIDs.</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-stephan-ai-agent-6g/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-audit-trail/</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -2775,7 +2775,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, October 2025; strong operator backing (Orange, Deutsche Telekom, Telefonica, China Mobile, Huawei). Requirements-oriented and important for 3GPP/IETF coordination. May be expired (April 2026); watch for an update.</t>
+          <t>Revision -00, 29 March 2026; orthogonal to delegation but important for compliance — standardized audit-log format is a genuine gap. Complements identity frameworks well. A sibling/alternative to the Kuehlewind audit architecture which takes a far more ambitious cross-layer approach.</t>
         </is>
       </c>
     </row>
@@ -2785,17 +2785,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>draft-jimenez-t2trg-iot-agent — Agentic AI Operation of Constrained RESTful Environments</t>
+          <t>draft-aiendpoint-ai-discovery — The AI Discovery Endpoint</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft (T2TRG affiliated) describing agentic AI (ReAct, smolagents) operating on CoAP/CoRE constrained-IoT environments, with a reference implementation provided.</t>
+          <t>An IETF individual draft defining a /.well-known/ai URI suffix for programmatic service capability discovery by AI agents — letting agents discover what an endpoint supports without having to parse human-oriented documentation; requests IANA well-known URI registration.</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jimenez-t2trg-iot-agent/</t>
+          <t>https://datatracker.ietf.org/doc/draft-aiendpoint-ai-discovery/</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 14 April 2026; unique in targeting constrained IoT environments. T2TRG affiliation and reference implementation are positive signals. Niche but fills an unaddressed gap.</t>
+          <t>Revision -00, March 2026; complementary to MCP discovery but broader (not MCP-specific). Needs differentiation from OpenAPI/service-description work to gain traction.</t>
         </is>
       </c>
     </row>
@@ -2815,17 +2815,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>draft-li-oauth-delegated-authorization — OAuth 2.0 Delegated Authorization</t>
+          <t>draft-hood-independent-agtp — Agent Transfer Protocol (AGTP)</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Huawei authors that extends OAuth 2.0 with a hierarchical 'delegation token' model so a client can mint subordinate, narrowly-scoped access tokens for delegated parties.</t>
+          <t>An IETF individual draft proposing a dedicated application-layer protocol for AI agent traffic on port 4480 (TCP/TLS and QUIC) with an agtp:// URI scheme, arguing that HTTP is insufficient because agent-generated intent-driven traffic is indistinguishable from human-initiated requests. Defines a Runtime Contract Negotiation Substrate (RCNS) with eighteen methods split into cognitive verbs (QUERY, DISCOVER, DESCRIBE, SUMMARIZE, PLAN, PROPOSE) and mechanics verbs (EXECUTE, DELEGATE, ESCALATE, CONFIRM, SUSPEND, NOTIFY), mandatory agent identity headers, and protocol-level authority scope declaration.</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-li-oauth-delegated-authorization/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-independent-agtp/</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, March 2026 (Informational); directly addresses over-privileged tokens and is one of the few drafts using the literal term 'delegated authorization'.</t>
+          <t>Revision -09, 28 Jun 2026 (was -08 May 2026); supersedes draft-hood-independent-atp. Companion specs in the same family: AGTP-API, AGTP-CERT, AGTP-MERCHANT, AGTP-IDENTIFIERS, AGTP-TRUST. Mandatory TLS 1.3+. Ambitious scope — a new transport layer rather than an HTTP profile. The cognitive/mechanics verb split is a distinctive design choice; contrasts with draft-sharif-agent-transport-protocol which layers async store-and-forward on top of existing transports rather than replacing them.</t>
         </is>
       </c>
     </row>
@@ -2845,17 +2845,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>draft-araut-oauth-transaction-tokens-for-agents — Transaction Tokens For Agents</t>
+          <t>draft-hood-agtp-ard — ARD Binding for AGTP: Agentic Resource Discovery over the Agent Transfer Protocol</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Ashay Raut (Amazon) profiling Transaction Tokens for agent-based workflows by adding 'act' for the agent identity, an 'agentic_ctx' claim carrying agent_type/intent/allowed_actions/environment_constraints, RFC 9396 RAR integration, and an 'actchain' claim for multi-agent delegation lineage.</t>
+          <t>Specifies how Agentic Resource Discovery (ARD) composes with AGTP, defining a catalog entry type for ARD manifests, aligning AGTP's identity model with ARD's trustManifest, and providing an AGTP-native binding for publishing ARD catalogs over AGTP substrate rather than HTTPS.</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-araut-oauth-transaction-tokens-for-agents/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-ard/</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -2865,7 +2865,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Revision -01 (May 2026) under the new slug — re-slugged from draft-oauth-transaction-tokens-for-agents-06; the -06 added the actchain delegation lineage, RAR-driven agentic_ctx, and a TTS check that blocks chain-splicing attacks. Conservative extension of the WG Transaction Tokens draft and an easier path to standardization.</t>
+          <t>Revision -00, 18 Jun 2026; author: Chris Hood (Nomotic). Extends the AGTP family (draft-hood-independent-agtp in corpus). The trustManifest identity alignment is the piece relevant to the agent identity thread; the rest is transport-layer plumbing for AGTP deployments.</t>
         </is>
       </c>
     </row>
@@ -2875,17 +2875,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>draft-oauth-ai-agents-on-behalf-of-user — On-Behalf-Of User Authorization for AI Agents</t>
+          <t>draft-hood-agtp-api — AGTP-API: Verbs, Paths, Endpoints, and Synthesis</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft adding requested_actor and actor_token parameters to the OAuth authorization-code flow so the user gives explicit consent per agent, with the resulting delegation chain documented in the access-token claims.</t>
+          <t>Establishes the full application-layer contract for AGTP agent–server interactions: approved method catalog, path grammar, endpoint primitives, semantic metadata blocks, server manifests, and runtime contract negotiation substrate. Defines how agents and servers negotiate capabilities and authority before action methods are invoked.</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-oauth-ai-agents-on-behalf-of-user/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-api/</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>Revision -02 was submitted August 2025; likely due for -03 refresh. Builds naturally on RFC 6749 + RFC 8693 + RFC 7636 PKCE — one of the most 'IETF-ready' delegation drafts and a strong WG-adoption candidate after the OAuth recharter.</t>
+          <t>Revision -01, May 26 2026; author: Chris Hood (Nomotic). The normative protocol contract layer for AGTP, complementing draft-hood-independent-agtp (transport) and draft-hood-agtp-trust (trust model). The AGTP family now spans 18 drafts; this is the API-layer anchor.</t>
         </is>
       </c>
     </row>
@@ -2905,17 +2905,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>draft-rosomakho-oauth-txn-challenge — OAuth Transaction Authorization Challenge</t>
+          <t>draft-hood-agtp-trust — AGTP Trust and Verification Specification</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>An OAuth mechanism enabling protected resources to demand transaction-specific authorization through challenges. When a request involves an agent or automated workflow, the RS returns a challenge to the client; the client presents it to the AS, which validates it, obtains human approval, and issues an access token with RFC 9396 authorization_details describing the approved operation. Positions as complementary to RFC 9470 (Step-Up Authentication) — that spec handles authentication freshness; this one handles authorization specificity.</t>
+          <t>Defines AGTP's three-tier trust model (Tier 1 Verified / Tier 2 Org-Asserted / Tier 3 Experimental) and a continuous behavioral trust score (0.0–1.0) used by infrastructure components for runtime trust-aware routing. Standardizes the evidence substrate, score format, freshness requirements, and consumer-side evaluation rules without mandating the scoring algorithm.</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rosomakho-oauth-txn-challenge/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-trust/</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, submitted 25 June 2026. Authors: Yaroslav Rosomakho (Zscaler), Brian Campbell (Ping Identity), Karl McGuinness (Independent), Pieter Kasselman (Defakto). Strong author lineup — Campbell is a prolific OAuth WG contributor, Kasselman co-authored Transaction Tokens and First-Party Apps, McGuinness brings the Mission-Bound OAuth context. The RS-initiated challenge model is distinct from ARAP (which operates at the PDP/PEP layer via AuthZEN) but addresses the same 'denial is not the end' problem — here at the OAuth RS/AS layer rather than the AuthZEN layer.</t>
+          <t>Revision -02, Jun 28 2026; author: Chris Hood (Nomotic). The continuous 0.0–1.0 trust score model contrasts with draft-sharif-attp's discrete L0–L4 levels and Larry Lewis's atp-core continuous scoring — three independent designs in the same design space.</t>
         </is>
       </c>
     </row>
@@ -2935,17 +2935,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>draft-lee-orprg-permit-receipts — Permit Receipts for Permit-Before-Commit Authorization</t>
+          <t>draft-hood-agtp-agent-cert — AGTP Agent Certificate Extension</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Defines requirements and an abstract data model for PermitReceipts: a verifier evaluates canonicalized effect requests, action digests, policy epochs, validity intervals, and revocation status before any protected effect is committed at an effect boundary. Covers verifier behavior, failure semantics, and candidate registries.</t>
+          <t>Specifies an X.509 v3 extension that cryptographically binds AGTP agent identity headers to TLS mutual authentication, enabling infrastructure components (Scope-Enforcement Points, load balancers, governance gateways) to verify agent identity at the network layer without application-layer access. Includes session-level revocation via AGTP NOTIFY broadcast.</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-lee-orprg-permit-receipts/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-agent-cert/</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 4 Jun 2026; author: Yong Bok Lee (Meridian Verity Group). The most complete standalone framework for pre-commit authorization in the current wave; intended to ground IETF discussion on scope and profiles. Seeks guidance on appropriate organizational placement.</t>
+          <t>Revision -03, Jun 28 2026; author: Chris Hood (Nomotic). The PKI-binding companion to the AGTP identity model; positions AGTP agent identity within existing X.509 / TLS infrastructure. Relevant to WebBotAuth comparison — both use PKI for bot/agent identity but at different layers.</t>
         </is>
       </c>
     </row>
@@ -2965,17 +2965,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>draft-nelson-agent-delegation-receipts — Delegation Receipt Protocol for AI Agent Authorization</t>
+          <t>draft-jernalczyk-intentweb-agent-manifest — IntentWeb AgentManifest</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Specifies the Delegation Receipt Protocol (DRP) where users sign Authorization Objects (containing scope boundaries, time constraints, instruction hashes, and model state commitments) that are published to an append-only log before the agent runtime gains control. Removes operators as trusted intermediaries by making the user's private key the sole signing authority.</t>
+          <t>Defines a JSON document that websites publish to describe identity, trusted knowledge, agent-facing capabilities, structured bindings, risk levels, consent requirements, authentication expectations, audit rules, and policies — enabling AI agents to comprehend website functionality and safely perform actions without scraping or fragile UI automation.</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-nelson-agent-delegation-receipts/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jernalczyk-intentweb-agent-manifest/</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>Revision -10, 13 Jun 2026; author: Ryan Nelson (Authproof). At version 10, the most iterated individual draft in the pre-action authorization space. The commitment-before-execution architecture — sign before the agent runs, not after — is distinctive and directly addresses the prompt-injection attack surface.</t>
+          <t>Revision -00, 6 Jul 2026; author: Mariusz Jernalczyk (IntentWeb). Website-side complement to agent identity drafts; sits in the Discovery &amp; Transport cluster alongside draft-hood-agtp-ard and the DAWN/.well-known discovery thread. Single author, no-affiliation submission — early stage but addresses a real discovery gap.</t>
         </is>
       </c>
     </row>
@@ -2995,17 +2995,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>draft-williams-intent-token — The Intent Token: A Cryptographic Authorization Primitive for Autonomous Agents</t>
+          <t>draft-fane-opena2a-aap — OpenA2A Agent Authorization Protocol (AAP)</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Specifies a cryptographic authorization primitive that binds an autonomous agent action to a cryptographically signed, human-declared authorization envelope before execution. Addresses the gap in OAuth 2.0 frameworks that govern access to resources but not what agents are permitted to do at the moment of action. Positioned as complementary to OAuth, not a replacement.</t>
+          <t>Establishes authorization mechanisms for AI agent systems through cryptographic identity assertions and scoped capability grants. Introduces a broker layer that separates credentials from the agent's reasoning context, specifically to prevent prompt injection attacks from leaking authorization state while enabling cross-agent delegation.</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-williams-intent-token/</t>
+          <t>https://datatracker.ietf.org/doc/draft-fane-opena2a-aap/</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 22 Jun 2026; author: Jeffrey Williams (Independent). Overlaps conceptually with draft-kroehl-agentic-trust-aae and draft-nelson-agent-delegation-receipts; worth tracking as a lighter-weight alternative to both.</t>
+          <t>Revision -00, Jul 6 2026; author: Abdel Fane (OpenA2A). Filed Jul 6 alongside a companion draft-fane-opena2a-aip which adds a fourth 'AIP' name collision to the existing Singla/Prakash/aip-agent-identity-protocol triple. The AAP authorization layer is the piece most relevant to OAuth boundary analysis.</t>
         </is>
       </c>
     </row>
@@ -3025,17 +3025,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>draft-pereira-licet-human-intent — LICET: Multi-Modal Physiological Human-Intent Verification for Autonomous AI Agent Authorization</t>
+          <t>draft-ni-a2a-ai-agent-security-requirements — Security Requirements for AI Agents</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Proposes a biometric HITL protocol fusing ECG, electrodermal activity, and Mahalanobis statistical distance to cryptographically verify genuine human intent — not just credential possession — before authorizing autonomous AI agent actions, with ZK proofs enabling third-party audit without exposing raw biometric data.</t>
+          <t>An IETF individual draft enumerating security requirements for AI agents, covering identity, authorization chaining across domains, and integration points with WIMSE, OAuth identity chaining, and the A2A OAuth profile.</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-pereira-licet-human-intent/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ni-a2a-ai-agent-security-requirements/</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 2 Jul 2026. The most novel and technically niche HITL proposal in the current wave — complements draft-rosenberg-aiproto-cheq (out-of-band HITL confirmation) and draft-sato-soos-hem (kernel-enforced escalation) by grounding human intent in physiological signal rather than credential or UI interaction.</t>
+          <t>Revision -01, February 2026; essential scaffolding for an eventual AI-agent WG. Well-connected to existing IETF work and authored by Ni and Liu, who also lead the WIMSE AI-agent identity draft.</t>
         </is>
       </c>
     </row>
@@ -3055,17 +3055,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>draft-reece-wimse-cross-org-delegation — Cross-Organizational Delegation for Workload and Agent Identity</t>
+          <t>draft-rosenberg-aiproto-framework — Framework, Use Cases and Requirements for AI Agent Protocols</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>A problem statement and requirements draft identifying that existing workload and token-based authorization mechanisms were designed for a single trust domain, describing the cross-organizational agent delegation gap, and enumerating requirements for solutions — without proposing specific technical approaches.</t>
+          <t>An IETF individual draft providing a comprehensive AI-agent communications framework that covers user↔agent, agent↔API, and agent↔agent interactions; surveys MCP, A2A, and Agntcy; and sets the stage for IETF standards activity.</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-reece-wimse-cross-org-delegation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-framework/</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -3075,7 +3075,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 25 Jun 2026; author: Morgan Reece (TowerGuardian Consulting). The problem-statement companion to the corpus's operational drafts; likely to feed into WIMSE WG scope expansion and is directly in scope for draft-kuehlewind-audit-architecture's composition graph.</t>
+          <t>Revision -00, October 2025; Rosenberg (Five9) and Jennings (Cisco) are credible long-time IETF contributors. Important landscape document but likely expired (April 2026); watch for a -01 refresh post-IETF 123.</t>
         </is>
       </c>
     </row>
@@ -3085,17 +3085,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>draft-jiang-wimse-heterogeneous-credential — Heterogeneous Credential Verification for Workload and Agentic Systems</t>
+          <t>draft-rosenberg-aiproto-cheq — CHEQ: A Protocol for Confirmation of AI Agent Decisions (HITL)</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Specifies mechanisms for representing credential sets, identifying credential types, determining appropriate verifiers, normalizing verification results across different formats (workload tokens, OAuth, X.509, attestation), and combining results into a single handling decision.</t>
+          <t>An IETF individual draft defining an out-of-band Human-in-the-Loop confirmation protocol for agent tool calls, eliminating LLM-hallucination risk for consequential actions and enabling sensitive operations (e.g., banking) without exposing data to the agent.</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jiang-wimse-heterogeneous-credential/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-cheq/</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 30 Jun 2026 (was -00 Jun 2026); authors: Yuning Jiang, Donghui Wang, Yurong Song, Faye Liu (Huawei). Solves the practical problem of agentic systems receiving credentials in multiple formats from different issuers. Fills a gap left by draft-ni-wimse-ai-agent-identity (corpus) which describes the identity problem but not multi-format credential handling.</t>
+          <t>Revision -00, October 2025; out-of-band HITL confirmation model is valuable and complements delegation frameworks. Likely expired (April 2026); worth tracking for a -01 refresh.</t>
         </is>
       </c>
     </row>
@@ -3115,27 +3115,27 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>draft-munoz-wimse-authorization-evidence — Signed Authorization-Evidence Records for WIMSE-Authorized AI Agent Actions</t>
+          <t>draft-sharif-agent-payment-trust — Trust Scoring and Identity Verification for AI Agent Payment Transactions (SUPERSEDED)</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Specifies a signed authorization-evidence record (Permit) for WIMSE-authorized AI actions, cryptographically binding to the dispatched request bytes via HTTP Message Signatures, OAuth access tokens, and Shared Signals Framework eventing — without modifying existing standards.</t>
+          <t>An IETF individual draft introducing an Agent Passport — a cryptographic delegation certificate intended to serve as the PSD2 'something you have' factor — and a trust-scoring model for payment transactions mapped to PCI DSS v4.0.1.</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-munoz-wimse-authorization-evidence/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-payment-trust/</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (individual, superseded)</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 15 May 2026; author: Christian Munoz (Keel API). Profiles WIMSE for AI agent actions and satisfies audit requirements; companion to the SCITT permit profile below. Extends the corpus WIMSE thread (draft-ni-wimse-ai-agent-identity) with a concrete evidence artifact.</t>
+          <t>SUPERSEDED by draft-sharif-attp-00 (April 2026). Retained for historical context — the Agent Passport concept is interesting but needs formal grounding; the ATTP successor generalizes it across transport bindings.</t>
         </is>
       </c>
     </row>
@@ -3145,17 +3145,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>draft-schwenkschuster-wimse-trust-domain-discovery — WIMSE Trust Domain Discovery</t>
+          <t>draft-stephan-ai-agent-6g — AI Agent Protocols for 6G Systems</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Fills a gap in the WIMSE architecture by defining how relying parties obtain cryptographic trust anchors for workload identity credentials; specifies the WIMSE Trust Bundle (a JSON document with freshness metadata) and a well-known HTTPS discovery endpoint resolving trust domain names to their trust bundles, following OpenID Connect Discovery / OAuth 2.0 patterns.</t>
+          <t>An IETF individual draft translating use cases and service requirements from 3GPP TR 22.870 into IETF agent-protocol requirements, covering autonomous vehicles, privacy preservation, and anomaly detection.</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-schwenkschuster-wimse-trust-domain-discovery/</t>
+          <t>https://datatracker.ietf.org/doc/draft-stephan-ai-agent-6g/</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 3 Jul 2026; authors: Arndt Schwenkschuster (Defakto Security), Yaroslav Rosomakho (Zscaler). Directly complements draft-schwenkschuster-wimse-credential-exchange (corpus). The kuehlewind-audit-architecture HUB assumes resolvable trust anchors — this provides the discovery mechanism. Rosomakho co-authorship ties it to draft-rosomakho-oauth-txn-challenge.</t>
+          <t>Revision -02, October 2025; strong operator backing (Orange, Deutsche Telekom, Telefonica, China Mobile, Huawei). Requirements-oriented and important for 3GPP/IETF coordination. May be expired (April 2026); watch for an update.</t>
         </is>
       </c>
     </row>
@@ -3175,17 +3175,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>draft-winmagic-wimse-condition-bounded-credentials — Condition-Bounded Credentials for Workload and Agent Identity</t>
+          <t>draft-jimenez-t2trg-iot-agent — Agentic AI Operation of Constrained RESTful Environments</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Proposes hardware-rooted, non-exfiltratable workload credentials whose validity is conditioned on attested runtime posture rather than expiration time — so a credential becomes invalid if the workload's attestation evidence degrades, regardless of the stated expiry.</t>
+          <t>An IETF individual draft (T2TRG affiliated) describing agentic AI (ReAct, smolagents) operating on CoAP/CoRE constrained-IoT environments, with a reference implementation provided.</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-winmagic-wimse-condition-bounded-credentials/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jimenez-t2trg-iot-agent/</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 6 Jul 2026; author: WinMagic. Extends the WIMSE credential model with posture-conditioned validity — distinct from time-bounded credentials in that security policy changes at the hardware/attestation layer instantly invalidate the credential. Bridges the RATS attestation thread and the WIMSE identity thread in the corpus.</t>
+          <t>Revision -00, 14 April 2026; unique in targeting constrained IoT environments. T2TRG affiliation and reference implementation are positive signals. Niche but fills an unaddressed gap.</t>
         </is>
       </c>
     </row>
@@ -3205,17 +3205,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>draft-munoz-scitt-permit-profile — A SCITT Profile for Pre-Execution AI Action Authorization Records</t>
+          <t>draft-li-oauth-delegated-authorization — OAuth 2.0 Delegated Authorization</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>SCITT profile for the Pre-Execution Authorization Record (Permit), documenting policy-evaluated decisions before AI agent action dispatch with cryptographic binding proving 'authorized request equals dispatched request.' Composes with adjacent profiles for human-authority binding, post-execution evidence, and content-refusal events via referencing mechanisms.</t>
+          <t>An IETF individual draft from Huawei authors that extends OAuth 2.0 with a hierarchical 'delegation token' model so a client can mint subordinate, narrowly-scoped access tokens for delegated parties.</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-munoz-scitt-permit-profile/</t>
+          <t>https://datatracker.ietf.org/doc/draft-li-oauth-delegated-authorization/</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 15 May 2026; author: Christian Munoz (Keel API). SCITT-anchored analog of the WIMSE evidence record; companion to draft-munoz-wimse-authorization-evidence from the same author. Connects to draft-sharif-agent-audit-trail and draft-kuehlewind-audit-architecture (both in corpus).</t>
+          <t>Revision -01, March 2026 (Informational); directly addresses over-privileged tokens and is one of the few drafts using the literal term 'delegated authorization'.</t>
         </is>
       </c>
     </row>
@@ -3235,17 +3235,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>draft-marques-asqav-compliance-receipts — Compliance Profile of Signed Action Receipts for AI Agents</t>
+          <t>draft-araut-oauth-transaction-tokens-for-agents — Transaction Tokens For Agents</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Establishes a compliance framework for signed action receipts from AI agents, mandating specific fields, cryptographic anchoring, hash-chain linkage, risk/incident classification, cross-agent envelope binding, and enforcement attestation with retention floors tied to EU AI Act, DORA, NIST AI RMF, HIPAA, SEC Rule 17a-4, and CIRCIA.</t>
+          <t>An IETF individual draft from Ashay Raut (Amazon) profiling Transaction Tokens for agent-based workflows by adding 'act' for the agent identity, an 'agentic_ctx' claim carrying agent_type/intent/allowed_actions/environment_constraints, RFC 9396 RAR integration, and an 'actchain' claim for multi-agent delegation lineage.</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-marques-asqav-compliance-receipts/</t>
+          <t>https://datatracker.ietf.org/doc/draft-araut-oauth-transaction-tokens-for-agents/</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -3255,7 +3255,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>Revision -06, 1 Jul 2026 (was -05 May 2026); author: João André Gomes Marques. The most legally grounded receipt profile in the wave — at revision 06, relatively mature. Complements draft-sharif-agent-audit-trail (corpus) with a multi-regulation compliance overlay.</t>
+          <t>Revision -01 (May 2026) under the new slug — re-slugged from draft-oauth-transaction-tokens-for-agents-06; the -06 added the actchain delegation lineage, RAR-driven agentic_ctx, and a TTS check that blocks chain-splicing attacks. Conservative extension of the WG Transaction Tokens draft and an easier path to standardization.</t>
         </is>
       </c>
     </row>
@@ -3265,17 +3265,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>draft-mih-scitt-agent-action-capsule — An Agent Action Capsule Profile for SCITT</t>
+          <t>draft-oauth-ai-agents-on-behalf-of-user — On-Behalf-Of User Authorization for AI Agents</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Defines a SCITT statement profile (Agent Action Capsule) documenting agent actions with outcome status (executed, blocked, denied, errored, timed out), evaluated constraints, committed-effect binding, and a human-in-the-loop flag; records a Capsule for every verdict including refusals. COSE Signed Statement format; registrable in SCITT Transparency Services.</t>
+          <t>An IETF individual draft adding requested_actor and actor_token parameters to the OAuth authorization-code flow so the user gives explicit consent per agent, with the resulting delegation chain documented in the access-token claims.</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mih-scitt-agent-action-capsule/</t>
+          <t>https://datatracker.ietf.org/doc/draft-oauth-ai-agents-on-behalf-of-user/</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, 6 Jul 2026 (was -01 Jun 2026); author: Steven Mih (Action State Group). -02 added an 'honest human-in-the-loop' flag distinguishing actual HITL from automated policy. Provides auditor-grade evidence that decision gates functioned; the HITL flag directly tracks the corpus theme.</t>
+          <t>Revision -02 was submitted August 2025; likely due for -03 refresh. Builds naturally on RFC 6749 + RFC 8693 + RFC 7636 PKCE — one of the most 'IETF-ready' delegation drafts and a strong WG-adoption candidate after the OAuth recharter.</t>
         </is>
       </c>
     </row>
@@ -3295,17 +3295,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>draft-car-rer-artifact — RER Run Artifact Format: Hash-Chained, Signed Records of AI Inference Execution</t>
+          <t>draft-rosomakho-oauth-txn-challenge — OAuth Transaction Authorization Challenge</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Specifies a cryptographically signed JSON record for AI inference runs including a signed envelope declaring permissions and limits, a hash-chained event log covering all model and tool calls, and a runtime signature binding envelope and log to the producing implementation. Enables offline verification by parties uninvolved in the original run.</t>
+          <t>An OAuth mechanism enabling protected resources to demand transaction-specific authorization through challenges. When a request involves an agent or automated workflow, the RS returns a challenge to the client; the client presents it to the AS, which validates it, obtains human approval, and issues an access token with RFC 9396 authorization_details describing the approved operation. Positions as complementary to RFC 9470 (Step-Up Authentication) — that spec handles authentication freshness; this one handles authorization specificity.</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-car-rer-artifact/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rosomakho-oauth-txn-challenge/</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 12 Jun 2026; author: Kayla Cardillo (Tech Enrichment). Relevant for post-hoc audit of what permissions an agent claimed during execution; companion to the SCITT profiles but more focused on inference traceability than authorization decisions.</t>
+          <t>Revision -00, submitted 25 June 2026. Authors: Yaroslav Rosomakho (Zscaler), Brian Campbell (Ping Identity), Karl McGuinness (Independent), Pieter Kasselman (Defakto). Strong author lineup — Campbell is a prolific OAuth WG contributor, Kasselman co-authored Transaction Tokens and First-Party Apps, McGuinness brings the Mission-Bound OAuth context. The RS-initiated challenge model is distinct from ARAP (which operates at the PDP/PEP layer via AuthZEN) but addresses the same 'denial is not the end' problem — here at the OAuth RS/AS layer rather than the AuthZEN layer.</t>
         </is>
       </c>
     </row>
@@ -3325,17 +3325,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>draft-noa-scitt-ai-agent-receipt — A SCITT Profile for AI-Agent Action Receipts</t>
+          <t>draft-lee-orprg-permit-receipts — Permit Receipts for Permit-Before-Commit Authorization</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Defines a minimal SCITT profile: COSE_Sign1 Signed Statements with canonicalized payloads, hash-chained for ordering, registrable in SCITT Transparency Services. Explicitly does NOT assert agent correctness, safety, or real-world outcomes — only tamper-evident, signature-verifiable records of action, principal, policy identity, and verdict.</t>
+          <t>Defines requirements and an abstract data model for PermitReceipts: a verifier evaluates canonicalized effect requests, action digests, policy epochs, validity intervals, and revocation status before any protected effect is committed at an effect boundary. Covers verifier behavior, failure semantics, and candidate registries.</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-noa-scitt-ai-agent-receipt/</t>
+          <t>https://datatracker.ietf.org/doc/draft-lee-orprg-permit-receipts/</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 23 Jun 2026; author: Tora Toraman (NordenSoft). The minimalist end of the SCITT profile spectrum; useful for corpus completeness alongside the more comprehensive draft-mih-scitt-agent-action-capsule.</t>
+          <t>Revision -00, 4 Jun 2026; author: Yong Bok Lee (Meridian Verity Group). The most complete standalone framework for pre-commit authorization in the current wave; intended to ground IETF discussion on scope and profiles. Seeks guidance on appropriate organizational placement.</t>
         </is>
       </c>
     </row>
@@ -3355,17 +3355,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>draft-rampalli-scitt-capsule-provenance-binding — Binding Per-Action Authorization and Memory Provenance into Agent Action Capsules</t>
+          <t>draft-nelson-agent-delegation-receipts — Delegation Receipt Protocol for AI Agent Authorization</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Specifies how to bind three components into AAC records: what was executed ('did'), whether it was authorized ('may'), and the source of the belief that motivated the action ('why-believed'); uses optional payload extensions carrying authorization token references, memory chain roots, and quarantine attestations without modifying AAC core protected-header claims.</t>
+          <t>Specifies the Delegation Receipt Protocol (DRP) where users sign Authorization Objects (containing scope boundaries, time constraints, instruction hashes, and model state commitments) that are published to an append-only log before the agent runtime gains control. Removes operators as trusted intermediaries by making the user's private key the sole signing authority.</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rampalli-scitt-capsule-provenance-binding/</t>
+          <t>https://datatracker.ietf.org/doc/draft-nelson-agent-delegation-receipts/</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -3375,7 +3375,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 5 Jul 2026; author: Karthik Rampalli (Glyphzero, Inc.). Extends draft-mih-scitt-agent-action-capsule with memory provenance — the 'why-believed' component is novel among SCITT profiles. Includes a defensive publication notice waiving patent claims on the core binding technique.</t>
+          <t>Revision -10, 13 Jun 2026; author: Ryan Nelson (Authproof). At version 10, the most iterated individual draft in the pre-action authorization space. The commitment-before-execution architecture — sign before the agent runs, not after — is distinctive and directly addresses the prompt-injection attack surface.</t>
         </is>
       </c>
     </row>
@@ -3385,17 +3385,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>draft-nobuo-scitt-composite-evidence-verification — Composite Evidence Verification for SCITT Statement Graphs</t>
+          <t>draft-williams-intent-token — The Intent Token: A Cryptographic Authorization Primitive for Autonomous Agents</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Defines a composite verifier function for checking collections of SCITT Signed Statements, receipts, object bindings, and relationship edges under a named verification profile; provides structured reporting on validation status, missing evidence, outdated information, and conflicting claims — targeting auditors needing to evaluate multiple interconnected statements.</t>
+          <t>Specifies a cryptographic authorization primitive that binds an autonomous agent action to a cryptographically signed, human-declared authorization envelope before execution. Addresses the gap in OAuth 2.0 frameworks that govern access to resources but not what agents are permitted to do at the moment of action. Positioned as complementary to OAuth, not a replacement.</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-nobuo-scitt-composite-evidence-verification/</t>
+          <t>https://datatracker.ietf.org/doc/draft-williams-intent-token/</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -3405,7 +3405,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 7 Jul 2026; author: Nobuo Aoki (SOKENDAI). Operates above individual SCITT profiles (AAC, permits, compliance receipts all in corpus) — the 'how do you verify all of them together' layer that draft-kuehlewind-audit-architecture implies but does not yet specify. Watch for Kühlewind/Birkholz pickup.</t>
+          <t>Revision -01, 22 Jun 2026; author: Jeffrey Williams (Independent). Overlaps conceptually with draft-kroehl-agentic-trust-aae and draft-nelson-agent-delegation-receipts; worth tracking as a lighter-weight alternative to both.</t>
         </is>
       </c>
     </row>
@@ -3415,17 +3415,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-mjwt — The Mandate JWT (MJWT) for Agentic AI Systems</t>
+          <t>draft-pereira-licet-human-intent — LICET: Multi-Modal Physiological Human-Intent Verification for Autonomous AI Agent Authorization</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Introduces the Mandate JWT — a WIMSE workload credential profile binding agent authority to specific Sovereign Object instances under named human principals, with cryptographically enforced delegation ceilings and a six-dimensional Narrowing Property preventing sub-agents from exceeding root authority.</t>
+          <t>Proposes a biometric HITL protocol fusing ECG, electrodermal activity, and Mahalanobis statistical distance to cryptographically verify genuine human intent — not just credential possession — before authorizing autonomous AI agent actions, with ZK proofs enabling third-party audit without exposing raw biometric data.</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-mjwt/</t>
+          <t>https://datatracker.ietf.org/doc/draft-pereira-licet-human-intent/</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -3435,7 +3435,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). The authorization token primitive for the SOOS governance protocol family. Directly comparable to draft-mcguinness-oauth-client-instance-assertion but uses a WIMSE/Sovereign Object substrate rather than OAuth.</t>
+          <t>Revision -01, 2 Jul 2026. The most novel and technically niche HITL proposal in the current wave — complements draft-rosenberg-aiproto-cheq (out-of-band HITL confirmation) and draft-sato-soos-hem (kernel-enforced escalation) by grounding human intent in physiological signal rather than credential or UI interaction.</t>
         </is>
       </c>
     </row>
@@ -3445,17 +3445,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-mad — Multi-Agent Delegation in Sovereign Object Systems</t>
+          <t>draft-reece-wimse-cross-org-delegation — Cross-Organizational Delegation for Workload and Agent Identity</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Specifies three core mechanisms for multi-agent delegation accountability: the Narrowing Property (capability non-amplification), five formally defined object topology patterns for runtime relationships, and cluster coordination primitives for parallel execution with aggregation rules. Version 02 adds revocation-during-execution handling and partial-completion routing to human oversight.</t>
+          <t>A problem statement and requirements draft identifying that existing workload and token-based authorization mechanisms were designed for a single trust domain, describing the cross-organizational agent delegation gap, and enumerating requirements for solutions — without proposing specific technical approaches.</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-mad/</t>
+          <t>https://datatracker.ietf.org/doc/draft-reece-wimse-cross-org-delegation/</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). Claims to address gaps the OpenID Foundation identifies as unsolved in multi-agent authorization. The five topology patterns are a useful vocabulary for describing agent-to-agent relationship structures.</t>
+          <t>Revision -00, 25 Jun 2026; author: Morgan Reece (TowerGuardian Consulting). The problem-statement companion to the corpus's operational drafts; likely to feed into WIMSE WG scope expansion and is directly in scope for draft-kuehlewind-audit-architecture's composition graph.</t>
         </is>
       </c>
     </row>
@@ -3475,17 +3475,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-hem — The Human Escalation Mechanism (HEM) for Agentic AI Systems</t>
+          <t>draft-jiang-wimse-heterogeneous-credential — Heterogeneous Credential Verification for Workload and Agentic Systems</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Defines a kernel-enforced mechanism placing agent sessions in a pending state when human judgment is required, routing structured escalation requests to designated human decision-makers, and prohibiting all state transitions until a human decision is received. Defines five decision types and a dual-layer architecture (LLM-HEM and SOOS-HEM).</t>
+          <t>Specifies mechanisms for representing credential sets, identifying credential types, determining appropriate verifiers, normalizing verification results across different formats (workload tokens, OAuth, X.509, attestation), and combining results into a single handling decision.</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-hem/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jiang-wimse-heterogeneous-credential/</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -3495,7 +3495,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>Revision -05, 30 Jun 2026 (was -04 Jun 2026); author: Tom Sato (MyAuberge K.K.). The most normative HITL protocol in the current wave; explicitly aligns with EU AI Act Article 14 requirements for high-risk AI system oversight. Counterpart to ARAP (AuthZEN WG) at the protocol level vs. the OAuth/AuthZEN layer.</t>
+          <t>Revision -01, 30 Jun 2026 (was -00 Jun 2026); authors: Yuning Jiang, Donghui Wang, Yurong Song, Faye Liu (Huawei). Solves the practical problem of agentic systems receiving credentials in multiple formats from different issuers. Fills a gap left by draft-ni-wimse-ai-agent-identity (corpus) which describes the identity problem but not multi-format credential handling.</t>
         </is>
       </c>
     </row>
@@ -3505,17 +3505,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-idp — The Intent Declaration Primitive (IDP) for Agentic AI Systems</t>
+          <t>draft-munoz-wimse-authorization-evidence — Signed Authorization-Evidence Records for WIMSE-Authorized AI Agent Actions</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Specifies a structured declaration mechanism committing AI agent intent to tamper-evident logs before actions are taken, enabling post-hoc review and EU AI Act Article 12 compliance for high-risk systems.</t>
+          <t>Specifies a signed authorization-evidence record (Permit) for WIMSE-authorized AI actions, cryptographically binding to the dispatched request bytes via HTTP Message Signatures, OAuth access tokens, and Shared Signals Framework eventing — without modifying existing standards.</t>
         </is>
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-idp/</t>
+          <t>https://datatracker.ietf.org/doc/draft-munoz-wimse-authorization-evidence/</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -3525,7 +3525,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>Revision -05, 30 Jun 2026 (was -04 Jun 2026); author: Tom Sato (MyAuberge K.K.). The log-before-execute pattern mirrors draft-nelson-agent-delegation-receipts but operates at the intent declaration level rather than the user-authorization level. Pairs with GAR (below) to form a complete pre/post audit trail.</t>
+          <t>Revision -00, 15 May 2026; author: Christian Munoz (Keel API). Profiles WIMSE for AI agent actions and satisfies audit requirements; companion to the SCITT permit profile below. Extends the corpus WIMSE thread (draft-ni-wimse-ai-agent-identity) with a concrete evidence artifact.</t>
         </is>
       </c>
     </row>
@@ -3535,17 +3535,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-gar — The Governance Audit Record (GAR) for Agentic AI Systems</t>
+          <t>draft-schwenkschuster-wimse-trust-domain-discovery — WIMSE Trust Domain Discovery</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Defines GAR, an audit framework with five audit types, a Session Audit Record, and an Audit Alert mechanism; collects, signs, and makes governance events from IDP, HEM, and associated SOOS primitives available for regulatory inspection via an append-only, non-suppressible SCITT-anchored audit stream with Authority Lifecycle Events covering the complete revocation-recovery cycle.</t>
+          <t>Fills a gap in the WIMSE architecture by defining how relying parties obtain cryptographic trust anchors for workload identity credentials; specifies the WIMSE Trust Bundle (a JSON document with freshness metadata) and a well-known HTTPS discovery endpoint resolving trust domain names to their trust bundles, following OpenID Connect Discovery / OAuth 2.0 patterns.</t>
         </is>
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-gar/</t>
+          <t>https://datatracker.ietf.org/doc/draft-schwenkschuster-wimse-trust-domain-discovery/</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>Revision -03, 28 Jun 2026 (was -02 Jun 10). -03 added OpenTelemetry attribute namespace for governance observability, a GAR Processor spec for converting OTel signals to audit records with integrity verification, four new Authority Lifecycle Event categories (policy conflict scenarios, statutory interpretation changes), and mandatory provenance fields for policy evaluation records. The integrator for the SOOS family, analogous to how draft-kuehlewind-audit-architecture integrates the broader IETF agent draft landscape.</t>
+          <t>Revision -00, 3 Jul 2026; authors: Arndt Schwenkschuster (Defakto Security), Yaroslav Rosomakho (Zscaler). Directly complements draft-schwenkschuster-wimse-credential-exchange (corpus). The kuehlewind-audit-architecture HUB assumes resolvable trust anchors — this provides the discovery mechanism. Rosomakho co-authorship ties it to draft-rosomakho-oauth-txn-challenge.</t>
         </is>
       </c>
     </row>
@@ -3565,17 +3565,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>draft-jiang-intent-security — Security Considerations and Requirements for Intent-Based Requests in Agentic Systems</t>
+          <t>draft-winmagic-wimse-condition-bounded-credentials — Condition-Bounded Credentials for Workload and Agent Identity</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Solution-agnostic threat analysis covering tampering, privilege escalation, constraint violations, and intent drift in intent-based agentic systems, with a reference model, attack scenarios, and security requirements covering authentication, admission control, constraint validation, and multi-hop integrity.</t>
+          <t>Proposes hardware-rooted, non-exfiltratable workload credentials whose validity is conditioned on attested runtime posture rather than expiration time — so a credential becomes invalid if the workload's attestation evidence degrades, regardless of the stated expiry.</t>
         </is>
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jiang-intent-security/</t>
+          <t>https://datatracker.ietf.org/doc/draft-winmagic-wimse-condition-bounded-credentials/</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -3585,7 +3585,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>Revision -03, 22 Jun 2026; authors: Yuning Jiang, Lun Li, Yurong Song, Faye Liu (Huawei). The threat-model companion to draft-jiang-oauth-intent-admission from the same group; likely intended to inform the broader IETF agentic AI security discussion.</t>
+          <t>Revision -01, 6 Jul 2026; author: WinMagic. Extends the WIMSE credential model with posture-conditioned validity — distinct from time-bounded credentials in that security policy changes at the hardware/attestation layer instantly invalidate the credential. Bridges the RATS attestation thread and the WIMSE identity thread in the corpus.</t>
         </is>
       </c>
     </row>
@@ -3595,17 +3595,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>draft-somoza-dmsc-atn-agent-trust-negotiation — Agent Trust Negotiation: Capability, Delegation, and Provenance Binding</t>
+          <t>draft-munoz-scitt-permit-profile — A SCITT Profile for Pre-Execution AI Action Authorization Records</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Specifies the Agent Trust Negotiation (ATN) protocol, which binds four artifacts — capability manifests, delegation chains, provenance attestations, and session receipts — to agent identities via a handshake state machine producing mutually verified, scope-bounded sessions with SCITT-suitable audit records.</t>
+          <t>SCITT profile for the Pre-Execution Authorization Record (Permit), documenting policy-evaluated decisions before AI agent action dispatch with cryptographic binding proving 'authorized request equals dispatched request.' Composes with adjacent profiles for human-authority binding, post-execution evidence, and content-refusal events via referencing mechanisms.</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-somoza-dmsc-atn-agent-trust-negotiation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-munoz-scitt-permit-profile/</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 29 May 2026; author: Enrique Somoza (Independent). Operates above discovery mechanisms and positions itself between the discovery layer (DAWN, MCP) and the authorization layer (WIMSE, OAuth). Relevant as an agent-to-agent trust establishment handshake protocol.</t>
+          <t>Revision -00, 15 May 2026; author: Christian Munoz (Keel API). SCITT-anchored analog of the WIMSE evidence record; companion to draft-munoz-wimse-authorization-evidence from the same author. Connects to draft-sharif-agent-audit-trail and draft-kuehlewind-audit-architecture (both in corpus).</t>
         </is>
       </c>
     </row>
@@ -3625,17 +3625,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>draft-mcgraw-httpapi-agent-budget — The Delegation HTTP Authentication Scheme for Request-Bound Authority</t>
+          <t>draft-marques-asqav-compliance-receipts — Compliance Profile of Signed Action Receipts for AI Agents</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Defines the 'Delegation' HTTP authentication scheme and response semantics for delegated-authority challenges using HTTP status codes and Problem Details, plus a CBOR/COSE proof format. The initial authority profile is 'Budget,' using post-quantum ML-DSA to prove spending or resource-consumption limits.</t>
+          <t>Establishes a compliance framework for signed action receipts from AI agents, mandating specific fields, cryptographic anchoring, hash-chain linkage, risk/incident classification, cross-agent envelope binding, and enforcement attestation with retention floors tied to EU AI Act, DORA, NIST AI RMF, HIPAA, SEC Rule 17a-4, and CIRCIA.</t>
         </is>
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcgraw-httpapi-agent-budget/</t>
+          <t>https://datatracker.ietf.org/doc/draft-marques-asqav-compliance-receipts/</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -3645,7 +3645,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, 15 Jun 2026; author: John Paul McGraw Jr. (TaskHawk Systems). HTTP-layer bounded delegation with post-quantum crypto; distinct from OAuth-layer delegation in that the authority proof travels in the Authorization header. Complements x401 (Industry tab) at the HTTP challenge-response layer.</t>
+          <t>Revision -06, 1 Jul 2026 (was -05 May 2026); author: João André Gomes Marques. The most legally grounded receipt profile in the wave — at revision 06, relatively mature. Complements draft-sharif-agent-audit-trail (corpus) with a multi-regulation compliance overlay.</t>
         </is>
       </c>
     </row>
@@ -3655,17 +3655,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>draft-vauban-x402-delegation-binding — x402 Delegation Binding for Agentic HTTP Pipelines</t>
+          <t>draft-mih-scitt-agent-action-capsule — An Agent Action Capsule Profile for SCITT</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>Addresses the security gap where x402 V2 payment grants issued to one agent could be misused by another in the same pipeline, introducing three binding mechanisms: a JCS-derived agent identity pseudonym, a nonce for anti-replay, and a depth-limiting field for transitive delegation.</t>
+          <t>Defines a SCITT statement profile (Agent Action Capsule) documenting agent actions with outcome status (executed, blocked, denied, errored, timed out), evaluated constraints, committed-effect binding, and a human-in-the-loop flag; records a Capsule for every verdict including refusals. COSE Signed Statement format; registrable in SCITT Transparency Services.</t>
         </is>
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-vauban-x402-delegation-binding/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mih-scitt-agent-action-capsule/</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 25 May 2026; author: Vauban Research. Narrowly scoped to payment pipelines but the delegation-binding pattern (pseudonymous identity + anti-replay + depth-limit) is applicable broadly. Validated across five language runtimes with A2A and MCP integration guidance.</t>
+          <t>Revision -02, 6 Jul 2026 (was -01 Jun 2026); author: Steven Mih (Action State Group). -02 added an 'honest human-in-the-loop' flag distinguishing actual HITL from automated policy. Provides auditor-grade evidence that decision gates functioned; the HITL flag directly tracks the corpus theme.</t>
         </is>
       </c>
     </row>
@@ -3685,17 +3685,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>draft-samal-vap — Verifiable Agent Protocol (VAP): Intent-Bound Admission Control and Audit for Agent Tool Invocation</t>
+          <t>draft-car-rer-artifact — RER Run Artifact Format: Hash-Chained, Signed Records of AI Inference Execution</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Specifies VAP as a defense-in-depth layer adding declarations of purpose and session budget commitments to tool invocation requests (targeting MCP-style protocols), enabling servers to perform admission control before execution via four messages carried in existing protocol metadata.</t>
+          <t>Specifies a cryptographically signed JSON record for AI inference runs including a signed envelope declaring permissions and limits, a hash-chained event log covering all model and tool calls, and a runtime signature binding envelope and log to the producing implementation. Enables offline verification by parties uninvolved in the original run.</t>
         </is>
       </c>
       <c r="D93" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-samal-vap/</t>
+          <t>https://datatracker.ietf.org/doc/draft-car-rer-artifact/</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -3705,7 +3705,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 3 Jun 2026; author: Kruttidipta Samal (Independent). Lightweight and protocol-agnostic; addresses erroneous agent behavior, cost control, and audit trails without replacing existing auth mechanisms. Practical tool-invocation-level authorization layer for MCP deployments.</t>
+          <t>Revision -01, 12 Jun 2026; author: Kayla Cardillo (Tech Enrichment). Relevant for post-hoc audit of what permissions an agent claimed during execution; companion to the SCITT profiles but more focused on inference traceability than authorization decisions.</t>
         </is>
       </c>
     </row>
@@ -3715,17 +3715,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>draft-khera-aurora — Agent Unification, Runtime, and Operational Responsibility Attestation (AURORA)</t>
+          <t>draft-noa-scitt-ai-agent-receipt — A SCITT Profile for AI-Agent Action Receipts</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>A two-layer framework unifying hardware-enclave-backed Runtime Integrity Attestation with scoped, cryptographically bound Authority Delegation; enables agents to prove both operational authority and runtime integrity simultaneously.</t>
+          <t>Defines a minimal SCITT profile: COSE_Sign1 Signed Statements with canonicalized payloads, hash-chained for ordering, registrable in SCITT Transparency Services. Explicitly does NOT assert agent correctness, safety, or real-world outcomes — only tamper-evident, signature-verifiable records of action, principal, policy identity, and verdict.</t>
         </is>
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-khera-aurora/</t>
+          <t>https://datatracker.ietf.org/doc/draft-noa-scitt-ai-agent-receipt/</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 5 Jun 2026; author: Ankur Khera. Addresses the gap where delegation tokens don't prove the runtime environment is trustworthy — relevant where delegation must be paired with platform attestation (enterprise/regulated deployments). Bridges the RATS attestation thread and the OAuth delegation thread.</t>
+          <t>Revision -00, 23 Jun 2026; author: Tora Toraman (NordenSoft). The minimalist end of the SCITT profile spectrum; useful for corpus completeness alongside the more comprehensive draft-mih-scitt-agent-action-capsule.</t>
         </is>
       </c>
     </row>
@@ -3745,17 +3745,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>draft-borthwick-msebenzi-environment-state — Verifiable Intent — environment.* Constraint Family</t>
+          <t>draft-rampalli-scitt-capsule-provenance-binding — Binding Per-Action Authorization and Memory Provenance into Agent Action Capsules</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Defines the environment.* constraint family for agent-authorization mandate vocabularies, covering external conditions at transaction execution time (venue availability, wallet funding) that existing transactional constraints cannot address. Extends agent authorization mandate frameworks with environmental precondition checking.</t>
+          <t>Specifies how to bind three components into AAC records: what was executed ('did'), whether it was authorized ('may'), and the source of the belief that motivated the action ('why-believed'); uses optional payload extensions carrying authorization token references, memory chain roots, and quarantine attestations without modifying AAC core protected-header claims.</t>
         </is>
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-borthwick-msebenzi-environment-state/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rampalli-scitt-capsule-provenance-binding/</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -3765,7 +3765,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 13 Jun 2026; authors: Douglas Cameron Borthwick (InsumerAPI), Michael Msebenzi (Headless Oracle). Narrow but practically important for financial and commerce agent workflows; connects to draft-mcgraw-httpapi-agent-budget and draft-vauban-x402-delegation-binding.</t>
+          <t>Revision -00, 5 Jul 2026; author: Karthik Rampalli (Glyphzero, Inc.). Extends draft-mih-scitt-agent-action-capsule with memory provenance — the 'why-believed' component is novel among SCITT profiles. Includes a defensive publication notice waiving patent claims on the core binding technique.</t>
         </is>
       </c>
     </row>
@@ -3775,17 +3775,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>draft-chen-oauth-agent-authz-use-cases — Agent Authorization Use Cases and Gap Analysis for OAuth 2.0</t>
+          <t>draft-nobuo-scitt-composite-evidence-verification — Composite Evidence Verification for SCITT Statement Graphs</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>A framework-level analysis enumerating agentic authorization use cases — delegated task execution, multi-agent coordination, long-running workflows, capability attenuation — and mapping each against current OAuth 2.0 mechanisms to identify gaps that require new extensions or profiles.</t>
+          <t>Defines a composite verifier function for checking collections of SCITT Signed Statements, receipts, object bindings, and relationship edges under a named verification profile; provides structured reporting on validation status, missing evidence, outdated information, and conflicting claims — targeting auditors needing to evaluate multiple interconnected statements.</t>
         </is>
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-chen-oauth-agent-authz-use-cases/</t>
+          <t>https://datatracker.ietf.org/doc/draft-nobuo-scitt-composite-evidence-verification/</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 5 Jul 2026; useful problem-statement companion to the OAuth recharter's 'Complex Delegation' milestone. Gap analysis directly motivates several other drafts in this corpus — a natural reference document for the OAuth WG scoping discussion.</t>
+          <t>Revision -00, 7 Jul 2026; author: Nobuo Aoki (SOKENDAI). Operates above individual SCITT profiles (AAC, permits, compliance receipts all in corpus) — the 'how do you verify all of them together' layer that draft-kuehlewind-audit-architecture implies but does not yet specify. Watch for Kühlewind/Birkholz pickup.</t>
         </is>
       </c>
     </row>
@@ -3805,17 +3805,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>draft-agnihotri-oauth-agent-impl-status — Implementation Status of OAuth Identity Chaining and Transaction Tokens</t>
+          <t>draft-sato-soos-mjwt — The Mandate JWT (MJWT) for Agentic AI Systems</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>An RFC 7942–compliant implementation status report tracking open-source implementations of draft-ietf-oauth-identity-chaining and draft-ietf-oauth-transaction-tokens against the relevant spec requirements.</t>
+          <t>Introduces the Mandate JWT — a WIMSE workload credential profile binding agent authority to specific Sovereign Object instances under named human principals, with cryptographically enforced delegation ceilings and a six-dimensional Narrowing Property preventing sub-agents from exceeding root authority.</t>
         </is>
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-agnihotri-oauth-agent-impl-status/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-mjwt/</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, Jun 2026; provides the implementation evidence required to advance both WG drafts toward IESG submission. Informational companion to the two WG drafts — not a protocol spec but tracking their standardization progress.</t>
+          <t>Revision -01, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). The authorization token primitive for the SOOS governance protocol family. Directly comparable to draft-mcguinness-oauth-client-instance-assertion but uses a WIMSE/Sovereign Object substrate rather than OAuth.</t>
         </is>
       </c>
     </row>
@@ -3835,17 +3835,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>draft-hardt-oauth-aauth-protocol — AAuth Protocol</t>
+          <t>draft-sato-soos-mad — Multi-Agent Delegation in Sovereign Object Systems</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>A new clean-sheet authorization protocol from Dick Hardt (original OAuth author) defining proof-of-possession by default, resource-signed challenges, agent identity without pre-registration, deferred 202 responses, and AS-to-AS federation for the agent ecosystem.</t>
+          <t>Specifies three core mechanisms for multi-agent delegation accountability: the Narrowing Property (capability non-amplification), five formally defined object topology patterns for runtime relationships, and cluster coordination primitives for parallel execution with aggregation rules. Version 02 adds revocation-during-execution handling and partial-completion routing to human oversight.</t>
         </is>
       </c>
       <c r="D98" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hardt-oauth-aauth-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-mad/</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>Revision -09, Jul 4 2026; slug gained 'oauth' infix at this revision (was draft-hardt-aauth-protocol). Now formally adds four resource access modes including agent governance. The design rationale section explicitly explains why AAuth is not GNAP, not OAuth, not DPoP and not mTLS — important read for anyone planning a new agent-auth stack. OUTLIER: zero OAuth dependencies.</t>
+          <t>Revision -02, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). Claims to address gaps the OpenID Foundation identifies as unsolved in multi-agent authorization. The five topology patterns are a useful vocabulary for describing agent-to-agent relationship structures.</t>
         </is>
       </c>
     </row>
@@ -3865,17 +3865,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>draft-chen-oauth-roadmap — Comprehensive Roadmap for OAuth 2.0 Standards and Drafts</t>
+          <t>draft-sato-soos-hem — The Human Escalation Mechanism (HEM) for Agentic AI Systems</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>An IETF informational draft that maps the entire OAuth 2.0 ecosystem of RFCs, BCPs, and active drafts into functional layers from core to extensions to industry profiles.</t>
+          <t>Defines a kernel-enforced mechanism placing agent sessions in a pending state when human judgment is required, routing structured escalation requests to designated human decision-makers, and prohibiting all state transitions until a human decision is received. Defines five decision types and a dual-layer architecture (LLM-HEM and SOOS-HEM).</t>
         </is>
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>https://www.ietf.org/archive/id/draft-chen-oauth-roadmap-00.html</t>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-hem/</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>Brand-new -00 draft (May 2026); the single most useful index when starting work in this area.</t>
+          <t>Revision -05, 30 Jun 2026 (was -04 Jun 2026); author: Tom Sato (MyAuberge K.K.). The most normative HITL protocol in the current wave; explicitly aligns with EU AI Act Article 14 requirements for high-risk AI system oversight. Counterpart to ARAP (AuthZEN WG) at the protocol level vs. the OAuth/AuthZEN layer.</t>
         </is>
       </c>
     </row>
@@ -3895,25 +3895,565 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
+          <t>draft-sato-soos-idp — The Intent Declaration Primitive (IDP) for Agentic AI Systems</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Specifies a structured declaration mechanism committing AI agent intent to tamper-evident logs before actions are taken, enabling post-hoc review and EU AI Act Article 12 compliance for high-risk systems.</t>
+        </is>
+      </c>
+      <c r="D100" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-idp/</t>
+        </is>
+      </c>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>Revision -05, 30 Jun 2026 (was -04 Jun 2026); author: Tom Sato (MyAuberge K.K.). The log-before-execute pattern mirrors draft-nelson-agent-delegation-receipts but operates at the intent declaration level rather than the user-authorization level. Pairs with GAR (below) to form a complete pre/post audit trail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>draft-sato-soos-gar — The Governance Audit Record (GAR) for Agentic AI Systems</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Defines GAR, an audit framework with five audit types, a Session Audit Record, and an Audit Alert mechanism; collects, signs, and makes governance events from IDP, HEM, and associated SOOS primitives available for regulatory inspection via an append-only, non-suppressible SCITT-anchored audit stream with Authority Lifecycle Events covering the complete revocation-recovery cycle.</t>
+        </is>
+      </c>
+      <c r="D101" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-gar/</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>Revision -03, 28 Jun 2026 (was -02 Jun 10). -03 added OpenTelemetry attribute namespace for governance observability, a GAR Processor spec for converting OTel signals to audit records with integrity verification, four new Authority Lifecycle Event categories (policy conflict scenarios, statutory interpretation changes), and mandatory provenance fields for policy evaluation records. The integrator for the SOOS family, analogous to how draft-kuehlewind-audit-architecture integrates the broader IETF agent draft landscape.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>draft-jiang-intent-security — Security Considerations and Requirements for Intent-Based Requests in Agentic Systems</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>Solution-agnostic threat analysis covering tampering, privilege escalation, constraint violations, and intent drift in intent-based agentic systems, with a reference model, attack scenarios, and security requirements covering authentication, admission control, constraint validation, and multi-hop integrity.</t>
+        </is>
+      </c>
+      <c r="D102" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-jiang-intent-security/</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>Revision -03, 22 Jun 2026; authors: Yuning Jiang, Lun Li, Yurong Song, Faye Liu (Huawei). The threat-model companion to draft-jiang-oauth-intent-admission from the same group; likely intended to inform the broader IETF agentic AI security discussion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>draft-li-dmsc-macp — Multi-agent Collaboration Protocol Suites Architecture</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>Defines a protocol suite and architectural framework for secure, scalable multi-agent collaboration covering trusted agent onboarding, capability-based discovery, distributed capability synchronization, and secure agent-to-agent interaction. Specifies a gateway-centric architecture where an Agent Gateway mediates capability negotiation and trust establishment between collaborating agents.</t>
+        </is>
+      </c>
+      <c r="D103" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-li-dmsc-macp/</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>Revision -05, 26 May 2026; active (expires Nov 2026); authors: Xueting Li (China Telecom), Bing Liu (Huawei), Jun Liu (Beijing U of Posts &amp; Telecom), Chenguang Du (Tsinghua), Lianhua Zhang (AsiaInfo). Replaces draft-li-dmsc-mcps-agw. Anchors a DMSC family of companion drafts covering intent-based interconnection, task protocol, gateway directory sync, semantic interaction, and gateway requirements. No explicit OAuth or WIMSE dependencies — operates at the agent coordination layer above transport, below authorization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="5" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>draft-li-dmsc-inf-architecture — Dynamic Multi-agent Secured Collaboration Infrastructure Architecture</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>Approaches DMSC from the network-infrastructure perspective: proposes capability-based forwarding and semantic routing at the network layer, where agent capability metadata influences packet-forwarding decisions rather than routing based solely on addresses. The most mature DMSC document at rev 07; predates and informs the MACP architecture draft.</t>
+        </is>
+      </c>
+      <c r="D104" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-li-dmsc-inf-architecture/</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F104" s="5" t="inlineStr">
+        <is>
+          <t>Revision -07, May 22 2026; authors: Xueting Li (China Telecom), Aijun Wang (China Telecom), Bing Liu (Huawei), Changwang Lin (New H3C). Infrastructure-layer complement to draft-li-dmsc-macp (protocol suite). The DMSC family now has 14+ companion drafts from Chinese telecom/academic groups — this is the architectural anchor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>draft-sz-dmsc-iaip — Intent-based Agent Interconnection Protocol at Agent Gateway</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Defines semantic capability advertisement and intent-driven routing at DMSC agent gateways: agents publish capability profiles in a structured format and the gateway matches incoming task intents to available agents, replacing fixed-address routing with dynamic semantic matching. The core routing-layer protocol for DMSC inter-agent communication.</t>
+        </is>
+      </c>
+      <c r="D105" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-sz-dmsc-iaip/</t>
+        </is>
+      </c>
+      <c r="E105" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F105" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, May 2026; authors: Sheng Sun, Xinyi Zhang (CAS/CNIC), Qiangzhou Gao (Huawei), Min Liu, Yuwei Wang (ICT, CAS). The intent-based routing mechanism that distinguishes DMSC from address-based protocols; relevant to the DAWN boundary question — DMSC embeds discovery in the gateway routing layer rather than treating it as a separate protocol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>draft-yang-dmsc-ioa-task-protocol — Internet of Agents Task Protocol for Heterogeneous Agent Collaboration</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>Establishes a session and task coordination layer with finite-state-machine-based dialogue management, dynamic team assembly, and nested team hierarchies for distributed heterogeneous agent collaboration. Addresses the multi-agent task lifecycle from assignment through completion and audit across heterogeneous agent implementations.</t>
+        </is>
+      </c>
+      <c r="D106" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-yang-dmsc-ioa-task-protocol/</t>
+        </is>
+      </c>
+      <c r="E106" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>Revision -03, Apr 21 2026; authors: Cheng Yang (BUPT), Zhiyuan Liu (Tsinghua), Aijun Wang (China Telecom). The task-coordination layer above the DMSC gateway routing; covers multi-domain and 6G/ITS scenarios. Distinct from OAuth-layer delegation in that it orchestrates task state rather than token issuance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>draft-dunbar-dmsc-gw-scenarios-gap-analysis — Deployment Scenarios and Gap Analysis for AI Agent Gateway</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Surveys single-domain to multi-domain deployment scenarios for AI Agent Gateways and identifies concrete gaps where existing protocols (specifically MCP and Google's A2A) cannot satisfy governance, policy enforcement, and cross-organizational trust requirements — particularly in regulated financial services and telecom environments.</t>
+        </is>
+      </c>
+      <c r="D107" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-dunbar-dmsc-gw-scenarios-gap-analysis/</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F107" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, Jul 2 2026; authors: Linda Dunbar (Futurewei), YiFei Wang (China Telecom), Bing Liu (Huawei). The most directly useful DMSC document for the boundary analysis: explicitly names MCP and A2A as insufficient and articulates where the DMSC gateway fills the gap. The regulated-environment focus (financial services, telco) distinguishes DMSC's use-case target from OAuth-centric approaches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="5" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>draft-somoza-dmsc-atn-agent-trust-negotiation — Agent Trust Negotiation: Capability, Delegation, and Provenance Binding</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>Specifies the Agent Trust Negotiation (ATN) protocol, which binds four artifacts — capability manifests, delegation chains, provenance attestations, and session receipts — to agent identities via a handshake state machine producing mutually verified, scope-bounded sessions with SCITT-suitable audit records.</t>
+        </is>
+      </c>
+      <c r="D108" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-somoza-dmsc-atn-agent-trust-negotiation/</t>
+        </is>
+      </c>
+      <c r="E108" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F108" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 29 May 2026; author: Enrique Somoza (Independent). Operates above discovery mechanisms and positions itself between the discovery layer (DAWN, MCP) and the authorization layer (WIMSE, OAuth). Relevant as an agent-to-agent trust establishment handshake protocol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>draft-mcgraw-httpapi-agent-budget — The Delegation HTTP Authentication Scheme for Request-Bound Authority</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>Defines the 'Delegation' HTTP authentication scheme and response semantics for delegated-authority challenges using HTTP status codes and Problem Details, plus a CBOR/COSE proof format. The initial authority profile is 'Budget,' using post-quantum ML-DSA to prove spending or resource-consumption limits.</t>
+        </is>
+      </c>
+      <c r="D109" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-mcgraw-httpapi-agent-budget/</t>
+        </is>
+      </c>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F109" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, 15 Jun 2026; author: John Paul McGraw Jr. (TaskHawk Systems). HTTP-layer bounded delegation with post-quantum crypto; distinct from OAuth-layer delegation in that the authority proof travels in the Authorization header. Complements x401 (Industry tab) at the HTTP challenge-response layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="5" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>draft-vauban-x402-delegation-binding — x402 Delegation Binding for Agentic HTTP Pipelines</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>Addresses the security gap where x402 V2 payment grants issued to one agent could be misused by another in the same pipeline, introducing three binding mechanisms: a JCS-derived agent identity pseudonym, a nonce for anti-replay, and a depth-limiting field for transitive delegation.</t>
+        </is>
+      </c>
+      <c r="D110" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-vauban-x402-delegation-binding/</t>
+        </is>
+      </c>
+      <c r="E110" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F110" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 25 May 2026; author: Vauban Research. Narrowly scoped to payment pipelines but the delegation-binding pattern (pseudonymous identity + anti-replay + depth-limit) is applicable broadly. Validated across five language runtimes with A2A and MCP integration guidance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>draft-samal-vap — Verifiable Agent Protocol (VAP): Intent-Bound Admission Control and Audit for Agent Tool Invocation</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>Specifies VAP as a defense-in-depth layer adding declarations of purpose and session budget commitments to tool invocation requests (targeting MCP-style protocols), enabling servers to perform admission control before execution via four messages carried in existing protocol metadata.</t>
+        </is>
+      </c>
+      <c r="D111" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-samal-vap/</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F111" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 3 Jun 2026; author: Kruttidipta Samal (Independent). Lightweight and protocol-agnostic; addresses erroneous agent behavior, cost control, and audit trails without replacing existing auth mechanisms. Practical tool-invocation-level authorization layer for MCP deployments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>draft-khera-aurora — Agent Unification, Runtime, and Operational Responsibility Attestation (AURORA)</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>A two-layer framework unifying hardware-enclave-backed Runtime Integrity Attestation with scoped, cryptographically bound Authority Delegation; enables agents to prove both operational authority and runtime integrity simultaneously.</t>
+        </is>
+      </c>
+      <c r="D112" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-khera-aurora/</t>
+        </is>
+      </c>
+      <c r="E112" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F112" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 5 Jun 2026; author: Ankur Khera. Addresses the gap where delegation tokens don't prove the runtime environment is trustworthy — relevant where delegation must be paired with platform attestation (enterprise/regulated deployments). Bridges the RATS attestation thread and the OAuth delegation thread.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>draft-borthwick-msebenzi-environment-state — Verifiable Intent — environment.* Constraint Family</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>Defines the environment.* constraint family for agent-authorization mandate vocabularies, covering external conditions at transaction execution time (venue availability, wallet funding) that existing transactional constraints cannot address. Extends agent authorization mandate frameworks with environmental precondition checking.</t>
+        </is>
+      </c>
+      <c r="D113" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-borthwick-msebenzi-environment-state/</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 13 Jun 2026; authors: Douglas Cameron Borthwick (InsumerAPI), Michael Msebenzi (Headless Oracle). Narrow but practically important for financial and commerce agent workflows; connects to draft-mcgraw-httpapi-agent-budget and draft-vauban-x402-delegation-binding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>draft-chen-oauth-agent-authz-use-cases — Agent Authorization Use Cases and Gap Analysis for OAuth 2.0</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>A framework-level analysis enumerating agentic authorization use cases — delegated task execution, multi-agent coordination, long-running workflows, capability attenuation — and mapping each against current OAuth 2.0 mechanisms to identify gaps that require new extensions or profiles.</t>
+        </is>
+      </c>
+      <c r="D114" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-chen-oauth-agent-authz-use-cases/</t>
+        </is>
+      </c>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 5 Jul 2026; useful problem-statement companion to the OAuth recharter's 'Complex Delegation' milestone. Gap analysis directly motivates several other drafts in this corpus — a natural reference document for the OAuth WG scoping discussion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>draft-agnihotri-oauth-agent-impl-status — Implementation Status of OAuth Identity Chaining and Transaction Tokens</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>An RFC 7942–compliant implementation status report tracking open-source implementations of draft-ietf-oauth-identity-chaining and draft-ietf-oauth-transaction-tokens against the relevant spec requirements.</t>
+        </is>
+      </c>
+      <c r="D115" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-agnihotri-oauth-agent-impl-status/</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, Jun 2026; provides the implementation evidence required to advance both WG drafts toward IESG submission. Informational companion to the two WG drafts — not a protocol spec but tracking their standardization progress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="5" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="5" t="inlineStr">
+        <is>
+          <t>draft-hardt-oauth-aauth-protocol — AAuth Protocol</t>
+        </is>
+      </c>
+      <c r="C116" s="5" t="inlineStr">
+        <is>
+          <t>A new clean-sheet authorization protocol from Dick Hardt (original OAuth author) defining proof-of-possession by default, resource-signed challenges, agent identity without pre-registration, deferred 202 responses, and AS-to-AS federation for the agent ecosystem.</t>
+        </is>
+      </c>
+      <c r="D116" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-hardt-oauth-aauth-protocol/</t>
+        </is>
+      </c>
+      <c r="E116" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F116" s="5" t="inlineStr">
+        <is>
+          <t>Revision -09, Jul 4 2026; slug gained 'oauth' infix at this revision (was draft-hardt-aauth-protocol). Now formally adds four resource access modes including agent governance. The design rationale section explicitly explains why AAuth is not GNAP, not OAuth, not DPoP and not mTLS — important read for anyone planning a new agent-auth stack. OUTLIER: zero OAuth dependencies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>draft-chen-oauth-roadmap — Comprehensive Roadmap for OAuth 2.0 Standards and Drafts</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>An IETF informational draft that maps the entire OAuth 2.0 ecosystem of RFCs, BCPs, and active drafts into functional layers from core to extensions to industry profiles.</t>
+        </is>
+      </c>
+      <c r="D117" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ietf.org/archive/id/draft-chen-oauth-roadmap-00.html</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F117" s="5" t="inlineStr">
+        <is>
+          <t>Brand-new -00 draft (May 2026); the single most useful index when starting work in this area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
           <t>Charter: WIMSE — Workload Identity in Multi-System Environments (charter-ietf-wimse-01)</t>
         </is>
       </c>
-      <c r="C100" s="5" t="inlineStr">
+      <c r="C118" s="5" t="inlineStr">
         <is>
           <t>The formal IETF charter for the WIMSE WG covering architecture, JOSE-based WIMSE tokens for service-to-service traffic, local token issuance, and token exchange profiles (likely based on RFC 8693) for cross-trust-domain workload identity.</t>
         </is>
       </c>
-      <c r="D100" s="9" t="inlineStr">
+      <c r="D118" s="9" t="inlineStr">
         <is>
           <t>https://datatracker.ietf.org/doc/charter-ietf-wimse/01/</t>
         </is>
       </c>
-      <c r="E100" s="5" t="inlineStr">
+      <c r="E118" s="5" t="inlineStr">
         <is>
           <t>IETF (WIMSE WG charter)</t>
         </is>
       </c>
-      <c r="F100" s="5" t="inlineStr">
+      <c r="F118" s="5" t="inlineStr">
         <is>
           <t>Approved 18 March 2026 (v01); explicitly liaises with OAuth, SCIM, SCITT, RATS, the OpenID Foundation, and CNCF/SPIFFE — the formal scope statement that anchors all WIMSE draft work.</t>
         </is>
@@ -4020,6 +4560,24 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId117"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Incorporated findings from Heather Flanagan
</commit_message>
<xml_diff>
--- a/delegated_authorization_research.xlsx
+++ b/delegated_authorization_research.xlsx
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="6" t="n">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="D11" s="7" t="n"/>
     </row>
@@ -906,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F118"/>
+  <dimension ref="A1:F132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1645,27 +1645,27 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-actor-profile — OAuth Actor Profile for Delegation</t>
+          <t>draft-ietf-oauth-client-id-metadata-document — OAuth Client ID Metadata Document</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Karl McGuinness's individual draft profiling the RFC 8693 'act' claim with required iss, optional sub_profile entity classification, and uniform processing across JWT assertion grants, JWT access tokens, and Transaction Tokens.</t>
+          <t>Defines a mechanism for OAuth clients to identify themselves to authorization servers via a URL as the client_id, pointing to a published JSON document containing client metadata — enabling dynamic client identification without prior registration.</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/html/draft-mcguinness-oauth-actor-profile-00</t>
+          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-client-id-metadata-document/</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (OAuth WG)</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Revision -00 published 30 April 2026; defines depth-1+ chain validation, cycle-aware construction, and bearer-to-PoP upgrade — the most complete actor-representation profile to date.</t>
+          <t>Revision -02, Jul 2026; OAuth WG-adopted. Directly relevant to AI agent deployments where agents may be registered via discoverable metadata documents rather than static registrations. Complements draft-king-dawn-requirements (discovery layer) by providing the OAuth-layer registration artifact.</t>
         </is>
       </c>
     </row>
@@ -1675,27 +1675,27 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>draft-mw-oauth-actor-chain — Cryptographically Verifiable Actor Chains for OAuth 2.0 Token Exchange</t>
+          <t>draft-ietf-oauth-refresh-token-expiration — OAuth 2.0 Refresh Token and Authorization Expiration</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft (Prasad/Krishnan/Lopez/Addepalli) defining six actor-chain profiles for RFC 8693 — Declared/Verified × Full/Subset/Actor-Only Disclosure — that preserve and cryptographically validate delegation-path continuity across successive token exchanges instead of relying on RFC 8693's informational-only nested act claims.</t>
+          <t>Extends OAuth 2.0 with new token endpoint response parameters specifying refresh token expiration and user authorization expiration, making expiry semantics explicit and interoperable across implementations.</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mw-oauth-actor-chain/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ietf-oauth-refresh-token-expiration/</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (OAuth WG)</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 30 Jun 2026 (was -00 May 2026; re-slugged from draft-mw-spice-actor-chain-05); a complementary alternative to the McGuinness Actor Profile that directly addresses RFC 8693's chain-splicing weakness by making the chain itself cryptographically verifiable rather than just informational.</t>
+          <t>Revision -03, Jul 2026; OAuth WG-adopted. Relevant to long-running agent sessions: explicit authorization expiration addresses the gap where refresh tokens survive past the user's intended authorization window — a known risk in agentic delegation scenarios.</t>
         </is>
       </c>
     </row>
@@ -1705,17 +1705,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-client-instance-assertion — OAuth Client Instance Assertion</t>
+          <t>draft-mcguinness-oauth-actor-profile — OAuth Actor Profile for Delegation</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Karl McGuinness's individual draft for representing a specific running instance of an OAuth client (rather than just the client registration) so authorization servers can bind grants to a concrete instance.</t>
+          <t>Karl McGuinness's individual draft profiling the RFC 8693 'act' claim with required iss, optional sub_profile entity classification, and uniform processing across JWT assertion grants, JWT access tokens, and Transaction Tokens.</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-client-instance-assertion/</t>
+          <t>https://datatracker.ietf.org/doc/html/draft-mcguinness-oauth-actor-profile-00</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Note: full draft text was not retrievable through automated fetch at time of writing — recommend reading directly. Companion to the Actor Profile draft and to attestation-based client auth.</t>
+          <t>Revision -00 published 30 April 2026; defines depth-1+ chain validation, cycle-aware construction, and bearer-to-PoP upgrade — the most complete actor-representation profile to date.</t>
         </is>
       </c>
     </row>
@@ -1735,17 +1735,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-resource-token-resp — OAuth 2.0 Resource Parameter in Access Token Response</t>
+          <t>draft-mw-oauth-actor-chain — Cryptographically Verifiable Actor Chains for OAuth 2.0 Token Exchange</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>A McGuinness/Skokan individual draft adding a 'resource' parameter to the OAuth access token response so clients can confirm which resource the issued token is valid for, mitigating resource mix-up attacks especially in deployments that use RFC 8707 Resource Indicators.</t>
+          <t>An IETF individual draft (Prasad/Krishnan/Lopez/Addepalli) defining six actor-chain profiles for RFC 8693 — Declared/Verified × Full/Subset/Actor-Only Disclosure — that preserve and cryptographically validate delegation-path continuity across successive token exchanges instead of relying on RFC 8693's informational-only nested act claims.</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-resource-token-resp/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mw-oauth-actor-chain/</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Revision -03 (March 2026). Filip Skokan added as co-author in -03. Complements RFC 8707 / RFC 9700 / RFC 9207 by adding issuance-time confirmation to the discovery-time mechanisms. Notable for the agent-authz corpus because dynamic resource discovery is a core agent pattern and resource-mix-up attacks are amplified when agents juggle many short-lived tokens.</t>
+          <t>Revision -01, 30 Jun 2026 (was -00 May 2026; re-slugged from draft-mw-spice-actor-chain-05); a complementary alternative to the McGuinness Actor Profile that directly addresses RFC 8693's chain-splicing weakness by making the chain itself cryptographically verifiable rather than just informational.</t>
         </is>
       </c>
     </row>
@@ -1765,17 +1765,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-rfc9728bis — Update to OAuth 2.0 Protected Resource Metadata Resource Identifier Validation</t>
+          <t>draft-mcguinness-oauth-client-instance-assertion — OAuth Client Instance Assertion</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>A McGuinness individual draft updating Section 3.3 of RFC 9728 (Protected Resource Metadata) so the resource value can be any URI sharing the same TLS origin as the requested URL whose path is a prefix of it — broadening the set of WWW-Authenticate response use cases without changing the rest of RFC 9728.</t>
+          <t>Karl McGuinness's individual draft for representing a specific running instance of an OAuth client (rather than just the client registration) so authorization servers can bind grants to a concrete instance.</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-rfc9728bis/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-client-instance-assertion/</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Revision -01 (Feb 2026). A small targeted correction to the PRM validation rule. Notable as supporting infrastructure for the McGuinness Mission-Bound OAuth work — PRM is the substrate for Resource AS / Resource Server discovery of required RAR types under that profile.</t>
+          <t>Note: full draft text was not retrievable through automated fetch at time of writing — recommend reading directly. Companion to the Actor Profile draft and to attestation-based client auth.</t>
         </is>
       </c>
     </row>
@@ -1795,17 +1795,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-token-xchg-target-svc-disco — OAuth 2.0 Token Exchange Target Service Discovery</t>
+          <t>draft-mcguinness-oauth-resource-token-resp — OAuth 2.0 Resource Parameter in Access Token Response</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>A McGuinness/Parecki individual draft defining a discovery endpoint that, given a subject token, returns the set of available target services (audiences, resources, scopes) the holder can request via RFC 8693 Token Exchange — accepting any registered subject_token_type so it supports advanced flows including identity chaining and cross-domain delegation.</t>
+          <t>A McGuinness/Skokan individual draft adding a 'resource' parameter to the OAuth access token response so clients can confirm which resource the issued token is valid for, mitigating resource mix-up attacks especially in deployments that use RFC 8707 Resource Indicators.</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-token-xchg-target-svc-disco/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-resource-token-resp/</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Revision -01 (Feb 2026), co-authored with Aaron Parecki (Okta). Fills a discovery gap that ID-JAG and the Transaction Token Chaining Profile both implicitly assume — clients today must know which audience to request, which doesn't compose with open-world agentic flows where the right downstream service is determined at runtime.</t>
+          <t>Revision -03 (March 2026). Filip Skokan added as co-author in -03. Complements RFC 8707 / RFC 9700 / RFC 9207 by adding issuance-time confirmation to the discovery-time mechanisms. Notable for the agent-authz corpus because dynamic resource discovery is a core agent pattern and resource-mix-up attacks are amplified when agents juggle many short-lived tokens.</t>
         </is>
       </c>
     </row>
@@ -1825,17 +1825,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-actor-receipts — OAuth Actor Receipts for Delegation Provenance</t>
+          <t>draft-mcguinness-oauth-rfc9728bis — Update to OAuth 2.0 Protected Resource Metadata Resource Identifier Validation</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>A McGuinness companion draft to the Actor Profile, aiming to provide per-hop signed receipts as the verifiable provenance layer that the Actor Profile (which keeps the 'act' chain informational) deliberately leaves out. Pulls over the provenance gap from the core profile so each principal in a delegation chain can produce independent cryptographic evidence.</t>
+          <t>A McGuinness individual draft updating Section 3.3 of RFC 9728 (Protected Resource Metadata) so the resource value can be any URI sharing the same TLS origin as the requested URL whose path is a prefix of it — broadening the set of WWW-Authenticate response use cases without changing the rest of RFC 9728.</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-actor-receipts/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-rfc9728bis/</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 4 Jul 2026; now formally on IETF Datatracker (was GitHub-only pre-publication through Jun 2026). Recommended companion to the Actor Profile when a deployment needs Verified Full Disclosure mode (per the Mission-Bound OAuth Runtime Enforcement Profile's Actor Provenance Module). Completes a triad with actor-profile and actor-proofs — receipts provide provenance, proofs provide cryptographic per-hop accountability.</t>
+          <t>Revision -01 (Feb 2026). A small targeted correction to the PRM validation rule. Notable as supporting infrastructure for the McGuinness Mission-Bound OAuth work — PRM is the substrate for Resource AS / Resource Server discovery of required RAR types under that profile.</t>
         </is>
       </c>
     </row>
@@ -1855,17 +1855,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-actor-proofs — OAuth Actor-Signed Hop Proofs</t>
+          <t>draft-mcguinness-token-xchg-target-svc-disco — OAuth 2.0 Token Exchange Target Service Discovery</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Introduces the 'actor_proofs' claim — a signed per-hop proof chain where each actor signs its own participation and the target binding it authorized for that hop; proofs are hash-chained and validated using actor verification keys from trusted sources, with optional references to sibling actor receipts.</t>
+          <t>A McGuinness/Parecki individual draft defining a discovery endpoint that, given a subject token, returns the set of available target services (audiences, resources, scopes) the holder can request via RFC 8693 Token Exchange — accepting any registered subject_token_type so it supports advanced flows including identity chaining and cross-domain delegation.</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-actor-proofs/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-token-xchg-target-svc-disco/</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 4 Jul 2026. Completes the actor triad with actor-profile (chain structure) and actor-receipts (provenance) — actor-proofs closes the cryptographic accountability gap. Filed the same day as ai-agent-instance, id-assertion-framework, and domain-authorized-issuer — McGuinness submitted four new I-Ds on Jul 4-6, bringing his total to 11 individual I-Ds on Datatracker.</t>
+          <t>Revision -01 (Feb 2026), co-authored with Aaron Parecki (Okta). Fills a discovery gap that ID-JAG and the Transaction Token Chaining Profile both implicitly assume — clients today must know which audience to request, which doesn't compose with open-world agentic flows where the right downstream service is determined at runtime.</t>
         </is>
       </c>
     </row>
@@ -1885,17 +1885,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-insufficient-claims — OAuth 2.0 Insufficient Claims Challenge</t>
+          <t>draft-mcguinness-oauth-actor-receipts — OAuth Actor Receipts for Delegation Provenance</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>A McGuinness individual draft defining an insufficient_claims error code and required_claims parameter enabling authorization servers and protected resources to signal precisely which claims are missing from a presented credential. Allows resource servers to request enriched credentials carrying specific missing attributes rather than returning a generic 401.</t>
+          <t>A McGuinness companion draft to the Actor Profile, aiming to provide per-hop signed receipts as the verifiable provenance layer that the Actor Profile (which keeps the 'act' chain informational) deliberately leaves out. Pulls over the provenance gap from the core profile so each principal in a delegation chain can produce independent cryptographic evidence.</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-insufficient-claims/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-actor-receipts/</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 27 May 2026. Enables just-in-time claim negotiation in multi-agent delegation chains where the acting party must assemble claims from multiple sources. Natural companion to the Actor Profile and Client Instance Assertion — those drafts define the identity structure; this one provides the feedback loop when that structure is incomplete at the RS.</t>
+          <t>Revision -00, 4 Jul 2026; now formally on IETF Datatracker (was GitHub-only pre-publication through Jun 2026). Recommended companion to the Actor Profile when a deployment needs Verified Full Disclosure mode (per the Mission-Bound OAuth Runtime Enforcement Profile's Actor Provenance Module). Completes a triad with actor-profile and actor-proofs — receipts provide provenance, proofs provide cryptographic per-hop accountability.</t>
         </is>
       </c>
     </row>
@@ -1915,17 +1915,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-ai-agent-instance — OAuth 2.0 AI Agent Instance Profile</t>
+          <t>draft-mcguinness-oauth-actor-proofs — OAuth Actor-Signed Hop Proofs</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Profiles OAuth 2.0 for deployments where a single client ID represents an agent platform running many concurrent agent instances; defines claims conveying attested agent instance identity and provenance from an agent attester to the AS, with delegation-chain semantics for sub-agents. Claims are carrier-independent, compatible with both Client Instance Assertions and Client Attestation JWT.</t>
+          <t>Introduces the 'actor_proofs' claim — a signed per-hop proof chain where each actor signs its own participation and the target binding it authorized for that hop; proofs are hash-chained and validated using actor verification keys from trusted sources, with optional references to sibling actor receipts.</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-ai-agent-instance/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-actor-proofs/</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 4 Jul 2026. Fills the gap between a registered OAuth client ID (platform-level) and a running agent instance (runtime-level) — the level at which delegation chains, attestation, and revocation actually operate. Companion to draft-mcguinness-oauth-client-instance-assertion (general instance framing) and draft-mcguinness-oauth-actor-profile (chain representation).</t>
+          <t>Revision -00, 4 Jul 2026. Completes the actor triad with actor-profile (chain structure) and actor-receipts (provenance) — actor-proofs closes the cryptographic accountability gap. Filed the same day as ai-agent-instance, id-assertion-framework, and domain-authorized-issuer — McGuinness submitted four new I-Ds on Jul 4-6, bringing his total to 11 individual I-Ds on Datatracker.</t>
         </is>
       </c>
     </row>
@@ -1945,17 +1945,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-id-assertion-framework — OAuth Identity Assertion Trust Framework</t>
+          <t>draft-mcguinness-oauth-insufficient-claims — OAuth 2.0 Insufficient Claims Challenge</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Addresses the gap where issuer authentication alone does not prove AS authority over subject namespaces; defines an Authority Delegation Model with independent trust-evaluation categories and an Identity Assertion Issuer Trust Policy (JSON document declaring required trust methods) that Resource ASes evaluate before accepting identity assertions.</t>
+          <t>A McGuinness individual draft defining an insufficient_claims error code and required_claims parameter enabling authorization servers and protected resources to signal precisely which claims are missing from a presented credential. Allows resource servers to request enriched credentials carrying specific missing attributes rather than returning a generic 401.</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-id-assertion-framework/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-insufficient-claims/</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 4 Jul 2026. Directly motivates and companions draft-mcguinness-oauth-domain-authorized-issuer (below) which provides a DNS-based trust method. Addresses the 'who is allowed to assert identities in this namespace?' question that ID-JAG and the identity-chaining WG draft assume resolved but do not specify.</t>
+          <t>Revision -00, 27 May 2026. Enables just-in-time claim negotiation in multi-agent delegation chains where the acting party must assemble claims from multiple sources. Natural companion to the Actor Profile and Client Instance Assertion — those drafts define the identity structure; this one provides the feedback loop when that structure is incomplete at the RS.</t>
         </is>
       </c>
     </row>
@@ -1975,17 +1975,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-domain-authorized-issuer — OAuth Domain-Authorized Issuer Trust Method</t>
+          <t>draft-mcguinness-oauth-ai-agent-instance — OAuth 2.0 AI Agent Instance Profile</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>DNS domain owners publish a policy (DNS TXT record at _oauth-issuer-policy.{domain} or HTTPS well-known fallback) listing the OAuth ASes authorized to assert identities in that namespace; Resource ASes use this to validate assertion issuers before accepting identity assertions or chaining tokens. Pattern echoes CAA/SPF/DKIM. Non-transitive — flat authorization, no delegation chains.</t>
+          <t>Profiles OAuth 2.0 for deployments where a single client ID represents an agent platform running many concurrent agent instances; defines claims conveying attested agent instance identity and provenance from an agent attester to the AS, with delegation-chain semantics for sub-agents. Claims are carrier-independent, compatible with both Client Instance Assertions and Client Attestation JWT.</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-domain-authorized-issuer/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-ai-agent-instance/</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 4 Jul 2026. Implements one trust method for draft-mcguinness-oauth-id-assertion-framework. DNS-based approach is lightweight and operationally familiar; the non-transitive design avoids the amplification risks of transitive trust chains. Closes the 'how do you know the AS is allowed to speak for this domain?' gap that cross-domain identity chaining has always assumed away.</t>
+          <t>Revision -00, 4 Jul 2026. Fills the gap between a registered OAuth client ID (platform-level) and a running agent instance (runtime-level) — the level at which delegation chains, attestation, and revocation actually operate. Companion to draft-mcguinness-oauth-client-instance-assertion (general instance framing) and draft-mcguinness-oauth-actor-profile (chain representation).</t>
         </is>
       </c>
     </row>
@@ -2005,17 +2005,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>draft-mcguinness-oauth-mission — Mission-Bound Authorization for OAuth 2.0</t>
+          <t>draft-mcguinness-oauth-id-assertion-framework — OAuth Identity Assertion Trust Framework</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Introduces 'Mission' — a durable, integrity-bound artifact stored at the AS representing an approved task; clients submit Mission Intent via PAR, ASes derive concrete permissions, and approvers grant consent via integrity anchors. Access tokens carry a 'mission' claim; issuance is gated by the Mission's lifecycle state, enabling revocation governance and audit trails for multi-step agent operations.</t>
+          <t>Addresses the gap where issuer authentication alone does not prove AS authority over subject namespaces; defines an Authority Delegation Model with independent trust-evaluation categories and an Identity Assertion Issuer Trust Policy (JSON document declaring required trust methods) that Resource ASes evaluate before accepting identity assertions.</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-mission/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-id-assertion-framework/</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 6 Jul 2026. This is the formal I-D target for the 'Mission-Bound OAuth MVP' blog post (May 2026, Industry tab) — the five-wire-addition protocol that makes the user-approved task a first-class OAuth object. Paired with the runtime enforcement profile (still not on Datatracker as of Jul 10). The Mission lifecycle (pending_approval → active → suspended → revoked → expired → completed → rejected) and the proposal_hash/consent_rendering_hash binding anchor what was approved versus what the user saw.</t>
+          <t>Revision -00, 4 Jul 2026. Directly motivates and companions draft-mcguinness-oauth-domain-authorized-issuer (below) which provides a DNS-based trust method. Addresses the 'who is allowed to assert identities in this namespace?' question that ID-JAG and the identity-chaining WG draft assume resolved but do not specify.</t>
         </is>
       </c>
     </row>
@@ -2035,17 +2035,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>draft-mishra-oauth-agent-grants — Delegated Agent Authorization Protocol (DAAP)</t>
+          <t>draft-mcguinness-oauth-domain-authorized-issuer — OAuth Domain-Authorized Issuer Trust Method</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft addressing runtime agent identity for dynamically-spawned agents, multi-agent sub-delegation with depth-limiting, and cascade revocation of an entire delegation subtree when any ancestor is revoked.</t>
+          <t>DNS domain owners publish a policy (DNS TXT record at _oauth-issuer-policy.{domain} or HTTPS well-known fallback) listing the OAuth ASes authorized to assert identities in that namespace; Resource ASes use this to validate assertion issuers before accepting identity assertions or chaining tokens. Pattern echoes CAA/SPF/DKIM. Non-transitive — flat authorization, no delegation chains.</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mishra-oauth-agent-grants/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-domain-authorized-issuer/</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Revision -01 (March 2026); registers new JWT claims (agt, dev, grnt, scp, bdg) — a more aggressive alternative to RFC 8693 with budget-bounded grants. Overlaps with draft-niyikiza-oauth-attenuating-agent-tokens; OAuth WG will likely expect consolidation.</t>
+          <t>Revision -00, 4 Jul 2026. Implements one trust method for draft-mcguinness-oauth-id-assertion-framework. DNS-based approach is lightweight and operationally familiar; the non-transitive design avoids the amplification risks of transitive trust chains. Closes the 'how do you know the AS is allowed to speak for this domain?' gap that cross-domain identity chaining has always assumed away.</t>
         </is>
       </c>
     </row>
@@ -2065,17 +2065,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>draft-kuehlewind-audit-architecture — Architecture for Auditing AI Agent Delegation and Interactions</t>
+          <t>draft-mcguinness-oauth-mission — Mission-Bound Authorization for OAuth 2.0</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Mirja Kühlewind (Ericsson, former IETF TSV-AD) and Henk Birkholz (Fraunhofer SIT, lead author of RFC 9334 RATS and SCITT architecture) defining four record types — Interaction, Action, Delegation, and Authorization Transition — and an Audit Context that propagates across OAuth + WIMSE + RATS + SCITT to make agent behaviour verifiably auditable end-to-end.</t>
+          <t>Introduces 'Mission' — a durable, integrity-bound artifact stored at the AS representing an approved task; clients submit Mission Intent via PAR, ASes derive concrete permissions, and approvers grant consent via integrity anchors. Access tokens carry a 'mission' claim; issuance is gated by the Mission's lifecycle state, enabling revocation governance and audit trails for multi-step agent operations.</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-kuehlewind-audit-architecture/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mcguinness-oauth-mission/</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Revision -00 published 18 May 2026; the cross-layer integration piece — explicitly composes the McGuinness Actor Profile, Transaction Tokens, identity-chaining, ID-JAG, WIMSE, RATS, and SCITT into a single auditable architecture with 11 proposed work items. The treats-Agent-as-untrusted threat model is what regulators (SOX, PSD2, EU AI Act) actually want.</t>
+          <t>Revision -00, 6 Jul 2026. This is the formal I-D target for the 'Mission-Bound OAuth MVP' blog post (May 2026, Industry tab) — the five-wire-addition protocol that makes the user-approved task a first-class OAuth object. Paired with the runtime enforcement profile (still not on Datatracker as of Jul 10). The Mission lifecycle (pending_approval → active → suspended → revoked → expired → completed → rejected) and the proposal_hash/consent_rendering_hash binding anchor what was approved versus what the user saw.</t>
         </is>
       </c>
     </row>
@@ -2095,17 +2095,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>draft-birkholz-verifiable-agent-conversations — Verifiable Agent Conversation Records</t>
+          <t>draft-mishra-oauth-agent-grants — Delegated Agent Authorization Protocol (DAAP)</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft (Birkholz/Heldt/Steele) defining a CDDL data format — with both JSON and CBOR encodings — for tamper-evident, verifiably-signed records of agent conversations, agent reasoning traces, tool calls, and system events that support long-term evidentiary value across chains of custody.</t>
+          <t>An IETF individual draft addressing runtime agent identity for dynamically-spawned agents, multi-agent sub-delegation with depth-limiting, and cascade revocation of an entire delegation subtree when any ancestor is revoked.</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-birkholz-verifiable-agent-conversations/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mishra-oauth-agent-grants/</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Revision -00 published 25 Feb 2026; presented at IETF 125 dispatch and hotrfc. The canonical Interaction-Record format for the Kuehlewind audit architecture. Motivating examples are concrete: agents acting beyond scope, CoT divergence, and 'sandbagging' during evaluations.</t>
+          <t>Revision -01 (March 2026); registers new JWT claims (agt, dev, grnt, scp, bdg) — a more aggressive alternative to RFC 8693 with budget-bounded grants. Overlaps with draft-niyikiza-oauth-attenuating-agent-tokens; OAuth WG will likely expect consolidation.</t>
         </is>
       </c>
     </row>
@@ -2125,17 +2125,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>draft-klrc-aiagent-auth — AI Agent Authentication and Authorization</t>
+          <t>draft-kuehlewind-audit-architecture — Architecture for Auditing AI Agent Delegation and Interactions</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft that does not invent new protocols but composes WIMSE/SPIFFE workload identity, OAuth 2.x, and OpenID SSF to authenticate and delegate authority to AI agents.</t>
+          <t>An IETF individual draft from Mirja Kühlewind (Ericsson, former IETF TSV-AD) and Henk Birkholz (Fraunhofer SIT, lead author of RFC 9334 RATS and SCITT architecture) defining four record types — Interaction, Action, Delegation, and Authorization Transition — and an Audit Context that propagates across OAuth + WIMSE + RATS + SCITT to make agent behaviour verifiably auditable end-to-end.</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/html/draft-klrc-aiagent-auth-00</t>
+          <t>https://datatracker.ietf.org/doc/draft-kuehlewind-audit-architecture/</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, March 2026; introduces 'Agent Identity Management System (AIMS)' and is the cleanest standards-based framing of agent-as-workload.</t>
+          <t>Revision -00 published 18 May 2026; the cross-layer integration piece — explicitly composes the McGuinness Actor Profile, Transaction Tokens, identity-chaining, ID-JAG, WIMSE, RATS, and SCITT into a single auditable architecture with 11 proposed work items. The treats-Agent-as-untrusted threat model is what regulators (SOX, PSD2, EU AI Act) actually want.</t>
         </is>
       </c>
     </row>
@@ -2155,17 +2155,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>draft-niyikiza-oauth-attenuating-agent-tokens — Attenuating Authorization Tokens for Agentic Delegation Chains</t>
+          <t>draft-birkholz-verifiable-agent-conversations — Verifiable Agent Conversation Records</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft extending RFC 9396 Rich Authorization Requests with monotonic attenuation at each delegation hop, offline chain verification, and a typed constraint vocabulary for tool-level argument restrictions.</t>
+          <t>An IETF individual draft (Birkholz/Heldt/Steele) defining a CDDL data format — with both JSON and CBOR encodings — for tamper-evident, verifiably-signed records of agent conversations, agent reasoning traces, tool calls, and system events that support long-term evidentiary value across chains of custody.</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-niyikiza-oauth-attenuating-agent-tokens/</t>
+          <t>https://datatracker.ietf.org/doc/draft-birkholz-verifiable-agent-conversations/</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, March 2026; arguably the strongest purely-OAuth-grounded delegation draft — offline verification is a key scalability property. Good path to OAuth WG adoption; overlaps with draft-mishra-oauth-agent-grants and will likely need to be consolidated with it.</t>
+          <t>Revision -00 published 25 Feb 2026; presented at IETF 125 dispatch and hotrfc. The canonical Interaction-Record format for the Kuehlewind audit architecture. Motivating examples are concrete: agents acting beyond scope, CoT divergence, and 'sandbagging' during evaluations.</t>
         </is>
       </c>
     </row>
@@ -2185,17 +2185,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>draft-singla-agent-identity-protocol — AIP: Decentralized Identity and Delegation for AI Agents</t>
+          <t>draft-klrc-aiagent-auth — AI Agent Authentication and Authorization</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft proposing a six-layer model (identity through reputation) for AI agents with W3C DID anchoring, a Delegation Depth counter, three Grant ceremony tiers (G1/G2/G3), DPoP proof-of-possession, and an MCP integration layer.</t>
+          <t>An IETF individual draft that does not invent new protocols but composes WIMSE/SPIFFE workload identity, OAuth 2.x, and OpenID SSF to authenticate and delegate authority to AI agents.</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-singla-agent-identity-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/html/draft-klrc-aiagent-auth-00</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 17 April 2026; the most comprehensive identity framework in the set. The W3C DID dependency will face IETF pushback, the 75+ page scope needs reduction, and the 'AIP' name collision with two other drafts (draft-prakash-aip, draft-aip-agent-identity-protocol) must be resolved.</t>
+          <t>Revision -00, March 2026; introduces 'Agent Identity Management System (AIMS)' and is the cleanest standards-based framing of agent-as-workload.</t>
         </is>
       </c>
     </row>
@@ -2215,17 +2215,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>draft-prakash-aip — AIP: Verifiable Delegation for AI Agent Systems</t>
+          <t>draft-niyikiza-oauth-attenuating-agent-tokens — Attenuating Authorization Tokens for Agentic Delegation Chains</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft introducing Invocation-Bound Capability Tokens (IBCTs) in two modes — compact (JWT/Ed25519) for single-hop and chained (Biscuit + Datalog) for multi-hop — with bindings for MCP, A2A, and HTTP APIs.</t>
+          <t>An IETF individual draft extending RFC 9396 Rich Authorization Requests with monotonic attenuation at each delegation hop, offline chain verification, and a typed constraint vocabulary for tool-level argument restrictions.</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-prakash-aip/</t>
+          <t>https://datatracker.ietf.org/doc/draft-niyikiza-oauth-attenuating-agent-tokens/</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 27 March 2026; technically strong — Biscuit + Datalog is well-suited to scope attenuation. The 'AIP' name collision with draft-singla-agent-identity-protocol and draft-aip-agent-identity-protocol is a blocking issue for WG adoption.</t>
+          <t>Revision -00, March 2026; arguably the strongest purely-OAuth-grounded delegation draft — offline verification is a key scalability property. Good path to OAuth WG adoption; overlaps with draft-mishra-oauth-agent-grants and will likely need to be consolidated with it.</t>
         </is>
       </c>
     </row>
@@ -2245,17 +2245,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>draft-goswami-agentic-jwt — Secure Intent Protocol: JWT-Compatible Agentic Identity and Workflow Management</t>
+          <t>draft-singla-agent-identity-protocol — AIP: Decentralized Identity and Delegation for AI Agents</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an Agentic JWT extension to OAuth 2.0 with a Supervisor Agent role for sub-agent coordination, explicitly addressing the 'intent-execution separation' gap and adding workflow-step authorization.</t>
+          <t>An IETF individual draft proposing a six-layer model (identity through reputation) for AI agents with W3C DID anchoring, a Delegation Depth counter, three Grant ceremony tiers (G1/G2/G3), DPoP proof-of-possession, and an MCP integration layer.</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-goswami-agentic-jwt/</t>
+          <t>https://datatracker.ietf.org/doc/draft-singla-agent-identity-protocol/</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, December 2025; the intent-execution-separation framing is insightful and distinguishing. The workflow-step authorization approach is novel but may face skepticism in the OAuth WG.</t>
+          <t>Revision -00, 17 April 2026; the most comprehensive identity framework in the set. The W3C DID dependency will face IETF pushback, the 75+ page scope needs reduction, and the 'AIP' name collision with two other drafts (draft-prakash-aip, draft-aip-agent-identity-protocol) must be resolved.</t>
         </is>
       </c>
     </row>
@@ -2275,17 +2275,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>draft-ni-wimse-ai-agent-identity — WIMSE Applicability for AI Agents</t>
+          <t>draft-prakash-aip — AIP: Verifiable Delegation for AI Agent Systems</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft mapping the WIMSE workload-identity architecture to AI-agent use cases and establishing credential-management mechanisms for agentic AI within the WIMSE framework.</t>
+          <t>An IETF individual draft introducing Invocation-Bound Capability Tokens (IBCTs) in two modes — compact (JWT/Ed25519) for single-hop and chained (Biscuit + Datalog) for multi-hop — with bindings for MCP, A2A, and HTTP APIs.</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ni-wimse-ai-agent-identity/</t>
+          <t>https://datatracker.ietf.org/doc/draft-prakash-aip/</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, February 2026; an important bridge between the WIMSE WG and the AI agent space. If an AI-agent WG is ever chartered, this applicability statement is essential groundwork. Co-authored with Liu, who also leads the related security-requirements draft.</t>
+          <t>Revision -00, 27 March 2026; technically strong — Biscuit + Datalog is well-suited to scope attenuation. The 'AIP' name collision with draft-singla-agent-identity-protocol and draft-aip-agent-identity-protocol is a blocking issue for WG adoption.</t>
         </is>
       </c>
     </row>
@@ -2305,17 +2305,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-identity-framework — Agent Identity Framework: Trust and Identity for Autonomous AI Agents</t>
+          <t>draft-goswami-agentic-jwt — Secure Intent Protocol: JWT-Compatible Agentic Identity and Workflow Management</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft proposing a five-layer model (identity, authorization, attestation, evidence, trust) for autonomous AI agents, with a gap analysis between current Internet standards and agent requirements.</t>
+          <t>An IETF individual draft defining an Agentic JWT extension to OAuth 2.0 with a Supervisor Agent role for sub-agent coordination, explicitly addressing the 'intent-execution separation' gap and adding workflow-step authorization.</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-identity-framework/</t>
+          <t>https://datatracker.ietf.org/doc/draft-goswami-agentic-jwt/</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 6 April 2026; more gap-analysis than protocol spec. Useful as problem statement. Five-layer model is a reasonable decomposition but insufficient as a standalone contribution. Part of the Sharif cluster (with -agent-audit-trail, -attp, etc.).</t>
+          <t>Revision -00, December 2025; the intent-execution-separation framing is insightful and distinguishing. The workflow-step authorization approach is novel but may face skepticism in the OAuth WG.</t>
         </is>
       </c>
     </row>
@@ -2335,17 +2335,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>draft-aip-agent-identity-protocol — AIP: Agentic Authentication and Authorized Policy Enforcement</t>
+          <t>draft-ni-wimse-ai-agent-identity — WIMSE Applicability for AI Agents</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an AIP Token signed per tool call (agent ID, tool, nonce, timestamp, signature), an AgentPolicy YAML format for per-tool argument constraints and DLP rules, and a Human-in-the-Loop proxy enforcement model.</t>
+          <t>An IETF individual draft mapping the WIMSE workload-identity architecture to AI-agent use cases and establishing credential-management mechanisms for agentic AI within the WIMSE framework.</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-aip-agent-identity-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ni-wimse-ai-agent-identity/</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 16 March 2026; implementation-focused. YAML policy approach is pragmatic but not interoperable-by-design. HITL integration is a valuable safety feature. Third member of the 'AIP' name-collision triple — must be resolved before any can progress.</t>
+          <t>Revision -02, February 2026; an important bridge between the WIMSE WG and the AI agent space. If an AI-agent WG is ever chartered, this applicability statement is essential groundwork. Co-authored with Liu, who also leads the related security-requirements draft.</t>
         </is>
       </c>
     </row>
@@ -2365,17 +2365,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>draft-liu-oauth-chain-delegation — Delegation Chain for OAuth 2.0</t>
+          <t>draft-sharif-agent-identity-framework — Agent Identity Framework: Trust and Identity for Autonomous AI Agents</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Introduces a delegation_chain JWT claim as a structured companion to RFC 8693's act claim; delegation_chain records the complete delegation history as an ordered array with per-hop authorization constraints and optional cryptographic confirmation from each delegating agent. Supports cross-domain delegation with integrated user consent interaction.</t>
+          <t>An IETF individual draft proposing a five-layer model (identity, authorization, attestation, evidence, trust) for autonomous AI agents, with a gap analysis between current Internet standards and agent requirements.</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-liu-oauth-chain-delegation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-identity-framework/</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 6 Jun 2026; authors: Dapeng Liu, Judy Zhu, Suresh Krishnan (Ericsson), Aaron Parecki (Okta). Provides the structured delegation lineage that act alone cannot express; strong overlap with draft-mw-oauth-actor-chain and draft-niyikiza-oauth-attenuating-agent-tokens — OAuth WG will likely expect consolidation across these three.</t>
+          <t>Revision -00, 6 April 2026; more gap-analysis than protocol spec. Useful as problem statement. Five-layer model is a reasonable decomposition but insufficient as a standalone contribution. Part of the Sharif cluster (with -agent-audit-trail, -attp, etc.).</t>
         </is>
       </c>
     </row>
@@ -2395,17 +2395,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>draft-fletcher-transaction-token-chaining-profile — Transaction Token Authorization Grant Profile for OAuth Identity and Authorization Chaining</t>
+          <t>draft-aip-agent-identity-protocol — AIP: Agentic Authentication and Authorized Policy Enforcement</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Establishes a framework for using Transaction Tokens as subject credentials in OAuth 2.0 Token Exchange requests (RFC 8693), enabling services within one trust domain to obtain JWT authorization grants for accessing resources across domain boundaries without exposing internal token formats.</t>
+          <t>An IETF individual draft defining an AIP Token signed per tool call (agent ID, tool, nonce, timestamp, signature), an AgentPolicy YAML format for per-tool argument constraints and DLP rules, and a Human-in-the-Loop proxy enforcement model.</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-fletcher-transaction-token-chaining-profile/</t>
+          <t>https://datatracker.ietf.org/doc/draft-aip-agent-identity-protocol/</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, 6 Jul 2026 (was -01 Jun 2026); authors: George Fletcher (Practical Identity LLC), Pieter Kasselman (Defakto Security), Sean O'Dell (CVS Health). Directly bridges draft-ietf-oauth-transaction-tokens and draft-ietf-oauth-identity-chaining (both in corpus), closing the 'how do TX Tokens actually cross domains' gap. Note: lead author is the corpus maintainer.</t>
+          <t>Revision -00, 16 March 2026; implementation-focused. YAML policy approach is pragmatic but not interoperable-by-design. HITL integration is a valuable safety feature. Third member of the 'AIP' name-collision triple — must be resolved before any can progress.</t>
         </is>
       </c>
     </row>
@@ -2425,17 +2425,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>draft-zhu-oauth-async-delegation — Sender-Constrained Delegation Handle for Asynchronous OAuth 2.0 Identity Chaining</t>
+          <t>draft-liu-oauth-chain-delegation — Delegation Chain for OAuth 2.0</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Introduces a Delegation Handle — a sender-constrained, audience-locked JWT issued by authorization servers — enabling acting clients to refresh chained access tokens without re-prompting an offline end user while maintaining strict policy bounds and identity chains.</t>
+          <t>Introduces a delegation_chain JWT claim as a structured companion to RFC 8693's act claim; delegation_chain records the complete delegation history as an ordered array with per-hop authorization constraints and optional cryptographic confirmation from each delegating agent. Supports cross-domain delegation with integrated user consent interaction.</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-zhu-oauth-async-delegation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-liu-oauth-chain-delegation/</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 22 May 2026; authors: Larry Zhu, Sam Currie (Atlassian). Addresses a concrete gap in agent delegation: what happens when the delegating human is not present to re-authorize. Directly relevant to long-running agentic workflows using draft-ietf-oauth-identity-chaining.</t>
+          <t>Revision -00, 6 Jun 2026; authors: Dapeng Liu, Judy Zhu, Suresh Krishnan (Ericsson), Aaron Parecki (Okta). Provides the structured delegation lineage that act alone cannot express; strong overlap with draft-mw-oauth-actor-chain and draft-niyikiza-oauth-attenuating-agent-tokens — OAuth WG will likely expect consolidation across these three.</t>
         </is>
       </c>
     </row>
@@ -2455,17 +2455,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>draft-chen-oauth-agent-revocation — OAuth 2.0 Agent Authorization Explicit Revocation</t>
+          <t>draft-fletcher-transaction-token-chaining-profile — Transaction Token Authorization Grant Profile for OAuth Identity and Authorization Chaining</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Extends RFC 7009 token revocation for agent-based scenarios: introduces batch revocation by agent ID, cascading revocation across delegation chains, conditional revocation options, and verifiable audit trails.</t>
+          <t>Establishes a framework for using Transaction Tokens as subject credentials in OAuth 2.0 Token Exchange requests (RFC 8693), enabling services within one trust domain to obtain JWT authorization grants for accessing resources across domain boundaries without exposing internal token formats.</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-chen-oauth-agent-revocation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-fletcher-transaction-token-chaining-profile/</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 27 Apr 2026; authors: Meiling Chen, Li Su (China Mobile). Fills the lifecycle management gap — existing RFC 7009 revocation is single-token and client-centric, but agent delegation chains require cascade semantics. Natural companion to draft-ietf-oauth-transaction-tokens and draft-niyikiza-oauth-attenuating-agent-tokens.</t>
+          <t>Revision -02, 6 Jul 2026 (was -01 Jun 2026); authors: George Fletcher (Practical Identity LLC), Pieter Kasselman (Defakto Security), Sean O'Dell (CVS Health). Directly bridges draft-ietf-oauth-transaction-tokens and draft-ietf-oauth-identity-chaining (both in corpus), closing the 'how do TX Tokens actually cross domains' gap. Note: lead author is the corpus maintainer.</t>
         </is>
       </c>
     </row>
@@ -2485,17 +2485,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>draft-jiang-oauth-intent-admission — Intent Admission Assertions for Agentic Systems</t>
+          <t>draft-zhu-oauth-async-delegation — Sender-Constrained Delegation Handle for Asynchronous OAuth 2.0 Identity Chaining</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Defines a signed, verifiable Intent Admission Assertion (IAA) that an admission point creates after verifying agent identity, evaluating permissions against policy, and — when required — obtaining explicit user consent; the IAA is transmitted to the execution endpoint which re-validates before proceeding. Leverages OAuth and RFC 9396 Rich Authorization Requests.</t>
+          <t>Introduces a Delegation Handle — a sender-constrained, audience-locked JWT issued by authorization servers — enabling acting clients to refresh chained access tokens without re-prompting an offline end user while maintaining strict policy bounds and identity chains.</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jiang-oauth-intent-admission/</t>
+          <t>https://datatracker.ietf.org/doc/draft-zhu-oauth-async-delegation/</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 23 Jun 2026; authors: Yuning Jiang, Lun Li, Yurong Song, Faye Liu (Huawei). The required_consent path maps directly to the HITL pattern central to the corpus. Companion to draft-jiang-intent-security (threat model) from the same Huawei group.</t>
+          <t>Revision -00, 22 May 2026; authors: Larry Zhu, Sam Currie (Atlassian). Addresses a concrete gap in agent delegation: what happens when the delegating human is not present to re-authorize. Directly relevant to long-running agentic workflows using draft-ietf-oauth-identity-chaining.</t>
         </is>
       </c>
     </row>
@@ -2515,17 +2515,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>draft-ni-oauth-batch-authorization-delegation — Batch Authorization Delegation</t>
+          <t>draft-emerson-oauth-user-mediated-delivery — User-Mediated Credential Delivery for AI Agents</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Defines a mechanism for delegating a batch of fine-grained, actor-bound permissions in a single request across multiple collaborating actors; uses RFC 9396 RAR to carry per-actor authorization_details and RFC 8693 Token Exchange for sub-agent delegation, targeting multi-agent orchestration where a leader-agent receives batch permissions and delegates subsets to sub-agents.</t>
+          <t>Proposes user-mediated credential delivery as a complementary OAuth authorization primitive for AI agent frameworks: rather than delivering credentials through automated channels controlled by the agent or its platform, places the authorization decision and credential delivery step in the user's hands even when the agent is autonomous.</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ni-oauth-batch-authorization-delegation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-emerson-oauth-user-mediated-delivery/</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 3 Jul 2026; authors: Ni Yuan, Peter Chunchi Liu (Huawei). Addresses the round-trip overhead problem in large-scale multi-agent orchestration — individual delegation exchanges per sub-agent don't scale. Complements draft-song-oauth-ai-agent-collaborate-authz (same Huawei group, coordination focus) and draft-niyikiza-oauth-attenuating-agent-tokens (attenuation semantics). The RAR-based batch approach aligns well with the OAuth WG's RAR investment.</t>
+          <t>Revision -00, Jul 2026; author: Matt Emerson. Novel complement to draft-zhu-oauth-async-delegation — where Zhu handles the case of offline delegation continuation, Emerson argues some credential deliveries should always route through the user even in automated pipelines. Addresses prompt-injection and social-engineering risks in agent credential chains.</t>
         </is>
       </c>
     </row>
@@ -2545,17 +2545,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>draft-liu-oauth-a2a-profile — Agent-to-Agent (A2A) Profile for OAuth Transaction Tokens</t>
+          <t>draft-chen-oauth-agent-revocation — OAuth 2.0 Agent Authorization Explicit Revocation</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Defines a profile for using OAuth Transaction Tokens in distributed agent-to-agent communication scenarios; specifies mechanisms for embedding call-chain context within tokens to preserve agent identity, authorization information, and operational flow across agent workloads in trusted environments.</t>
+          <t>Extends RFC 7009 token revocation for agent-based scenarios: introduces batch revocation by agent ID, cascading revocation across delegation chains, conditional revocation options, and verifiable audit trails.</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-liu-oauth-a2a-profile/</t>
+          <t>https://datatracker.ietf.org/doc/draft-chen-oauth-agent-revocation/</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>EXPIRED. Revision -00, Oct 2025; authors: Peter Chunchi Liu, Ni Yuan (Huawei) — same author pair as draft-ni-oauth-batch-authorization-delegation. Directly profiles draft-ietf-oauth-transaction-tokens for A2A use; overlaps significantly with draft-araut-oauth-transaction-tokens-for-agents. Never revised; likely deferred rather than abandoned given both authors remain active in the corpus through Jul 2026.</t>
+          <t>Revision -00, 27 Apr 2026; authors: Meiling Chen, Li Su (China Mobile). Fills the lifecycle management gap — existing RFC 7009 revocation is single-token and client-centric, but agent delegation chains require cascade semantics. Natural companion to draft-ietf-oauth-transaction-tokens and draft-niyikiza-oauth-attenuating-agent-tokens.</t>
         </is>
       </c>
     </row>
@@ -2575,17 +2575,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>draft-song-oauth-ai-agent-collaborate-authz — OAuth 2.0 Extension for Multi-AI Agent Collaboration</t>
+          <t>draft-jiang-oauth-intent-admission — Intent Admission Assertions for Agentic Systems</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Extends OAuth 2.0 for coordinated multi-agent task groups: defines a collaborative authorization flow allowing a lead agent to obtain delegation tokens for sub-agents, with shared task context, coordinated scope attenuation, and cross-agent session binding.</t>
+          <t>Defines a signed, verifiable Intent Admission Assertion (IAA) that an admission point creates after verifying agent identity, evaluating permissions against policy, and — when required — obtaining explicit user consent; the IAA is transmitted to the execution endpoint which re-validates before proceeding. Leverages OAuth and RFC 9396 Rich Authorization Requests.</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-song-oauth-ai-agent-collaborate-authz/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jiang-oauth-intent-admission/</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, Jun/Jul 2026; authors: Yurong Song (Huawei) and colleagues. Addresses the multi-agent coordination gap at the OAuth layer — complements draft-jiang-oauth-intent-admission from the same Huawei group. Distinct from single-hop delegation drafts in explicitly modeling lead-agent-to-sub-agent scope sharing.</t>
+          <t>Revision -00, 23 Jun 2026; authors: Yuning Jiang, Lun Li, Yurong Song, Faye Liu (Huawei). The required_consent path maps directly to the HITL pattern central to the corpus. Companion to draft-jiang-intent-security (threat model) from the same Huawei group.</t>
         </is>
       </c>
     </row>
@@ -2605,17 +2605,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>draft-kroehl-agentic-trust-aae — Agent Authorization Envelope (AAE)</t>
+          <t>draft-ni-oauth-batch-authorization-delegation — Batch Authorization Delegation</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Specifies the AAE, a structured authorization container with three mandatory components — MANDATE, CONSTRAINTS, and VALIDITY — providing a machine-evaluable, cryptographically verifiable authorization assertion using W3C DIDs and Verifiable Credentials.</t>
+          <t>Defines a mechanism for delegating a batch of fine-grained, actor-bound permissions in a single request across multiple collaborating actors; uses RFC 9396 RAR to carry per-actor authorization_details and RFC 8693 Token Exchange for sub-agent delegation, targeting multi-agent orchestration where a leader-agent receives batch permissions and delegates subsets to sub-agents.</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-kroehl-agentic-trust-aae/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ni-oauth-batch-authorization-delegation/</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 21 May 2026; author: Lars Kersten Kroehl (CryptoKRI GmbH). Occupies similar design space to draft-mcguinness-oauth-actor-profile but uses a DID/VC substrate rather than OAuth — provides a useful alternative approach for non-OAuth deployments.</t>
+          <t>Revision -00, 3 Jul 2026; authors: Ni Yuan, Peter Chunchi Liu (Huawei). Addresses the round-trip overhead problem in large-scale multi-agent orchestration — individual delegation exchanges per sub-agent don't scale. Complements draft-song-oauth-ai-agent-collaborate-authz (same Huawei group, coordination focus) and draft-niyikiza-oauth-attenuating-agent-tokens (attenuation semantics). The RAR-based batch approach aligns well with the OAuth WG's RAR investment.</t>
         </is>
       </c>
     </row>
@@ -2635,17 +2635,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>draft-pidlisnyi-aps — Agent Passport System (APS)</t>
+          <t>draft-liu-oauth-a2a-profile — Agent-to-Agent (A2A) Profile for OAuth Transaction Tokens</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Specifies Ed25519-based agent passports, scoped delegation chains with constraints across seven dimensions (a lattice model where delegation monotonically narrows capabilities), cascade revocation, a three-signature policy chain, signed receipts, and MCP bindings; includes reference implementations in TypeScript and Python.</t>
+          <t>Defines a profile for using OAuth Transaction Tokens in distributed agent-to-agent communication scenarios; specifies mechanisms for embedding call-chain context within tokens to preserve agent identity, authorization information, and operational flow across agent workloads in trusted environments.</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-pidlisnyi-aps/</t>
+          <t>https://datatracker.ietf.org/doc/draft-liu-oauth-a2a-profile/</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 14 May 2026; author: Tymofii Pidlisnyi (AEOESS). Among the most comprehensive standalone agent authz specs in the wave — the seven-dimension constraint lattice and MCP binding make it directly implementable against Model Context Protocol deployments alongside draft-serra-mcp-discovery-uri.</t>
+          <t>EXPIRED. Revision -00, Oct 2025; authors: Peter Chunchi Liu, Ni Yuan (Huawei) — same author pair as draft-ni-oauth-batch-authorization-delegation. Directly profiles draft-ietf-oauth-transaction-tokens for A2A use; overlaps significantly with draft-araut-oauth-transaction-tokens-for-agents. Never revised; likely deferred rather than abandoned given both authors remain active in the corpus through Jul 2026.</t>
         </is>
       </c>
     </row>
@@ -2665,17 +2665,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>draft-serra-mcp-discovery-uri — The mcp URI Scheme and MCP Server Discovery Mechanism</t>
+          <t>draft-song-oauth-ai-agent-collaborate-authz — OAuth 2.0 Extension for Multi-AI Agent Collaboration</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an 'mcp://' URI scheme combined with /.well-known/mcp-server (RFC 8615) and a DNS TXT fallback for discovery of Model Context Protocol servers.</t>
+          <t>Extends OAuth 2.0 for coordinated multi-agent task groups: defines a collaborative authorization flow allowing a lead agent to obtain delegation tokens for sub-agents, with shared task context, coordinated scope attenuation, and cross-agent session binding.</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-serra-mcp-discovery-uri/</t>
+          <t>https://datatracker.ietf.org/doc/draft-song-oauth-ai-agent-collaborate-authz/</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Already at revision -04 (March 2026), suggesting active iteration; narrow scope, clean design, and the strongest IANA-registration candidate in the set. OAuth 2.1 for auth is deliberately out of scope.</t>
+          <t>Revision -02, Jun/Jul 2026; authors: Yurong Song (Huawei) and colleagues. Addresses the multi-agent coordination gap at the OAuth layer — complements draft-jiang-oauth-intent-admission from the same Huawei group. Distinct from single-hop delegation drafts in explicitly modeling lead-agent-to-sub-agent scope sharing.</t>
         </is>
       </c>
     </row>
@@ -2695,17 +2695,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-attp — ATTP: Agent Trust Transport Protocol</t>
+          <t>draft-kroehl-agentic-trust-aae — Agent Authorization Envelope (AAE)</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining trust levels L0–L4 mapped to PSD2 Strong Customer Authentication requirements, with bindings for MCP (MCPS), REST, A2A, gRPC, and GraphQL; supersedes draft-sharif-agent-payment-trust.</t>
+          <t>Specifies the AAE, a structured authorization container with three mandatory components — MANDATE, CONSTRAINTS, and VALIDITY — providing a machine-evaluable, cryptographically verifiable authorization assertion using W3C DIDs and Verifiable Credentials.</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-attp/</t>
+          <t>https://datatracker.ietf.org/doc/draft-kroehl-agentic-trust-aae/</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, April 2026; regulatory mapping appendices (PSD2, PCI DSS) are notable — one of the few drafts engaging financial regulation directly. Ambitious scope. Part of the Sharif cluster.</t>
+          <t>Revision -00, 21 May 2026; author: Lars Kersten Kroehl (CryptoKRI GmbH). Occupies similar design space to draft-mcguinness-oauth-actor-profile but uses a DID/VC substrate rather than OAuth — provides a useful alternative approach for non-OAuth deployments.</t>
         </is>
       </c>
     </row>
@@ -2725,17 +2725,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-transport-protocol — Agent Transport Protocol (ATP): Async Store-and-Forward for AI Agents</t>
+          <t>draft-pidlisnyi-aps — Agent Passport System (APS)</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining async store-and-forward messaging semantics with cryptographic identity per relay hop, trust scoring at ingress, capability negotiation, and interop with Google A2A, MCP, and FIPA ACL; transport-agnostic over TCP/TLS/QUIC.</t>
+          <t>Specifies Ed25519-based agent passports, scoped delegation chains with constraints across seven dimensions (a lattice model where delegation monotonically narrows capabilities), cascade revocation, a three-signature policy chain, signed receipts, and MCP bindings; includes reference implementations in TypeScript and Python.</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-transport-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-pidlisnyi-aps/</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 28 March 2026; addresses a real gap — most agent protocols assume synchronous availability, and store-and-forward is appropriate for long-running agentic tasks. Scope is broad and needs narrowing.</t>
+          <t>Revision -01, 14 May 2026; author: Tymofii Pidlisnyi (AEOESS). Among the most comprehensive standalone agent authz specs in the wave — the seven-dimension constraint lattice and MCP binding make it directly implementable against Model Context Protocol deployments alongside draft-serra-mcp-discovery-uri.</t>
         </is>
       </c>
     </row>
@@ -2755,17 +2755,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-audit-trail — Agent Audit Trail (AAT): Standard Logging Format for Autonomous AI Systems</t>
+          <t>draft-serra-mcp-discovery-uri — The mcp URI Scheme and MCP Server Discovery Mechanism</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining a JSON-based audit record with mandatory fields (agent identity, action classification, outcome tracking, trust level) using RFC 8785 JSON Canonicalization and RFC 9562 UUIDs.</t>
+          <t>An IETF individual draft defining an 'mcp://' URI scheme combined with /.well-known/mcp-server (RFC 8615) and a DNS TXT fallback for discovery of Model Context Protocol servers.</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-audit-trail/</t>
+          <t>https://datatracker.ietf.org/doc/draft-serra-mcp-discovery-uri/</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -2775,7 +2775,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 29 March 2026; orthogonal to delegation but important for compliance — standardized audit-log format is a genuine gap. Complements identity frameworks well. A sibling/alternative to the Kuehlewind audit architecture which takes a far more ambitious cross-layer approach.</t>
+          <t>Already at revision -04 (March 2026), suggesting active iteration; narrow scope, clean design, and the strongest IANA-registration candidate in the set. OAuth 2.1 for auth is deliberately out of scope.</t>
         </is>
       </c>
     </row>
@@ -2785,17 +2785,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>draft-aiendpoint-ai-discovery — The AI Discovery Endpoint</t>
+          <t>draft-sharif-attp — ATTP: Agent Trust Transport Protocol</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining a /.well-known/ai URI suffix for programmatic service capability discovery by AI agents — letting agents discover what an endpoint supports without having to parse human-oriented documentation; requests IANA well-known URI registration.</t>
+          <t>An IETF individual draft defining trust levels L0–L4 mapped to PSD2 Strong Customer Authentication requirements, with bindings for MCP (MCPS), REST, A2A, gRPC, and GraphQL; supersedes draft-sharif-agent-payment-trust.</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-aiendpoint-ai-discovery/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-attp/</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, March 2026; complementary to MCP discovery but broader (not MCP-specific). Needs differentiation from OpenAPI/service-description work to gain traction.</t>
+          <t>Revision -00, April 2026; regulatory mapping appendices (PSD2, PCI DSS) are notable — one of the few drafts engaging financial regulation directly. Ambitious scope. Part of the Sharif cluster.</t>
         </is>
       </c>
     </row>
@@ -2815,17 +2815,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>draft-hood-independent-agtp — Agent Transfer Protocol (AGTP)</t>
+          <t>draft-sharif-agent-transport-protocol — Agent Transport Protocol (ATP): Async Store-and-Forward for AI Agents</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft proposing a dedicated application-layer protocol for AI agent traffic on port 4480 (TCP/TLS and QUIC) with an agtp:// URI scheme, arguing that HTTP is insufficient because agent-generated intent-driven traffic is indistinguishable from human-initiated requests. Defines a Runtime Contract Negotiation Substrate (RCNS) with eighteen methods split into cognitive verbs (QUERY, DISCOVER, DESCRIBE, SUMMARIZE, PLAN, PROPOSE) and mechanics verbs (EXECUTE, DELEGATE, ESCALATE, CONFIRM, SUSPEND, NOTIFY), mandatory agent identity headers, and protocol-level authority scope declaration.</t>
+          <t>An IETF individual draft defining async store-and-forward messaging semantics with cryptographic identity per relay hop, trust scoring at ingress, capability negotiation, and interop with Google A2A, MCP, and FIPA ACL; transport-agnostic over TCP/TLS/QUIC.</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hood-independent-agtp/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-transport-protocol/</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Revision -09, 28 Jun 2026 (was -08 May 2026); supersedes draft-hood-independent-atp. Companion specs in the same family: AGTP-API, AGTP-CERT, AGTP-MERCHANT, AGTP-IDENTIFIERS, AGTP-TRUST. Mandatory TLS 1.3+. Ambitious scope — a new transport layer rather than an HTTP profile. The cognitive/mechanics verb split is a distinctive design choice; contrasts with draft-sharif-agent-transport-protocol which layers async store-and-forward on top of existing transports rather than replacing them.</t>
+          <t>Revision -00, 28 March 2026; addresses a real gap — most agent protocols assume synchronous availability, and store-and-forward is appropriate for long-running agentic tasks. Scope is broad and needs narrowing.</t>
         </is>
       </c>
     </row>
@@ -2845,17 +2845,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>draft-hood-agtp-ard — ARD Binding for AGTP: Agentic Resource Discovery over the Agent Transfer Protocol</t>
+          <t>draft-sharif-agent-audit-trail — Agent Audit Trail (AAT): Standard Logging Format for Autonomous AI Systems</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Specifies how Agentic Resource Discovery (ARD) composes with AGTP, defining a catalog entry type for ARD manifests, aligning AGTP's identity model with ARD's trustManifest, and providing an AGTP-native binding for publishing ARD catalogs over AGTP substrate rather than HTTPS.</t>
+          <t>An IETF individual draft defining a JSON-based audit record with mandatory fields (agent identity, action classification, outcome tracking, trust level) using RFC 8785 JSON Canonicalization and RFC 9562 UUIDs.</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-ard/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-audit-trail/</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -2865,7 +2865,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 18 Jun 2026; author: Chris Hood (Nomotic). Extends the AGTP family (draft-hood-independent-agtp in corpus). The trustManifest identity alignment is the piece relevant to the agent identity thread; the rest is transport-layer plumbing for AGTP deployments.</t>
+          <t>Revision -00, 29 March 2026; orthogonal to delegation but important for compliance — standardized audit-log format is a genuine gap. Complements identity frameworks well. A sibling/alternative to the Kuehlewind audit architecture which takes a far more ambitious cross-layer approach.</t>
         </is>
       </c>
     </row>
@@ -2875,17 +2875,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>draft-hood-agtp-api — AGTP-API: Verbs, Paths, Endpoints, and Synthesis</t>
+          <t>draft-aiendpoint-ai-discovery — The AI Discovery Endpoint</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Establishes the full application-layer contract for AGTP agent–server interactions: approved method catalog, path grammar, endpoint primitives, semantic metadata blocks, server manifests, and runtime contract negotiation substrate. Defines how agents and servers negotiate capabilities and authority before action methods are invoked.</t>
+          <t>An IETF individual draft defining a /.well-known/ai URI suffix for programmatic service capability discovery by AI agents — letting agents discover what an endpoint supports without having to parse human-oriented documentation; requests IANA well-known URI registration.</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-api/</t>
+          <t>https://datatracker.ietf.org/doc/draft-aiendpoint-ai-discovery/</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, May 26 2026; author: Chris Hood (Nomotic). The normative protocol contract layer for AGTP, complementing draft-hood-independent-agtp (transport) and draft-hood-agtp-trust (trust model). The AGTP family now spans 18 drafts; this is the API-layer anchor.</t>
+          <t>Revision -00, March 2026; complementary to MCP discovery but broader (not MCP-specific). Needs differentiation from OpenAPI/service-description work to gain traction.</t>
         </is>
       </c>
     </row>
@@ -2905,17 +2905,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>draft-hood-agtp-trust — AGTP Trust and Verification Specification</t>
+          <t>draft-hood-independent-agtp — Agent Transfer Protocol (AGTP)</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Defines AGTP's three-tier trust model (Tier 1 Verified / Tier 2 Org-Asserted / Tier 3 Experimental) and a continuous behavioral trust score (0.0–1.0) used by infrastructure components for runtime trust-aware routing. Standardizes the evidence substrate, score format, freshness requirements, and consumer-side evaluation rules without mandating the scoring algorithm.</t>
+          <t>An IETF individual draft proposing a dedicated application-layer protocol for AI agent traffic on port 4480 (TCP/TLS and QUIC) with an agtp:// URI scheme, arguing that HTTP is insufficient because agent-generated intent-driven traffic is indistinguishable from human-initiated requests. Defines a Runtime Contract Negotiation Substrate (RCNS) with eighteen methods split into cognitive verbs (QUERY, DISCOVER, DESCRIBE, SUMMARIZE, PLAN, PROPOSE) and mechanics verbs (EXECUTE, DELEGATE, ESCALATE, CONFIRM, SUSPEND, NOTIFY), mandatory agent identity headers, and protocol-level authority scope declaration.</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-trust/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-independent-agtp/</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, Jun 28 2026; author: Chris Hood (Nomotic). The continuous 0.0–1.0 trust score model contrasts with draft-sharif-attp's discrete L0–L4 levels and Larry Lewis's atp-core continuous scoring — three independent designs in the same design space.</t>
+          <t>Revision -09, 28 Jun 2026 (was -08 May 2026); supersedes draft-hood-independent-atp. Companion specs in the same family: AGTP-API, AGTP-CERT, AGTP-MERCHANT, AGTP-IDENTIFIERS, AGTP-TRUST. Mandatory TLS 1.3+. Ambitious scope — a new transport layer rather than an HTTP profile. The cognitive/mechanics verb split is a distinctive design choice; contrasts with draft-sharif-agent-transport-protocol which layers async store-and-forward on top of existing transports rather than replacing them.</t>
         </is>
       </c>
     </row>
@@ -2935,17 +2935,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>draft-hood-agtp-agent-cert — AGTP Agent Certificate Extension</t>
+          <t>draft-hood-agtp-ard — ARD Binding for AGTP: Agentic Resource Discovery over the Agent Transfer Protocol</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Specifies an X.509 v3 extension that cryptographically binds AGTP agent identity headers to TLS mutual authentication, enabling infrastructure components (Scope-Enforcement Points, load balancers, governance gateways) to verify agent identity at the network layer without application-layer access. Includes session-level revocation via AGTP NOTIFY broadcast.</t>
+          <t>Specifies how Agentic Resource Discovery (ARD) composes with AGTP, defining a catalog entry type for ARD manifests, aligning AGTP's identity model with ARD's trustManifest, and providing an AGTP-native binding for publishing ARD catalogs over AGTP substrate rather than HTTPS.</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-agent-cert/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-ard/</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>Revision -03, Jun 28 2026; author: Chris Hood (Nomotic). The PKI-binding companion to the AGTP identity model; positions AGTP agent identity within existing X.509 / TLS infrastructure. Relevant to WebBotAuth comparison — both use PKI for bot/agent identity but at different layers.</t>
+          <t>Revision -00, 18 Jun 2026; author: Chris Hood (Nomotic). Extends the AGTP family (draft-hood-independent-agtp in corpus). The trustManifest identity alignment is the piece relevant to the agent identity thread; the rest is transport-layer plumbing for AGTP deployments.</t>
         </is>
       </c>
     </row>
@@ -2965,17 +2965,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>draft-jernalczyk-intentweb-agent-manifest — IntentWeb AgentManifest</t>
+          <t>draft-hood-agtp-api — AGTP-API: Verbs, Paths, Endpoints, and Synthesis</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Defines a JSON document that websites publish to describe identity, trusted knowledge, agent-facing capabilities, structured bindings, risk levels, consent requirements, authentication expectations, audit rules, and policies — enabling AI agents to comprehend website functionality and safely perform actions without scraping or fragile UI automation.</t>
+          <t>Establishes the full application-layer contract for AGTP agent–server interactions: approved method catalog, path grammar, endpoint primitives, semantic metadata blocks, server manifests, and runtime contract negotiation substrate. Defines how agents and servers negotiate capabilities and authority before action methods are invoked.</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jernalczyk-intentweb-agent-manifest/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-api/</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 6 Jul 2026; author: Mariusz Jernalczyk (IntentWeb). Website-side complement to agent identity drafts; sits in the Discovery &amp; Transport cluster alongside draft-hood-agtp-ard and the DAWN/.well-known discovery thread. Single author, no-affiliation submission — early stage but addresses a real discovery gap.</t>
+          <t>Revision -01, May 26 2026; author: Chris Hood (Nomotic). The normative protocol contract layer for AGTP, complementing draft-hood-independent-agtp (transport) and draft-hood-agtp-trust (trust model). The AGTP family now spans 18 drafts; this is the API-layer anchor.</t>
         </is>
       </c>
     </row>
@@ -2995,17 +2995,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>draft-fane-opena2a-aap — OpenA2A Agent Authorization Protocol (AAP)</t>
+          <t>draft-hood-agtp-trust — AGTP Trust and Verification Specification</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Establishes authorization mechanisms for AI agent systems through cryptographic identity assertions and scoped capability grants. Introduces a broker layer that separates credentials from the agent's reasoning context, specifically to prevent prompt injection attacks from leaking authorization state while enabling cross-agent delegation.</t>
+          <t>Defines AGTP's three-tier trust model (Tier 1 Verified / Tier 2 Org-Asserted / Tier 3 Experimental) and a continuous behavioral trust score (0.0–1.0) used by infrastructure components for runtime trust-aware routing. Standardizes the evidence substrate, score format, freshness requirements, and consumer-side evaluation rules without mandating the scoring algorithm.</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-fane-opena2a-aap/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-trust/</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, Jul 6 2026; author: Abdel Fane (OpenA2A). Filed Jul 6 alongside a companion draft-fane-opena2a-aip which adds a fourth 'AIP' name collision to the existing Singla/Prakash/aip-agent-identity-protocol triple. The AAP authorization layer is the piece most relevant to OAuth boundary analysis.</t>
+          <t>Revision -02, Jun 28 2026; author: Chris Hood (Nomotic). The continuous 0.0–1.0 trust score model contrasts with draft-sharif-attp's discrete L0–L4 levels and Larry Lewis's atp-core continuous scoring — three independent designs in the same design space.</t>
         </is>
       </c>
     </row>
@@ -3025,17 +3025,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>draft-ni-a2a-ai-agent-security-requirements — Security Requirements for AI Agents</t>
+          <t>draft-hood-agtp-agent-cert — AGTP Agent Certificate Extension</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft enumerating security requirements for AI agents, covering identity, authorization chaining across domains, and integration points with WIMSE, OAuth identity chaining, and the A2A OAuth profile.</t>
+          <t>Specifies an X.509 v3 extension that cryptographically binds AGTP agent identity headers to TLS mutual authentication, enabling infrastructure components (Scope-Enforcement Points, load balancers, governance gateways) to verify agent identity at the network layer without application-layer access. Includes session-level revocation via AGTP NOTIFY broadcast.</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-ni-a2a-ai-agent-security-requirements/</t>
+          <t>https://datatracker.ietf.org/doc/draft-hood-agtp-agent-cert/</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, February 2026; essential scaffolding for an eventual AI-agent WG. Well-connected to existing IETF work and authored by Ni and Liu, who also lead the WIMSE AI-agent identity draft.</t>
+          <t>Revision -03, Jun 28 2026; author: Chris Hood (Nomotic). The PKI-binding companion to the AGTP identity model; positions AGTP agent identity within existing X.509 / TLS infrastructure. Relevant to WebBotAuth comparison — both use PKI for bot/agent identity but at different layers.</t>
         </is>
       </c>
     </row>
@@ -3055,17 +3055,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>draft-rosenberg-aiproto-framework — Framework, Use Cases and Requirements for AI Agent Protocols</t>
+          <t>draft-jernalczyk-intentweb-agent-manifest — IntentWeb AgentManifest</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft providing a comprehensive AI-agent communications framework that covers user↔agent, agent↔API, and agent↔agent interactions; surveys MCP, A2A, and Agntcy; and sets the stage for IETF standards activity.</t>
+          <t>Defines a JSON document that websites publish to describe identity, trusted knowledge, agent-facing capabilities, structured bindings, risk levels, consent requirements, authentication expectations, audit rules, and policies — enabling AI agents to comprehend website functionality and safely perform actions without scraping or fragile UI automation.</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-framework/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jernalczyk-intentweb-agent-manifest/</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -3075,7 +3075,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, October 2025; Rosenberg (Five9) and Jennings (Cisco) are credible long-time IETF contributors. Important landscape document but likely expired (April 2026); watch for a -01 refresh post-IETF 123.</t>
+          <t>Revision -00, 6 Jul 2026; author: Mariusz Jernalczyk (IntentWeb). Website-side complement to agent identity drafts; sits in the Discovery &amp; Transport cluster alongside draft-hood-agtp-ard and the DAWN/.well-known discovery thread. Single author, no-affiliation submission — early stage but addresses a real discovery gap.</t>
         </is>
       </c>
     </row>
@@ -3085,17 +3085,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>draft-rosenberg-aiproto-cheq — CHEQ: A Protocol for Confirmation of AI Agent Decisions (HITL)</t>
+          <t>draft-bu-agentproto-security-principal-binding — Security Principal and Verifier Binding for Agent Communication Protocols</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft defining an out-of-band Human-in-the-Loop confirmation protocol for agent tool calls, eliminating LLM-hallucination risk for consequential actions and enabling sensitive operations (e.g., banking) without exposing data to the agent.</t>
+          <t>Addresses how agent communication protocols carry claims about user authority, agent instance identity, tool or external-resource identity, delegation state, session continuity, and action evidence; each claim has a different verifier, freshness requirement, failure mode, and security consequence, requiring explicit binding rather than collapsing all claims into a single assertion.</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-cheq/</t>
+          <t>https://datatracker.ietf.org/doc/draft-bu-agentproto-security-principal-binding/</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, October 2025; out-of-band HITL confirmation model is valuable and complements delegation frameworks. Likely expired (April 2026); worth tracking for a -01 refresh.</t>
+          <t>Revision -02, Jul 2026. Fills a gap in the AGTP family (draft-hood-independent-agtp in corpus) and is relevant to any agent communication protocol carrying mixed-provenance claims. The verifier-separation model is the missing security architecture layer between protocol transport and authorization enforcement.</t>
         </is>
       </c>
     </row>
@@ -3115,27 +3115,27 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>draft-sharif-agent-payment-trust — Trust Scoring and Identity Verification for AI Agent Payment Transactions (SUPERSEDED)</t>
+          <t>draft-fane-opena2a-aap — OpenA2A Agent Authorization Protocol (AAP)</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft introducing an Agent Passport — a cryptographic delegation certificate intended to serve as the PSD2 'something you have' factor — and a trust-scoring model for payment transactions mapped to PCI DSS v4.0.1.</t>
+          <t>Establishes authorization mechanisms for AI agent systems through cryptographic identity assertions and scoped capability grants. Introduces a broker layer that separates credentials from the agent's reasoning context, specifically to prevent prompt injection attacks from leaking authorization state while enabling cross-agent delegation.</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-payment-trust/</t>
+          <t>https://datatracker.ietf.org/doc/draft-fane-opena2a-aap/</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual, superseded)</t>
+          <t>IETF (individual)</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>SUPERSEDED by draft-sharif-attp-00 (April 2026). Retained for historical context — the Agent Passport concept is interesting but needs formal grounding; the ATTP successor generalizes it across transport bindings.</t>
+          <t>Revision -00, Jul 6 2026; author: Abdel Fane (OpenA2A). Filed Jul 6 alongside a companion draft-fane-opena2a-aip which adds a fourth 'AIP' name collision to the existing Singla/Prakash/aip-agent-identity-protocol triple. The AAP authorization layer is the piece most relevant to OAuth boundary analysis.</t>
         </is>
       </c>
     </row>
@@ -3145,17 +3145,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>draft-stephan-ai-agent-6g — AI Agent Protocols for 6G Systems</t>
+          <t>draft-ni-a2a-ai-agent-security-requirements — Security Requirements for AI Agents</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft translating use cases and service requirements from 3GPP TR 22.870 into IETF agent-protocol requirements, covering autonomous vehicles, privacy preservation, and anomaly detection.</t>
+          <t>An IETF individual draft enumerating security requirements for AI agents, covering identity, authorization chaining across domains, and integration points with WIMSE, OAuth identity chaining, and the A2A OAuth profile.</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-stephan-ai-agent-6g/</t>
+          <t>https://datatracker.ietf.org/doc/draft-ni-a2a-ai-agent-security-requirements/</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, October 2025; strong operator backing (Orange, Deutsche Telekom, Telefonica, China Mobile, Huawei). Requirements-oriented and important for 3GPP/IETF coordination. May be expired (April 2026); watch for an update.</t>
+          <t>Revision -01, February 2026; essential scaffolding for an eventual AI-agent WG. Well-connected to existing IETF work and authored by Ni and Liu, who also lead the WIMSE AI-agent identity draft.</t>
         </is>
       </c>
     </row>
@@ -3175,17 +3175,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>draft-jimenez-t2trg-iot-agent — Agentic AI Operation of Constrained RESTful Environments</t>
+          <t>draft-rosenberg-aiproto-framework — Framework, Use Cases and Requirements for AI Agent Protocols</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft (T2TRG affiliated) describing agentic AI (ReAct, smolagents) operating on CoAP/CoRE constrained-IoT environments, with a reference implementation provided.</t>
+          <t>An IETF individual draft providing a comprehensive AI-agent communications framework that covers user↔agent, agent↔API, and agent↔agent interactions; surveys MCP, A2A, and Agntcy; and sets the stage for IETF standards activity.</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jimenez-t2trg-iot-agent/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-framework/</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 14 April 2026; unique in targeting constrained IoT environments. T2TRG affiliation and reference implementation are positive signals. Niche but fills an unaddressed gap.</t>
+          <t>Revision -00, October 2025; Rosenberg (Five9) and Jennings (Cisco) are credible long-time IETF contributors. Important landscape document but likely expired (April 2026); watch for a -01 refresh post-IETF 123.</t>
         </is>
       </c>
     </row>
@@ -3205,17 +3205,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>draft-li-oauth-delegated-authorization — OAuth 2.0 Delegated Authorization</t>
+          <t>draft-rosenberg-aiproto-cheq — CHEQ: A Protocol for Confirmation of AI Agent Decisions (HITL)</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Huawei authors that extends OAuth 2.0 with a hierarchical 'delegation token' model so a client can mint subordinate, narrowly-scoped access tokens for delegated parties.</t>
+          <t>An IETF individual draft defining an out-of-band Human-in-the-Loop confirmation protocol for agent tool calls, eliminating LLM-hallucination risk for consequential actions and enabling sensitive operations (e.g., banking) without exposing data to the agent.</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-li-oauth-delegated-authorization/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rosenberg-aiproto-cheq/</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, March 2026 (Informational); directly addresses over-privileged tokens and is one of the few drafts using the literal term 'delegated authorization'.</t>
+          <t>Revision -00, October 2025; out-of-band HITL confirmation model is valuable and complements delegation frameworks. Likely expired (April 2026); worth tracking for a -01 refresh.</t>
         </is>
       </c>
     </row>
@@ -3235,27 +3235,27 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>draft-araut-oauth-transaction-tokens-for-agents — Transaction Tokens For Agents</t>
+          <t>draft-sharif-agent-payment-trust — Trust Scoring and Identity Verification for AI Agent Payment Transactions (SUPERSEDED)</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft from Ashay Raut (Amazon) profiling Transaction Tokens for agent-based workflows by adding 'act' for the agent identity, an 'agentic_ctx' claim carrying agent_type/intent/allowed_actions/environment_constraints, RFC 9396 RAR integration, and an 'actchain' claim for multi-agent delegation lineage.</t>
+          <t>An IETF individual draft introducing an Agent Passport — a cryptographic delegation certificate intended to serve as the PSD2 'something you have' factor — and a trust-scoring model for payment transactions mapped to PCI DSS v4.0.1.</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-araut-oauth-transaction-tokens-for-agents/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sharif-agent-payment-trust/</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>IETF (individual)</t>
+          <t>IETF (individual, superseded)</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>Revision -01 (May 2026) under the new slug — re-slugged from draft-oauth-transaction-tokens-for-agents-06; the -06 added the actchain delegation lineage, RAR-driven agentic_ctx, and a TTS check that blocks chain-splicing attacks. Conservative extension of the WG Transaction Tokens draft and an easier path to standardization.</t>
+          <t>SUPERSEDED by draft-sharif-attp-00 (April 2026). Retained for historical context — the Agent Passport concept is interesting but needs formal grounding; the ATTP successor generalizes it across transport bindings.</t>
         </is>
       </c>
     </row>
@@ -3265,17 +3265,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>draft-oauth-ai-agents-on-behalf-of-user — On-Behalf-Of User Authorization for AI Agents</t>
+          <t>draft-stephan-ai-agent-6g — AI Agent Protocols for 6G Systems</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>An IETF individual draft adding requested_actor and actor_token parameters to the OAuth authorization-code flow so the user gives explicit consent per agent, with the resulting delegation chain documented in the access-token claims.</t>
+          <t>An IETF individual draft translating use cases and service requirements from 3GPP TR 22.870 into IETF agent-protocol requirements, covering autonomous vehicles, privacy preservation, and anomaly detection.</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-oauth-ai-agents-on-behalf-of-user/</t>
+          <t>https://datatracker.ietf.org/doc/draft-stephan-ai-agent-6g/</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Revision -02 was submitted August 2025; likely due for -03 refresh. Builds naturally on RFC 6749 + RFC 8693 + RFC 7636 PKCE — one of the most 'IETF-ready' delegation drafts and a strong WG-adoption candidate after the OAuth recharter.</t>
+          <t>Revision -02, October 2025; strong operator backing (Orange, Deutsche Telekom, Telefonica, China Mobile, Huawei). Requirements-oriented and important for 3GPP/IETF coordination. May be expired (April 2026); watch for an update.</t>
         </is>
       </c>
     </row>
@@ -3295,17 +3295,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>draft-rosomakho-oauth-txn-challenge — OAuth Transaction Authorization Challenge</t>
+          <t>draft-jimenez-t2trg-iot-agent — Agentic AI Operation of Constrained RESTful Environments</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>An OAuth mechanism enabling protected resources to demand transaction-specific authorization through challenges. When a request involves an agent or automated workflow, the RS returns a challenge to the client; the client presents it to the AS, which validates it, obtains human approval, and issues an access token with RFC 9396 authorization_details describing the approved operation. Positions as complementary to RFC 9470 (Step-Up Authentication) — that spec handles authentication freshness; this one handles authorization specificity.</t>
+          <t>An IETF individual draft (T2TRG affiliated) describing agentic AI (ReAct, smolagents) operating on CoAP/CoRE constrained-IoT environments, with a reference implementation provided.</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rosomakho-oauth-txn-challenge/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jimenez-t2trg-iot-agent/</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, submitted 25 June 2026. Authors: Yaroslav Rosomakho (Zscaler), Brian Campbell (Ping Identity), Karl McGuinness (Independent), Pieter Kasselman (Defakto). Strong author lineup — Campbell is a prolific OAuth WG contributor, Kasselman co-authored Transaction Tokens and First-Party Apps, McGuinness brings the Mission-Bound OAuth context. The RS-initiated challenge model is distinct from ARAP (which operates at the PDP/PEP layer via AuthZEN) but addresses the same 'denial is not the end' problem — here at the OAuth RS/AS layer rather than the AuthZEN layer.</t>
+          <t>Revision -00, 14 April 2026; unique in targeting constrained IoT environments. T2TRG affiliation and reference implementation are positive signals. Niche but fills an unaddressed gap.</t>
         </is>
       </c>
     </row>
@@ -3325,17 +3325,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>draft-lee-orprg-permit-receipts — Permit Receipts for Permit-Before-Commit Authorization</t>
+          <t>draft-li-oauth-delegated-authorization — OAuth 2.0 Delegated Authorization</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Defines requirements and an abstract data model for PermitReceipts: a verifier evaluates canonicalized effect requests, action digests, policy epochs, validity intervals, and revocation status before any protected effect is committed at an effect boundary. Covers verifier behavior, failure semantics, and candidate registries.</t>
+          <t>An IETF individual draft from Huawei authors that extends OAuth 2.0 with a hierarchical 'delegation token' model so a client can mint subordinate, narrowly-scoped access tokens for delegated parties.</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-lee-orprg-permit-receipts/</t>
+          <t>https://datatracker.ietf.org/doc/draft-li-oauth-delegated-authorization/</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 4 Jun 2026; author: Yong Bok Lee (Meridian Verity Group). The most complete standalone framework for pre-commit authorization in the current wave; intended to ground IETF discussion on scope and profiles. Seeks guidance on appropriate organizational placement.</t>
+          <t>Revision -01, March 2026 (Informational); directly addresses over-privileged tokens and is one of the few drafts using the literal term 'delegated authorization'.</t>
         </is>
       </c>
     </row>
@@ -3355,17 +3355,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>draft-nelson-agent-delegation-receipts — Delegation Receipt Protocol for AI Agent Authorization</t>
+          <t>draft-araut-oauth-transaction-tokens-for-agents — Transaction Tokens For Agents</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Specifies the Delegation Receipt Protocol (DRP) where users sign Authorization Objects (containing scope boundaries, time constraints, instruction hashes, and model state commitments) that are published to an append-only log before the agent runtime gains control. Removes operators as trusted intermediaries by making the user's private key the sole signing authority.</t>
+          <t>An IETF individual draft from Ashay Raut (Amazon) profiling Transaction Tokens for agent-based workflows by adding 'act' for the agent identity, an 'agentic_ctx' claim carrying agent_type/intent/allowed_actions/environment_constraints, RFC 9396 RAR integration, and an 'actchain' claim for multi-agent delegation lineage.</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-nelson-agent-delegation-receipts/</t>
+          <t>https://datatracker.ietf.org/doc/draft-araut-oauth-transaction-tokens-for-agents/</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -3375,7 +3375,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>Revision -10, 13 Jun 2026; author: Ryan Nelson (Authproof). At version 10, the most iterated individual draft in the pre-action authorization space. The commitment-before-execution architecture — sign before the agent runs, not after — is distinctive and directly addresses the prompt-injection attack surface.</t>
+          <t>Revision -01 (May 2026) under the new slug — re-slugged from draft-oauth-transaction-tokens-for-agents-06; the -06 added the actchain delegation lineage, RAR-driven agentic_ctx, and a TTS check that blocks chain-splicing attacks. Conservative extension of the WG Transaction Tokens draft and an easier path to standardization.</t>
         </is>
       </c>
     </row>
@@ -3385,17 +3385,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>draft-williams-intent-token — The Intent Token: A Cryptographic Authorization Primitive for Autonomous Agents</t>
+          <t>draft-oauth-ai-agents-on-behalf-of-user — On-Behalf-Of User Authorization for AI Agents</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Specifies a cryptographic authorization primitive that binds an autonomous agent action to a cryptographically signed, human-declared authorization envelope before execution. Addresses the gap in OAuth 2.0 frameworks that govern access to resources but not what agents are permitted to do at the moment of action. Positioned as complementary to OAuth, not a replacement.</t>
+          <t>An IETF individual draft adding requested_actor and actor_token parameters to the OAuth authorization-code flow so the user gives explicit consent per agent, with the resulting delegation chain documented in the access-token claims.</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-williams-intent-token/</t>
+          <t>https://datatracker.ietf.org/doc/draft-oauth-ai-agents-on-behalf-of-user/</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -3405,7 +3405,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 22 Jun 2026; author: Jeffrey Williams (Independent). Overlaps conceptually with draft-kroehl-agentic-trust-aae and draft-nelson-agent-delegation-receipts; worth tracking as a lighter-weight alternative to both.</t>
+          <t>Revision -02 was submitted August 2025; likely due for -03 refresh. Builds naturally on RFC 6749 + RFC 8693 + RFC 7636 PKCE — one of the most 'IETF-ready' delegation drafts and a strong WG-adoption candidate after the OAuth recharter.</t>
         </is>
       </c>
     </row>
@@ -3415,17 +3415,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>draft-pereira-licet-human-intent — LICET: Multi-Modal Physiological Human-Intent Verification for Autonomous AI Agent Authorization</t>
+          <t>draft-rosomakho-oauth-txn-challenge — OAuth Transaction Authorization Challenge</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Proposes a biometric HITL protocol fusing ECG, electrodermal activity, and Mahalanobis statistical distance to cryptographically verify genuine human intent — not just credential possession — before authorizing autonomous AI agent actions, with ZK proofs enabling third-party audit without exposing raw biometric data.</t>
+          <t>An OAuth mechanism enabling protected resources to demand transaction-specific authorization through challenges. When a request involves an agent or automated workflow, the RS returns a challenge to the client; the client presents it to the AS, which validates it, obtains human approval, and issues an access token with RFC 9396 authorization_details describing the approved operation. Positions as complementary to RFC 9470 (Step-Up Authentication) — that spec handles authentication freshness; this one handles authorization specificity.</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-pereira-licet-human-intent/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rosomakho-oauth-txn-challenge/</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -3435,7 +3435,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 2 Jul 2026. The most novel and technically niche HITL proposal in the current wave — complements draft-rosenberg-aiproto-cheq (out-of-band HITL confirmation) and draft-sato-soos-hem (kernel-enforced escalation) by grounding human intent in physiological signal rather than credential or UI interaction.</t>
+          <t>Revision -00, submitted 25 June 2026. Authors: Yaroslav Rosomakho (Zscaler), Brian Campbell (Ping Identity), Karl McGuinness (Independent), Pieter Kasselman (Defakto). Strong author lineup — Campbell is a prolific OAuth WG contributor, Kasselman co-authored Transaction Tokens and First-Party Apps, McGuinness brings the Mission-Bound OAuth context. The RS-initiated challenge model is distinct from ARAP (which operates at the PDP/PEP layer via AuthZEN) but addresses the same 'denial is not the end' problem — here at the OAuth RS/AS layer rather than the AuthZEN layer.</t>
         </is>
       </c>
     </row>
@@ -3445,17 +3445,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>draft-reece-wimse-cross-org-delegation — Cross-Organizational Delegation for Workload and Agent Identity</t>
+          <t>draft-lee-orprg-permit-receipts — Permit Receipts for Permit-Before-Commit Authorization</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>A problem statement and requirements draft identifying that existing workload and token-based authorization mechanisms were designed for a single trust domain, describing the cross-organizational agent delegation gap, and enumerating requirements for solutions — without proposing specific technical approaches.</t>
+          <t>Defines requirements and an abstract data model for PermitReceipts: a verifier evaluates canonicalized effect requests, action digests, policy epochs, validity intervals, and revocation status before any protected effect is committed at an effect boundary. Covers verifier behavior, failure semantics, and candidate registries.</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-reece-wimse-cross-org-delegation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-lee-orprg-permit-receipts/</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 25 Jun 2026; author: Morgan Reece (TowerGuardian Consulting). The problem-statement companion to the corpus's operational drafts; likely to feed into WIMSE WG scope expansion and is directly in scope for draft-kuehlewind-audit-architecture's composition graph.</t>
+          <t>Revision -00, 4 Jun 2026; author: Yong Bok Lee (Meridian Verity Group). The most complete standalone framework for pre-commit authorization in the current wave; intended to ground IETF discussion on scope and profiles. Seeks guidance on appropriate organizational placement.</t>
         </is>
       </c>
     </row>
@@ -3475,17 +3475,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>draft-jiang-wimse-heterogeneous-credential — Heterogeneous Credential Verification for Workload and Agentic Systems</t>
+          <t>draft-nelson-agent-delegation-receipts — Delegation Receipt Protocol for AI Agent Authorization</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Specifies mechanisms for representing credential sets, identifying credential types, determining appropriate verifiers, normalizing verification results across different formats (workload tokens, OAuth, X.509, attestation), and combining results into a single handling decision.</t>
+          <t>Specifies the Delegation Receipt Protocol (DRP) where users sign Authorization Objects (containing scope boundaries, time constraints, instruction hashes, and model state commitments) that are published to an append-only log before the agent runtime gains control. Removes operators as trusted intermediaries by making the user's private key the sole signing authority.</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jiang-wimse-heterogeneous-credential/</t>
+          <t>https://datatracker.ietf.org/doc/draft-nelson-agent-delegation-receipts/</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -3495,7 +3495,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 30 Jun 2026 (was -00 Jun 2026); authors: Yuning Jiang, Donghui Wang, Yurong Song, Faye Liu (Huawei). Solves the practical problem of agentic systems receiving credentials in multiple formats from different issuers. Fills a gap left by draft-ni-wimse-ai-agent-identity (corpus) which describes the identity problem but not multi-format credential handling.</t>
+          <t>Revision -10, 13 Jun 2026; author: Ryan Nelson (Authproof). At version 10, the most iterated individual draft in the pre-action authorization space. The commitment-before-execution architecture — sign before the agent runs, not after — is distinctive and directly addresses the prompt-injection attack surface.</t>
         </is>
       </c>
     </row>
@@ -3505,17 +3505,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>draft-munoz-wimse-authorization-evidence — Signed Authorization-Evidence Records for WIMSE-Authorized AI Agent Actions</t>
+          <t>draft-williams-intent-token — The Intent Token: A Cryptographic Authorization Primitive for Autonomous Agents</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Specifies a signed authorization-evidence record (Permit) for WIMSE-authorized AI actions, cryptographically binding to the dispatched request bytes via HTTP Message Signatures, OAuth access tokens, and Shared Signals Framework eventing — without modifying existing standards.</t>
+          <t>Specifies a cryptographic authorization primitive that binds an autonomous agent action to a cryptographically signed, human-declared authorization envelope before execution. Addresses the gap in OAuth 2.0 frameworks that govern access to resources but not what agents are permitted to do at the moment of action. Positioned as complementary to OAuth, not a replacement.</t>
         </is>
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-munoz-wimse-authorization-evidence/</t>
+          <t>https://datatracker.ietf.org/doc/draft-williams-intent-token/</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -3525,7 +3525,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 15 May 2026; author: Christian Munoz (Keel API). Profiles WIMSE for AI agent actions and satisfies audit requirements; companion to the SCITT permit profile below. Extends the corpus WIMSE thread (draft-ni-wimse-ai-agent-identity) with a concrete evidence artifact.</t>
+          <t>Revision -01, 22 Jun 2026; author: Jeffrey Williams (Independent). Overlaps conceptually with draft-kroehl-agentic-trust-aae and draft-nelson-agent-delegation-receipts; worth tracking as a lighter-weight alternative to both.</t>
         </is>
       </c>
     </row>
@@ -3535,17 +3535,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>draft-schwenkschuster-wimse-trust-domain-discovery — WIMSE Trust Domain Discovery</t>
+          <t>draft-pereira-licet-human-intent — LICET: Multi-Modal Physiological Human-Intent Verification for Autonomous AI Agent Authorization</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Fills a gap in the WIMSE architecture by defining how relying parties obtain cryptographic trust anchors for workload identity credentials; specifies the WIMSE Trust Bundle (a JSON document with freshness metadata) and a well-known HTTPS discovery endpoint resolving trust domain names to their trust bundles, following OpenID Connect Discovery / OAuth 2.0 patterns.</t>
+          <t>Proposes a biometric HITL protocol fusing ECG, electrodermal activity, and Mahalanobis statistical distance to cryptographically verify genuine human intent — not just credential possession — before authorizing autonomous AI agent actions, with ZK proofs enabling third-party audit without exposing raw biometric data.</t>
         </is>
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-schwenkschuster-wimse-trust-domain-discovery/</t>
+          <t>https://datatracker.ietf.org/doc/draft-pereira-licet-human-intent/</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 3 Jul 2026; authors: Arndt Schwenkschuster (Defakto Security), Yaroslav Rosomakho (Zscaler). Directly complements draft-schwenkschuster-wimse-credential-exchange (corpus). The kuehlewind-audit-architecture HUB assumes resolvable trust anchors — this provides the discovery mechanism. Rosomakho co-authorship ties it to draft-rosomakho-oauth-txn-challenge.</t>
+          <t>Revision -01, 2 Jul 2026. The most novel and technically niche HITL proposal in the current wave — complements draft-rosenberg-aiproto-cheq (out-of-band HITL confirmation) and draft-sato-soos-hem (kernel-enforced escalation) by grounding human intent in physiological signal rather than credential or UI interaction.</t>
         </is>
       </c>
     </row>
@@ -3565,17 +3565,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>draft-winmagic-wimse-condition-bounded-credentials — Condition-Bounded Credentials for Workload and Agent Identity</t>
+          <t>draft-reece-wimse-cross-org-delegation — Cross-Organizational Delegation for Workload and Agent Identity</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Proposes hardware-rooted, non-exfiltratable workload credentials whose validity is conditioned on attested runtime posture rather than expiration time — so a credential becomes invalid if the workload's attestation evidence degrades, regardless of the stated expiry.</t>
+          <t>A problem statement and requirements draft identifying that existing workload and token-based authorization mechanisms were designed for a single trust domain, describing the cross-organizational agent delegation gap, and enumerating requirements for solutions — without proposing specific technical approaches.</t>
         </is>
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-winmagic-wimse-condition-bounded-credentials/</t>
+          <t>https://datatracker.ietf.org/doc/draft-reece-wimse-cross-org-delegation/</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -3585,7 +3585,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 6 Jul 2026; author: WinMagic. Extends the WIMSE credential model with posture-conditioned validity — distinct from time-bounded credentials in that security policy changes at the hardware/attestation layer instantly invalidate the credential. Bridges the RATS attestation thread and the WIMSE identity thread in the corpus.</t>
+          <t>Revision -00, 25 Jun 2026; author: Morgan Reece (TowerGuardian Consulting). The problem-statement companion to the corpus's operational drafts; likely to feed into WIMSE WG scope expansion and is directly in scope for draft-kuehlewind-audit-architecture's composition graph.</t>
         </is>
       </c>
     </row>
@@ -3595,17 +3595,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>draft-munoz-scitt-permit-profile — A SCITT Profile for Pre-Execution AI Action Authorization Records</t>
+          <t>draft-jiang-wimse-heterogeneous-credential — Heterogeneous Credential Verification for Workload and Agentic Systems</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>SCITT profile for the Pre-Execution Authorization Record (Permit), documenting policy-evaluated decisions before AI agent action dispatch with cryptographic binding proving 'authorized request equals dispatched request.' Composes with adjacent profiles for human-authority binding, post-execution evidence, and content-refusal events via referencing mechanisms.</t>
+          <t>Specifies mechanisms for representing credential sets, identifying credential types, determining appropriate verifiers, normalizing verification results across different formats (workload tokens, OAuth, X.509, attestation), and combining results into a single handling decision.</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-munoz-scitt-permit-profile/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jiang-wimse-heterogeneous-credential/</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 15 May 2026; author: Christian Munoz (Keel API). SCITT-anchored analog of the WIMSE evidence record; companion to draft-munoz-wimse-authorization-evidence from the same author. Connects to draft-sharif-agent-audit-trail and draft-kuehlewind-audit-architecture (both in corpus).</t>
+          <t>Revision -01, 30 Jun 2026 (was -00 Jun 2026); authors: Yuning Jiang, Donghui Wang, Yurong Song, Faye Liu (Huawei). Solves the practical problem of agentic systems receiving credentials in multiple formats from different issuers. Fills a gap left by draft-ni-wimse-ai-agent-identity (corpus) which describes the identity problem but not multi-format credential handling.</t>
         </is>
       </c>
     </row>
@@ -3625,17 +3625,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>draft-marques-asqav-compliance-receipts — Compliance Profile of Signed Action Receipts for AI Agents</t>
+          <t>draft-munoz-wimse-authorization-evidence — Signed Authorization-Evidence Records for WIMSE-Authorized AI Agent Actions</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Establishes a compliance framework for signed action receipts from AI agents, mandating specific fields, cryptographic anchoring, hash-chain linkage, risk/incident classification, cross-agent envelope binding, and enforcement attestation with retention floors tied to EU AI Act, DORA, NIST AI RMF, HIPAA, SEC Rule 17a-4, and CIRCIA.</t>
+          <t>Specifies a signed authorization-evidence record (Permit) for WIMSE-authorized AI actions, cryptographically binding to the dispatched request bytes via HTTP Message Signatures, OAuth access tokens, and Shared Signals Framework eventing — without modifying existing standards.</t>
         </is>
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-marques-asqav-compliance-receipts/</t>
+          <t>https://datatracker.ietf.org/doc/draft-munoz-wimse-authorization-evidence/</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -3645,7 +3645,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>Revision -06, 1 Jul 2026 (was -05 May 2026); author: João André Gomes Marques. The most legally grounded receipt profile in the wave — at revision 06, relatively mature. Complements draft-sharif-agent-audit-trail (corpus) with a multi-regulation compliance overlay.</t>
+          <t>Revision -00, 15 May 2026; author: Christian Munoz (Keel API). Profiles WIMSE for AI agent actions and satisfies audit requirements; companion to the SCITT permit profile below. Extends the corpus WIMSE thread (draft-ni-wimse-ai-agent-identity) with a concrete evidence artifact.</t>
         </is>
       </c>
     </row>
@@ -3655,17 +3655,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>draft-mih-scitt-agent-action-capsule — An Agent Action Capsule Profile for SCITT</t>
+          <t>draft-schwenkschuster-wimse-trust-domain-discovery — WIMSE Trust Domain Discovery</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>Defines a SCITT statement profile (Agent Action Capsule) documenting agent actions with outcome status (executed, blocked, denied, errored, timed out), evaluated constraints, committed-effect binding, and a human-in-the-loop flag; records a Capsule for every verdict including refusals. COSE Signed Statement format; registrable in SCITT Transparency Services.</t>
+          <t>Fills a gap in the WIMSE architecture by defining how relying parties obtain cryptographic trust anchors for workload identity credentials; specifies the WIMSE Trust Bundle (a JSON document with freshness metadata) and a well-known HTTPS discovery endpoint resolving trust domain names to their trust bundles, following OpenID Connect Discovery / OAuth 2.0 patterns.</t>
         </is>
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mih-scitt-agent-action-capsule/</t>
+          <t>https://datatracker.ietf.org/doc/draft-schwenkschuster-wimse-trust-domain-discovery/</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, 6 Jul 2026 (was -01 Jun 2026); author: Steven Mih (Action State Group). -02 added an 'honest human-in-the-loop' flag distinguishing actual HITL from automated policy. Provides auditor-grade evidence that decision gates functioned; the HITL flag directly tracks the corpus theme.</t>
+          <t>Revision -00, 3 Jul 2026; authors: Arndt Schwenkschuster (Defakto Security), Yaroslav Rosomakho (Zscaler). Directly complements draft-schwenkschuster-wimse-credential-exchange (corpus). The kuehlewind-audit-architecture HUB assumes resolvable trust anchors — this provides the discovery mechanism. Rosomakho co-authorship ties it to draft-rosomakho-oauth-txn-challenge.</t>
         </is>
       </c>
     </row>
@@ -3685,17 +3685,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>draft-car-rer-artifact — RER Run Artifact Format: Hash-Chained, Signed Records of AI Inference Execution</t>
+          <t>draft-winmagic-wimse-condition-bounded-credentials — Condition-Bounded Credentials for Workload and Agent Identity</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Specifies a cryptographically signed JSON record for AI inference runs including a signed envelope declaring permissions and limits, a hash-chained event log covering all model and tool calls, and a runtime signature binding envelope and log to the producing implementation. Enables offline verification by parties uninvolved in the original run.</t>
+          <t>Proposes hardware-rooted, non-exfiltratable workload credentials whose validity is conditioned on attested runtime posture rather than expiration time — so a credential becomes invalid if the workload's attestation evidence degrades, regardless of the stated expiry.</t>
         </is>
       </c>
       <c r="D93" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-car-rer-artifact/</t>
+          <t>https://datatracker.ietf.org/doc/draft-winmagic-wimse-condition-bounded-credentials/</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -3705,7 +3705,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 12 Jun 2026; author: Kayla Cardillo (Tech Enrichment). Relevant for post-hoc audit of what permissions an agent claimed during execution; companion to the SCITT profiles but more focused on inference traceability than authorization decisions.</t>
+          <t>Revision -01, 6 Jul 2026; author: WinMagic. Extends the WIMSE credential model with posture-conditioned validity — distinct from time-bounded credentials in that security policy changes at the hardware/attestation layer instantly invalidate the credential. Bridges the RATS attestation thread and the WIMSE identity thread in the corpus.</t>
         </is>
       </c>
     </row>
@@ -3715,17 +3715,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>draft-noa-scitt-ai-agent-receipt — A SCITT Profile for AI-Agent Action Receipts</t>
+          <t>draft-munoz-scitt-permit-profile — A SCITT Profile for Pre-Execution AI Action Authorization Records</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>Defines a minimal SCITT profile: COSE_Sign1 Signed Statements with canonicalized payloads, hash-chained for ordering, registrable in SCITT Transparency Services. Explicitly does NOT assert agent correctness, safety, or real-world outcomes — only tamper-evident, signature-verifiable records of action, principal, policy identity, and verdict.</t>
+          <t>SCITT profile for the Pre-Execution Authorization Record (Permit), documenting policy-evaluated decisions before AI agent action dispatch with cryptographic binding proving 'authorized request equals dispatched request.' Composes with adjacent profiles for human-authority binding, post-execution evidence, and content-refusal events via referencing mechanisms.</t>
         </is>
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-noa-scitt-ai-agent-receipt/</t>
+          <t>https://datatracker.ietf.org/doc/draft-munoz-scitt-permit-profile/</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 23 Jun 2026; author: Tora Toraman (NordenSoft). The minimalist end of the SCITT profile spectrum; useful for corpus completeness alongside the more comprehensive draft-mih-scitt-agent-action-capsule.</t>
+          <t>Revision -00, 15 May 2026; author: Christian Munoz (Keel API). SCITT-anchored analog of the WIMSE evidence record; companion to draft-munoz-wimse-authorization-evidence from the same author. Connects to draft-sharif-agent-audit-trail and draft-kuehlewind-audit-architecture (both in corpus).</t>
         </is>
       </c>
     </row>
@@ -3745,17 +3745,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>draft-rampalli-scitt-capsule-provenance-binding — Binding Per-Action Authorization and Memory Provenance into Agent Action Capsules</t>
+          <t>draft-marques-asqav-compliance-receipts — Compliance Profile of Signed Action Receipts for AI Agents</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Specifies how to bind three components into AAC records: what was executed ('did'), whether it was authorized ('may'), and the source of the belief that motivated the action ('why-believed'); uses optional payload extensions carrying authorization token references, memory chain roots, and quarantine attestations without modifying AAC core protected-header claims.</t>
+          <t>Establishes a compliance framework for signed action receipts from AI agents, mandating specific fields, cryptographic anchoring, hash-chain linkage, risk/incident classification, cross-agent envelope binding, and enforcement attestation with retention floors tied to EU AI Act, DORA, NIST AI RMF, HIPAA, SEC Rule 17a-4, and CIRCIA.</t>
         </is>
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-rampalli-scitt-capsule-provenance-binding/</t>
+          <t>https://datatracker.ietf.org/doc/draft-marques-asqav-compliance-receipts/</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -3765,7 +3765,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 5 Jul 2026; author: Karthik Rampalli (Glyphzero, Inc.). Extends draft-mih-scitt-agent-action-capsule with memory provenance — the 'why-believed' component is novel among SCITT profiles. Includes a defensive publication notice waiving patent claims on the core binding technique.</t>
+          <t>Revision -06, 1 Jul 2026 (was -05 May 2026); author: João André Gomes Marques. The most legally grounded receipt profile in the wave — at revision 06, relatively mature. Complements draft-sharif-agent-audit-trail (corpus) with a multi-regulation compliance overlay.</t>
         </is>
       </c>
     </row>
@@ -3775,17 +3775,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>draft-nobuo-scitt-composite-evidence-verification — Composite Evidence Verification for SCITT Statement Graphs</t>
+          <t>draft-mih-scitt-agent-action-capsule — An Agent Action Capsule Profile for SCITT</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>Defines a composite verifier function for checking collections of SCITT Signed Statements, receipts, object bindings, and relationship edges under a named verification profile; provides structured reporting on validation status, missing evidence, outdated information, and conflicting claims — targeting auditors needing to evaluate multiple interconnected statements.</t>
+          <t>Defines a SCITT statement profile (Agent Action Capsule) documenting agent actions with outcome status (executed, blocked, denied, errored, timed out), evaluated constraints, committed-effect binding, and a human-in-the-loop flag; records a Capsule for every verdict including refusals. COSE Signed Statement format; registrable in SCITT Transparency Services.</t>
         </is>
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-nobuo-scitt-composite-evidence-verification/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mih-scitt-agent-action-capsule/</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 7 Jul 2026; author: Nobuo Aoki (SOKENDAI). Operates above individual SCITT profiles (AAC, permits, compliance receipts all in corpus) — the 'how do you verify all of them together' layer that draft-kuehlewind-audit-architecture implies but does not yet specify. Watch for Kühlewind/Birkholz pickup.</t>
+          <t>Revision -02, 6 Jul 2026 (was -01 Jun 2026); author: Steven Mih (Action State Group). -02 added an 'honest human-in-the-loop' flag distinguishing actual HITL from automated policy. Provides auditor-grade evidence that decision gates functioned; the HITL flag directly tracks the corpus theme.</t>
         </is>
       </c>
     </row>
@@ -3805,17 +3805,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-mjwt — The Mandate JWT (MJWT) for Agentic AI Systems</t>
+          <t>draft-mih-sato-agent-accountability-composition — Agent Accountability: Composition and Conformance</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Introduces the Mandate JWT — a WIMSE workload credential profile binding agent authority to specific Sovereign Object instances under named human principals, with cryptographically enforced delegation ceilings and a six-dimensional Narrowing Property preventing sub-agents from exceeding root authority.</t>
+          <t>Addresses how to answer accountability questions about cross-domain autonomous agent actions for auditors and regulators who do not trust the operator; defines a composition model assembling multiple independently verifiable artifacts (workload credentials, delegation tokens, action capsules, attestation results) into a single accountability record with a conformance evaluation framework.</t>
         </is>
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-mjwt/</t>
+          <t>https://datatracker.ietf.org/doc/draft-mih-sato-agent-accountability-composition/</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). The authorization token primitive for the SOOS governance protocol family. Directly comparable to draft-mcguinness-oauth-client-instance-assertion but uses a WIMSE/Sovereign Object substrate rather than OAuth.</t>
+          <t>Revision -00, Jul 2026; authors: Steven Mih (Action State Group) + Tom Sato (MyAuberge K.K.) — collaboration between the two principal authors of draft-mih-scitt-agent-action-capsule (corpus) and the SOOS governance suite (corpus). Operates above individual SCITT profiles; the accountability-composition layer the kuehlewind-audit-architecture HUB depends on but does not yet specify.</t>
         </is>
       </c>
     </row>
@@ -3835,17 +3835,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-mad — Multi-Agent Delegation in Sovereign Object Systems</t>
+          <t>draft-car-rer-artifact — RER Run Artifact Format: Hash-Chained, Signed Records of AI Inference Execution</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>Specifies three core mechanisms for multi-agent delegation accountability: the Narrowing Property (capability non-amplification), five formally defined object topology patterns for runtime relationships, and cluster coordination primitives for parallel execution with aggregation rules. Version 02 adds revocation-during-execution handling and partial-completion routing to human oversight.</t>
+          <t>Specifies a cryptographically signed JSON record for AI inference runs including a signed envelope declaring permissions and limits, a hash-chained event log covering all model and tool calls, and a runtime signature binding envelope and log to the producing implementation. Enables offline verification by parties uninvolved in the original run.</t>
         </is>
       </c>
       <c r="D98" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-mad/</t>
+          <t>https://datatracker.ietf.org/doc/draft-car-rer-artifact/</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). Claims to address gaps the OpenID Foundation identifies as unsolved in multi-agent authorization. The five topology patterns are a useful vocabulary for describing agent-to-agent relationship structures.</t>
+          <t>Revision -01, 12 Jun 2026; author: Kayla Cardillo (Tech Enrichment). Relevant for post-hoc audit of what permissions an agent claimed during execution; companion to the SCITT profiles but more focused on inference traceability than authorization decisions.</t>
         </is>
       </c>
     </row>
@@ -3865,17 +3865,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-hem — The Human Escalation Mechanism (HEM) for Agentic AI Systems</t>
+          <t>draft-noa-scitt-ai-agent-receipt — A SCITT Profile for AI-Agent Action Receipts</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Defines a kernel-enforced mechanism placing agent sessions in a pending state when human judgment is required, routing structured escalation requests to designated human decision-makers, and prohibiting all state transitions until a human decision is received. Defines five decision types and a dual-layer architecture (LLM-HEM and SOOS-HEM).</t>
+          <t>Defines a minimal SCITT profile: COSE_Sign1 Signed Statements with canonicalized payloads, hash-chained for ordering, registrable in SCITT Transparency Services. Explicitly does NOT assert agent correctness, safety, or real-world outcomes — only tamper-evident, signature-verifiable records of action, principal, policy identity, and verdict.</t>
         </is>
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-hem/</t>
+          <t>https://datatracker.ietf.org/doc/draft-noa-scitt-ai-agent-receipt/</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>Revision -05, 30 Jun 2026 (was -04 Jun 2026); author: Tom Sato (MyAuberge K.K.). The most normative HITL protocol in the current wave; explicitly aligns with EU AI Act Article 14 requirements for high-risk AI system oversight. Counterpart to ARAP (AuthZEN WG) at the protocol level vs. the OAuth/AuthZEN layer.</t>
+          <t>Revision -00, 23 Jun 2026; author: Tora Toraman (NordenSoft). The minimalist end of the SCITT profile spectrum; useful for corpus completeness alongside the more comprehensive draft-mih-scitt-agent-action-capsule.</t>
         </is>
       </c>
     </row>
@@ -3895,17 +3895,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-idp — The Intent Declaration Primitive (IDP) for Agentic AI Systems</t>
+          <t>draft-rampalli-scitt-capsule-provenance-binding — Binding Per-Action Authorization and Memory Provenance into Agent Action Capsules</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>Specifies a structured declaration mechanism committing AI agent intent to tamper-evident logs before actions are taken, enabling post-hoc review and EU AI Act Article 12 compliance for high-risk systems.</t>
+          <t>Specifies how to bind three components into AAC records: what was executed ('did'), whether it was authorized ('may'), and the source of the belief that motivated the action ('why-believed'); uses optional payload extensions carrying authorization token references, memory chain roots, and quarantine attestations without modifying AAC core protected-header claims.</t>
         </is>
       </c>
       <c r="D100" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-idp/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rampalli-scitt-capsule-provenance-binding/</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>Revision -05, 30 Jun 2026 (was -04 Jun 2026); author: Tom Sato (MyAuberge K.K.). The log-before-execute pattern mirrors draft-nelson-agent-delegation-receipts but operates at the intent declaration level rather than the user-authorization level. Pairs with GAR (below) to form a complete pre/post audit trail.</t>
+          <t>Revision -00, 5 Jul 2026; author: Karthik Rampalli (Glyphzero, Inc.). Extends draft-mih-scitt-agent-action-capsule with memory provenance — the 'why-believed' component is novel among SCITT profiles. Includes a defensive publication notice waiving patent claims on the core binding technique.</t>
         </is>
       </c>
     </row>
@@ -3925,17 +3925,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>draft-sato-soos-gar — The Governance Audit Record (GAR) for Agentic AI Systems</t>
+          <t>draft-rampalli-cross-org-delegation-mapping — A Layered Requirements Mapping for Cross-Organization Agent Delegation</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Defines GAR, an audit framework with five audit types, a Session Audit Record, and an Audit Alert mechanism; collects, signs, and makes governance events from IDP, HEM, and associated SOOS primitives available for regulatory inspection via an append-only, non-suppressible SCITT-anchored audit stream with Authority Lifecycle Events covering the complete revocation-recovery cycle.</t>
+          <t>Records a comparative mapping of two evidence layers for cross-organization AI agent delegation — per-hop delegation chains (PEDIGREE model) and named-human authorization roots (EMILIA Protocol binding and evidence-graph drafts) — evaluated against the nine requirements of draft-reece-wimse-cross-org-delegation under a multi-tier organizational architecture.</t>
         </is>
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sato-soos-gar/</t>
+          <t>https://datatracker.ietf.org/doc/draft-rampalli-cross-org-delegation-mapping/</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -3945,7 +3945,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>Revision -03, 28 Jun 2026 (was -02 Jun 10). -03 added OpenTelemetry attribute namespace for governance observability, a GAR Processor spec for converting OTel signals to audit records with integrity verification, four new Authority Lifecycle Event categories (policy conflict scenarios, statutory interpretation changes), and mandatory provenance fields for policy evaluation records. The integrator for the SOOS family, analogous to how draft-kuehlewind-audit-architecture integrates the broader IETF agent draft landscape.</t>
+          <t>Revision -05, Jul 2026; author: Karthik Rampalli (Glyphzero, Inc.) — same author as draft-rampalli-scitt-capsule-provenance-binding (corpus). Rev-05 signals active iteration; the mapping bridges two otherwise disconnected design families and is the first document to formally cross-reference EMILIA Protocol against WIMSE cross-org requirements.</t>
         </is>
       </c>
     </row>
@@ -3955,17 +3955,17 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>draft-jiang-intent-security — Security Considerations and Requirements for Intent-Based Requests in Agentic Systems</t>
+          <t>draft-nobuo-scitt-composite-evidence-verification — Composite Evidence Verification for SCITT Statement Graphs</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>Solution-agnostic threat analysis covering tampering, privilege escalation, constraint violations, and intent drift in intent-based agentic systems, with a reference model, attack scenarios, and security requirements covering authentication, admission control, constraint validation, and multi-hop integrity.</t>
+          <t>Defines a composite verifier function for checking collections of SCITT Signed Statements, receipts, object bindings, and relationship edges under a named verification profile; provides structured reporting on validation status, missing evidence, outdated information, and conflicting claims — targeting auditors needing to evaluate multiple interconnected statements.</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-jiang-intent-security/</t>
+          <t>https://datatracker.ietf.org/doc/draft-nobuo-scitt-composite-evidence-verification/</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>Revision -03, 22 Jun 2026; authors: Yuning Jiang, Lun Li, Yurong Song, Faye Liu (Huawei). The threat-model companion to draft-jiang-oauth-intent-admission from the same group; likely intended to inform the broader IETF agentic AI security discussion.</t>
+          <t>Revision -00, 7 Jul 2026; author: Nobuo Aoki (SOKENDAI). Operates above individual SCITT profiles (AAC, permits, compliance receipts all in corpus) — the 'how do you verify all of them together' layer that draft-kuehlewind-audit-architecture implies but does not yet specify. Watch for Kühlewind/Birkholz pickup.</t>
         </is>
       </c>
     </row>
@@ -3985,17 +3985,17 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>draft-li-dmsc-macp — Multi-agent Collaboration Protocol Suites Architecture</t>
+          <t>draft-schrock-ep-authorization-receipts — Authorization Receipts for High-Risk Agent Actions</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Defines a protocol suite and architectural framework for secure, scalable multi-agent collaboration covering trusted agent onboarding, capability-based discovery, distributed capability synchronization, and secure agent-to-agent interaction. Specifies a gateway-centric architecture where an Agent Gateway mediates capability negotiation and trust establishment between collaborating agents.</t>
+          <t>Defines the EMILIA Protocol (EP) authorization receipt — a COSE_Sign1 artifact that cryptographically binds a named human principal to a specific high-risk agent action before execution, providing auditors and counterparties a tamper-evident record that a real human authorized the consequential step.</t>
         </is>
       </c>
       <c r="D103" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-li-dmsc-macp/</t>
+          <t>https://datatracker.ietf.org/doc/draft-schrock-ep-authorization-receipts/</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
@@ -4005,7 +4005,7 @@
       </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
-          <t>Revision -05, 26 May 2026; active (expires Nov 2026); authors: Xueting Li (China Telecom), Bing Liu (Huawei), Jun Liu (Beijing U of Posts &amp; Telecom), Chenguang Du (Tsinghua), Lianhua Zhang (AsiaInfo). Replaces draft-li-dmsc-mcps-agw. Anchors a DMSC family of companion drafts covering intent-based interconnection, task protocol, gateway directory sync, semantic interaction, and gateway requirements. No explicit OAuth or WIMSE dependencies — operates at the agent coordination layer above transport, below authorization.</t>
+          <t>Revision -06, Jul 2026. The base artifact for the EMILIA Protocol family; companion drafts draft-schrock-ep-authorization-evidence-chain, draft-schrock-ep-action-evidence-graph, draft-schrock-ep-quorum, and draft-schrock-ep-evidence-record all build on or reference this receipt format. Rev-06 indicates active iteration. Draft-rampalli-cross-org-delegation-mapping (corpus) formally maps EMILIA Protocol receipts against the nine reece-wimse-cross-org-delegation requirements.</t>
         </is>
       </c>
     </row>
@@ -4015,17 +4015,17 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>draft-li-dmsc-inf-architecture — Dynamic Multi-agent Secured Collaboration Infrastructure Architecture</t>
+          <t>draft-schrock-ep-action-evidence-graph — Action Evidence Graphs and Evidence Policy Replay for High-Risk Agent Actions (EP-AEG)</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>Approaches DMSC from the network-infrastructure perspective: proposes capability-based forwarding and semantic routing at the network layer, where agent capability metadata influences packet-forwarding decisions rather than routing based solely on addresses. The most mature DMSC document at rev 07; predates and informs the MACP architecture draft.</t>
+          <t>Composes the full set of signed artifacts about an AI agent action — workload identity credentials, delegation tokens, transaction tokens, runtime attestation results, pre-execution policy permits, and EMILIA Protocol authorization receipts — into a single verifiable action evidence graph; defines evidence policy replay for auditing past actions against policy versions current at the time.</t>
         </is>
       </c>
       <c r="D104" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-li-dmsc-inf-architecture/</t>
+          <t>https://datatracker.ietf.org/doc/draft-schrock-ep-action-evidence-graph/</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -4035,7 +4035,7 @@
       </c>
       <c r="F104" s="5" t="inlineStr">
         <is>
-          <t>Revision -07, May 22 2026; authors: Xueting Li (China Telecom), Aijun Wang (China Telecom), Bing Liu (Huawei), Changwang Lin (New H3C). Infrastructure-layer complement to draft-li-dmsc-macp (protocol suite). The DMSC family now has 14+ companion drafts from Chinese telecom/academic groups — this is the architectural anchor.</t>
+          <t>Revision -00, Jul 2026. The graph composition layer above the individual SCITT profiles and receipts already in corpus; the 'single verifiable artifact' problem that draft-nobuo-scitt-composite-evidence-verification (corpus) approaches from the SCITT statement side. Together these two drafts define the evidence graph landscape.</t>
         </is>
       </c>
     </row>
@@ -4045,17 +4045,17 @@
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>draft-sz-dmsc-iaip — Intent-based Agent Interconnection Protocol at Agent Gateway</t>
+          <t>draft-schrock-ep-authorization-evidence-chain — Authorization Evidence Chains: Composing Heterogeneous Agent-Authorization Receipts (EP-AEC)</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Defines semantic capability advertisement and intent-driven routing at DMSC agent gateways: agents publish capability profiles in a structured format and the gateway matches incoming task intents to available agents, replacing fixed-address routing with dynamic semantic matching. The core routing-layer protocol for DMSC inter-agent communication.</t>
+          <t>Defines a mechanism for composing EMILIA Protocol authorization receipts from different systems and issuers into a single authorization evidence chain, enabling auditors to verify a heterogeneous chain of human approvals across organizational boundaries without requiring a common receipt format.</t>
         </is>
       </c>
       <c r="D105" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-sz-dmsc-iaip/</t>
+          <t>https://datatracker.ietf.org/doc/draft-schrock-ep-authorization-evidence-chain/</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -4065,7 +4065,7 @@
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, May 2026; authors: Sheng Sun, Xinyi Zhang (CAS/CNIC), Qiangzhou Gao (Huawei), Min Liu, Yuwei Wang (ICT, CAS). The intent-based routing mechanism that distinguishes DMSC from address-based protocols; relevant to the DAWN boundary question — DMSC embeds discovery in the gateway routing layer rather than treating it as a separate protocol.</t>
+          <t>Revision -02, Jul 2026. The cross-system interoperability layer for EMILIA Protocol receipts; directly addresses the scenario where draft-reece-wimse-cross-org-delegation (corpus) operates and authorization evidence must span administrative domains. Rev-02 indicates active development.</t>
         </is>
       </c>
     </row>
@@ -4075,17 +4075,17 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>draft-yang-dmsc-ioa-task-protocol — Internet of Agents Task Protocol for Heterogeneous Agent Collaboration</t>
+          <t>draft-schrock-ep-quorum — Multi-Party Quorum Authorization for High-Risk Agent Actions (EP-QUORUM)</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>Establishes a session and task coordination layer with finite-state-machine-based dialogue management, dynamic team assembly, and nested team hierarchies for distributed heterogeneous agent collaboration. Addresses the multi-agent task lifecycle from assignment through completion and audit across heterogeneous agent implementations.</t>
+          <t>Defines EP-QUORUM, a multi-party authorization profile for EMILIA Protocol authorization receipts; extends the base receipt (which binds one human to one action) to require a quorum of named human approvals before an action may proceed, with configurable thresholds, role requirements, and time-bounded approval windows.</t>
         </is>
       </c>
       <c r="D106" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-yang-dmsc-ioa-task-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-schrock-ep-quorum/</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -4095,7 +4095,7 @@
       </c>
       <c r="F106" s="5" t="inlineStr">
         <is>
-          <t>Revision -03, Apr 21 2026; authors: Cheng Yang (BUPT), Zhiyuan Liu (Tsinghua), Aijun Wang (China Telecom). The task-coordination layer above the DMSC gateway routing; covers multi-domain and 6G/ITS scenarios. Distinct from OAuth-layer delegation in that it orchestrates task state rather than token issuance.</t>
+          <t>Revision -02, Jul 2026. The enterprise governance complement to the base EP receipt; relevant for high-risk regulated workflows (financial transactions, medical orders, critical infrastructure changes) where single-human authorization is insufficient. Rev-02 indicates active iteration.</t>
         </is>
       </c>
     </row>
@@ -4105,17 +4105,17 @@
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>draft-dunbar-dmsc-gw-scenarios-gap-analysis — Deployment Scenarios and Gap Analysis for AI Agent Gateway</t>
+          <t>draft-schrock-ep-evidence-record — Long-Term, Crypto-Agile Preservation of Authorization Evidence (EP-EVIDENCE-RECORD)</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Surveys single-domain to multi-domain deployment scenarios for AI Agent Gateways and identifies concrete gaps where existing protocols (specifically MCP and Google's A2A) cannot satisfy governance, policy enforcement, and cross-organizational trust requirements — particularly in regulated financial services and telecom environments.</t>
+          <t>Defines a long-term, crypto-agile record format for preserving EMILIA Protocol authorization evidence under regulatory retention mandates; addresses algorithm deprecation over multi-year retention periods (DORA 5-year, HIPAA 6-year, SEC 17a-4 requirements) using a re-signing model that preserves evidentiary chain of custody.</t>
         </is>
       </c>
       <c r="D107" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-dunbar-dmsc-gw-scenarios-gap-analysis/</t>
+          <t>https://datatracker.ietf.org/doc/draft-schrock-ep-evidence-record/</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -4125,7 +4125,7 @@
       </c>
       <c r="F107" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, Jul 2 2026; authors: Linda Dunbar (Futurewei), YiFei Wang (China Telecom), Bing Liu (Huawei). The most directly useful DMSC document for the boundary analysis: explicitly names MCP and A2A as insufficient and articulates where the DMSC gateway fills the gap. The regulated-environment focus (financial services, telco) distinguishes DMSC's use-case target from OAuth-centric approaches.</t>
+          <t>Revision -01, Jul 2026. The regulatory compliance layer for EMILIA Protocol; directly connects to the kuehlewind-audit-architecture HUB (corpus) requirement for audit evidence that survives algorithm sunset. The DORA/HIPAA/SEC citation grounds the spec in concrete regulatory obligations.</t>
         </is>
       </c>
     </row>
@@ -4135,17 +4135,17 @@
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>draft-somoza-dmsc-atn-agent-trust-negotiation — Agent Trust Negotiation: Capability, Delegation, and Provenance Binding</t>
+          <t>draft-tsyrulnikov-rats-attested-inference-receipt — Attested Inference Receipt (AIR): A COSE/CWT Profile for Confidential AI Inference</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>Specifies the Agent Trust Negotiation (ATN) protocol, which binds four artifacts — capability manifests, delegation chains, provenance attestations, and session receipts — to agent identities via a handshake state machine producing mutually verified, scope-bounded sessions with SCITT-suitable audit records.</t>
+          <t>Defines the Attested Inference Receipt (AIR), a COSE_Sign1 envelope carrying CWT claims profiled per the Entity Attestation Token (EAT) framework; an AIR receipt cryptographically binds model identity, input/output hashes, TEE attestation evidence, and operational telemetry into a single signed artifact verifiable by parties not present at inference time.</t>
         </is>
       </c>
       <c r="D108" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-somoza-dmsc-atn-agent-trust-negotiation/</t>
+          <t>https://datatracker.ietf.org/doc/draft-tsyrulnikov-rats-attested-inference-receipt/</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -4155,7 +4155,7 @@
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 29 May 2026; author: Enrique Somoza (Independent). Operates above discovery mechanisms and positions itself between the discovery layer (DAWN, MCP) and the authorization layer (WIMSE, OAuth). Relevant as an agent-to-agent trust establishment handshake protocol.</t>
+          <t>Revision -02, Jul 2026. The RATS-layer complement to the SCITT profiles in corpus: where SCITT profiles (mih-scitt-agent-action-capsule, marques-asqav-compliance-receipts) record authorization and governance events, AIR records what the model actually computed — model identity, I/O content hashes, and TEE attestation linking the computation to trusted hardware. Together they address the full audit evidence stack.</t>
         </is>
       </c>
     </row>
@@ -4165,17 +4165,17 @@
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>draft-mcgraw-httpapi-agent-budget — The Delegation HTTP Authentication Scheme for Request-Bound Authority</t>
+          <t>draft-sato-soos-mjwt — The Mandate JWT (MJWT) for Agentic AI Systems</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Defines the 'Delegation' HTTP authentication scheme and response semantics for delegated-authority challenges using HTTP status codes and Problem Details, plus a CBOR/COSE proof format. The initial authority profile is 'Budget,' using post-quantum ML-DSA to prove spending or resource-consumption limits.</t>
+          <t>Introduces the Mandate JWT — a WIMSE workload credential profile binding agent authority to specific Sovereign Object instances under named human principals, with cryptographically enforced delegation ceilings and a six-dimensional Narrowing Property preventing sub-agents from exceeding root authority.</t>
         </is>
       </c>
       <c r="D109" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-mcgraw-httpapi-agent-budget/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-mjwt/</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="F109" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, 15 Jun 2026; author: John Paul McGraw Jr. (TaskHawk Systems). HTTP-layer bounded delegation with post-quantum crypto; distinct from OAuth-layer delegation in that the authority proof travels in the Authorization header. Complements x401 (Industry tab) at the HTTP challenge-response layer.</t>
+          <t>Revision -01, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). The authorization token primitive for the SOOS governance protocol family. Directly comparable to draft-mcguinness-oauth-client-instance-assertion but uses a WIMSE/Sovereign Object substrate rather than OAuth.</t>
         </is>
       </c>
     </row>
@@ -4195,17 +4195,17 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>draft-vauban-x402-delegation-binding — x402 Delegation Binding for Agentic HTTP Pipelines</t>
+          <t>draft-sato-soos-mad — Multi-Agent Delegation in Sovereign Object Systems</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>Addresses the security gap where x402 V2 payment grants issued to one agent could be misused by another in the same pipeline, introducing three binding mechanisms: a JCS-derived agent identity pseudonym, a nonce for anti-replay, and a depth-limiting field for transitive delegation.</t>
+          <t>Specifies three core mechanisms for multi-agent delegation accountability: the Narrowing Property (capability non-amplification), five formally defined object topology patterns for runtime relationships, and cluster coordination primitives for parallel execution with aggregation rules. Version 02 adds revocation-during-execution handling and partial-completion routing to human oversight.</t>
         </is>
       </c>
       <c r="D110" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-vauban-x402-delegation-binding/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-mad/</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">
@@ -4215,7 +4215,7 @@
       </c>
       <c r="F110" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 25 May 2026; author: Vauban Research. Narrowly scoped to payment pipelines but the delegation-binding pattern (pseudonymous identity + anti-replay + depth-limit) is applicable broadly. Validated across five language runtimes with A2A and MCP integration guidance.</t>
+          <t>Revision -02, 10 Jun 2026; author: Tom Sato (MyAuberge K.K.). Claims to address gaps the OpenID Foundation identifies as unsolved in multi-agent authorization. The five topology patterns are a useful vocabulary for describing agent-to-agent relationship structures.</t>
         </is>
       </c>
     </row>
@@ -4225,17 +4225,17 @@
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>draft-samal-vap — Verifiable Agent Protocol (VAP): Intent-Bound Admission Control and Audit for Agent Tool Invocation</t>
+          <t>draft-sato-soos-hem — The Human Escalation Mechanism (HEM) for Agentic AI Systems</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Specifies VAP as a defense-in-depth layer adding declarations of purpose and session budget commitments to tool invocation requests (targeting MCP-style protocols), enabling servers to perform admission control before execution via four messages carried in existing protocol metadata.</t>
+          <t>Defines a kernel-enforced mechanism placing agent sessions in a pending state when human judgment is required, routing structured escalation requests to designated human decision-makers, and prohibiting all state transitions until a human decision is received. Defines five decision types and a dual-layer architecture (LLM-HEM and SOOS-HEM).</t>
         </is>
       </c>
       <c r="D111" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-samal-vap/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-hem/</t>
         </is>
       </c>
       <c r="E111" s="5" t="inlineStr">
@@ -4245,7 +4245,7 @@
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 3 Jun 2026; author: Kruttidipta Samal (Independent). Lightweight and protocol-agnostic; addresses erroneous agent behavior, cost control, and audit trails without replacing existing auth mechanisms. Practical tool-invocation-level authorization layer for MCP deployments.</t>
+          <t>Revision -05, 30 Jun 2026 (was -04 Jun 2026); author: Tom Sato (MyAuberge K.K.). The most normative HITL protocol in the current wave; explicitly aligns with EU AI Act Article 14 requirements for high-risk AI system oversight. Counterpart to ARAP (AuthZEN WG) at the protocol level vs. the OAuth/AuthZEN layer.</t>
         </is>
       </c>
     </row>
@@ -4255,17 +4255,17 @@
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>draft-khera-aurora — Agent Unification, Runtime, and Operational Responsibility Attestation (AURORA)</t>
+          <t>draft-sato-soos-idp — The Intent Declaration Primitive (IDP) for Agentic AI Systems</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
-          <t>A two-layer framework unifying hardware-enclave-backed Runtime Integrity Attestation with scoped, cryptographically bound Authority Delegation; enables agents to prove both operational authority and runtime integrity simultaneously.</t>
+          <t>Specifies a structured declaration mechanism committing AI agent intent to tamper-evident logs before actions are taken, enabling post-hoc review and EU AI Act Article 12 compliance for high-risk systems.</t>
         </is>
       </c>
       <c r="D112" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-khera-aurora/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-idp/</t>
         </is>
       </c>
       <c r="E112" s="5" t="inlineStr">
@@ -4275,7 +4275,7 @@
       </c>
       <c r="F112" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 5 Jun 2026; author: Ankur Khera. Addresses the gap where delegation tokens don't prove the runtime environment is trustworthy — relevant where delegation must be paired with platform attestation (enterprise/regulated deployments). Bridges the RATS attestation thread and the OAuth delegation thread.</t>
+          <t>Revision -05, 30 Jun 2026 (was -04 Jun 2026); author: Tom Sato (MyAuberge K.K.). The log-before-execute pattern mirrors draft-nelson-agent-delegation-receipts but operates at the intent declaration level rather than the user-authorization level. Pairs with GAR (below) to form a complete pre/post audit trail.</t>
         </is>
       </c>
     </row>
@@ -4285,17 +4285,17 @@
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>draft-borthwick-msebenzi-environment-state — Verifiable Intent — environment.* Constraint Family</t>
+          <t>draft-sato-soos-gar — The Governance Audit Record (GAR) for Agentic AI Systems</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Defines the environment.* constraint family for agent-authorization mandate vocabularies, covering external conditions at transaction execution time (venue availability, wallet funding) that existing transactional constraints cannot address. Extends agent authorization mandate frameworks with environmental precondition checking.</t>
+          <t>Defines GAR, an audit framework with five audit types, a Session Audit Record, and an Audit Alert mechanism; collects, signs, and makes governance events from IDP, HEM, and associated SOOS primitives available for regulatory inspection via an append-only, non-suppressible SCITT-anchored audit stream with Authority Lifecycle Events covering the complete revocation-recovery cycle.</t>
         </is>
       </c>
       <c r="D113" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-borthwick-msebenzi-environment-state/</t>
+          <t>https://datatracker.ietf.org/doc/draft-sato-soos-gar/</t>
         </is>
       </c>
       <c r="E113" s="5" t="inlineStr">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="F113" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 13 Jun 2026; authors: Douglas Cameron Borthwick (InsumerAPI), Michael Msebenzi (Headless Oracle). Narrow but practically important for financial and commerce agent workflows; connects to draft-mcgraw-httpapi-agent-budget and draft-vauban-x402-delegation-binding.</t>
+          <t>Revision -03, 28 Jun 2026 (was -02 Jun 10). -03 added OpenTelemetry attribute namespace for governance observability, a GAR Processor spec for converting OTel signals to audit records with integrity verification, four new Authority Lifecycle Event categories (policy conflict scenarios, statutory interpretation changes), and mandatory provenance fields for policy evaluation records. The integrator for the SOOS family, analogous to how draft-kuehlewind-audit-architecture integrates the broader IETF agent draft landscape.</t>
         </is>
       </c>
     </row>
@@ -4315,17 +4315,17 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>draft-chen-oauth-agent-authz-use-cases — Agent Authorization Use Cases and Gap Analysis for OAuth 2.0</t>
+          <t>draft-jiang-intent-security — Security Considerations and Requirements for Intent-Based Requests in Agentic Systems</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>A framework-level analysis enumerating agentic authorization use cases — delegated task execution, multi-agent coordination, long-running workflows, capability attenuation — and mapping each against current OAuth 2.0 mechanisms to identify gaps that require new extensions or profiles.</t>
+          <t>Solution-agnostic threat analysis covering tampering, privilege escalation, constraint violations, and intent drift in intent-based agentic systems, with a reference model, attack scenarios, and security requirements covering authentication, admission control, constraint validation, and multi-hop integrity.</t>
         </is>
       </c>
       <c r="D114" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-chen-oauth-agent-authz-use-cases/</t>
+          <t>https://datatracker.ietf.org/doc/draft-jiang-intent-security/</t>
         </is>
       </c>
       <c r="E114" s="5" t="inlineStr">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="F114" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 5 Jul 2026; useful problem-statement companion to the OAuth recharter's 'Complex Delegation' milestone. Gap analysis directly motivates several other drafts in this corpus — a natural reference document for the OAuth WG scoping discussion.</t>
+          <t>Revision -03, 22 Jun 2026; authors: Yuning Jiang, Lun Li, Yurong Song, Faye Liu (Huawei). The threat-model companion to draft-jiang-oauth-intent-admission from the same group; likely intended to inform the broader IETF agentic AI security discussion.</t>
         </is>
       </c>
     </row>
@@ -4345,17 +4345,17 @@
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>draft-agnihotri-oauth-agent-impl-status — Implementation Status of OAuth Identity Chaining and Transaction Tokens</t>
+          <t>draft-haberkamp-ipp — Intent Provenance Protocol (IPP)</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>An RFC 7942–compliant implementation status report tracking open-source implementations of draft-ietf-oauth-identity-chaining and draft-ietf-oauth-transaction-tokens against the relevant spec requirements.</t>
+          <t>Specifies a cryptographic infrastructure standard for carrying verified human intent through chains of autonomous AI agent actions; defines the Intent Token, a signed, bounded, and tamper-evident data structure that travels with every agentic action so downstream agents and resource servers can verify that the chain traces to a real human authorization.</t>
         </is>
       </c>
       <c r="D115" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-agnihotri-oauth-agent-impl-status/</t>
+          <t>https://datatracker.ietf.org/doc/draft-haberkamp-ipp/</t>
         </is>
       </c>
       <c r="E115" s="5" t="inlineStr">
@@ -4365,7 +4365,7 @@
       </c>
       <c r="F115" s="5" t="inlineStr">
         <is>
-          <t>Revision -02, Jun 2026; provides the implementation evidence required to advance both WG drafts toward IESG submission. Informational companion to the two WG drafts — not a protocol spec but tracking their standardization progress.</t>
+          <t>Revision -01, Jul 2026. Addresses the 'intent drift' threat class from draft-jiang-intent-security (corpus) with a concrete token artifact; complements the EMILIA Protocol receipts (authorization at the action level) with an intent record at the delegation chain level. The traveling Intent Token model is distinct from both SOOS Mandate JWTs (Sato, governance substrate) and McGuinness Actor Profiles (delegation chain encoding in existing OAuth tokens).</t>
         </is>
       </c>
     </row>
@@ -4375,17 +4375,17 @@
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>draft-hardt-oauth-aauth-protocol — AAuth Protocol</t>
+          <t>draft-li-dmsc-macp — Multi-agent Collaboration Protocol Suites Architecture</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>A new clean-sheet authorization protocol from Dick Hardt (original OAuth author) defining proof-of-possession by default, resource-signed challenges, agent identity without pre-registration, deferred 202 responses, and AS-to-AS federation for the agent ecosystem.</t>
+          <t>Defines a protocol suite and architectural framework for secure, scalable multi-agent collaboration covering trusted agent onboarding, capability-based discovery, distributed capability synchronization, and secure agent-to-agent interaction. Specifies a gateway-centric architecture where an Agent Gateway mediates capability negotiation and trust establishment between collaborating agents.</t>
         </is>
       </c>
       <c r="D116" s="9" t="inlineStr">
         <is>
-          <t>https://datatracker.ietf.org/doc/draft-hardt-oauth-aauth-protocol/</t>
+          <t>https://datatracker.ietf.org/doc/draft-li-dmsc-macp/</t>
         </is>
       </c>
       <c r="E116" s="5" t="inlineStr">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="F116" s="5" t="inlineStr">
         <is>
-          <t>Revision -09, Jul 4 2026; slug gained 'oauth' infix at this revision (was draft-hardt-aauth-protocol). Now formally adds four resource access modes including agent governance. The design rationale section explicitly explains why AAuth is not GNAP, not OAuth, not DPoP and not mTLS — important read for anyone planning a new agent-auth stack. OUTLIER: zero OAuth dependencies.</t>
+          <t>Revision -05, 26 May 2026; active (expires Nov 2026); authors: Xueting Li (China Telecom), Bing Liu (Huawei), Jun Liu (Beijing U of Posts &amp; Telecom), Chenguang Du (Tsinghua), Lianhua Zhang (AsiaInfo). Replaces draft-li-dmsc-mcps-agw. Anchors a DMSC family of companion drafts covering intent-based interconnection, task protocol, gateway directory sync, semantic interaction, and gateway requirements. No explicit OAuth or WIMSE dependencies — operates at the agent coordination layer above transport, below authorization.</t>
         </is>
       </c>
     </row>
@@ -4405,17 +4405,17 @@
       </c>
       <c r="B117" s="5" t="inlineStr">
         <is>
-          <t>draft-chen-oauth-roadmap — Comprehensive Roadmap for OAuth 2.0 Standards and Drafts</t>
+          <t>draft-li-dmsc-inf-architecture — Dynamic Multi-agent Secured Collaboration Infrastructure Architecture</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>An IETF informational draft that maps the entire OAuth 2.0 ecosystem of RFCs, BCPs, and active drafts into functional layers from core to extensions to industry profiles.</t>
+          <t>Approaches DMSC from the network-infrastructure perspective: proposes capability-based forwarding and semantic routing at the network layer, where agent capability metadata influences packet-forwarding decisions rather than routing based solely on addresses. The most mature DMSC document at rev 07; predates and informs the MACP architecture draft.</t>
         </is>
       </c>
       <c r="D117" s="9" t="inlineStr">
         <is>
-          <t>https://www.ietf.org/archive/id/draft-chen-oauth-roadmap-00.html</t>
+          <t>https://datatracker.ietf.org/doc/draft-li-dmsc-inf-architecture/</t>
         </is>
       </c>
       <c r="E117" s="5" t="inlineStr">
@@ -4425,7 +4425,7 @@
       </c>
       <c r="F117" s="5" t="inlineStr">
         <is>
-          <t>Brand-new -00 draft (May 2026); the single most useful index when starting work in this area.</t>
+          <t>Revision -07, May 22 2026; authors: Xueting Li (China Telecom), Aijun Wang (China Telecom), Bing Liu (Huawei), Changwang Lin (New H3C). Infrastructure-layer complement to draft-li-dmsc-macp (protocol suite). The DMSC family now has 14+ companion drafts from Chinese telecom/academic groups — this is the architectural anchor.</t>
         </is>
       </c>
     </row>
@@ -4435,25 +4435,445 @@
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
+          <t>draft-sz-dmsc-iaip — Intent-based Agent Interconnection Protocol at Agent Gateway</t>
+        </is>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>Defines semantic capability advertisement and intent-driven routing at DMSC agent gateways: agents publish capability profiles in a structured format and the gateway matches incoming task intents to available agents, replacing fixed-address routing with dynamic semantic matching. The core routing-layer protocol for DMSC inter-agent communication.</t>
+        </is>
+      </c>
+      <c r="D118" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-sz-dmsc-iaip/</t>
+        </is>
+      </c>
+      <c r="E118" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F118" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, May 2026; authors: Sheng Sun, Xinyi Zhang (CAS/CNIC), Qiangzhou Gao (Huawei), Min Liu, Yuwei Wang (ICT, CAS). The intent-based routing mechanism that distinguishes DMSC from address-based protocols; relevant to the DAWN boundary question — DMSC embeds discovery in the gateway routing layer rather than treating it as a separate protocol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>draft-yang-dmsc-ioa-task-protocol — Internet of Agents Task Protocol for Heterogeneous Agent Collaboration</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>Establishes a session and task coordination layer with finite-state-machine-based dialogue management, dynamic team assembly, and nested team hierarchies for distributed heterogeneous agent collaboration. Addresses the multi-agent task lifecycle from assignment through completion and audit across heterogeneous agent implementations.</t>
+        </is>
+      </c>
+      <c r="D119" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-yang-dmsc-ioa-task-protocol/</t>
+        </is>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F119" s="5" t="inlineStr">
+        <is>
+          <t>Revision -03, Apr 21 2026; authors: Cheng Yang (BUPT), Zhiyuan Liu (Tsinghua), Aijun Wang (China Telecom). The task-coordination layer above the DMSC gateway routing; covers multi-domain and 6G/ITS scenarios. Distinct from OAuth-layer delegation in that it orchestrates task state rather than token issuance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="5" t="inlineStr">
+        <is>
+          <t>draft-dunbar-dmsc-gw-scenarios-gap-analysis — Deployment Scenarios and Gap Analysis for AI Agent Gateway</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>Surveys single-domain to multi-domain deployment scenarios for AI Agent Gateways and identifies concrete gaps where existing protocols (specifically MCP and Google's A2A) cannot satisfy governance, policy enforcement, and cross-organizational trust requirements — particularly in regulated financial services and telecom environments.</t>
+        </is>
+      </c>
+      <c r="D120" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-dunbar-dmsc-gw-scenarios-gap-analysis/</t>
+        </is>
+      </c>
+      <c r="E120" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F120" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, Jul 2 2026; authors: Linda Dunbar (Futurewei), YiFei Wang (China Telecom), Bing Liu (Huawei). The most directly useful DMSC document for the boundary analysis: explicitly names MCP and A2A as insufficient and articulates where the DMSC gateway fills the gap. The regulated-environment focus (financial services, telco) distinguishes DMSC's use-case target from OAuth-centric approaches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>draft-somoza-dmsc-atn-agent-trust-negotiation — Agent Trust Negotiation: Capability, Delegation, and Provenance Binding</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>Specifies the Agent Trust Negotiation (ATN) protocol, which binds four artifacts — capability manifests, delegation chains, provenance attestations, and session receipts — to agent identities via a handshake state machine producing mutually verified, scope-bounded sessions with SCITT-suitable audit records.</t>
+        </is>
+      </c>
+      <c r="D121" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-somoza-dmsc-atn-agent-trust-negotiation/</t>
+        </is>
+      </c>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F121" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 29 May 2026; author: Enrique Somoza (Independent). Operates above discovery mechanisms and positions itself between the discovery layer (DAWN, MCP) and the authorization layer (WIMSE, OAuth). Relevant as an agent-to-agent trust establishment handshake protocol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="5" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="5" t="inlineStr">
+        <is>
+          <t>draft-mcgraw-httpapi-agent-budget — The Delegation HTTP Authentication Scheme for Request-Bound Authority</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>Defines the 'Delegation' HTTP authentication scheme and response semantics for delegated-authority challenges using HTTP status codes and Problem Details, plus a CBOR/COSE proof format. The initial authority profile is 'Budget,' using post-quantum ML-DSA to prove spending or resource-consumption limits.</t>
+        </is>
+      </c>
+      <c r="D122" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-mcgraw-httpapi-agent-budget/</t>
+        </is>
+      </c>
+      <c r="E122" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F122" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, 15 Jun 2026; author: John Paul McGraw Jr. (TaskHawk Systems). HTTP-layer bounded delegation with post-quantum crypto; distinct from OAuth-layer delegation in that the authority proof travels in the Authorization header. Complements x401 (Industry tab) at the HTTP challenge-response layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>draft-vauban-x402-delegation-binding — x402 Delegation Binding for Agentic HTTP Pipelines</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>Addresses the security gap where x402 V2 payment grants issued to one agent could be misused by another in the same pipeline, introducing three binding mechanisms: a JCS-derived agent identity pseudonym, a nonce for anti-replay, and a depth-limiting field for transitive delegation.</t>
+        </is>
+      </c>
+      <c r="D123" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-vauban-x402-delegation-binding/</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 25 May 2026; author: Vauban Research. Narrowly scoped to payment pipelines but the delegation-binding pattern (pseudonymous identity + anti-replay + depth-limit) is applicable broadly. Validated across five language runtimes with A2A and MCP integration guidance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>draft-samal-vap — Verifiable Agent Protocol (VAP): Intent-Bound Admission Control and Audit for Agent Tool Invocation</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>Specifies VAP as a defense-in-depth layer adding declarations of purpose and session budget commitments to tool invocation requests (targeting MCP-style protocols), enabling servers to perform admission control before execution via four messages carried in existing protocol metadata.</t>
+        </is>
+      </c>
+      <c r="D124" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-samal-vap/</t>
+        </is>
+      </c>
+      <c r="E124" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F124" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 3 Jun 2026; author: Kruttidipta Samal (Independent). Lightweight and protocol-agnostic; addresses erroneous agent behavior, cost control, and audit trails without replacing existing auth mechanisms. Practical tool-invocation-level authorization layer for MCP deployments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>draft-khera-aurora — Agent Unification, Runtime, and Operational Responsibility Attestation (AURORA)</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>A two-layer framework unifying hardware-enclave-backed Runtime Integrity Attestation with scoped, cryptographically bound Authority Delegation; enables agents to prove both operational authority and runtime integrity simultaneously.</t>
+        </is>
+      </c>
+      <c r="D125" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-khera-aurora/</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>Revision -00, 5 Jun 2026; author: Ankur Khera. Addresses the gap where delegation tokens don't prove the runtime environment is trustworthy — relevant where delegation must be paired with platform attestation (enterprise/regulated deployments). Bridges the RATS attestation thread and the OAuth delegation thread.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="5" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>draft-borthwick-msebenzi-environment-state — Verifiable Intent — environment.* Constraint Family</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>Defines the environment.* constraint family for agent-authorization mandate vocabularies, covering external conditions at transaction execution time (venue availability, wallet funding) that existing transactional constraints cannot address. Extends agent authorization mandate frameworks with environmental precondition checking.</t>
+        </is>
+      </c>
+      <c r="D126" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-borthwick-msebenzi-environment-state/</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F126" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 13 Jun 2026; authors: Douglas Cameron Borthwick (InsumerAPI), Michael Msebenzi (Headless Oracle). Narrow but practically important for financial and commerce agent workflows; connects to draft-mcgraw-httpapi-agent-budget and draft-vauban-x402-delegation-binding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>draft-chen-oauth-agent-authz-use-cases — Agent Authorization Use Cases and Gap Analysis for OAuth 2.0</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>A framework-level analysis enumerating agentic authorization use cases — delegated task execution, multi-agent coordination, long-running workflows, capability attenuation — and mapping each against current OAuth 2.0 mechanisms to identify gaps that require new extensions or profiles.</t>
+        </is>
+      </c>
+      <c r="D127" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-chen-oauth-agent-authz-use-cases/</t>
+        </is>
+      </c>
+      <c r="E127" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F127" s="5" t="inlineStr">
+        <is>
+          <t>Revision -01, 5 Jul 2026; useful problem-statement companion to the OAuth recharter's 'Complex Delegation' milestone. Gap analysis directly motivates several other drafts in this corpus — a natural reference document for the OAuth WG scoping discussion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="5" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="5" t="inlineStr">
+        <is>
+          <t>draft-agnihotri-oauth-agent-impl-status — Implementation Status of OAuth Identity Chaining and Transaction Tokens</t>
+        </is>
+      </c>
+      <c r="C128" s="5" t="inlineStr">
+        <is>
+          <t>An RFC 7942–compliant implementation status report tracking open-source implementations of draft-ietf-oauth-identity-chaining and draft-ietf-oauth-transaction-tokens against the relevant spec requirements.</t>
+        </is>
+      </c>
+      <c r="D128" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-agnihotri-oauth-agent-impl-status/</t>
+        </is>
+      </c>
+      <c r="E128" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F128" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, Jun 2026; provides the implementation evidence required to advance both WG drafts toward IESG submission. Informational companion to the two WG drafts — not a protocol spec but tracking their standardization progress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>draft-hardt-oauth-aauth-protocol — AAuth Protocol</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>A new clean-sheet authorization protocol from Dick Hardt (original OAuth author) defining proof-of-possession by default, resource-signed challenges, agent identity without pre-registration, deferred 202 responses, and AS-to-AS federation for the agent ecosystem.</t>
+        </is>
+      </c>
+      <c r="D129" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-hardt-oauth-aauth-protocol/</t>
+        </is>
+      </c>
+      <c r="E129" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F129" s="5" t="inlineStr">
+        <is>
+          <t>Revision -09, Jul 4 2026; slug gained 'oauth' infix at this revision (was draft-hardt-aauth-protocol). Now formally adds four resource access modes including agent governance. The design rationale section explicitly explains why AAuth is not GNAP, not OAuth, not DPoP and not mTLS — important read for anyone planning a new agent-auth stack. OUTLIER: zero OAuth dependencies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="5" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>draft-chen-oauth-roadmap — Comprehensive Roadmap for OAuth 2.0 Standards and Drafts</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>An IETF informational draft that maps the entire OAuth 2.0 ecosystem of RFCs, BCPs, and active drafts into functional layers from core to extensions to industry profiles.</t>
+        </is>
+      </c>
+      <c r="D130" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ietf.org/archive/id/draft-chen-oauth-roadmap-00.html</t>
+        </is>
+      </c>
+      <c r="E130" s="5" t="inlineStr">
+        <is>
+          <t>IETF (individual)</t>
+        </is>
+      </c>
+      <c r="F130" s="5" t="inlineStr">
+        <is>
+          <t>Brand-new -00 draft (May 2026); the single most useful index when starting work in this area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>draft-ietf-wimse-workload-creds — WIMSE Workload Credentials</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>Defines the credential format and issuance profile for workload credentials in the WIMSE architecture, covering service-to-service authentication token types, local issuance mechanisms, and token exchange profiles for cross-trust-domain workload identity scenarios.</t>
+        </is>
+      </c>
+      <c r="D131" s="9" t="inlineStr">
+        <is>
+          <t>https://datatracker.ietf.org/doc/draft-ietf-wimse-workload-creds/</t>
+        </is>
+      </c>
+      <c r="E131" s="5" t="inlineStr">
+        <is>
+          <t>IETF (WIMSE WG)</t>
+        </is>
+      </c>
+      <c r="F131" s="5" t="inlineStr">
+        <is>
+          <t>Revision -02, Jul 2026; WIMSE WG-adopted. The credential issuance companion to draft-ietf-wimse-arch (architecture) and draft-ietf-wimse-identifier (identifiers) already in corpus. Three WG drafts now cover the full WIMSE stack: arch → identifier → workload-creds. Relevant to the WIMSE agent extension family (ni-wimse, reece, jiang, schwenkschuster) which assumes a credential format this draft now specifies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="5" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="5" t="inlineStr">
+        <is>
           <t>Charter: WIMSE — Workload Identity in Multi-System Environments (charter-ietf-wimse-01)</t>
         </is>
       </c>
-      <c r="C118" s="5" t="inlineStr">
+      <c r="C132" s="5" t="inlineStr">
         <is>
           <t>The formal IETF charter for the WIMSE WG covering architecture, JOSE-based WIMSE tokens for service-to-service traffic, local token issuance, and token exchange profiles (likely based on RFC 8693) for cross-trust-domain workload identity.</t>
         </is>
       </c>
-      <c r="D118" s="9" t="inlineStr">
+      <c r="D132" s="9" t="inlineStr">
         <is>
           <t>https://datatracker.ietf.org/doc/charter-ietf-wimse/01/</t>
         </is>
       </c>
-      <c r="E118" s="5" t="inlineStr">
+      <c r="E132" s="5" t="inlineStr">
         <is>
           <t>IETF (WIMSE WG charter)</t>
         </is>
       </c>
-      <c r="F118" s="5" t="inlineStr">
+      <c r="F132" s="5" t="inlineStr">
         <is>
           <t>Approved 18 March 2026 (v01); explicitly liaises with OAuth, SCIM, SCITT, RATS, the OpenID Foundation, and CNCF/SPIFFE — the formal scope statement that anchors all WIMSE draft work.</t>
         </is>
@@ -4578,6 +4998,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId116"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D132" r:id="rId131"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>